<commit_message>
Update headlines archive — 2026-03-24
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D61"/>
+  <dimension ref="A1:D121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1790,8 +1790,1328 @@
         </is>
       </c>
     </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Kemenpar Ungkap 4,2 Juta Warga DKI Tak Mudik, Harap Bisa Liburan di Jakarta</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8414069/kemenpar-ungkap-4-2-juta-warga-dki-tak-mudik-harap-bisa-liburan-di-jakarta</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Viral Pasutri Lebaran di Kampungnya Masing-masing untuk Hindari Ribut</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/bali/berita/d-8414053/viral-pasutri-lebaran-di-kampungnya-masing-masing-untuk-hindari-ribut</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Video Kereta Api Tambahan Lebaran Masih Beroperasi Sampai 1 April 2026</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260324-260324119/video-kereta-api-tambahan-lebaran-masih-beroperasi-sampai-1-april-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Mudik Rudy Jadi Lebih Tenang, Motor Aman Dititip di Polsek Setu</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8413681/mudik-rudy-jadi-lebih-tenang-motor-aman-dititip-di-polsek-setu</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Video Klopp Bantah Rumor Latih Real Madrid: Semua Itu Omong Kosong!</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/detiktv/d-8414095/video-klopp-bantah-rumor-latih-real-madrid-semua-itu-omong-kosong</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Ngeri! Satu Lagi Bukti Ultra Processed Food Bisa 'Membunuh' Secara Perlahan</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8413778/ngeri-satu-lagi-bukti-ultra-processed-food-bisa-membunuh-secara-perlahan</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Timur Tengah Konflik, Pesawat-Pesawat Parkir di Bandara Terpencil Ini</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.detik.com/travel-news/d-8413598/timur-tengah-konflik-pesawat-pesawat-parkir-di-bandara-terpencil-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Viral SPBU di Atas Gedung Bikin Penasaran, Begini Penjelasan Pertamina</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8413584/viral-spbu-di-atas-gedung-bikin-penasaran-begini-penjelasan-pertamina</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Rencana Besar Prabowo Genjot Ekonomi RI Tembus 8% Pakai 'Mesin' Ini</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8413416/rencana-besar-prabowo-genjot-ekonomi-ri-tembus-8-pakai-mesin-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Rudal Iran Hantam Kota Dekat Tel Aviv Israel, 12 Orang Terluka</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8414100/rudal-iran-hantam-kota-dekat-tel-aviv-israel-12-orang-terluka</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Ledakan Terdengar di Beirut Lebanon, Sebabkan Kepanikan</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8414097/ledakan-terdengar-di-beirut-lebanon-sebabkan-kepanikan</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Filipina Deklarasi Darurat Energi Buntut Perang AS-Israel dan Iran</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8414037/filipina-deklarasi-darurat-energi-buntut-perang-as-israel-dan-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Pemerintah Pastikan Sekolah Tetap Tatap Muka di Tengah Krisis Global</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8414030/pemerintah-pastikan-sekolah-tetap-tatap-muka-di-tengah-krisis-global</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Video: Mo Salah Angkat Kaki dari Liverpool Akhir Musim Ini!</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260325-260325006/video-mo-salah-angkat-kaki-dari-liverpool-akhir-musim-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>5 Fakta Pengemudi Fortuner di PIK Tabrak 4 Motor hingga 2 Orang Tewas</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8414048/5-fakta-pengemudi-fortuner-di-pik-tabrak-4-motor-hingga-2-orang-tewas</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>Reaksi Warga Tel Aviv Melihat Permukiman Luluh Lantak Dihantam Rudal Iran</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1919115/reaksi-warga-tel-aviv-melihat-permukiman-luluh-lantak-dihantam-rudal-iran?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>Tindak Pidana Anak Meningkat: PR Besar Sistem Peradilan Anak</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/tindak-pidana-anak-meningkat-pr-besar-sistem-peradilan-anak?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>Komdigi Siagakan 500 Posko, Pastikan Layanan Telekomunikasi dan Internet Tetap Lancar</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/24/21015761/komdigi-siagakan-500-posko-pastikan-layanan-telekomunikasi-dan-internet</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>Infrastruktur Jalan Prima Selama Lebaran 2026, Pemprov Jateng Tuai Apresiasi Pemudik</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/03/24/202859178/infrastruktur-jalan-prima-selama-lebaran-2026-pemprov-jateng-tuai-apresiasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>Cara Satgas PRR Pastikan Bantuan Hunian bagi Penyintas Bencana Tepat Guna dan Tepat Sasaran</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/24/20135341/cara-satgas-prr-pastikan-bantuan-hunian-bagi-penyintas-bencana-tepat-guna</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>Dampak Perang Iran Disebut Lebih Parah dari Tiga Krisis Minyak Dunia dalam Sejarah</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1919090/dampak-perang-iran-disebut-lebih-parah-dari-tiga-krisis-minyak-dunia-dalam-sejarah?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Titik Nol Jogja Setelah Tanpa Bus-Bus Besar</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/agustinapurwantini/69c0a68b34777c0632086ab3/titik-nol-jogja-setelah-tanpa-bus-besar-besar</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Terlihat Sopan, Tapi Salah? Ini Bedanya Enryo dan Hairyo di Kantor Jepang</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5694/terlihat-sopan-tapi-salah-ini-bedanya-enryo-dan-hairyo-di-kantor-jepang</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Potret Bus PO Haryanto dan 5 Mobil Rusak Usai Tabrakan Beruntun di Tol Batang</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/jawa-tengah/read/2026/03/16/160000688/berita-foto--potret-bus-po-haryanto-dan-5-mobil-rusak-usai-tabrakan</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Arus Balik, One Way Mulai dari Tol Kalikangkung Semarang</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094290/arus-balik-one-way-mulai-dari-tol-kalikangkung-semarang</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>BGN: Kelengkapan Sertifikasi Jadi Acuan Penentuan Gradasi Dapur MBG</t>
+        </is>
+      </c>
+      <c r="D93" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094288/bgn-kelengkapan-sertifikasi-jadi-acuan-penentuan-gradasi-dapur-mbg</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Didit Prabowo Dapat Kejutan Ulang Tahun dari Megawati-Puan</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094278/didit-prabowo-dapat-kejutan-ulang-tahun-dari-megawati-puan</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Menko PMK Pratikno: Belajar Siswa Diutamakan Tatap Muka</t>
+        </is>
+      </c>
+      <c r="D95" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094257/menko-pmk-pratikno-belajar-siswa-diutamakan-tatap-muka</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Pembelajaran Siswa Normal, Pratikno Singgung Learning Loss</t>
+        </is>
+      </c>
+      <c r="D96" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094253/pembelajaran-siswa-normal-pratikno-singgung-learning-loss</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Kwarnas Estimasi Biaya Rp 67 Juta bagi Peserta Jambore Dunia</t>
+        </is>
+      </c>
+      <c r="D97" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094241/kwarnas-estimasi-biaya-rp-67-juta-bagi-peserta-jambore-dunia</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Pansus 12 DPRD Bandung Dorong Raperda Kesejahteraan Sosial</t>
+        </is>
+      </c>
+      <c r="D98" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094237/pansus-12-dprd-bandung-dorong-raperda-kesejahteraan-sosial</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Jalan Mulus Era Rudy Susmanto Dongkrak Wisata Nirmala</t>
+        </is>
+      </c>
+      <c r="D99" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094236/jalan-mulus-era-rudy-susmanto-dongkrak-wisata-nirmala</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>PM Malaysia Anwar Ibrahim Ungkap Isi Pembicaraan dengan Prabowo</t>
+        </is>
+      </c>
+      <c r="D100" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094235/pm-malaysia-anwar-ibrahim-ungkap-isi-pembicaraan-dengan-prabowo</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Abdul Mu'ti Pastikan Tak Ada Pembelajaran Daring bagi Siswa</t>
+        </is>
+      </c>
+      <c r="D101" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094230/abdul-muti-pastikan-tak-ada-pembelajaran-daring-bagi-siswa</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Program Air Bersih PNM Dorong Produktivitas Usaha Masyarakat</t>
+        </is>
+      </c>
+      <c r="D102" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094225/program-air-bersih-pnm-dorong-produktivitas-usaha-masyarakat</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>TAUD Desak Penuntutan Kasus Andrie Yunus ke Peradilan Umum</t>
+        </is>
+      </c>
+      <c r="D103" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094222/taud-desak-penuntutan-kasus-andrie-yunus-ke-peradilan-umum</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Kementrans Perkuat Sinergi Indonesia-Qatar untuk Pembangunan Sarana Pendidikan Terpadu di Rempang</t>
+        </is>
+      </c>
+      <c r="D104" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094220/kementrans-perkuat-sinergi-indonesia-qatar-untuk-pembangunan-sarana-pendidikan-terpadu-di-rempang</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>BGN Menindak 1.251 SPPG yang Melanggar Standar</t>
+        </is>
+      </c>
+      <c r="D105" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094216/bgn-menindak-1-251-sppg-yang-melanggar-standar</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>SETARA Kritik Diskriminasi Akibat Perbedaan Idul Fitri</t>
+        </is>
+      </c>
+      <c r="D106" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094205/setara-kritik-diskriminasi-akibat-perbedaan-idul-fitri</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Soekarno-Hatta handles nearly two million passengers over Eid period</t>
+        </is>
+      </c>
+      <c r="D107" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409726/soekarno-hatta-handles-nearly-two-million-passengers-over-eid-period</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Asia's economy expected to expand 4.5 pct in 2026: report</t>
+        </is>
+      </c>
+      <c r="D108" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409722/asias-economy-expected-to-expand-45-pct-in-2026-report</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Body of missing British diver found off Gili Air</t>
+        </is>
+      </c>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409718/body-of-missing-british-diver-found-off-gili-air</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>RI Govt confirms 2026 Hajj departures remain on schedule</t>
+        </is>
+      </c>
+      <c r="D110" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409714/ri-govt-confirms-2026-hajj-departures-remain-on-schedule</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>The 'main players' who keep Jakarta alive at Eid</t>
+        </is>
+      </c>
+      <c r="D111" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409710/the-main-players-who-keep-jakarta-alive-at-eid</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>RI Govt urges safe fleets for Eid return travel surge</t>
+        </is>
+      </c>
+      <c r="D112" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409706/ri-govt-urges-safe-fleets-for-eid-return-travel-surge</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Indonesian police urge staggered Eid return with WFA</t>
+        </is>
+      </c>
+      <c r="D113" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409702/indonesian-police-urge-staggered-eid-return-with-wfa</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Jakarta plans to revitalize Kampung Rambutan Terminal after flooding</t>
+        </is>
+      </c>
+      <c r="D114" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409698/jakarta-plans-to-revitalize-kampung-rambutan-terminal-after-flooding</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>Indonesia sees FIFA Series as test of hosting capacity</t>
+        </is>
+      </c>
+      <c r="D115" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409694/indonesia-sees-fifa-series-as-test-of-hosting-capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>Police chief, ministers launch one-way traffic for Eid return flow</t>
+        </is>
+      </c>
+      <c r="D116" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409690/police-chief-ministers-launch-one-way-traffic-for-eid-return-flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>Traffic accidents decline during 2026 Eid homecoming: Minister</t>
+        </is>
+      </c>
+      <c r="D117" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409686/traffic-accidents-decline-during-2026-eid-homecoming-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Police chief calls for optimal service during Eid return flow</t>
+        </is>
+      </c>
+      <c r="D118" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409682/police-chief-calls-for-optimal-service-during-eid-return-flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Indonesia's fuel supply secure during Eid travel: BPH Migas</t>
+        </is>
+      </c>
+      <c r="D119" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409678/indonesias-fuel-supply-secure-during-eid-travel-bph-migas</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Bali internet speeds exceed national average during holidays</t>
+        </is>
+      </c>
+      <c r="D120" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409674/bali-internet-speeds-exceed-national-average-during-holidays</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>Wednesday, 25 March 2026</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>KPK cites GERD in former minister Yaqut house arrest decision</t>
+        </is>
+      </c>
+      <c r="D121" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409670/kpk-cites-gerd-in-former-minister-yaqut-house-arrest-decision</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D61"/>
+  <autoFilter ref="A1:D121"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -1853,6 +3173,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId58"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId59"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D64" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D65" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D81" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D82" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D83" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D84" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D85" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D86" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D87" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D88" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D89" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D90" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D91" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D92" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D93" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D94" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D95" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D96" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D97" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D98" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D99" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D100" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D101" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D102" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D103" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D104" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D105" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D106" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D107" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D108" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D109" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D110" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D111" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D112" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D113" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D114" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D115" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D116" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D117" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D118" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId120"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-03-25
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$181</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D121"/>
+  <dimension ref="A1:D181"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3110,8 +3110,1328 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Puncak Arus Balik Diprediksi 28-29 Maret</t>
+        </is>
+      </c>
+      <c r="D122" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8415597/puncak-arus-balik-diprediksi-28-29-maret</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Kreatif, Kisah Mudik dan Kuliner Khas Lebaran Dibalut Jadi Animasi</t>
+        </is>
+      </c>
+      <c r="D123" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jatim/kuliner/d-8415526/kreatif-kisah-mudik-dan-kuliner-khas-lebaran-dibalut-jadi-animasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Rumah Ditinggal Mudik di Jagakarsa Dibobol, Pelaku Kepergok Warga</t>
+        </is>
+      </c>
+      <c r="D124" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8415359/rumah-ditinggal-mudik-di-jagakarsa-dibobol-pelaku-kepergok-warga</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Video: Situasi Arus Balik Lebaran di Stasiun Pasar Senen</t>
+        </is>
+      </c>
+      <c r="D125" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260325-260325047/video-situasi-arus-balik-lebaran-di-stasiun-pasar-senen</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Video Dean James Dicoret dari Timnas di Tengah Polemik Paspor Belanda</t>
+        </is>
+      </c>
+      <c r="D126" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/detiktv/d-8415659/video-dean-james-dicoret-dari-timnas-di-tengah-polemik-paspor-belanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>Bangga! TN Komodo Runner-up dalam Daftar 10 Tempat Terindah Dunia</t>
+        </is>
+      </c>
+      <c r="D127" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.detik.com/travel-news/d-8415273/bangga-tn-komodo-runner-up-dalam-daftar-10-tempat-terindah-dunia</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Video Hendrik 'Joget MBG' Mengaku Belum Balik Modal Bangun Dapur</t>
+        </is>
+      </c>
+      <c r="D128" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8415417/video-hendrik-joget-mbg-mengaku-belum-balik-modal-bangun-dapur</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>Video: Makna Pertemuan Anies dengan SBY-AHY hingga Didit Prabowo</t>
+        </is>
+      </c>
+      <c r="D129" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8415472/video-makna-pertemuan-anies-dengan-sby-ahy-hingga-didit-prabowo</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Purbaya Buka-bukaan soal Coretax: Salah Desain!</t>
+        </is>
+      </c>
+      <c r="D130" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8415524/purbaya-buka-bukaan-soal-coretax-salah-desain</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Iran Bolehkan Negara Sahabat Lewati Selat Hormuz: Hanya Tertutup Bagi Musuh!</t>
+        </is>
+      </c>
+      <c r="D131" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8415660/iran-bolehkan-negara-sahabat-lewati-selat-hormuz-hanya-tertutup-bagi-musuh</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Iran Ogah Negosiasi dengan AS, Tegaskan Akan Terus Melawan</t>
+        </is>
+      </c>
+      <c r="D132" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8415657/iran-ogah-negosiasi-dengan-as-tegaskan-akan-terus-melawan</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>AS Minta Iran Akui Kekalahan, Peringatkan Serangan Lanjutan Lebih Keras</t>
+        </is>
+      </c>
+      <c r="D133" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8415652/as-minta-iran-akui-kekalahan-peringatkan-serangan-lanjutan-lebih-keras</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>Ulah Pengemudi Fortuner Ugal-ugalan hingga Tabrakan di Tol Andara</t>
+        </is>
+      </c>
+      <c r="D134" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8415579/ulah-pengemudi-fortuner-ugal-ugalan-hingga-tabrakan-di-tol-andara</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>Cerita Pemecatan Brutal Ange Postecoglu</t>
+        </is>
+      </c>
+      <c r="D135" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8415643/cerita-pemecatan-brutal-ange-postecoglu</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>Purbaya Diam-diam Guyur Rp 100 T ke Bank Sebelum Lebaran</t>
+        </is>
+      </c>
+      <c r="D136" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8415313/purbaya-diam-diam-guyur-rp-100-t-ke-bank-sebelum-lebaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>Prabowo Minta Percepatan Kendaraan Listrik, Ini Kata Toyota</t>
+        </is>
+      </c>
+      <c r="D137" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1919355/prabowo-minta-percepatan-kendaraan-listrik-ini-kata-toyota?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Pertamina Oil Scandal: What is the Chronology and What is the Impact?</t>
+        </is>
+      </c>
+      <c r="D138" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/en-skandal-minyak-pertamina-bagaimana-kronologi-dan-apa-dampaknya?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>DLH Semarang Minta Maaf, Tumpahan Sampah di Jalan Sultan Agung Cepat Dibersihkan</t>
+        </is>
+      </c>
+      <c r="D139" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/03/25/185507678/dlh-semarang-minta-maaf-tumpahan-sampah-di-jalan-sultan-agung-cepat</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>Sembari Tunggu Data Rampung, Pemerintah Percepat Penyaluran Bantuan Pemulihan di Sumatera</t>
+        </is>
+      </c>
+      <c r="D140" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/25/18320071/sembari-tunggu-data-rampung-pemerintah-percepat-penyaluran-bantuan-pemulihan</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>Kasatgas PRR Dorong Percepatan Pemulihan Bencana Sumatera lewat Kolaborasi Antardaerah</t>
+        </is>
+      </c>
+      <c r="D141" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/25/17461781/kasatgas-prr-dorong-percepatan-pemulihan-bencana-sumatera-lewat-kolaborasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D142" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D143" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D144" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D145" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>China Kirim Bus Listrik Canggih ke Meksiko Dukung Piala Dunia 2026</t>
+        </is>
+      </c>
+      <c r="D146" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1919315/china-kirim-bus-listrik-canggih-ke-meksiko-dukung-piala-dunia-2026?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>Produktif Kerja Pasca Lebaran: Kembali Fokus!</t>
+        </is>
+      </c>
+      <c r="D147" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/pristiwan/69c337ed34777c26c3619a72/produktif-kerja-pasca-lebaran-kembali-fokus</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>Culture</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>Perbedaan Geisha dan Maiko, dari Tahap Pelatihan hingga Penampilan Tradisional</t>
+        </is>
+      </c>
+      <c r="D148" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5626/perbedaan-geisha-dan-maiko-dari-tahap-pelatihan-hingga-penampilan-tradisional</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D149" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D150" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Potret Bus PO Haryanto dan 5 Mobil Rusak Usai Tabrakan Beruntun di Tol Batang</t>
+        </is>
+      </c>
+      <c r="D151" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/jawa-tengah/read/2026/03/16/160000688/berita-foto--potret-bus-po-haryanto-dan-5-mobil-rusak-usai-tabrakan</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>Tourism</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>Liburan ke Bali, Cokelat Falala Oleh-Olehnya</t>
+        </is>
+      </c>
+      <c r="D152" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094501/liburan-ke-bali-cokelat-falala-oleh-olehnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B153" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>Kapuspen: TNI Tak Menoleransi Prajurit yang Melanggar Hukum</t>
+        </is>
+      </c>
+      <c r="D153" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094500/kapuspen-tni-tak-menoleransi-prajurit-yang-melanggar-hukum</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>Soal Anies ke Cikeas, Demokrat: Murni Silaturahmi</t>
+        </is>
+      </c>
+      <c r="D154" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094499/soal-anies-ke-cikeas-demokrat-murni-silaturahmi</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>Kepala Bais TNI Serahkan Jabatan Buntut Kasus Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D155" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094488/kepala-bais-tni-serahkan-jabatan-buntut-kasus-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>Soal Penerapan WFH, Tito Karnavian: Tunggu Arahan Presiden</t>
+        </is>
+      </c>
+      <c r="D156" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094475/soal-penerapan-wfh-tito-karnavian-tunggu-arahan-presiden</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>Anies Bertemu SBY di Cikeas, Bahas Apa?</t>
+        </is>
+      </c>
+      <c r="D157" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094469/anies-bertemu-sby-di-cikeas-bahas-apa</t>
+        </is>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B158" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C158" t="inlineStr">
+        <is>
+          <t>SPPG Milik Pria Viral Joget Dihentikan Sementara</t>
+        </is>
+      </c>
+      <c r="D158" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094442/sppg-milik-pria-viral-joget-dihentikan-sementara</t>
+        </is>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B159" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
+          <t>Alasan Pemprov Jatim Tetapkan Rabu sebagai WFH bagi ASN</t>
+        </is>
+      </c>
+      <c r="D159" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094440/alasan-pemprov-jatim-tetapkan-rabu-sebagai-wfh-bagi-asn</t>
+        </is>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B160" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C160" t="inlineStr">
+        <is>
+          <t>Konsumsi BBM Pertamax Series Naik Signifikan Saat Musim Lebaran</t>
+        </is>
+      </c>
+      <c r="D160" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094435/konsumsi-bbm-pertamax-series-naik-signifikan-saat-musim-lebaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>Tito: Semua Menteri Sudah Sepakat WFH Satu Hari Sepekan</t>
+        </is>
+      </c>
+      <c r="D161" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094429/tito-semua-menteri-sudah-sepakat-wfh-satu-hari-sepekan</t>
+        </is>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B162" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C162" t="inlineStr">
+        <is>
+          <t>Khofifah Pilih WFH Tiap Rabu untuk ASN Jawa Timur</t>
+        </is>
+      </c>
+      <c r="D162" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094425/khofifah-pilih-wfh-tiap-rabu-untuk-asn-jawa-timur</t>
+        </is>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B163" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
+          <t>Tito: 171 Jiwa Masih Tinggal di Tenda Pengungsian Aceh</t>
+        </is>
+      </c>
+      <c r="D163" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094417/tito-171-jiwa-masih-tinggal-di-tenda-pengungsian-aceh</t>
+        </is>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B164" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C164" t="inlineStr">
+        <is>
+          <t>Datangi Rumah Jokowi, Budi Arie Projo: Silaturahmi Lebaran</t>
+        </is>
+      </c>
+      <c r="D164" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094410/datangi-rumah-jokowi-budi-arie-projo-silaturahmi-lebaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B165" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C165" t="inlineStr">
+        <is>
+          <t>Menteri Abdul Mu'ti: Rencana Pembelajaran Daring Dibatalkan</t>
+        </is>
+      </c>
+      <c r="D165" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094406/menteri-abdul-muti-rencana-pembelajaran-daring-dibatalkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B166" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
+          <t>Mengapa Pemerintah Perlu Buat TGPF di Kasus Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D166" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094400/mengapa-pemerintah-perlu-buat-tgpf-di-kasus-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B167" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C167" t="inlineStr">
+        <is>
+          <t>KPAI urges govt to enforce child online safety rules</t>
+        </is>
+      </c>
+      <c r="D167" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409846/kpai-urges-govt-to-enforce-child-online-safety-rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B168" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C168" t="inlineStr">
+        <is>
+          <t>Free meal efficiency could save up Rp40 trln a year: minister</t>
+        </is>
+      </c>
+      <c r="D168" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409842/free-meal-efficiency-could-save-up-rp40-trln-a-year-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B169" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C169" t="inlineStr">
+        <is>
+          <t>Govt speeds up Sumatra recovery with cross-region collaboration</t>
+        </is>
+      </c>
+      <c r="D169" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409838/govt-speeds-up-sumatra-recovery-with-cross-region-collaboration</t>
+        </is>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B170" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>Two suspects sought in killing of Dutch national in Bali</t>
+        </is>
+      </c>
+      <c r="D170" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409834/two-suspects-sought-in-killing-of-dutch-national-in-bali</t>
+        </is>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B171" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>Indonesia to expand MBG with over 90 kitchens in Jayawijaya</t>
+        </is>
+      </c>
+      <c r="D171" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409830/indonesia-to-expand-mbg-with-over-90-kitchens-in-jayawijaya</t>
+        </is>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>Indonesia disburses $41 million aid for Sumatra disaster victims</t>
+        </is>
+      </c>
+      <c r="D172" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409826/indonesia-disburses-41-million-aid-for-sumatra-disaster-victims</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>Saudi ambassador to Indonesia condemns Iran's attacks on Gulf states</t>
+        </is>
+      </c>
+      <c r="D173" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409822/saudi-ambassador-to-indonesia-condemns-irans-attacks-on-gulf-states</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>Indonesia expects arrival of second A400M aircraft</t>
+        </is>
+      </c>
+      <c r="D174" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409818/indonesia-expects-arrival-of-second-a400m-aircraft</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>BNPB building 36,000 homes for flood victims in Sumatra</t>
+        </is>
+      </c>
+      <c r="D175" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409814/bnpb-building-36000-homes-for-flood-victims-in-sumatra</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>Traffic conditions improve, police end one-way system for return flow</t>
+        </is>
+      </c>
+      <c r="D176" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409810/traffic-conditions-improve-police-end-one-way-system-for-return-flow</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>SBC Medical Announces Next-Generation Wellness Strategy “SBC Wellness 2.0”</t>
+        </is>
+      </c>
+      <c r="D177" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409806/sbc-medical-announces-next-generation-wellness-strategy-sbc-wellness-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>Bali Governor seeks end to Suwung-like landfills by 2027</t>
+        </is>
+      </c>
+      <c r="D178" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409802/bali-governor-seeks-end-to-suwung-like-landfills-by-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>Sumatra rehabilitation budget need estimated at Rp130 trillion: govt</t>
+        </is>
+      </c>
+      <c r="D179" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409798/sumatra-rehabilitation-budget-need-estimated-at-rp130-trillion-govt</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B180" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>Saudi envoy says 2026 Hajj to proceed despite Mideast tensions</t>
+        </is>
+      </c>
+      <c r="D180" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409794/saudi-envoy-says-2026-hajj-to-proceed-despite-mideast-tensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" t="inlineStr">
+        <is>
+          <t>Thursday, 26 March 2026</t>
+        </is>
+      </c>
+      <c r="B181" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>Police foil 67 kg drug smuggling in Port of Merak during Eid travel</t>
+        </is>
+      </c>
+      <c r="D181" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409790/police-foil-67-kg-drug-smuggling-in-port-of-merak-during-eid-travel</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D121"/>
+  <autoFilter ref="A1:D181"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -3233,6 +4553,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D119" r:id="rId118"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D120" r:id="rId119"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D121" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D122" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D123" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D124" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D125" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D126" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D127" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D128" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D129" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D130" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D131" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D132" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D133" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D134" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D135" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D136" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D137" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D138" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D139" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D140" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D141" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D142" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D143" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D144" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D145" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D146" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D147" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D148" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D149" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D150" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D151" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D152" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D153" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D154" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D155" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D156" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D157" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D158" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D159" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D160" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D161" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D162" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D163" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D164" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D165" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D166" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D167" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D168" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D169" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D170" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D171" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D172" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D173" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D174" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D175" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D176" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D177" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D178" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D179" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D180" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D181" r:id="rId180"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-03-26
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$181</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$241</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D181"/>
+  <dimension ref="A1:D241"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -4430,8 +4430,1328 @@
         </is>
       </c>
     </row>
+    <row r="182">
+      <c r="A182" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B182" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>Video Curhat Pedagang di Nagreg, Omzet Turun Meski Lalin Padat</t>
+        </is>
+      </c>
+      <c r="D182" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260326-260326056/video-curhat-pedagang-di-nagreg-omzet-turun-meski-lalin-padat</t>
+        </is>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B183" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>Video: GT Parungkuda Masih Jadi Titik Tumpu Kepadatan di H+5 Lebaran</t>
+        </is>
+      </c>
+      <c r="D183" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260326-260326049/video-gt-parungkuda-masih-jadi-titik-tumpu-kepadatan-di-h5-lebaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B184" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>Video Pemudik Masih Ramaikan Stasiun Gambir H+5 Lebaran</t>
+        </is>
+      </c>
+      <c r="D184" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260326-260326035/video-pemudik-masih-ramaikan-stasiun-gambir-h5-lebaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B185" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>2 Maling di Kendari Diamuk Massa Usai Kepergok Satroni Rumah Ditinggal Mudik</t>
+        </is>
+      </c>
+      <c r="D185" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/sulsel/hukum-dan-kriminal/d-8416183/2-maling-di-kendari-diamuk-massa-usai-kepergok-satroni-rumah-ditinggal-mudik</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B186" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>Negara Tetangga Darurat BBM, Bahlil Pastikan RI Aman</t>
+        </is>
+      </c>
+      <c r="D186" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8417082/negara-tetangga-darurat-bbm-bahlil-pastikan-ri-aman</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B187" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>Malaysia Pangkas Kuota BBM Subsidi 1 April, Jadi 200 Liter/Bulan</t>
+        </is>
+      </c>
+      <c r="D187" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8417063/malaysia-pangkas-kuota-bbm-subsidi-1-april-jadi-200-liter-bulan</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B188" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>Blusukan ke Bantaran Rel Senen, Prabowo Janji Bangun Hunian Layak</t>
+        </is>
+      </c>
+      <c r="D188" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8416969/blusukan-ke-bantaran-rel-senen-prabowo-janji-bangun-hunian-layak</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B189" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>Sekali Foto Kencan, Cristiano Ronaldo &amp; Georgina Pamer Harta Rp 250 Miliar</t>
+        </is>
+      </c>
+      <c r="D189" s="2" t="inlineStr">
+        <is>
+          <t>https://wolipop.detik.com/entertainment-news/d-8416660/sekali-foto-kencan-cristiano-ronaldo-georgina-pamer-harta-rp-250-miliar</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>Kapal Tanker Malaysia Boleh Lewat Hormuz, Anwar Ibrahim Ungkap Jurus Nego Iran</t>
+        </is>
+      </c>
+      <c r="D190" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8416927/kapal-tanker-malaysia-boleh-lewat-hormuz-anwar-ibrahim-ungkap-jurus-nego-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Video Trump Sebut Iran Kasih AS 'Hadiah': 10 Kapal Minyak Lolos Hormuz</t>
+        </is>
+      </c>
+      <c r="D191" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260327-260327002/video-trump-sebut-iran-kasih-as-hadiah-10-kapal-minyak-lolos-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Ibunda Anji Meninggal Dunia</t>
+        </is>
+      </c>
+      <c r="D192" s="2" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8417067/ibunda-anji-meninggal-dunia</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Kakorlantas hingga Menhub Akan Rapat Persiapan Puncak Arus Balik Gelombang Kedua</t>
+        </is>
+      </c>
+      <c r="D193" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8417147/kakorlantas-hingga-menhub-akan-rapat-persiapan-puncak-arus-balik-gelombang-kedua</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Malaysia Pangkas Kuota BBM Subsidi 1 April, Jadi 200 Liter/Bulan</t>
+        </is>
+      </c>
+      <c r="D194" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8417063/malaysia-pangkas-kuota-bbm-subsidi-1-april-jadi-200-liter-bulan</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Video Momen Kakorlantas Putar Balik Truk Sumbu 3 demi Kelancaran Arus Balik</t>
+        </is>
+      </c>
+      <c r="D195" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260326-260326094/video-momen-kakorlantas-putar-balik-truk-sumbu-3-demi-kelancaran-arus-balik</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Video Iran Ingin Perang Berakhir: Tapi dengan Syarat Kami</t>
+        </is>
+      </c>
+      <c r="D196" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260326-260326054/video-iran-ingin-perang-berakhir-tapi-dengan-syarat-kami</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Israel Klaim Tewaskan Komandan Angkatan Laut IRGC dalam Serangan Terbaru ke Iran</t>
+        </is>
+      </c>
+      <c r="D197" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1919568/israel-klaim-tewaskan-komandan-angkatan-laut-irgc-dalam-serangan-terbaru-ke-iran?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Prodi Apa yang Paling Diburu di UTBK SNBT 2026?</t>
+        </is>
+      </c>
+      <c r="D198" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/prodi-apa-yang-paling-diburu-di-snbt-utbk-2026?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Mendagri–Menteri PKP Tinjau Program BSPS di Humbahas, Target Perbaikan Rumah di Sumut Naik Drastis</t>
+        </is>
+      </c>
+      <c r="D199" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/26/21052391/mendagrimenteri-pkp-tinjau-program-bsps-di-humbahas-target-perbaikan-rumah</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Ekonomi RI Tangguh di Tengah Badai Global, Kemenko Perekonomian Beberkan Indikatornya</t>
+        </is>
+      </c>
+      <c r="D200" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/26/20084161/ekonomi-ri-tangguh-di-tengah-badai-global-kemenko-perekonomian-beberkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Banjir Rendam Sejumlah Wilayah, Pemkot Semarang Perkuat Pengelolaan Pintu Air dan Tanggul</t>
+        </is>
+      </c>
+      <c r="D201" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/03/26/200319878/banjir-rendam-sejumlah-wilayah-pemkot-semarang-perkuat-pengelolaan-pintu</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D202" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D203" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D204" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D205" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Gedung Putih "Bingung" dengan Klaim Trump dapat Hadiah dari Iran</t>
+        </is>
+      </c>
+      <c r="D206" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1919515/gedung-putih-bingung-dengan-klaim-trump-dapat-hadiah-dari-iran?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Cerpen: Di Bawah Langit Pisa</t>
+        </is>
+      </c>
+      <c r="D207" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/noviar8266/69c2503934777c5b131ae8e2/cerpen-di-bawah-langit-pisa</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Ingin Riset di Jepang? Ini Panduan Lengkap Visa Peneliti dan Cara Mengajukannya</t>
+        </is>
+      </c>
+      <c r="D208" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5699/ingin-riset-di-jepang-ini-panduan-lengkap-visa-peneliti-dan-cara-mengajukannya</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D209" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D210" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Potret Bus PO Haryanto dan 5 Mobil Rusak Usai Tabrakan Beruntun di Tol Batang</t>
+        </is>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/jawa-tengah/read/2026/03/16/160000688/berita-foto--potret-bus-po-haryanto-dan-5-mobil-rusak-usai-tabrakan</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Pembatas 138 Km, Gubernur Lampung Sebut Bukti Komitmen Presiden Atasi Konflik Gajah Way Kambas</t>
+        </is>
+      </c>
+      <c r="D212" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094700/pembatas-138-km-gubernur-lampung-sebut-bukti-komitmen-presiden-atasi-konflik-gajah-way-kambas</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>PLN Berhasil Amankan Pasokan Listrik Nasional Saat Salat Idul Fitri 1447 H</t>
+        </is>
+      </c>
+      <c r="D213" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094691/pln-berhasil-amankan-pasokan-listrik-nasional-saat-salat-idul-fitri-1447-h</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Disebut Rentan Rusak, Ini Fakta Penggunaan AC Inverter</t>
+        </is>
+      </c>
+      <c r="D214" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094685/disebut-rentan-rusak-ini-fakta-penggunaan-ac-inverter</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Prabowo Mengundang PM Malaysia Anwar Ibrahim ke Jakarta</t>
+        </is>
+      </c>
+      <c r="D215" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094679/prabowo-mengundang-pm-malaysia-anwar-ibrahim-ke-jakarta</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Gadai BPKB Mobil di SEVA, Jadi Alternatif Pinjaman Dana Tunai Tanpa Jual Kendaraan</t>
+        </is>
+      </c>
+      <c r="D216" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094678/gadai-bpkb-mobil-di-seva-jadi-alternatif-pinjaman-dana-tunai-tanpa-jual-kendaraan</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Hadir di 400 Kota di Indonesia, Maxim Tingkatkan Mobilitas Transportasi di Tanah Air</t>
+        </is>
+      </c>
+      <c r="D217" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094675/hadir-di-400-kota-di-indonesia-maxim-tingkatkan-mobilitas-transportasi-di-tanah-air</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Amnesty Desak Prabowo dan DPR Bentuk TPF Kasus Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D218" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094674/amnesty-desak-prabowo-dan-dpr-bentuk-tpf-kasus-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B219" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C219" t="inlineStr">
+        <is>
+          <t>Pemprov Jabar Liburkan Ribuan Sopir Angkot di Sukabumi</t>
+        </is>
+      </c>
+      <c r="D219" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094656/pemprov-jabar-liburkan-ribuan-sopir-angkot-di-sukabumi</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B220" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C220" t="inlineStr">
+        <is>
+          <t>Gibran Menyambangi Sejumlah Ponpes saat Mudik ke Solo</t>
+        </is>
+      </c>
+      <c r="D220" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094655/gibran-menyambangi-sejumlah-ponpes-saat-mudik-ke-solo</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B221" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C221" t="inlineStr">
+        <is>
+          <t>Kesadaran Investasi Emas Masyarakat Meningkat, Transaksi Pegadaian Meningkat Jelang Lebaran</t>
+        </is>
+      </c>
+      <c r="D221" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094646/kesadaran-investasi-emas-masyarakat-meningkat-transaksi-pegadaian-meningkat-jelang-lebaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B222" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C222" t="inlineStr">
+        <is>
+          <t>Koalisi: Pencopotan Kabais Tak Beri Keadilan bagi Andrie</t>
+        </is>
+      </c>
+      <c r="D222" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094643/koalisi-pencopotan-kabais-tak-beri-keadilan-bagi-andrie</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B223" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C223" t="inlineStr">
+        <is>
+          <t>Komnas HAM: Pemulihan Andrie Yunus Bisa Sampai 2 Tahun</t>
+        </is>
+      </c>
+      <c r="D223" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094639/komnas-ham-pemulihan-andrie-yunus-bisa-sampai-2-tahun</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B224" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C224" t="inlineStr">
+        <is>
+          <t>Ning Ita Instruksikan ASN Kota Mojokerto "Gowes" Setiap Hari Jumat</t>
+        </is>
+      </c>
+      <c r="D224" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094620/ning-ita-instruksikan-asn-kota-mojokerto-gowes-setiap-hari-jumat</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>Prabowo Menyoroti Industri Mineral Belum Adil untuk Negara</t>
+        </is>
+      </c>
+      <c r="D225" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094609/prabowo-menyoroti-industri-mineral-belum-adil-untuk-negara</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B226" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C226" t="inlineStr">
+        <is>
+          <t>KontraS Ungkap Kondisi Terkini Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D226" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094607/kontras-ungkap-kondisi-terkini-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B227" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C227" t="inlineStr">
+        <is>
+          <t>Way Kambas National Park pilot for innovative climate financing</t>
+        </is>
+      </c>
+      <c r="D227" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409982/way-kambas-national-park-pilot-for-innovative-climate-financing</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B228" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C228" t="inlineStr">
+        <is>
+          <t>Two Bengal tiger cubs at Bandung Zoo die of panleukopenia</t>
+        </is>
+      </c>
+      <c r="D228" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409978/two-bengal-tiger-cubs-at-bandung-zoo-die-of-panleukopenia</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B229" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C229" t="inlineStr">
+        <is>
+          <t>Govt to include 30 new schools in Garuda Top School program for 2026</t>
+        </is>
+      </c>
+      <c r="D229" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409974/govt-to-include-30-new-schools-in-garuda-top-school-program-for-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>WSBP Reports Operating Revenue of Rp1.57 Trillion in 2025, Drives Efficiency and Optimizes Operational Performance</t>
+        </is>
+      </c>
+      <c r="D230" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409970/wsbp-reports-operating-revenue-of-rp157-trillion-in-2025-drives-efficiency-and-optimizes-operational-performance</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B231" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C231" t="inlineStr">
+        <is>
+          <t>Indonesia's diesel import halt buffers supply against global risks</t>
+        </is>
+      </c>
+      <c r="D231" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409966/indonesias-diesel-import-halt-buffers-supply-against-global-risks</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B232" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C232" t="inlineStr">
+        <is>
+          <t>Indonesian Navy weighs missile options for new warship</t>
+        </is>
+      </c>
+      <c r="D232" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409962/indonesian-navy-weighs-missile-options-for-new-warship</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B233" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C233" t="inlineStr">
+        <is>
+          <t>Resignation over attack seen as "good example," MP says</t>
+        </is>
+      </c>
+      <c r="D233" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409958/resignation-over-attack-seen-as-good-example-mp-says</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B234" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C234" t="inlineStr">
+        <is>
+          <t>Racing for peace: Indonesia’s move to blunt Mideast escalation</t>
+        </is>
+      </c>
+      <c r="D234" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409954/racing-for-peace-indonesias-move-to-blunt-mideast-escalation</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>Task force prioritizes river restoration in Sumatra recovery</t>
+        </is>
+      </c>
+      <c r="D235" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409950/task-force-prioritizes-river-restoration-in-sumatra-recovery</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B236" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C236" t="inlineStr">
+        <is>
+          <t>Prabowo, Anwar to discuss geopolitics in Jakarta talks Friday</t>
+        </is>
+      </c>
+      <c r="D236" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409946/prabowo-anwar-to-discuss-geopolitics-in-jakarta-talks-friday</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B237" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C237" t="inlineStr">
+        <is>
+          <t>Prabowo orders resource push to secure energy autonomy</t>
+        </is>
+      </c>
+      <c r="D237" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409942/prabowo-orders-resource-push-to-secure-energy-autonomy</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B238" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C238" t="inlineStr">
+        <is>
+          <t>Four months on, Sumatra moves from emergency to reconstruction</t>
+        </is>
+      </c>
+      <c r="D238" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409938/four-months-on-sumatra-moves-from-emergency-to-reconstruction</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B239" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C239" t="inlineStr">
+        <is>
+          <t>MPR calls for reform in energy subsidies to improve targeting</t>
+        </is>
+      </c>
+      <c r="D239" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409934/mpr-calls-for-reform-in-energy-subsidies-to-improve-targeting</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B240" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C240" t="inlineStr">
+        <is>
+          <t>Indonesia channels Rp22.6 billion for Samosir housing upgrades</t>
+        </is>
+      </c>
+      <c r="D240" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409930/indonesia-channels-rp226-billion-for-samosir-housing-upgrades</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>Friday, 27 March 2026</t>
+        </is>
+      </c>
+      <c r="B241" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C241" t="inlineStr">
+        <is>
+          <t>President Prabowo says overseas visits to protect people's interests</t>
+        </is>
+      </c>
+      <c r="D241" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/409926/president-prabowo-says-overseas-visits-to-protect-peoples-interests</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D181"/>
+  <autoFilter ref="A1:D241"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -4613,6 +5933,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D179" r:id="rId178"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D180" r:id="rId179"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D181" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D182" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D183" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D184" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D185" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D186" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D187" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D188" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D189" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D190" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D191" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D192" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D193" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D194" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D195" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D196" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D197" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D198" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D199" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D200" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D201" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D202" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D203" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D204" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D205" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D206" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D207" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D208" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D209" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D210" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D211" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D212" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D213" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D214" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D215" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D216" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D217" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D218" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D219" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D220" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D221" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D222" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D223" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D224" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D225" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D226" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D227" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D228" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D229" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D230" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D231" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D232" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D233" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D234" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D235" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D236" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D237" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D238" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D239" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D240" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D241" r:id="rId240"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-03-27
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$241</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$301</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D241"/>
+  <dimension ref="A1:D301"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -5750,8 +5750,1328 @@
         </is>
       </c>
     </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B242" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C242" t="inlineStr">
+        <is>
+          <t>Niat Hati Mudik ke Jogja, Mobil Pemudik Nahas Malah Nyemplung ke Parit</t>
+        </is>
+      </c>
+      <c r="D242" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.detik.com/travel-news/d-8418276/niat-hati-mudik-ke-jogja-mobil-pemudik-nahas-malah-nyemplung-ke-parit</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B243" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C243" t="inlineStr">
+        <is>
+          <t>Video Arus Lalu Lintas Menuju Jalur Wisata Kota Batu Ramai Lancar</t>
+        </is>
+      </c>
+      <c r="D243" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260327-260327043/video-arus-lalu-lintas-menuju-jalur-wisata-kota-batu-ramai-lancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B244" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C244" t="inlineStr">
+        <is>
+          <t>Tantangan Arus Mudik Kepulauan</t>
+        </is>
+      </c>
+      <c r="D244" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/kolom/d-8417531/tantangan-arus-mudik-kepulauan</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B245" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C245" t="inlineStr">
+        <is>
+          <t>Video 48 Ribu Pemudik Kereta Api Tiba di Jakarta pada H+6 Lebaran</t>
+        </is>
+      </c>
+      <c r="D245" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260327-260327013/-video-48-ribu-pemudik-kereta-api-tiba-di-jakarta-pada-h6-lebaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B246" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C246" t="inlineStr">
+        <is>
+          <t>Indonesia Vs Saint Kitts &amp; Nevis: Garuda Unggul 2-0 di Babak I</t>
+        </is>
+      </c>
+      <c r="D246" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8418513/indonesia-vs-saint-kitts-nevis-garuda-unggul-2-0-di-babak-i</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B247" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C247" t="inlineStr">
+        <is>
+          <t>Lagi Post Holiday Blues? Mending Isi Waktu dengan Selesaikan Game Asah Otak Ini</t>
+        </is>
+      </c>
+      <c r="D247" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/asah-otak/d-8418459/lagi-post-holiday-blues-mending-isi-waktu-dengan-selesaikan-game-asah-otak-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B248" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C248" t="inlineStr">
+        <is>
+          <t>Dokter Internship di Cianjur Meninggal, Disebut Alami Komplikasi Berat Campak</t>
+        </is>
+      </c>
+      <c r="D248" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8418400/dokter-internship-di-cianjur-meninggal-disebut-alami-komplikasi-berat-campak</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B249" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C249" t="inlineStr">
+        <is>
+          <t>Kisah Pilu Pekerja Pabrik Batu Bata Pakistan, Jual Ginjal Demi Lunasi Utang</t>
+        </is>
+      </c>
+      <c r="D249" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8418317/kisah-pilu-pekerja-pabrik-batu-bata-pakistan-jual-ginjal-demi-lunasi-utang</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B250" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C250" t="inlineStr">
+        <is>
+          <t>Purbaya Bongkar Aksi Nakal di Balik Coretax: Masukin Vendor Diam-diam!</t>
+        </is>
+      </c>
+      <c r="D250" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8418306/purbaya-bongkar-aksi-nakal-di-balik-coretax-masukin-vendor-diam-diam</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C251" t="inlineStr">
+        <is>
+          <t>Mahasiswi di Sumsel Ditahan Polisi Usai Buka HP Rekan Kerja dan Kirim Foto</t>
+        </is>
+      </c>
+      <c r="D251" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8418704/mahasiswi-di-sumsel-ditahan-polisi-usai-buka-hp-rekan-kerja-dan-kirim-foto</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C252" t="inlineStr">
+        <is>
+          <t>Staf Bawaslu OKU Ditemukan Tewas di Rumahnya, Ada Luka di Leher</t>
+        </is>
+      </c>
+      <c r="D252" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8415658/staf-bawaslu-oku-ditemukan-tewas-di-rumahnya-ada-luka-di-leher</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B253" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C253" t="inlineStr">
+        <is>
+          <t>Ngeluh Sesak Nafas dan Punggung Sakit, Tahanan di Sumsel Meninggal</t>
+        </is>
+      </c>
+      <c r="D253" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8411797/ngeluh-sesak-nafas-dan-punggung-sakit-tahanan-di-sumsel-meninggal</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B254" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C254" t="inlineStr">
+        <is>
+          <t>Hasil Practice MotoGP Amerika 2026: Marc Marquez Tercepat</t>
+        </is>
+      </c>
+      <c r="D254" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/moto-gp/d-8418705/hasil-practice-motogp-amerika-2026-marc-marquez-tercepat</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B255" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C255" t="inlineStr">
+        <is>
+          <t>Arus Balik Gelombang 2, Korlantas Siapkan Skema Perpanjang One Way</t>
+        </is>
+      </c>
+      <c r="D255" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8418702/arus-balik-gelombang-2-korlantas-siapkan-skema-perpanjang-one-way</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B256" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C256" t="inlineStr">
+        <is>
+          <t>Polisi Buru I Dewa Ketut Wiranida Terkait Peredaran Ekstasi di Kelab Bali</t>
+        </is>
+      </c>
+      <c r="D256" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8418535/polisi-buru-i-dewa-ketut-wiranida-terkait-peredaran-ekstasi-di-kelab-bali</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B257" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C257" t="inlineStr">
+        <is>
+          <t>Contraflow Tol Japek Diperpanjang Atasi Kemacetan Arus Balik Lebaran 2026</t>
+        </is>
+      </c>
+      <c r="D257" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1919781/contraflow-tol-japek-diperpanjang-atasi-kemacetan-arus-balik-lebaran-2026?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B258" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C258" t="inlineStr">
+        <is>
+          <t>Ketika Semua Pihak Bisa Berinvestasi: Apakah Pasar Modal Benar-benar Memajukan Perekonomian?</t>
+        </is>
+      </c>
+      <c r="D258" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/ketika-semua-pihak-bisa-berinvestasi-apakah-pasar-modal-benar-benar-memajukan-perekonomian-2?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B259" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C259" t="inlineStr">
+        <is>
+          <t>Dorong Penyaluran Bantuan di Tapanuli Tengah Tepat Waktu, Tito Tekankan Percepatan Pendataan Kerusakan Rumah</t>
+        </is>
+      </c>
+      <c r="D259" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/27/21405521/dorong-penyaluran-bantuan-di-tapanuli-tengah-tepat-waktu-tito-tekankan</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B260" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C260" t="inlineStr">
+        <is>
+          <t>Atlet Pencak Silat Rentan Cedera, BPJS Ketenagakerjaan Dorong Perlindungan Jaminan Sosial</t>
+        </is>
+      </c>
+      <c r="D260" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/27/19471061/atlet-pencak-silat-rentan-cedera-bpjs-ketenagakerjaan-dorong-perlindungan</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B261" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C261" t="inlineStr">
+        <is>
+          <t>Serahkan 120 Unit Huntap bagi Penyintas Bencana di Tapsel, Kasatgas Tito Apresiasi Kecepatan Pendataan Bupati</t>
+        </is>
+      </c>
+      <c r="D261" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/27/19032591/serahkan-120-unit-huntap-bagi-penyintas-bencana-di-tapsel-kasatgas-tito</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B262" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C262" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D262" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B263" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C263" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D263" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B264" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C264" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D264" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B265" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C265" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D265" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B266" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C266" t="inlineStr">
+        <is>
+          <t>Arus Balik Lebaran 2026: 480.000 Kendaraan Belum Kembali ke Jakarta</t>
+        </is>
+      </c>
+      <c r="D266" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1919742/arus-balik-lebaran-2026-480000-kendaraan-belum-kembali-ke-jakarta?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B267" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C267" t="inlineStr">
+        <is>
+          <t>Sepulang Mudik, Mendapati Sepucuk Surat Dari Pak Anies Baswedan</t>
+        </is>
+      </c>
+      <c r="D267" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/rintawulandarii/69c36bbc34777c7cc666ef24/sepulang-mudik-mendapati-sepucuk-surat-dari-pak-anies-baswedan</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B268" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C268" t="inlineStr">
+        <is>
+          <t>6 Spot Terbaik Melihat Gunung Fuji di Shizuoka, dari Pantai hingga Puncak Bukit</t>
+        </is>
+      </c>
+      <c r="D268" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5705/6-spot-terbaik-melihat-gunung-fuji-di-shizuoka-dari-pantai-hingga-puncak-bukit</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B269" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C269" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D269" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B270" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C270" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D270" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B271" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C271" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Ikuti Google Maps Niat Hindari Macet ke Tol Purwomartani, Pemudik Malah Masuk Jalan Persawahan</t>
+        </is>
+      </c>
+      <c r="D271" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/jawa-tengah/read/2026/03/27/061500188/berita-foto--ikuti-google-maps-niat-hindari-macet-ke-tol</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B272" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C272" t="inlineStr">
+        <is>
+          <t>Anwar Ibrahim Beberkan Obrolan dengan Prabowo</t>
+        </is>
+      </c>
+      <c r="D272" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094847/anwar-ibrahim-beberkan-obrolan-dengan-prabowo</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B273" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C273" t="inlineStr">
+        <is>
+          <t>ASN Didorong Hemat Energi, Bupati Rudy Susmanto Berlakukan WFH Tiap Jumat</t>
+        </is>
+      </c>
+      <c r="D273" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094845/asn-didorong-hemat-energi-bupati-rudy-susmanto-berlakukan-wfh-tiap-jumat</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B274" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C274" t="inlineStr">
+        <is>
+          <t>Prabowo Bertemu Anwar Ibrahim, Teddy: Bahas Isu Strategis</t>
+        </is>
+      </c>
+      <c r="D274" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094842/prabowo-bertemu-anwar-ibrahim-teddy-bahas-isu-strategis</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B275" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C275" t="inlineStr">
+        <is>
+          <t>Radea Respati: Evaluasi ASN Kunci Tingkatkan Responsivitas Pemerintah</t>
+        </is>
+      </c>
+      <c r="D275" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094841/radea-respati-evaluasi-asn-kunci-tingkatkan-responsivitas-pemerintah</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B276" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C276" t="inlineStr">
+        <is>
+          <t>Purbaya Ungkap Anak Buah "Nakal" Jadi Alasan Coretax Lemot</t>
+        </is>
+      </c>
+      <c r="D276" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094838/purbaya-ungkap-anak-buah-nakal-jadi-alasan-coretax-lemot</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B277" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C277" t="inlineStr">
+        <is>
+          <t>Prabowo Menerima Menteri Keamanan Negara Cina</t>
+        </is>
+      </c>
+      <c r="D277" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094828/prabowo-menerima-menteri-keamanan-negara-cina</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B278" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C278" t="inlineStr">
+        <is>
+          <t>GEM Group Dorong Hilirisasi Nikel, Perkuat Posisi Indonesia di Rantai Pasok Baterai Global</t>
+        </is>
+      </c>
+      <c r="D278" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094820/gem-group-dorong-hilirisasi-nikel-perkuat-posisi-indonesia-di-rantai-pasok-baterai-global</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B279" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C279" t="inlineStr">
+        <is>
+          <t>Ketua DPRD Kabupaten Bogor: Silaturahmi Tingkatkan Kualitas Kerja dan Pelayanan Publik</t>
+        </is>
+      </c>
+      <c r="D279" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094819/ketua-dprd-kabupaten-bogor-silaturahmi-tingkatkan-kualitas-kerja-dan-pelayanan-publik</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B280" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C280" t="inlineStr">
+        <is>
+          <t>Komnas HAM Minta Eks Kepala BAIS TNI Diperiksa Kasus Andrie</t>
+        </is>
+      </c>
+      <c r="D280" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094812/komnas-ham-minta-eks-kepala-bais-tni-diperiksa-kasus-andrie</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B281" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C281" t="inlineStr">
+        <is>
+          <t>Anwar Ibrahim Kunjungi Prabowo: Bahas Situasi Regional</t>
+        </is>
+      </c>
+      <c r="D281" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094803/anwar-ibrahim-kunjungi-prabowo-bahas-situasi-regional</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B282" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C282" t="inlineStr">
+        <is>
+          <t>Tanggapan Panitia SNPMB Ihwal Keluhan Lokasi UTBK 2026</t>
+        </is>
+      </c>
+      <c r="D282" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094797/tanggapan-panitia-snpmb-ihwal-keluhan-lokasi-utbk-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B283" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C283" t="inlineStr">
+        <is>
+          <t>Prabowo Bertemu Ray Dalio di Istana, Bahas Apa?</t>
+        </is>
+      </c>
+      <c r="D283" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094796/prabowo-bertemu-ray-dalio-di-istana-bahas-apa</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B284" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C284" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota Padang akan Kurangi Volume Timbunan Sampah dengan Bangun PSEL</t>
+        </is>
+      </c>
+      <c r="D284" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094792/pemerintah-kota-padang-akan-kurangi-volume-timbunan-sampah-dengan-bangun-psel</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B285" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C285" t="inlineStr">
+        <is>
+          <t>Airlangga: Kebijakan WFH 1 Hari Sepekan Ditetapkan Bulan Ini</t>
+        </is>
+      </c>
+      <c r="D285" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094790/airlangga-kebijakan-wfh-1-hari-sepekan-ditetapkan-bulan-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B286" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C286" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota Padang akan Kurangi VolumeTimbunan Sampah dengan Bangun PSEL</t>
+        </is>
+      </c>
+      <c r="D286" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094789/pemerintah-kota-padang-akan-kurangi-volumetimbunan-sampah-dengan-bangun-psel</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B287" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C287" t="inlineStr">
+        <is>
+          <t>Indonesia, China boost security ties amid global tensions</t>
+        </is>
+      </c>
+      <c r="D287" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410086/indonesia-china-boost-security-ties-amid-global-tensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B288" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C288" t="inlineStr">
+        <is>
+          <t>Indonesian President Prabowo welcomes Malaysian PM Anwar in Jakarta</t>
+        </is>
+      </c>
+      <c r="D288" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410082/indonesian-president-prabowo-welcomes-malaysian-pm-anwar-in-jakarta</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B289" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C289" t="inlineStr">
+        <is>
+          <t>Indonesian govt flags Wikimedia Commons, urges ESP registration</t>
+        </is>
+      </c>
+      <c r="D289" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410078/indonesian-govt-flags-wikimedia-commons-urges-esp-registration</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B290" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C290" t="inlineStr">
+        <is>
+          <t>Chinese national arrested for drug smuggling at Soekarno-Hatta airport</t>
+        </is>
+      </c>
+      <c r="D290" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410074/chinese-national-arrested-for-drug-smuggling-at-soekarno-hatta-airport</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B291" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C291" t="inlineStr">
+        <is>
+          <t>Prabowo hosts China's state security minister for stability talks</t>
+        </is>
+      </c>
+      <c r="D291" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410070/prabowo-hosts-chinas-state-security-minister-for-stability-talks</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B292" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C292" t="inlineStr">
+        <is>
+          <t>RI in intense talk with Iran to ensure Pertamina tankers leave Hormuz</t>
+        </is>
+      </c>
+      <c r="D292" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410066/ri-in-intense-talk-with-iran-to-ensure-pertamina-tankers-leave-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B293" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C293" t="inlineStr">
+        <is>
+          <t>Prabowo, Dalio discuss Danantara's role as driver of economic growth</t>
+        </is>
+      </c>
+      <c r="D293" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410062/prabowo-dalio-discuss-danantaras-role-as-driver-of-economic-growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B294" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C294" t="inlineStr">
+        <is>
+          <t>Ministry hopes women, child protection can start from villages</t>
+        </is>
+      </c>
+      <c r="D294" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410058/ministry-hopes-women-child-protection-can-start-from-villages</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B295" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C295" t="inlineStr">
+        <is>
+          <t>Gov't to announce one-day weekly WFH policy before March end</t>
+        </is>
+      </c>
+      <c r="D295" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410054/govt-to-announce-one-day-weekly-wfh-policy-before-march-end</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B296" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C296" t="inlineStr">
+        <is>
+          <t>Prabowo-Anwar meeting in Jakarta to discuss Iran-Israel-US conflict</t>
+        </is>
+      </c>
+      <c r="D296" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410050/prabowo-anwar-meeting-in-jakarta-to-discuss-iran-israel-us-conflict</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B297" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C297" t="inlineStr">
+        <is>
+          <t>1,790 athletes to compete in Sanya Asian Beach Games</t>
+        </is>
+      </c>
+      <c r="D297" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410046/1790-athletes-to-compete-in-sanya-asian-beach-games</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B298" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C298" t="inlineStr">
+        <is>
+          <t>Polyplastics’ DURACON(R) POM Adopted for Ground-breaking Crawler Transport System</t>
+        </is>
+      </c>
+      <c r="D298" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410042/polyplastics-duraconr-pom-adopted-for-ground-breaking-crawler-transport-system</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B299" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C299" t="inlineStr">
+        <is>
+          <t>Indonesia's Parliament to cut electricity overnight starting March 30</t>
+        </is>
+      </c>
+      <c r="D299" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410038/indonesias-parliament-to-cut-electricity-overnight-starting-march-30</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B300" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C300" t="inlineStr">
+        <is>
+          <t>NX Group Integrates Business Companies in Indonesia</t>
+        </is>
+      </c>
+      <c r="D300" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410034/nx-group-integrates-business-companies-in-indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>Saturday, 28 March 2026</t>
+        </is>
+      </c>
+      <c r="B301" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C301" t="inlineStr">
+        <is>
+          <t>Indonesia sets 2 million cattle target to boost meat, milk production</t>
+        </is>
+      </c>
+      <c r="D301" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410030/indonesia-sets-2-million-cattle-target-to-boost-meat-milk-production</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D241"/>
+  <autoFilter ref="A1:D301"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -5993,6 +7313,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D239" r:id="rId238"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D240" r:id="rId239"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D241" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D242" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D243" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D244" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D245" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D246" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D247" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D248" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D249" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D250" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D251" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D252" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D253" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D254" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D255" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D256" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D257" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D258" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D259" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D260" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D261" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D262" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D263" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D264" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D265" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D266" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D267" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D268" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D269" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D270" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D271" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D272" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D273" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D274" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D275" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D276" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D277" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D278" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D279" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D280" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D281" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D282" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D283" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D284" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D285" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D286" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D287" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D288" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D289" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D290" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D291" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D292" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D293" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D294" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D295" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D296" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D297" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D298" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D299" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D300" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D301" r:id="rId300"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-03-28
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$301</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$361</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D301"/>
+  <dimension ref="A1:D361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -7070,8 +7070,1328 @@
         </is>
       </c>
     </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B302" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C302" t="inlineStr">
+        <is>
+          <t>Video: H+7 Lebaran, 52 Ribu Penumpang KA Tiba di Jakarta</t>
+        </is>
+      </c>
+      <c r="D302" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260328-260328013/video-h7-lebaran-52-ribu-penumpang-ka-tiba-di-jakarta-</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B303" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C303" t="inlineStr">
+        <is>
+          <t>Video: Arus Balik Lebaran, 1.145 Pemudik Kembali ke Terminal Kampung Rambutan</t>
+        </is>
+      </c>
+      <c r="D303" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260328-260328010/video-arus-balik-lebaran-1145-pemudik-kembali-ke-terminal-kampung-rambutan</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B304" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C304" t="inlineStr">
+        <is>
+          <t>Video KuTips: Susah Tidur Habis Liburan? Coba Metode Pernapasan 4-7-8 Deh!</t>
+        </is>
+      </c>
+      <c r="D304" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/detiktv/d-8418758/video-kutips-susah-tidur-habis-liburan-coba-metode-pernapasan-4-7-8-deh</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B305" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C305" t="inlineStr">
+        <is>
+          <t>Cerita Viral Mudik Naik Motor, Istri Diikat Sarung agar Tetap Aman</t>
+        </is>
+      </c>
+      <c r="D305" s="2" t="inlineStr">
+        <is>
+          <t>https://wolipop.detik.com/entertainment-news/d-8418136/cerita-viral-mudik-naik-motor-istri-diikat-sarung-agar-tetap-aman</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B306" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C306" t="inlineStr">
+        <is>
+          <t>Tiket Indonesia Vs Bulgaria Masih Tersedia, Segini Harganya</t>
+        </is>
+      </c>
+      <c r="D306" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8419501/tiket-indonesia-vs-bulgaria-masih-tersedia-segini-harganya</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B307" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C307" t="inlineStr">
+        <is>
+          <t>Tiap Makan Menunya Itu-itu Saja? Ada Bagusnya, Riset Bilang Itu Bikin Cepat Kurus</t>
+        </is>
+      </c>
+      <c r="D307" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/diet/d-8419439/tiap-makan-menunya-itu-itu-saja-ada-bagusnya-riset-bilang-itu-bikin-cepat-kurus</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B308" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C308" t="inlineStr">
+        <is>
+          <t>Tak Melulu Buntung, Konflik Timur Tengah Bisa Bikin Wisata ASEAN Untung</t>
+        </is>
+      </c>
+      <c r="D308" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.detik.com/travel-news/d-8419324/tak-melulu-buntung-konflik-timur-tengah-bisa-bikin-wisata-asean-untung</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B309" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C309" t="inlineStr">
+        <is>
+          <t>Ini Ole Romeny yang Baru</t>
+        </is>
+      </c>
+      <c r="D309" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8419362/ini-ole-romeny-yang-baru</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B310" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C310" t="inlineStr">
+        <is>
+          <t>Video: Lebaran Jadi Lebar-an? Ini Tips Diet Biar BB Balik Lagi</t>
+        </is>
+      </c>
+      <c r="D310" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/detiktv/d-8419492/video-lebaran-jadi-lebar-an-ini-tips-diet-biar-bb-balik-lagi</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B311" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C311" t="inlineStr">
+        <is>
+          <t>Fortuner Bawa 5 Pemudik Nyemplung ke Saluran Irigasi di OKU Timur Sulsel</t>
+        </is>
+      </c>
+      <c r="D311" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8419860/fortuner-bawa-5-pemudik-nyemplung-ke-saluran-irigasi-di-oku-timur-sulsel</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B312" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C312" t="inlineStr">
+        <is>
+          <t>Arus Balik Lebaran, 22 Persen Kendaraan Belum Kembali ke Jakarta</t>
+        </is>
+      </c>
+      <c r="D312" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8419027/arus-balik-lebaran-22-persen-kendaraan-belum-kembali-ke-jakarta</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B313" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C313" t="inlineStr">
+        <is>
+          <t>Pemotor Remaja di Puncak Bogor Tewas Usai Jatuh Lalu Tertabrak Motor Lain</t>
+        </is>
+      </c>
+      <c r="D313" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8418881/pemotor-remaja-di-puncak-bogor-tewas-usai-jatuh-lalu-tertabrak-motor-lain</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B314" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C314" t="inlineStr">
+        <is>
+          <t>Chemistry Beckham-Romeny</t>
+        </is>
+      </c>
+      <c r="D314" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sportstyle/d-8419552/chemistry-beckham-romeny</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B315" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C315" t="inlineStr">
+        <is>
+          <t>Hasil Sprint Race MotoGP Amerika 2026: Jorge Martin Pemenangnya</t>
+        </is>
+      </c>
+      <c r="D315" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/moto-gp/d-8419859/hasil-sprint-race-motogp-amerika-2026-jorge-martin-pemenangnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>Kasus Pembunuhan Bule Belanda di Bali, 2 WNA Ditetapkan Tersangka!</t>
+        </is>
+      </c>
+      <c r="D316" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/bali/hukum-dan-kriminal/d-8419526/kasus-pembunuhan-bule-belanda-di-bali-2-wna-ditetapkan-tersangka</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>Museum Sejarah Jakarta di Kota Tua Jadi Favorit Wisatawan Habiskan Libur Lebaran</t>
+        </is>
+      </c>
+      <c r="D317" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1919878/museum-sejarah-jakarta-di-kota-tua-jadi-favorit-wisatawan-habiskan-libur-lebaran?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>Iran dan Resiliensi Intelektual</t>
+        </is>
+      </c>
+      <c r="D318" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/iran-dan-resiliensi-intelektual?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>Menteri PU Tinjau Langsung Lokasi Banjir di Brebes, Bupati Paramitha: Ini Kepedulian Pemerintah Pusat</t>
+        </is>
+      </c>
+      <c r="D319" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/03/28/223901378/menteri-pu-tinjau-langsung-lokasi-banjir-di-brebes-bupati-paramitha-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>Satgas PRR Terus Percepat Pembersihan Lumpur dan Rehabilitasi Sawah di Aceh, Sumut, dan Sumbar</t>
+        </is>
+      </c>
+      <c r="D320" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/28/21055401/satgas-prr-terus-percepat-pembersihan-lumpur-dan-rehabilitasi-sawah-di-aceh</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>Atasi Masalah Sampah, Pemkot Semarang Tanda Tangani Kerja Sama Penyelenggaraan PSEL</t>
+        </is>
+      </c>
+      <c r="D321" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/03/28/190755878/atasi-masalah-sampah-pemkot-semarang-tanda-tangani-kerja-sama</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D322" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D323" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D324" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D325" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>Mengenal Balendra Shah, Eks Rapper Pembangkang Jadi PM Nepal yang Baru</t>
+        </is>
+      </c>
+      <c r="D326" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1919842/mengenal-balendra-shah-eks-rapper-pembangkang-jadi-pm-nepal-yang-baru?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>Kenangan yang Tersisa dari Pabrik Benang Sutra Regaloh</t>
+        </is>
+      </c>
+      <c r="D327" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/hestri09924/69c74251ed64153d2229b133/kenangan-yang-tersisa-dari-pabrik-benang-sutra-regaloh</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>Festival Inuyama di Jepang, Tradisi Arak-arakan Kereta Hias Sejak Zaman Edo</t>
+        </is>
+      </c>
+      <c r="D328" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5709/festival-inuyama-di-jepang-tradisi-arak-arakan-kereta-hias-sejak-zaman-edo</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D329" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D330" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Ikuti Google Maps Niat Hindari Macet ke Tol Purwomartani, Pemudik Malah Masuk Jalan Persawahan</t>
+        </is>
+      </c>
+      <c r="D331" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/jawa-tengah/read/2026/03/27/061500188/berita-foto--ikuti-google-maps-niat-hindari-macet-ke-tol</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>Anggota DPR Desak Kasus Andrie Ditetapkan Pelanggaran HAM</t>
+        </is>
+      </c>
+      <c r="D332" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094970/anggota-dpr-desak-kasus-andrie-ditetapkan-pelanggaran-ham</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>Arus Balik Bakauheni-Merak Terkendali, 72 Persen Pemudik Sudah Kembali ke Jawa</t>
+        </is>
+      </c>
+      <c r="D333" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094966/arus-balik-bakauheni-merak-terkendali-72-persen-pemudik-sudah-kembali-ke-jawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>Kemenag Kecam Kasus Penganiayaan Murid TPQ di Probolinggo</t>
+        </is>
+      </c>
+      <c r="D334" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094965/kemenag-kecam-kasus-penganiayaan-murid-tpq-di-probolinggo</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>Dukung Earth Hour 2026, BNI Padamkan Lampu Serentak dan Perkuat Komitmen Rendah Emisi</t>
+        </is>
+      </c>
+      <c r="D335" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094963/dukung-earth-hour-2026-bni-padamkan-lampu-serentak-dan-perkuat-komitmen-rendah-emisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>PP Tunas Berlaku, Meutya Minta Platform Digital Mengikuti</t>
+        </is>
+      </c>
+      <c r="D336" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094961/pp-tunas-berlaku-meutya-minta-platform-digital-mengikuti</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>Gubernur Mirza Dampingi Kapolri Pantau Arus Balik di Bakauheni: Situasi Terkendali</t>
+        </is>
+      </c>
+      <c r="D337" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094958/gubernur-mirza-dampingi-kapolri-pantau-arus-balik-di-bakauheni-situasi-terkendali</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>Menhan Sjafrie Akan Pimpin Pemakaman Juwono Sudarsono</t>
+        </is>
+      </c>
+      <c r="D338" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094951/menhan-sjafrie-akan-pimpin-pemakaman-juwono-sudarsono</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>Peran Kemenag dalam Pembatasan Akses Anak di Medsos</t>
+        </is>
+      </c>
+      <c r="D339" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094940/peran-kemenag-dalam-pembatasan-akses-anak-di-medsos</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>Mantan Menteri Pertahanan Juwono Sudarsono Meninggal</t>
+        </is>
+      </c>
+      <c r="D340" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094938/mantan-menteri-pertahanan-juwono-sudarsono-meninggal</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>Kuota Mahasiswa S1 ITB 2026 Dipangkas Sebanyak 12 Persen</t>
+        </is>
+      </c>
+      <c r="D341" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094934/kuota-mahasiswa-s1-itb-2026-dipangkas-sebanyak-12-persen</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>Prabowo Instruksikan Pasar Murah Digelar di Monas</t>
+        </is>
+      </c>
+      <c r="D342" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094930/prabowo-instruksikan-pasar-murah-digelar-di-monas</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>Anggota DPR: WFH Bukan Solusi Tunggal Hemat Energi</t>
+        </is>
+      </c>
+      <c r="D343" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094929/anggota-dpr-wfh-bukan-solusi-tunggal-hemat-energi</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>Raja Juli Dampingi Prabowo ke Jepang-Korea Selatan</t>
+        </is>
+      </c>
+      <c r="D344" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094924/raja-juli-dampingi-prabowo-ke-jepang-korea-selatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>Gus Ipul: 2.708 Pegawai Kemensos Bolos Kerja Setelah Lebaran</t>
+        </is>
+      </c>
+      <c r="D345" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094918/gus-ipul-2-708-pegawai-kemensos-bolos-kerja-setelah-lebaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>Penjelasan TNI AD Soal Isi Video Viral Prajurit Beli Narkoba</t>
+        </is>
+      </c>
+      <c r="D346" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2094917/penjelasan-tni-ad-soal-isi-video-viral-prajurit-beli-narkoba</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>Indonesia's Hajj preparations for 2026 near 100 percent completion</t>
+        </is>
+      </c>
+      <c r="D347" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410226/indonesias-hajj-preparations-for-2026-near-100-percent-completion</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>Indonesia's NTT targets June completion for Nat'l Salt Industry Center</t>
+        </is>
+      </c>
+      <c r="D348" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410222/indonesias-ntt-targets-june-completion-for-natl-salt-industry-center</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>Indonesia pushes downstream strategy to boost economy, end raw exports</t>
+        </is>
+      </c>
+      <c r="D349" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410218/indonesia-pushes-downstream-strategy-to-boost-economy-end-raw-exports</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>Bali's survival strategies as global conflict disrupts travel</t>
+        </is>
+      </c>
+      <c r="D350" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410214/balis-survival-strategies-as-global-conflict-disrupts-travel</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>Bali Police name two Brazilians as suspects in Dutch man's killing</t>
+        </is>
+      </c>
+      <c r="D351" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410210/bali-police-name-two-brazilians-as-suspects-in-dutch-mans-killing</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>Bali Immigration thwarts escape attempt of British Interpol fugitive</t>
+        </is>
+      </c>
+      <c r="D352" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410206/bali-immigration-thwarts-escape-attempt-of-british-interpol-fugitive</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>Indonesia's Eid travel accidents drop 7.8 pct despite surge: Police</t>
+        </is>
+      </c>
+      <c r="D353" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410202/indonesias-eid-travel-accidents-drop-78-pct-despite-surge-police</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>Teachers urged to bolster digital literacy for 'Tunas' regulation</t>
+        </is>
+      </c>
+      <c r="D354" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410198/teachers-urged-to-bolster-digital-literacy-for-tunas-regulation</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>Indonesia braces for Eid return peak at Ketapang Port East Java</t>
+        </is>
+      </c>
+      <c r="D355" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410194/indonesia-braces-for-eid-return-peak-at-ketapang-port-east-java</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>Indonesian restaurants shine in Asia’s 50 Best 2026</t>
+        </is>
+      </c>
+      <c r="D356" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410190/indonesian-restaurants-shine-in-asias-50-best-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>Govt to study impact of child protection rule</t>
+        </is>
+      </c>
+      <c r="D357" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410186/govt-to-study-impact-of-child-protection-rule</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>Yadea's Strong Sales Surge Worldwide Drives the Shift Toward Green Mobility</t>
+        </is>
+      </c>
+      <c r="D358" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410182/yadeas-strong-sales-surge-worldwide-drives-the-shift-toward-green-mobility</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>[MWC 2026] Preparing for AI Calling: Ookla's Vision for Updated Voice Quality Standards</t>
+        </is>
+      </c>
+      <c r="D359" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410178/mwc-2026-preparing-for-ai-calling-ooklas-vision-for-updated-voice-quality-standards</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>Indonesia starts talks to secure tanker passage through Hormuz</t>
+        </is>
+      </c>
+      <c r="D360" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410174/indonesia-starts-talks-to-secure-tanker-passage-through-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>Sunday, 29 March 2026</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>MTR Lab and ZGC Science City Ltd Establish Ecosystem Partnership</t>
+        </is>
+      </c>
+      <c r="D361" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410170/mtr-lab-and-zgc-science-city-ltd-establish-ecosystem-partnership</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D301"/>
+  <autoFilter ref="A1:D361"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -7373,6 +8693,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D299" r:id="rId298"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D300" r:id="rId299"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D301" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D302" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D303" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D304" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D305" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D306" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D307" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D308" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D309" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D310" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D311" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D312" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D313" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D314" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D315" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D316" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D317" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D318" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D319" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D320" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D321" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D322" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D323" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D324" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D325" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D326" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D327" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D328" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D329" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D330" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D331" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D332" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D333" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D334" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D335" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D336" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D337" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D338" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D339" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D340" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D341" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D342" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D343" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D344" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D345" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D346" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D347" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D348" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D349" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D350" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D351" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D352" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D353" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D354" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D355" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D356" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D357" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D358" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D359" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D360" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D361" r:id="rId360"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-03-29
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$361</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$421</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D361"/>
+  <dimension ref="A1:D421"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -8390,8 +8390,1328 @@
         </is>
       </c>
     </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>Video Stasiun Pasar Senen Masih Dipadati Pemudik pada H+7 Lebaran</t>
+        </is>
+      </c>
+      <c r="D362" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260329-260329011/video-stasiun-pasar-senen-masih-dipadati-pemudik-pada-h7-lebaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>Antrean BBM di SPBU Massemba Enrekang Mengular hingga 1 Km Sejak Pagi</t>
+        </is>
+      </c>
+      <c r="D363" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/sulsel/berita/d-8420312/antrean-bbm-di-spbu-massemba-enrekang-mengular-hingga-1-km-sejak-pagi</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>Video: Tips Mengelola Konsentrasi dan Kebugaran Tubuh di Tengah Perjalanan Panjang</t>
+        </is>
+      </c>
+      <c r="D364" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260329-260329004/video-tips-mengelola-konsentrasi-dan-kebugaran-tubuh-di-tengah-perjalanan-panjang--</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>Video: H+7 Lebaran, 52 Ribu Penumpang KA Tiba di Jakarta</t>
+        </is>
+      </c>
+      <c r="D365" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260328-260328013/video-h7-lebaran-52-ribu-penumpang-ka-tiba-di-jakarta-</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>Rusia Setop Ekspor Bensin Mulai April!</t>
+        </is>
+      </c>
+      <c r="D366" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8420661/rusia-setop-ekspor-bensin-mulai-april</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>Cerita Wanita Tasikmalaya Harus Makan Lewat Selang, Berawal dari Sakit Tenggorokan</t>
+        </is>
+      </c>
+      <c r="D367" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/true-story/d-8420425/cerita-wanita-tasikmalaya-harus-makan-lewat-selang-berawal-dari-sakit-tenggorokan</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>8 Jam Mewah Georgina Rodriguez, Pacar Ronaldo, Setara Rumah Miliaran</t>
+        </is>
+      </c>
+      <c r="D368" s="2" t="inlineStr">
+        <is>
+          <t>https://wolipop.detik.com/celeb-style/d-8420111/8-jam-mewah-georgina-rodriguez-pacar-ronaldo-setara-rumah-miliaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>OECD Prediksi Ekonomi Global Makin Loyo Gara-gara Perang Timur Tengah</t>
+        </is>
+      </c>
+      <c r="D369" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8420451/oecd-prediksi-ekonomi-global-makin-loyo-gara-gara-perang-timur-tengah</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>Akses Medsos Resmi Dibatasi, Pemerintah Bakal Evaluasi Dampaknya ke Mental Anak</t>
+        </is>
+      </c>
+      <c r="D370" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8420352/akses-medsos-resmi-dibatasi-pemerintah-bakal-evaluasi-dampaknya-ke-mental-anak</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>Hasil MotoGP Amerika Serikat 2026: Bezzecchi Juara, Marc Marquez ke-5</t>
+        </is>
+      </c>
+      <c r="D371" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/moto-gp/d-8420961/hasil-motogp-amerika-serikat-2026-bezzecchi-juara-marc-marquez-ke-5</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>Link Live Streaming MotoGP Amerika dan Balapan Veda Ega</t>
+        </is>
+      </c>
+      <c r="D372" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/moto-gp/d-8420460/link-live-streaming-motogp-amerika-dan-balapan-veda-ega</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>Starting Grid MotoGP Amerika 2026: Perubahan usai Penalti</t>
+        </is>
+      </c>
+      <c r="D373" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/moto-gp/d-8420379/starting-grid-motogp-amerika-2026-perubahan-usai-penalti</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>Veda Ega Crash, Gagal Finis di Moto3 Amerika Serikat</t>
+        </is>
+      </c>
+      <c r="D374" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/moto-gp/d-8420938/veda-ega-crash-gagal-finis-di-moto3-amerika-serikat</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>Daniel Sturridge Sapa Fans Liverpool di Jakarta</t>
+        </is>
+      </c>
+      <c r="D375" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8420956/daniel-sturridge-sapa-fans-liverpool-di-jakarta</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>Igor Tudor Resmi Tinggalkan Tottenham Hotspur</t>
+        </is>
+      </c>
+      <c r="D376" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8420915/igor-tudor-resmi-tinggalkan-tottenham-hotspur</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>Jejak Stasiun Mampang yang Pernah Layani Warga Menteng</t>
+        </is>
+      </c>
+      <c r="D377" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1920003/jejak-stasiun-mampang-yang-pernah-layani-warga-menteng?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>Ketika Perang Membuat Bumi Makin Panas</t>
+        </is>
+      </c>
+      <c r="D378" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/ketika-perang-semakin-membakar-bumi?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>Kunjungi PLBN Long Nawang, Wakil Menteri Digital Sarawak Bahas Penguatan Konektivitas Perbatasan</t>
+        </is>
+      </c>
+      <c r="D379" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/29/19340651/kunjungi-plbn-long-nawang-wakil-menteri-digital-sarawak-bahas-penguatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>Arus Balik Lebaran 1447 H di PLBN Skouw Melandai, Posko Kesehatan Tetap Siaga hingga Akhir Maret</t>
+        </is>
+      </c>
+      <c r="D380" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/29/18460071/arus-balik-lebaran-1447-h-di-plbn-skouw-melandai-posko-kesehatan-tetap-siaga</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>PLBN Jagoi Babang Terima Kunjungan Panglima Tentera Darat Malaysia, Perkuat Koordinasi Pengamanan Perbatasan</t>
+        </is>
+      </c>
+      <c r="D381" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/29/18382261/plbn-jagoi-babang-terima-kunjungan-panglima-tentera-darat-malaysia-perkuat</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D382" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D383" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D384" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D385" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>Taktik Iran Kuras Pertahanan Berlapis Israel, Kini Stok Rudal Pencegat IDF Menipis?</t>
+        </is>
+      </c>
+      <c r="D386" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1919983/taktik-iran-kuras-pertahanan-berlapis-israel-kini-stok-rudal-pencegat-idf-menipis?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>Berceritalah</t>
+        </is>
+      </c>
+      <c r="D387" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/pramahyjore9775/69c520c7c925c4558b386912/berceritalah</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>Resep Somage, Bola-bola Tepung Soba dengan Kuah dan Sayuran</t>
+        </is>
+      </c>
+      <c r="D388" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5717/resep-somage-bola-bola-tepung-soba-dengan-kuah-dan-sayuran</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D389" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D390" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Ikuti Google Maps Niat Hindari Macet ke Tol Purwomartani, Pemudik Malah Masuk Jalan Persawahan</t>
+        </is>
+      </c>
+      <c r="D391" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/jawa-tengah/read/2026/03/27/061500188/berita-foto--ikuti-google-maps-niat-hindari-macet-ke-tol</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>Prabowo Melawat ke Jepang Atas Undangan Kaisar Naruhito</t>
+        </is>
+      </c>
+      <c r="D392" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095113/prabowo-melawat-ke-jepang-atas-undangan-kaisar-naruhito</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>SETARA: Hanya TGPF Opsi Penyelesaian Kasus Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D393" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095112/setara-hanya-tgpf-opsi-penyelesaian-kasus-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>Tiba di Jepang, Prabowo Akan Temui Kaisar Naruhito-PM Sanae</t>
+        </is>
+      </c>
+      <c r="D394" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095110/tiba-di-jepang-prabowo-akan-temui-kaisar-naruhito-pm-sanae</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>Pramono Dukung Prabowo Bangun Hunian untuk Warga Pinggir Rel</t>
+        </is>
+      </c>
+      <c r="D395" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095098/pramono-dukung-prabowo-bangun-hunian-untuk-warga-pinggir-rel</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>Pramono: DKI Berusaha Agar PPPK Tak Diberhentikan</t>
+        </is>
+      </c>
+      <c r="D396" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095095/pramono-dki-berusaha-agar-pppk-tak-diberhentikan</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>Siswa di Daerah 3T dan Rawan Stunting Dapat MBG 6 Hari</t>
+        </is>
+      </c>
+      <c r="D397" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095082/siswa-di-daerah-3t-dan-rawan-stunting-dapat-mbg-6-hari</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>Prabowo ke Jepang Bahas Perdagangan hingga Teknologi</t>
+        </is>
+      </c>
+      <c r="D398" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095078/prabowo-ke-jepang-bahas-perdagangan-hingga-teknologi</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>Terima Hercules di Kantornya, Seskab Teddy: Kawan Lama</t>
+        </is>
+      </c>
+      <c r="D399" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095071/terima-hercules-di-kantornya-seskab-teddy-kawan-lama</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>Menhub Dudy Pastikan Arus Balik di Pelabuhan Bakauheni Lancar</t>
+        </is>
+      </c>
+      <c r="D400" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095070/menhub-dudy-pastikan-arus-balik-di-pelabuhan-bakauheni-lancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>Prabowo Bahas Usul Penghematan Energi dengan Para Menteri</t>
+        </is>
+      </c>
+      <c r="D401" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095059/prabowo-bahas-usul-penghematan-energi-dengan-para-menteri</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>DPR Berhemat, Nurul: Jangan Sampai Ganggu Kinerja Legislatif</t>
+        </is>
+      </c>
+      <c r="D402" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095055/dpr-berhemat-nurul-jangan-sampai-ganggu-kinerja-legislatif</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>Bercermin dari Suara Rakyat Maluku Utara</t>
+        </is>
+      </c>
+      <c r="D403" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095046/bercermin-dari-suara-rakyat-maluku-utara</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>Prabowo Terbang ke Jepang, Bakal Bertemu Kaisar Naruhito</t>
+        </is>
+      </c>
+      <c r="D404" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095043/prabowo-terbang-ke-jepang-bakal-bertemu-kaisar-naruhito</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>Pemerintah Kota Banda Aceh : Kerja Maksimal Meski Terimpit Fiskal</t>
+        </is>
+      </c>
+      <c r="D405" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095030/pemerintah-kota-banda-aceh-kerja-maksimal-meski-terimpit-fiskal</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>Pasar Murah di Monas Berpeluang Jadi Agenda Rutin</t>
+        </is>
+      </c>
+      <c r="D406" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095029/pasar-murah-di-monas-berpeluang-jadi-agenda-rutin</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>Bulog, BRIN expand tech partnership for food security</t>
+        </is>
+      </c>
+      <c r="D407" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410306/bulog-brin-expand-tech-partnership-for-food-security</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>Russian fleets arrive in Jakarta for joint drills with Indonesian Navy</t>
+        </is>
+      </c>
+      <c r="D408" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410302/russian-fleets-arrive-in-jakarta-for-joint-drills-with-indonesian-navy</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>President Prabowo arrives in Tokyo for first official Japan visit</t>
+        </is>
+      </c>
+      <c r="D409" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410298/president-prabowo-arrives-in-tokyo-for-first-official-japan-visit</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>Indonesia builds facilities for 34,000 village co-ops, 2,500 finished</t>
+        </is>
+      </c>
+      <c r="D410" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410294/indonesia-builds-facilities-for-34000-village-co-ops-2500-finished</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>Indonesia coordinates for safety of its vessels in Strait of Hormuz</t>
+        </is>
+      </c>
+      <c r="D411" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410290/indonesia-coordinates-for-safety-of-its-vessels-in-strait-of-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>Legislator hails 'Tunas' Regulation as investment in children</t>
+        </is>
+      </c>
+      <c r="D412" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410286/legislator-hails-tunas-regulation-as-investment-in-children</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>Prabowo eyes trade, technology, forestry ties through Japan visit</t>
+        </is>
+      </c>
+      <c r="D413" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410282/prabowo-eyes-trade-technology-forestry-ties-through-japan-visit</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>Ministry promotes 'Seven Great Habits' amid under-16 social media ban</t>
+        </is>
+      </c>
+      <c r="D414" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410278/ministry-promotes-seven-great-habits-amid-under-16-social-media-ban</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>Indonesia's BGN to maintain six-day MBG rollout in priority regions</t>
+        </is>
+      </c>
+      <c r="D415" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410274/indonesias-bgn-to-maintain-six-day-mbg-rollout-in-priority-regions</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>Prabowo bound for Japan to meet Emperor Naruhito, PM Takaichi</t>
+        </is>
+      </c>
+      <c r="D416" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410270/prabowo-bound-for-japan-to-meet-emperor-naruhito-pm-takaichi</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>Batam immigration officer probed for extortion against foreigners</t>
+        </is>
+      </c>
+      <c r="D417" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410266/batam-immigration-officer-probed-for-extortion-against-foreigners</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>Lightning strike kills one, injures nine at Lumajang beaches</t>
+        </is>
+      </c>
+      <c r="D418" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410262/lightning-strike-kills-one-injures-nine-at-lumajang-beaches</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>SBY honors Juwono Sudarsono's role in military-civilian unity</t>
+        </is>
+      </c>
+      <c r="D419" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410258/sby-honors-juwono-sudarsonos-role-in-military-civilian-unity</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>Gov't ensures optimal rice production ahead of dry season</t>
+        </is>
+      </c>
+      <c r="D420" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410254/govt-ensures-optimal-rice-production-ahead-of-dry-season</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>Monday, 30 March 2026</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>Minister ensures smooth Eid return flow on Sumatra-Java crossing</t>
+        </is>
+      </c>
+      <c r="D421" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410250/minister-ensures-smooth-eid-return-flow-on-sumatra-java-crossing</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D361"/>
+  <autoFilter ref="A1:D421"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -8753,6 +10073,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D359" r:id="rId358"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D360" r:id="rId359"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D361" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D362" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D363" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D364" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D365" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D366" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D367" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D368" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D369" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D370" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D371" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D372" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D373" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D374" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D375" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D376" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D377" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D378" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D379" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D380" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D381" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D382" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D383" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D384" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D385" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D386" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D387" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D388" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D389" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D390" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D391" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D392" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D393" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D394" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D395" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D396" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D397" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D398" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D399" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D400" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D401" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D402" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D403" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D404" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D405" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D406" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D407" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D408" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D409" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D410" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D411" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D412" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D413" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D414" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D415" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D416" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D417" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D418" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D419" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D420" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D421" r:id="rId420"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-03-30
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$421</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$481</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D421"/>
+  <dimension ref="A1:D481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -9710,8 +9710,1328 @@
         </is>
       </c>
     </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>Bahlil Buka Suara soal Peluang BBM Nonsubsidi Naik: Ikut Harga Pasar!</t>
+        </is>
+      </c>
+      <c r="D422" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8422449/bahlil-buka-suara-soal-peluang-bbm-nonsubsidi-naik-ikut-harga-pasar</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>Video Arti di Balik Nama AHY Junior: Arjuna Hanyokrokusumo Yudhoyono</t>
+        </is>
+      </c>
+      <c r="D423" s="2" t="inlineStr">
+        <is>
+          <t>https://wolipop.detik.com/detiktv/d-8422425/video-arti-di-balik-nama-ahy-junior-arjuna-hanyokrokusumo-yudhoyono</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>Momen Suporter Rebutan Foto Bareng 'Jay Idzes' dan 'Bepe' di GBK!</t>
+        </is>
+      </c>
+      <c r="D424" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sportstyle/d-8422385/momen-suporter-rebutan-foto-bareng-jay-idzes-dan-bepe-di-gbk</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>Manchester City Siapkan Rp 4 Triliun Beli Dua Gelandang Ini</t>
+        </is>
+      </c>
+      <c r="D425" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8422051/manchester-city-siapkan-rp-4-triliun-beli-dua-gelandang-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>Banjir Berulang di Kota Lele</t>
+        </is>
+      </c>
+      <c r="D426" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/spotlight/d-8422221/banjir-berulang-di-kota-lele</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>Video: Dengar Lagi Pernyataan Prabowo soal Israel Harus Dijamin Keamanannya</t>
+        </is>
+      </c>
+      <c r="D427" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8422566/video-dengar-lagi-pernyataan-prabowo-soal-israel-harus-dijamin-keamanannya</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>Video: Komandan Iran yang Pimpin Penutupan Selat Hormuz Tewas</t>
+        </is>
+      </c>
+      <c r="D428" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8422342/video-komandan-iran-yang-pimpin-penutupan-selat-hormuz-tewas</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>Video: Identitas Prajurit TNI yang Gugur-Luka Akibat Serangan Israel di Lebanon</t>
+        </is>
+      </c>
+      <c r="D429" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8422013/video-identitas-prajurit-tni-yang-gugur-luka-akibat-serangan-israel-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>Indonesia Vs Bulgaria: RI Kalah 0-1 di Final FIFA Series 2026</t>
+        </is>
+      </c>
+      <c r="D430" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8422437/indonesia-vs-bulgaria-ri-kalah-0-1-di-final-fifa-series-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>Trump Ngaku AS Sedang Negosiasi dengan Ketua Parlemen Iran</t>
+        </is>
+      </c>
+      <c r="D431" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8422565/trump-ngaku-as-sedang-negosiasi-dengan-ketua-parlemen-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>Kabar Potensi Invasi Darat AS Tak Bikin Hiu-hiu Teluk Persia Gentar</t>
+        </is>
+      </c>
+      <c r="D432" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8422443/kabar-potensi-invasi-darat-as-tak-bikin-hiu-hiu-teluk-persia-gentar</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>Video Timnas Indonesia Dibungkam Bulgaria di Final FIFA Series</t>
+        </is>
+      </c>
+      <c r="D433" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260330-260330132/video-timnas-indonesia-dibungkam-bulgaria-di-final-fifa-series</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>Video: Momen Polisi Gagalkan Penyelundupan 50 Kg Sabu dan 20 Ribu Ekstasi</t>
+        </is>
+      </c>
+      <c r="D434" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260331-260331002/video-momen-polisi-gagalkan-penyelundupan-50-kg-sabu-dan-20-ribu-ekstasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>Video: Kapal Nazila 05 Tenggelam di Maluku Utara, 27 ABK Hilang</t>
+        </is>
+      </c>
+      <c r="D435" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260331-260331003/video-kapal-nazila-05-tenggelam-di-maluku-utara-27-abk-hilang</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>Jerman Vs Ghana: Nationalelf Menang Tipis 2-1</t>
+        </is>
+      </c>
+      <c r="D436" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8422564/jerman-vs-ghana-nationalelf-menang-tipis-2-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>B50 Jadi Strategi Energi Nasional di Tengah Konflik Timur Tengah</t>
+        </is>
+      </c>
+      <c r="D437" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1920310/b50-jadi-strategi-energi-nasional-di-tengah-konflik-timur-tengah?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>Pembalakan Hutan dan Kerusakan Lingkungan Picu Amuk Alam di Sulawesi Selatan</t>
+        </is>
+      </c>
+      <c r="D438" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/pembalakan-hutan-dan-kerusakan-lingkungan-picu-amuk-alam-di-sulawesi-selatan?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>Mendagri Tito Apresiasi BSPS, Program Mulia Bantu Masyarakat Kurang Mampu</t>
+        </is>
+      </c>
+      <c r="D439" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/30/22061201/mendagri-tito-apresiasi-bsps-program-mulia-bantu-masyarakat-kurang-mampu</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>Usai Idul Fitri 1447 Hijriah, Mendagri Minta ASN Kemendagri dan BNPP Tingkatkan Kinerja</t>
+        </is>
+      </c>
+      <c r="D440" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/30/19385751/usai-idul-fitri-1447-hijriah-mendagri-minta-asn-kemendagri-dan-bnpp</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>Rapat dengan DPR, Mendagri Tito Jelaskan Capaian Kinerja Strategis Kemendagri</t>
+        </is>
+      </c>
+      <c r="D441" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/30/17541511/rapat-dengan-dpr-mendagri-tito-jelaskan-capaian-kinerja-strategis-kemendagri</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D442" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D443" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D444" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D445" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>Penampakan Kapal Perang Rusia Tiba di Jakarta</t>
+        </is>
+      </c>
+      <c r="D446" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1920271/penampakan-kapal-perang-rusia-tiba-di-jakarta?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>"Comforting Sounds", Mew, dan Konser Perpisahan</t>
+        </is>
+      </c>
+      <c r="D447" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/dewi_puspa/69c8d65ded6415081549c032/comforting-sounds-mew-dan-konser-perpisahan</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>Sakura di Tokyo Mekar Lebih Cepat dari Biasanya, Lonjakan Pengunjung Picu Pembatasan di Spot Populer</t>
+        </is>
+      </c>
+      <c r="D448" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5722/sakura-di-tokyo-mekar-lebih-cepat-dari-biasanya-lonjakan-pengunjung-picu-pembatasan-di-spot-populer</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D449" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D450" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Ikuti Google Maps Niat Hindari Macet ke Tol Purwomartani, Pemudik Malah Masuk Jalan Persawahan</t>
+        </is>
+      </c>
+      <c r="D451" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/jawa-tengah/read/2026/03/27/061500188/berita-foto--ikuti-google-maps-niat-hindari-macet-ke-tol</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>Menlu Sugiono Minta UNIFIL Investigasi Insiden di Lebanon</t>
+        </is>
+      </c>
+      <c r="D452" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095367/menlu-sugiono-minta-unifil-investigasi-insiden-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>Bentuk Manajemen Mikro ala Prabowo</t>
+        </is>
+      </c>
+      <c r="D453" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095353/bentuk-manajemen-mikro-ala-prabowo</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>Lokasi Pemakaman Prajurit TNI yang Tewas di Lebanon</t>
+        </is>
+      </c>
+      <c r="D454" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095343/lokasi-pemakaman-prajurit-tni-yang-tewas-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>Imigrasi Ngurah Rai Tangkap Buronan Interpol Asal Inggris</t>
+        </is>
+      </c>
+      <c r="D455" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095341/imigrasi-ngurah-rai-tangkap-buronan-interpol-asal-inggris</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>Prabowo: Jepang Bagian dari Perjalanan Pembangunan Indonesia</t>
+        </is>
+      </c>
+      <c r="D456" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095340/prabowo-jepang-bagian-dari-perjalanan-pembangunan-indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>Sastra Winara: Halalbihalal Jadi Momentum Perkuat Kedaulatan Rakyat</t>
+        </is>
+      </c>
+      <c r="D457" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095338/sastra-winara-halalbihalal-jadi-momentum-perkuat-kedaulatan-rakyat</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>DPRD Sebut Pemerataan Infrastruktur Kunci Sukses Kunjungan ke Objek Wisata Bogor Meningkat</t>
+        </is>
+      </c>
+      <c r="D458" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095336/dprd-sebut-pemerataan-infrastruktur-kunci-sukses-kunjungan-ke-objek-wisata-bogor-meningkat</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>Menhub Dudy: Jumlah Orang Melakukan Perjalanan Selama Masa Angkutan Lebaran Capai 147,55 Juta</t>
+        </is>
+      </c>
+      <c r="D459" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095335/menhub-dudy-jumlah-orang-melakukan-perjalanan-selama-masa-angkutan-lebaran-capai-14755-juta</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>Praka Rizal Sempat Telepon Ayah sebelum Gugur di Lebanon</t>
+        </is>
+      </c>
+      <c r="D460" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095331/praka-rizal-sempat-telepon-ayah-sebelum-gugur-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>Anggota Komisi I Desak TNI Evaluasi Prajurit di Lebanon</t>
+        </is>
+      </c>
+      <c r="D461" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095330/anggota-komisi-i-desak-tni-evaluasi-prajurit-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>Prabowo Saksikan Pengusaha Jepang-Indonesia Teken 10 MoU</t>
+        </is>
+      </c>
+      <c r="D462" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095328/prabowo-saksikan-pengusaha-jepang-indonesia-teken-10-mou</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>Bupati Bogor Tinjau UPT Balai Kesejahteraan Sosial Citeureup</t>
+        </is>
+      </c>
+      <c r="D463" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095326/bupati-bogor-tinjau-upt-balai-kesejahteraan-sosial-citeureup</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>PT Pegadaian Resmi Lakukan Ekspansi Internasional ke Timor Leste</t>
+        </is>
+      </c>
+      <c r="D464" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095316/pt-pegadaian-resmi-lakukan-ekspansi-internasional-ke-timor-leste</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>Apresiasi Kinerja Satpol PP Kota Bandung dalam Penegakan Perda dan Pelayanan Masyarakat</t>
+        </is>
+      </c>
+      <c r="D465" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095312/apresiasi-kinerja-satpol-pp-kota-bandung-dalam-penegakan-perda-dan-pelayanan-masyarakat</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>Lewat Halalbihalal, Gubernur Lampung Ajak Tingkatkan Kepedulian Sosial</t>
+        </is>
+      </c>
+      <c r="D466" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095310/lewat-halalbihalal-gubernur-lampung-ajak-tingkatkan-kepedulian-sosial</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>Prabowo invites Japanese investors to expand investment in Indonesia</t>
+        </is>
+      </c>
+      <c r="D467" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410506/prabowo-invites-japanese-investors-to-expand-investment-in-indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>Indonesia, JICA deepen forestry partnership to support climate action</t>
+        </is>
+      </c>
+      <c r="D468" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410502/indonesia-jica-deepen-forestry-partnership-to-support-climate-action</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>Indonesia records 147.55 million travelers during 2026 Eid season</t>
+        </is>
+      </c>
+      <c r="D469" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410498/indonesia-records-14755-million-travelers-during-2026-eid-season</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>Bali Police name 7 foreign nationals as suspects in Ukrainian murder</t>
+        </is>
+      </c>
+      <c r="D470" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410494/bali-police-name-7-foreign-nationals-as-suspects-in-ukrainian-murder</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>Indonesian soldier killed in Lebanon, TNI reaffirms UN mission</t>
+        </is>
+      </c>
+      <c r="D471" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410490/indonesian-soldier-killed-in-lebanon-tni-reaffirms-un-mission</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>Reverse migration to cities seen risking demographic dividend: BKKBN</t>
+        </is>
+      </c>
+      <c r="D472" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410486/reverse-migration-to-cities-seen-risking-demographic-dividend-bkkbn</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>RI Govt probes intern deaths, to review hospital policies</t>
+        </is>
+      </c>
+      <c r="D473" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410482/ri-govtprobes-intern-deaths-to-review-hospital-policies</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>Indonesian students urged to walk, cycle to support energy efficiency</t>
+        </is>
+      </c>
+      <c r="D474" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410478/indonesian-students-urged-to-walk-cycle-to-support-energy-efficiency</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>Indonesian tourism pivots to Asian travelers amid Middle East conflict</t>
+        </is>
+      </c>
+      <c r="D475" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410474/indonesian-tourism-pivots-to-asian-travelers-amid-middle-east-conflict</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>SBC Medical Announces Fourth Quarter and Full Year 2025 Financial Results</t>
+        </is>
+      </c>
+      <c r="D476" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410470/sbc-medical-announces-fourth-quarter-and-full-year-2025-financial-results</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>RI, Saudi discuss hajj flight cost rise, prioritize pilgrims' safety</t>
+        </is>
+      </c>
+      <c r="D477" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410466/ri-saudi-discuss-hajj-flight-cost-rise-prioritize-pilgrims-safety</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>Social assistance digitalization to boost accuracy: minister</t>
+        </is>
+      </c>
+      <c r="D478" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410462/social-assistance-digitalization-to-boost-accuracy-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>Deputy minister reviews hajj health service readiness in Mecca</t>
+        </is>
+      </c>
+      <c r="D479" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410458/deputy-minister-reviews-hajj-health-service-readiness-in-mecca</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>Schools urged to reinforce responsible gadget use culture</t>
+        </is>
+      </c>
+      <c r="D480" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410454/schools-urged-to-reinforce-responsible-gadget-use-culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>Tuesday, 31 March 2026</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>Indonesian lawmaker sees ‘dupe’ trend as boost for local brands</t>
+        </is>
+      </c>
+      <c r="D481" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410450/indonesian-lawmaker-sees-dupe-trend-as-boost-for-local-brands</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D421"/>
+  <autoFilter ref="A1:D481"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -10133,6 +11453,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D419" r:id="rId418"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D420" r:id="rId419"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D421" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D422" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D423" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D424" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D425" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D426" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D427" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D428" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D429" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D430" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D431" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D432" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D433" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D434" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D435" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D436" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D437" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D438" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D439" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D440" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D441" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D442" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D443" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D444" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D445" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D446" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D447" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D448" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D449" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D450" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D451" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D452" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D453" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D454" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D455" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D456" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D457" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D458" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D459" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D460" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D461" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D462" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D463" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D464" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D465" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D466" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D467" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D468" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D469" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D470" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D471" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D472" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D473" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D474" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D475" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D476" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D477" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D478" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D479" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D480" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D481" r:id="rId480"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-03-31
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$481</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$541</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D481"/>
+  <dimension ref="A1:D541"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -11030,8 +11030,1328 @@
         </is>
       </c>
     </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>Italia Gagal ke Piala Dunia 2026!</t>
+        </is>
+      </c>
+      <c r="D482" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8424217/italia-gagal-ke-piala-dunia-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>Video Bahlil Pastikan Cadangan BBM RI Aman</t>
+        </is>
+      </c>
+      <c r="D483" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/detiktv/d-8424081/video-bahlil-pastikan-cadangan-bbm-ri-aman</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>Swasta Wajib WFH Mulai April, Ini Bidang Pekerjaan yang Dikecualikan</t>
+        </is>
+      </c>
+      <c r="D484" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8423940/swasta-wajib-wfh-mulai-april-ini-bidang-pekerjaan-yang-dikecualikan</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>Mobil Pribadi Isi BBM Subsidi Dibatasi 50 Liter/Hari, Berlaku Mulai 1 April</t>
+        </is>
+      </c>
+      <c r="D485" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8424059/mobil-pribadi-isi-bbm-subsidi-dibatasi-50-liter-hari-berlaku-mulai-1-april</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>Video Pemerintah Tetapkan ASN WFH Setiap Jumat</t>
+        </is>
+      </c>
+      <c r="D486" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/detiktv/d-8423945/video-pemerintah-tetapkan-asn-wfh-setiap-jumat</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>Italia Gagal ke Piala Dunia 2026!</t>
+        </is>
+      </c>
+      <c r="D487" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8424217/italia-gagal-ke-piala-dunia-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>Ancelotti Berharap Italia Lolos ke Piala Dunia</t>
+        </is>
+      </c>
+      <c r="D488" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8423582/ancelotti-berharap-italia-lolos-ke-piala-dunia</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>Bosnia Akan Parkir Bus kalau Sudah Ungguli Italia</t>
+        </is>
+      </c>
+      <c r="D489" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8423304/bosnia-akan-parkir-bus-kalau-sudah-ungguli-italia</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>4 Prajurit TNI Penyiram Air Keras ke Andrie Yunus Dijerat Pasal Penganiayaan</t>
+        </is>
+      </c>
+      <c r="D490" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8424162/4-prajurit-tni-penyiram-air-keras-ke-andrie-yunus-dijerat-pasal-penganiayaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>Swedia Vs Polandia: Gol Gyokeres Bawa Timnya ke Piala Dunia 2026</t>
+        </is>
+      </c>
+      <c r="D491" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8424215/swedia-vs-polandia-gol-gyokeres-bawa-timnya-ke-piala-dunia-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>4 Prajurit TNI Tersangka Kasus Andrie Yunus Ditahan di Lapas Maximum Security</t>
+        </is>
+      </c>
+      <c r="D492" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8424116/4-prajurit-tni-tersangka-kasus-andrie-yunus-ditahan-di-lapas-maximum-security</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>Video: Warga 'Panic Buying' BBM, Antrean SPBU di Purwakarta Picu Kemacetan</t>
+        </is>
+      </c>
+      <c r="D493" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260401-260401004/video-warga-panic-buying-bbm-antrean-spbu-di-purwakarta-picu-kemacetan</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>Video Bahlil Pastikan Cadangan BBM RI Aman</t>
+        </is>
+      </c>
+      <c r="D494" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260331-260331157/video-bahlil-pastikan-cadangan-bbm-ri-aman</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>Video: Bahlil Pastikan RI Punya Alternatif Impor Minyak-LPG Selain dari Timur Tengah</t>
+        </is>
+      </c>
+      <c r="D495" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260331-260331165/video-bahlil-pastikan-ri-punya-alternatif-impor-minyak-lpg-selain-dari-timur-tengah</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>Paus Dengar Trump Sedang Cari 'Jalan Keluar' Akhiri Perang dengan Iran</t>
+        </is>
+      </c>
+      <c r="D496" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8424213/paus-dengar-trump-sedang-cari-jalan-keluar-akhiri-perang-dengan-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>Jepang Kerahkan Rudal Jarak Jauh Pertamanya, untuk Apa?</t>
+        </is>
+      </c>
+      <c r="D497" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1920536/jepang-kerahkan-rudal-jarak-jauh-pertamanya-untuk-apa?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>Rokok Elektronik Memicu Kanker</t>
+        </is>
+      </c>
+      <c r="D498" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/rokok-elektrik-memicu-kanker?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>Perkuat Implementasi Sistem Jaminan Produk Halal, BPJPH Tingkatkan Kompetensi Penyelia Halal</t>
+        </is>
+      </c>
+      <c r="D499" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/31/20304391/perkuat-implementasi-sistem-jaminan-produk-halal-bpjph-tingkatkan-kompetensi</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>Sambut Peluncuran BSPS, Bupati Maesyal: Sejalan dengan Program Kabupaten Tangerang</t>
+        </is>
+      </c>
+      <c r="D500" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/03/31/191547978/sambut-peluncuran-bsps-bupati-maesyal-sejalan-dengan-program-kabupaten</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>Sumur Bor Terus Bertambah, Air Bersih Mengalir di Wilayah Terdampak Bencana Sumatera</t>
+        </is>
+      </c>
+      <c r="D501" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/03/31/18350291/sumur-bor-terus-bertambah-air-bersih-mengalir-di-wilayah-terdampak-bencana</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D502" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D503" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D504" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D505" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>Prabowo Berduka Atas Tewasnya 3 Prajurit TNI di Lebanon</t>
+        </is>
+      </c>
+      <c r="D506" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1920498/prabowo-berduka-atas-tewasnya-3-prajurit-tni-di-lebanon?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>Tahukah Anda Khasiat dari Ginseng?</t>
+        </is>
+      </c>
+      <c r="D507" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/lilianalie2123/698d75b7ed64150a4b540242/tahukah-anda-khasiat-dari-ginseng</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>Komodo Akan Dikembangbiakkan Jepang, Ditempatkan di Kebun Binatang Shizuoka</t>
+        </is>
+      </c>
+      <c r="D508" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5729/komodo-akan-dikembangbiakkan-jepang-ditempatkan-di-kebun-binatang-shizuoka</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D509" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D510" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Ikuti Google Maps Niat Hindari Macet ke Tol Purwomartani, Pemudik Malah Masuk Jalan Persawahan</t>
+        </is>
+      </c>
+      <c r="D511" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/jawa-tengah/read/2026/03/27/061500188/berita-foto--ikuti-google-maps-niat-hindari-macet-ke-tol</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>Solo Kaji Bike to Work hingga Transportasi Umum bagi ASN</t>
+        </is>
+      </c>
+      <c r="D512" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095612/solo-kaji-bike-to-work-hingga-transportasi-umum-bagi-asn</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>Alur Pemulangan Jenazah Praka Farizal ke Indonesia</t>
+        </is>
+      </c>
+      <c r="D513" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095609/alur-pemulangan-jenazah-praka-farizal-ke-indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>Pertamina-INPEX Perkuat Sinergi Proyek LNG Abadi Masela</t>
+        </is>
+      </c>
+      <c r="D514" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095605/pertamina-inpex-perkuat-sinergi-proyek-lng-abadi-masela</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>Prabowo Lanjutkan Perjalanan Dinas ke Seoul</t>
+        </is>
+      </c>
+      <c r="D515" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095600/prabowo-lanjutkan-perjalanan-dinas-ke-seoul</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>Pemerintah Terapkan WFH Setiap Jumat untuk ASN</t>
+        </is>
+      </c>
+      <c r="D516" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095599/pemerintah-terapkan-wfh-setiap-jumat-untuk-asn</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>Tiga Prajurit TNI Gugur di Lebanon, Ketum PPP Mardiono Sampaikan Duka Mendalam</t>
+        </is>
+      </c>
+      <c r="D517" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095594/tiga-prajurit-tni-gugur-di-lebanon-ketum-ppp-mardiono-sampaikan-duka-mendalam</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>Harapan Dasco terhadap PAN di Pemerintahan Prabowo</t>
+        </is>
+      </c>
+      <c r="D518" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095591/harapan-dasco-terhadap-pan-di-pemerintahan-prabowo</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>Pemerintah Aktifkan Kembali 625 Ribu Penerima BPJS Kesehatan</t>
+        </is>
+      </c>
+      <c r="D519" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095586/pemerintah-aktifkan-kembali-625-ribu-penerima-bpjs-kesehatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>Mensos Punya Data Rumah Sakit yang Tolak Pasien Cuci Darah</t>
+        </is>
+      </c>
+      <c r="D520" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095579/mensos-punya-data-rumah-sakit-yang-tolak-pasien-cuci-darah</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>DPR Ingatkan Masyarakat Tak Timbun BBM</t>
+        </is>
+      </c>
+      <c r="D521" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095573/dpr-ingatkan-masyarakat-tak-timbun-bbm</t>
+        </is>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Audiensi dengan Ditjen ESDM, Pemkot Bontang Usulkan Tambahan 4.034 Jargas</t>
+        </is>
+      </c>
+      <c r="D522" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095572/audiensi-dengan-ditjen-esdm-pemkot-bontang-usulkan-tambahan-4-034-jargas</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Prabowo Undang PM Jepang Sanae Takaichi ke Indonesia</t>
+        </is>
+      </c>
+      <c r="D523" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095571/prabowo-undang-pm-jepang-sanae-takaichi-ke-indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Perjalanan Kota Bontang Wujudkan City Gas di Indonesia</t>
+        </is>
+      </c>
+      <c r="D524" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095566/perjalanan-kota-bontang-wujudkan-city-gas-di-indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Prajurit TNI Gugur, Prabowo Ucapkan Duka Lewat Instagram</t>
+        </is>
+      </c>
+      <c r="D525" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095561/prajurit-tni-gugur-prabowo-ucapkan-duka-lewat-instagram</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Prabowo: Indonesia dan Jepang Siap Jadi Mediator Konflik</t>
+        </is>
+      </c>
+      <c r="D526" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095560/prabowo-indonesia-dan-jepang-siap-jadi-mediator-konflik</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Indonesia implements Friday WFH for civil servants to cut energy use</t>
+        </is>
+      </c>
+      <c r="D527" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410625/indonesia-implements-friday-wfh-for-civil-servants-to-cut-energy-use</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Indonesia rolls out Friday WFH policy to boost energy efficiency</t>
+        </is>
+      </c>
+      <c r="D528" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410621/indonesia-rolls-out-friday-wfh-policy-to-boost-energy-efficiency</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>President Prabowo arrives in Seoul for official South Korea visit</t>
+        </is>
+      </c>
+      <c r="D529" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410617/president-prabowo-arrives-in-seoul-for-official-south-korea-visit</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Indonesia pushes development of competitive female entrepreneurs</t>
+        </is>
+      </c>
+      <c r="D530" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410613/indonesia-pushes-development-of-competitive-female-entrepreneurs</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>MPR proposes withdrawal of RI's peacekeeping troops from Lebanon</t>
+        </is>
+      </c>
+      <c r="D531" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410609/mpr-proposes-withdrawal-of-ris-peacekeeping-troops-from-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Papua pushes fish exports as government builds ports and cold storage</t>
+        </is>
+      </c>
+      <c r="D532" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410605/papua-pushes-fish-exports-as-government-builds-ports-and-cold-storage</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>BGN suspends 1,256 free meal kitchens in eastern Indonesia</t>
+        </is>
+      </c>
+      <c r="D533" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410601/bgn-suspends-1256-free-meal-kitchens-in-eastern-indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Police arrest British national on red notice at Ngurah Rai Airport</t>
+        </is>
+      </c>
+      <c r="D534" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410597/police-arrest-british-national-on-red-notice-at-ngurah-rai-airport</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>BGN imposes stricter SOPs to improve free meal program quality</t>
+        </is>
+      </c>
+      <c r="D535" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410595/bgn-imposes-stricter-sops-to-improve-free-meal-program-quality</t>
+        </is>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Indonesia imports 160,000 co-op trucks from India, China, Japan</t>
+        </is>
+      </c>
+      <c r="D536" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410594/indonesia-imports-160000-co-op-trucks-from-india-china-japan</t>
+        </is>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Indonesia mourns three TNI UNIFIL Peacekeepers who fell in Lebanon</t>
+        </is>
+      </c>
+      <c r="D537" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410593/indonesia-mourns-three-tni-unifil-peacekeepers-who-fell-in-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Indonesia, Japan agree to bolster multifaceted cooperation</t>
+        </is>
+      </c>
+      <c r="D538" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410589/indonesia-japan-agree-to-bolster-multifaceted-cooperation</t>
+        </is>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Prabowo envisions Indonesia, Japan to shape global stability</t>
+        </is>
+      </c>
+      <c r="D539" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410587/prabowo-envisions-indonesia-japan-to-shape-global-stability</t>
+        </is>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Indonesia, Japan pledge deeper partnership, joint peace efforts</t>
+        </is>
+      </c>
+      <c r="D540" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410585/indonesia-japan-pledge-deeper-partnership-joint-peace-efforts</t>
+        </is>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>Wednesday, 01 April 2026</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Govt ensures public services not disrupted by one-day WFH scheme</t>
+        </is>
+      </c>
+      <c r="D541" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410583/govt-ensures-public-services-not-disrupted-by-one-day-wfh-scheme</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D481"/>
+  <autoFilter ref="A1:D541"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -11513,6 +12833,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D479" r:id="rId478"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D480" r:id="rId479"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D481" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D482" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D483" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D484" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D485" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D486" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D487" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D488" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D489" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D490" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D491" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D492" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D493" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D494" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D495" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D496" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D497" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D498" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D499" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D500" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D501" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D502" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D503" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D504" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D505" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D506" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D507" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D508" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D509" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D510" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D511" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D512" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D513" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D514" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D515" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D516" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D517" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D518" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D519" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D520" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D521" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D522" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D523" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D524" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D525" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D526" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D527" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D528" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D529" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D530" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D531" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D532" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D533" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D534" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D535" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D536" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D537" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D538" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D539" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D540" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D541" r:id="rId540"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-01
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$541</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$586</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D541"/>
+  <dimension ref="A1:D586"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -12350,8 +12350,998 @@
         </is>
       </c>
     </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Iran Ancam Serang 18 Perusahaan Teknologi AS dari Apple Sampai Tesla</t>
+        </is>
+      </c>
+      <c r="D542" s="2" t="inlineStr">
+        <is>
+          <t>https://inet.detik.com/cyberlife/d-8425831/iran-ancam-serang-18-perusahaan-teknologi-as-dari-apple-sampai-tesla</t>
+        </is>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Pemerintah Minta Swasta WFH Sehari Sepekan, Pengusaha Buka Suara</t>
+        </is>
+      </c>
+      <c r="D543" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8425726/pemerintah-minta-swasta-wfh-sehari-sepekan-pengusaha-buka-suara</t>
+        </is>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Gattuso: Saya Tidak Pantas Bilang Sepakbola Italia Harus Berubah</t>
+        </is>
+      </c>
+      <c r="D544" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8425044/gattuso-saya-tidak-pantas-bilang-sepakbola-italia-harus-berubah</t>
+        </is>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Video Amsal Sitepu Ucap Terima Kasih ke Prabowo Usai Divonis Bebas</t>
+        </is>
+      </c>
+      <c r="D545" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8425568/video-amsal-sitepu-ucap-terima-kasih-ke-prabowo-usai-divonis-bebas</t>
+        </is>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Inggris Dibungkam Jepang, Tuchel: Ini Bukan Kiamat</t>
+        </is>
+      </c>
+      <c r="D546" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8425042/inggris-dibungkam-jepang-tuchel-ini-bukan-kiamat</t>
+        </is>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Jasad Bayi Ditemukan Warga Sambas di Masjid, Ada Pesan 'Tolong Dimakamkan'</t>
+        </is>
+      </c>
+      <c r="D547" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8425920/jasad-bayi-ditemukan-warga-sambas-di-masjid-ada-pesan-tolong-dimakamkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Istri Tewas dan Suami Kritis dalam Rumah di Karawang, Penyebabnya Misterius</t>
+        </is>
+      </c>
+      <c r="D548" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8423464/istri-tewas-dan-suami-kritis-dalam-rumah-di-karawang-penyebabnya-misterius</t>
+        </is>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Geger Mayat Pria Ditemukan di Pasar Malioboro Jambi, Ada Bekas Luka Sajam</t>
+        </is>
+      </c>
+      <c r="D549" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8420955/geger-mayat-pria-ditemukan-di-pasar-malioboro-jambi-ada-bekas-luka-sajam</t>
+        </is>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Duduk Perkara Taksi Pelat B Ditilang karena Cari Penumpang di Bogor</t>
+        </is>
+      </c>
+      <c r="D550" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8425829/duduk-perkara-taksi-pelat-b-ditilang-karena-cari-penumpang-di-bogor</t>
+        </is>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Italia Gagal Lagi ke Piala Dunia, Pelatih Timnas Argentina Terpukul</t>
+        </is>
+      </c>
+      <c r="D551" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8425904/italia-gagal-lagi-ke-piala-dunia-pelatih-timnas-argentina-terpukul</t>
+        </is>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Oleh-oleh Prabowo dari Korea: Kerja Sama Energi Bersih &amp; Mineral</t>
+        </is>
+      </c>
+      <c r="D552" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8425838/oleh-oleh-prabowo-dari-korea-kerja-sama-energi-bersih-mineral</t>
+        </is>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Video Amsal Sitepu Ucap Terima Kasih ke Prabowo Usai Divonis Bebas</t>
+        </is>
+      </c>
+      <c r="D553" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260401-260401196/video-amsal-sitepu-ucap-terima-kasih-ke-prabowo-usai-divonis-bebas</t>
+        </is>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Video: Kesaksian Masinis saat KA Ciremai Anjlok gegara Rel Terkena Longsor</t>
+        </is>
+      </c>
+      <c r="D554" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260401-260401222/video-kesaksian-masinis-saat-ka-ciremai-anjlok-gegara-rel-terkena-longsor</t>
+        </is>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Video Eks Kadis PUPR Sumut Divonis 5,5 Tahun Bui di Kasus Korupsi Jalan</t>
+        </is>
+      </c>
+      <c r="D555" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260401-260401220/video-eks-kadis-pupr-sumut-divonis-5-5-tahun-bui-di-kasus-korupsi-jalan</t>
+        </is>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Dari Jepang-Korsel, Prabowo Bawa 'Oleh-oleh' Investasi Rp 575 T</t>
+        </is>
+      </c>
+      <c r="D556" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8425919/dari-jepang-korsel-prabowo-bawa-oleh-oleh-investasi-rp-575-t</t>
+        </is>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Kejaksaan RI Berkolaborasi, Kawal Keberhasilan Program MBG</t>
+        </is>
+      </c>
+      <c r="D557" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095851/kejaksaan-ri-berkolaborasi-kawal-keberhasilan-program-mbg</t>
+        </is>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Komnas HAM Minta Polisi Lanjutkan Penyidikan Kasus Andrie</t>
+        </is>
+      </c>
+      <c r="D558" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095850/komnas-ham-minta-polisi-lanjutkan-penyidikan-kasus-andrie</t>
+        </is>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Menteri Abdul Mu'ti Imbau Murid Bersepeda ke Sekolah</t>
+        </is>
+      </c>
+      <c r="D559" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095844/menteri-abdul-muti-imbau-murid-bersepeda-ke-sekolah</t>
+        </is>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Prabowo: Indonesia dan Korea Negara Middle Power</t>
+        </is>
+      </c>
+      <c r="D560" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095843/prabowo-indonesia-dan-korea-negara-middle-power</t>
+        </is>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Komnas HAM: Tak Ada Koordinasi TNI-Polri di Kasus Andrie</t>
+        </is>
+      </c>
+      <c r="D561" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095840/komnas-ham-tak-ada-koordinasi-tni-polri-di-kasus-andrie</t>
+        </is>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Gus Ipul Kawal Pembangunan Sekolah Rakyat di OKU Timur dan Sambas</t>
+        </is>
+      </c>
+      <c r="D562" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095839/gus-ipul-kawal-pembangunan-sekolah-rakyat-di-oku-timur-dan-sambas</t>
+        </is>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Wali Kota Semarang Minta Dukungan Ulama Sukseskan MTQ Nasional ke-31</t>
+        </is>
+      </c>
+      <c r="D563" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095835/wali-kota-semarang-minta-dukungan-ulama-sukseskan-mtq-nasional-ke-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Taspen Group Hadirkan Program Bedah Rumah Gratis di NTT</t>
+        </is>
+      </c>
+      <c r="D564" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095830/taspen-group-hadirkan-program-bedah-rumah-gratis-di-ntt</t>
+        </is>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Pengobatan Rutin Lebih Tenang Berkat Layanan JKN</t>
+        </is>
+      </c>
+      <c r="D565" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095823/pengobatan-rutin-lebih-tenang-berkat-layanan-jkn</t>
+        </is>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>PGN Dorong BBG Jadi Opsi Ekonomis Bagi Kendaraan</t>
+        </is>
+      </c>
+      <c r="D566" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095822/pgn-dorong-bbg-jadi-opsi-ekonomis-bagi-kendaraan</t>
+        </is>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Komnas HAM Gali Keterangan TNI Soal Kasus Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D567" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095819/komnas-ham-gali-keterangan-tni-soal-kasus-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Pegadaian Perkuat Layanan Digital melalui Tring!</t>
+        </is>
+      </c>
+      <c r="D568" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095816/pegadaian-perkuat-layanan-digital-melalui-tring</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>DPRD DKI Jakarta Soroti Pembenahan Layanan Dasar Warga</t>
+        </is>
+      </c>
+      <c r="D569" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095813/dprd-dki-jakarta-soroti-pembenahan-layanan-dasar-warga</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Pramono Anung Larang ASN Pakai Kendaraan Pribadi saat WFH</t>
+        </is>
+      </c>
+      <c r="D570" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095807/pramono-anung-larang-asn-pakai-kendaraan-pribadi-saat-wfh</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Abdul Mu'ti: Ada Sanksi untuk Murid yang Curang Saat TKA</t>
+        </is>
+      </c>
+      <c r="D571" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2095803/abdul-muti-ada-sanksi-untuk-murid-yang-curang-saat-tka</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Indonesia honors fallen UN peacekeepers with promotions, compensation</t>
+        </is>
+      </c>
+      <c r="D572" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410769/indonesia-honors-fallen-un-peacekeepers-with-promotions-compensation</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>February's trade surplus supports external economic growth: BI</t>
+        </is>
+      </c>
+      <c r="D573" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410765/februarys-trade-surplus-supports-external-economic-growth-bi</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Ministry calls for regions' responsiveness in addressing unemployment</t>
+        </is>
+      </c>
+      <c r="D574" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410761/ministry-calls-for-regions-responsiveness-in-addressing-unemployment</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Prabowo highlights strategic results from meeting with S Korea's Lee</t>
+        </is>
+      </c>
+      <c r="D575" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410757/prabowo-highlights-strategic-results-from-meeting-with-s-koreas-lee</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Minister encourages village digitalization to promote local products</t>
+        </is>
+      </c>
+      <c r="D576" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410753/minister-encourages-village-digitalization-to-promote-local-products</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Indonesia, South Korea launch cross-border QR-based payment system</t>
+        </is>
+      </c>
+      <c r="D577" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410749/indonesia-south-korea-launch-cross-border-qr-based-payment-system</t>
+        </is>
+      </c>
+    </row>
+    <row r="578">
+      <c r="A578" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B578" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C578" t="inlineStr">
+        <is>
+          <t>Indonesia diversifies energy sources to reduce Middle East dependence</t>
+        </is>
+      </c>
+      <c r="D578" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410745/indonesia-diversifies-energy-sources-to-reduce-middle-east-dependence</t>
+        </is>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B579" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C579" t="inlineStr">
+        <is>
+          <t>RI, Japan deepen cooperation on forestry, conservation, climate action</t>
+        </is>
+      </c>
+      <c r="D579" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410741/ri-japan-deepen-cooperation-on-forestry-conservation-climate-action</t>
+        </is>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B580" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C580" t="inlineStr">
+        <is>
+          <t>Prabowo quotes Korean proverb to highlight RI–South Korea friendship</t>
+        </is>
+      </c>
+      <c r="D580" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410737/prabowo-quotes-korean-proverb-to-highlight-ri-south-korea-friendship</t>
+        </is>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B581" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C581" t="inlineStr">
+        <is>
+          <t>President Prabowo receives South Korea's top honorary award</t>
+        </is>
+      </c>
+      <c r="D581" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410733/president-prabowo-receives-south-koreas-top-honorary-award</t>
+        </is>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B582" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C582" t="inlineStr">
+        <is>
+          <t>Indonesia prepares action plan to anticipate rising urbanization</t>
+        </is>
+      </c>
+      <c r="D582" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410729/indonesia-prepares-action-plan-to-anticipate-rising-urbanization</t>
+        </is>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B583" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C583" t="inlineStr">
+        <is>
+          <t>Indonesia condemns Israel's death penalty law for Palestinian prisoner</t>
+        </is>
+      </c>
+      <c r="D583" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410725/indonesia-condemns-israels-death-penalty-law-for-palestinian-prisoner</t>
+        </is>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B584" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C584" t="inlineStr">
+        <is>
+          <t>BNN deploys 1,800 facilitators to boost grassroots anti-drug efforts</t>
+        </is>
+      </c>
+      <c r="D584" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410721/bnn-deploys-1800-facilitators-to-boost-grassroots-anti-drug-efforts</t>
+        </is>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B585" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C585" t="inlineStr">
+        <is>
+          <t>Indonesia, South Korea align to boost digital services, AI growth</t>
+        </is>
+      </c>
+      <c r="D585" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410717/indonesia-south-korea-align-to-boost-digital-services-ai-growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" t="inlineStr">
+        <is>
+          <t>Thursday, 02 April 2026</t>
+        </is>
+      </c>
+      <c r="B586" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C586" t="inlineStr">
+        <is>
+          <t>Indonesia, South Korea ministers seal clean energy cooperation</t>
+        </is>
+      </c>
+      <c r="D586" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410713/indonesia-south-korea-ministers-seal-clean-energy-cooperation</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D541"/>
+  <autoFilter ref="A1:D586"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -12893,6 +13883,51 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D539" r:id="rId538"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D540" r:id="rId539"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D541" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D542" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D543" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D544" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D545" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D546" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D547" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D548" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D549" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D550" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D551" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D552" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D553" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D554" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D555" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D556" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D557" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D558" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D559" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D560" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D561" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D562" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D563" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D564" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D565" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D566" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D567" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D568" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D569" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D570" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D571" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D572" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D573" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D574" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D575" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D576" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D577" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D578" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D579" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D580" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D581" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D582" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D583" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D584" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D585" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D586" r:id="rId585"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-02
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$586</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$646</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D586"/>
+  <dimension ref="A1:D646"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -13340,8 +13340,1328 @@
         </is>
       </c>
     </row>
+    <row r="587">
+      <c r="A587" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B587" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C587" t="inlineStr">
+        <is>
+          <t>Video: Misi Artemis II NASA Meluncur ke Bulan, Bawa 4 Astronaut</t>
+        </is>
+      </c>
+      <c r="D587" s="2" t="inlineStr">
+        <is>
+          <t>https://inet.detik.com/detiktv/d-8427361/video-misi-artemis-ii-nasa-meluncur-ke-bulan-bawa-4-astronaut</t>
+        </is>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B588" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C588" t="inlineStr">
+        <is>
+          <t>Video Kepala BGN Tegaskan Tak Menjual Susu Berlabel MBG di Minimarket</t>
+        </is>
+      </c>
+      <c r="D588" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/detiktv/d-8427341/video-kepala-bgn-tegaskan-tak-menjual-susu-berlabel-mbg-di-minimarket</t>
+        </is>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B589" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C589" t="inlineStr">
+        <is>
+          <t>Cek! Aturan Pembatasan Bawa Minuman Beralkohol &amp; Rokok dari Luar Negeri</t>
+        </is>
+      </c>
+      <c r="D589" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8427342/cek-aturan-pembatasan-bawa-minuman-beralkohol-rokok-dari-luar-negeri</t>
+        </is>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>Bayar Tol Tanpa Setop Belum Jadi Juga, Kini Mau Diuji Coba Lagi</t>
+        </is>
+      </c>
+      <c r="D590" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8427308/bayar-tol-tanpa-setop-belum-jadi-juga-kini-mau-diuji-coba-lagi</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>Ternyata Ini Biang Kerok Penumpukan Penumpang di Stasiun KRL</t>
+        </is>
+      </c>
+      <c r="D591" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8427303/ternyata-ini-biang-kerok-penumpukan-penumpang-di-stasiun-krl</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>Trump Pecat Jaksa Agung AS Usai Ramai Dikritik soal Epstein Files</t>
+        </is>
+      </c>
+      <c r="D592" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8427477/trump-pecat-jaksa-agung-as-usai-ramai-dikritik-soal-epstein-files</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>Trump Umumkan Serangan ke Iran Lagi, Jembatan Tertinggi di Timteng Hancur</t>
+        </is>
+      </c>
+      <c r="D593" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8427471/trump-umumkan-serangan-ke-iran-lagi-jembatan-tertinggi-di-timteng-hancur</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>5 Berita Terpopuler Internasional Hari Ini</t>
+        </is>
+      </c>
+      <c r="D594" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8427158/5-berita-terpopuler-internasional-hari-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>China Tunjuk Hidung AS soal Selat Hormuz Ditutup</t>
+        </is>
+      </c>
+      <c r="D595" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8427404/china-tunjuk-hidung-as-soal-selat-hormuz-ditutup</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>De Zerbi Ingin Bertahan Lama di Tottenham</t>
+        </is>
+      </c>
+      <c r="D596" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8427474/de-zerbi-ingin-bertahan-lama-di-tottenham</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>Enzo dari Fans Berat Jadi Rekan Setim Messi di Timnas Argentina</t>
+        </is>
+      </c>
+      <c r="D597" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8427473/enzo-dari-fans-berat-jadi-rekan-setim-messi-di-timnas-argentina</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>Video Kajari Karo Minta Maaf Atas Kasus Amsal Sitepu</t>
+        </is>
+      </c>
+      <c r="D598" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260402-260402228/video-kajari-karo-minta-maaf-atas-kasus-amsal-sitepu</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>Video: Empat Anak TK Tewas Ditikam di Kampala, Pelaku Ditangkap</t>
+        </is>
+      </c>
+      <c r="D599" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260403-260403002/video-empat-anak-tk-tewas-ditikam-di-kampala-pelaku-ditangkap</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>Video KPK Geledah Rumah Ono Surono di Indramayu, Sejumlah Dokumen Disita</t>
+        </is>
+      </c>
+      <c r="D600" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260402-260402208/video-kpk-geledah-rumah-ono-surono-di-indramayu-sejumlah-dokumen-disita</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>Video: Penampakan Tas dari Kolagen T-Rex di Belanda</t>
+        </is>
+      </c>
+      <c r="D601" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260403-260403003/video-penampakan-tas-dari-kolagen-t-rex-di-belanda</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>KPK Geledah Rumah Ono Surono di Indramayu, Angkut 2 Koper dan 1 Kardus Berkas</t>
+        </is>
+      </c>
+      <c r="D602" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1921033/kpk-geledah-rumah-ono-surono-di-indramayu-angkut-2-koper-dan-1-kardus-berkas?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>Anti-Scam Center Dibentuk, Apakah Uang Korban Bisa Kembali?</t>
+        </is>
+      </c>
+      <c r="D603" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/anti-scam-center-dibentuk-apakah-uang-korban-bisa-kembali?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>Pengiriman Perdana Bumbu Pasta dan Makanan RTE Tandai Awal Pengelolaan Ekonomi Haji dan Umrah Terintegrasi</t>
+        </is>
+      </c>
+      <c r="D604" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/02/19261911/pengiriman-perdana-bumbu-pasta-dan-makanan-rte-tandai-awal-pengelolaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>7 Siswa SMAK 7 Penabur Masuk Kelas Internasional UI 2026 lewat Jalur Talent Scouting</t>
+        </is>
+      </c>
+      <c r="D605" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/edu/read/2026/04/02/181607671/7-siswa-smak-7-penabur-masuk-kelas-internasional-ui-2026-lewat-jalur-talent</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>Pemerintah Perkuat Kemitraan Indonesia–Republik Korea melalui 10 MoU Senilai Rp 173 Triliun</t>
+        </is>
+      </c>
+      <c r="D606" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/02/18070001/pemerintah-perkuat-kemitraan-indonesiarepublik-korea-melalui-10-mou-senilai</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D607" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D608" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D609" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D610" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>Reaksi Iran dan China soal AS yang Ingin Mundur Perang</t>
+        </is>
+      </c>
+      <c r="D611" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1921012/reaksi-iran-dan-china-soal-as-yang-ingin-mundur-perang?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>Tiap Tetes BBM, Refleksi Kecil tentang Tanggung Jawab Besar</t>
+        </is>
+      </c>
+      <c r="D612" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/untay74418/69cdda48c925c47774334192/tiap-tetes-bbm-refleksi-kecil-tentang-tanggung-jawab-besar</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>Pengendara Sepeda di Jepang Bisa Kena Tilang, Denda Maksimal Rp 1,3 Juta</t>
+        </is>
+      </c>
+      <c r="D613" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5745/pengendara-sepeda-di-jepang-bisa-kena-tilang-denda-maksimal-rp-1-3-juta</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D614" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D615" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>Berita Foto: Dampak Gempa M 7,6 Bitung–Manado, Korban Tewas Ditemukan di Reruntuhan</t>
+        </is>
+      </c>
+      <c r="D616" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/02/123000278/berita-foto-dampak-gempa-m-76-bitungmanado-korban-tewas-ditemukan-di</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>Hasil Pertemuan Komite SMK IDN Bogor dengan Ombudsman RI</t>
+        </is>
+      </c>
+      <c r="D617" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096086/hasil-pertemuan-komite-smk-idn-bogor-dengan-ombudsman-ri</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>Anggota DPR Desak Pemerintah Pulihkan Korban Pelanggaran HAM</t>
+        </is>
+      </c>
+      <c r="D618" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096084/anggota-dpr-desak-pemerintah-pulihkan-korban-pelanggaran-ham</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>Andrie Yunus Kirim Pesan: Panjang Umur Perjuangan</t>
+        </is>
+      </c>
+      <c r="D619" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096080/andrie-yunus-kirim-pesan-panjang-umur-perjuangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>Legislator PDIP Kritik Mandeknya Penuntasan HAM Berat</t>
+        </is>
+      </c>
+      <c r="D620" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096071/legislator-pdip-kritik-mandeknya-penuntasan-ham-berat</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>BMKG Catat 93 Gempa Susulan Usai Gempa M 7,6 di Bitung</t>
+        </is>
+      </c>
+      <c r="D621" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096065/bmkg-catat-93-gempa-susulan-usai-gempa-m-76-di-bitung</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>Kemenimipas Awasi Kondisi WNI yang Terdampak Perang Iran</t>
+        </is>
+      </c>
+      <c r="D622" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096056/kemenimipas-awasi-kondisi-wni-yang-terdampak-perang-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>Jenazah Tiga Prajurit TNI dari Lebanon Tiba Akhir Pekan</t>
+        </is>
+      </c>
+      <c r="D623" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096053/jenazah-tiga-prajurit-tni-dari-lebanon-tiba-akhir-pekan</t>
+        </is>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B624" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C624" t="inlineStr">
+        <is>
+          <t>BPBD Maluku Utara Laporkan SituasiTerkini Pascagempa M7,6</t>
+        </is>
+      </c>
+      <c r="D624" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096050/bpbd-maluku-utara-laporkan-situasiterkini-pascagempa-m76</t>
+        </is>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B625" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C625" t="inlineStr">
+        <is>
+          <t>Aktivis Papua Desak Komnas HAM Telisik Kasus Dogiyai</t>
+        </is>
+      </c>
+      <c r="D625" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096045/aktivis-papua-desak-komnas-ham-telisik-kasus-dogiyai</t>
+        </is>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B626" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C626" t="inlineStr">
+        <is>
+          <t>Semarang Jadi Tuan Rumah Event Olahraga Nasional April 2026</t>
+        </is>
+      </c>
+      <c r="D626" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096042/semarang-jadi-tuan-rumah-event-olahraga-nasional-april-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B627" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C627" t="inlineStr">
+        <is>
+          <t>Mendagri Pantau ASN WFH Lewat Geolokasi, Ponsel Harus Aktif</t>
+        </is>
+      </c>
+      <c r="D627" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096038/mendagri-pantau-asn-wfh-lewat-geolokasi-ponsel-harus-aktif</t>
+        </is>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B628" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C628" t="inlineStr">
+        <is>
+          <t>BNPB Desak Sulut-Malut Tetapkan Status Darurat Gempa</t>
+        </is>
+      </c>
+      <c r="D628" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096037/bnpb-desak-sulut-malut-tetapkan-status-darurat-gempa</t>
+        </is>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B629" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C629" t="inlineStr">
+        <is>
+          <t>DPRD DKI Jakarta Dukung Indonesia Jetsport World Series 2026 yang Digelar Agustus Mendatang</t>
+        </is>
+      </c>
+      <c r="D629" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096035/dprd-dki-jakarta-dukung-indonesia-jetsport-world-series-2026-yang-digelar-agustus-mendatang</t>
+        </is>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B630" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C630" t="inlineStr">
+        <is>
+          <t>DPRD DKI Jakarta Dukung Masyarakat Ikut Kelola Sampah</t>
+        </is>
+      </c>
+      <c r="D630" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096027/dprd-dki-jakarta-dukung-masyarakat-ikut-kelola-sampah</t>
+        </is>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B631" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C631" t="inlineStr">
+        <is>
+          <t>Praka Farizal Akan Dimakamkan di TMP Giripeni</t>
+        </is>
+      </c>
+      <c r="D631" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096026/praka-farizal-akan-dimakamkan-di-tmp-giripeni</t>
+        </is>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B632" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C632" t="inlineStr">
+        <is>
+          <t>Indonesia, Saudi Arabia strengthen bilateral relations through culture</t>
+        </is>
+      </c>
+      <c r="D632" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410981/indonesia-saudi-arabia-strengthen-bilateral-relations-through-culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B633" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C633" t="inlineStr">
+        <is>
+          <t>Minister says 2026 Eid homecoming and return travel run more smoothly</t>
+        </is>
+      </c>
+      <c r="D633" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410977/minister-says-2026-eid-homecoming-and-return-travel-run-more-smoothly</t>
+        </is>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B634" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C634" t="inlineStr">
+        <is>
+          <t>Indonesia maintains energy stability with proportional measures: staff</t>
+        </is>
+      </c>
+      <c r="D634" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410973/indonesia-maintains-energy-stability-with-proportional-measures-staff</t>
+        </is>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B635" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C635" t="inlineStr">
+        <is>
+          <t>Land productivity key to food self-sufficiency: deputy minister</t>
+        </is>
+      </c>
+      <c r="D635" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410969/land-productivity-key-to-food-self-sufficiency-deputy-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B636" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C636" t="inlineStr">
+        <is>
+          <t>Downstreaming drives Indonesia's palm oil export growth: minister</t>
+        </is>
+      </c>
+      <c r="D636" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410965/downstreaming-drives-indonesias-palm-oil-export-growth-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B637" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C637" t="inlineStr">
+        <is>
+          <t>BGN warns 2,100 MBG kitchens to improve services</t>
+        </is>
+      </c>
+      <c r="D637" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410961/bgn-warns-2100-mbg-kitchens-to-improve-services</t>
+        </is>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B638" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C638" t="inlineStr">
+        <is>
+          <t>Govt ensures local jobs in Waingapu shrimp farm project</t>
+        </is>
+      </c>
+      <c r="D638" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410957/govt-ensures-local-jobs-in-waingapu-shrimp-farm-project</t>
+        </is>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B639" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C639" t="inlineStr">
+        <is>
+          <t>Garuda Indonesia sets Bali as hub for eastern, international routes</t>
+        </is>
+      </c>
+      <c r="D639" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410953/garuda-indonesia-sets-bali-as-hub-for-eastern-international-routes</t>
+        </is>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B640" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C640" t="inlineStr">
+        <is>
+          <t>MPR urges universities to adopt recommendations on women's protection</t>
+        </is>
+      </c>
+      <c r="D640" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410949/mpr-urges-universities-to-adopt-recommendations-on-womens-protection</t>
+        </is>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B641" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C641" t="inlineStr">
+        <is>
+          <t>VP sends off Digital Warriors to expand digital education in 3T areas</t>
+        </is>
+      </c>
+      <c r="D641" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410945/vp-sends-off-digital-warriors-to-expand-digital-education-in-3t-areas</t>
+        </is>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B642" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C642" t="inlineStr">
+        <is>
+          <t>Komnas HAM issues 8,599 certificates for grave rights abuse victims</t>
+        </is>
+      </c>
+      <c r="D642" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410941/komnas-ham-issues-8599-certificates-for-grave-rights-abuse-victims</t>
+        </is>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B643" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C643" t="inlineStr">
+        <is>
+          <t>House Speaker calls for productivity amid Friday WFH policy</t>
+        </is>
+      </c>
+      <c r="D643" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410937/house-speaker-calls-for-productivity-amid-friday-wfh-policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B644" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C644" t="inlineStr">
+        <is>
+          <t>2027 infrastructure development to support 8 percent growth: minister</t>
+        </is>
+      </c>
+      <c r="D644" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410933/2027-infrastructure-development-to-support-8-percent-growth-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B645" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C645" t="inlineStr">
+        <is>
+          <t>Indonesia foils illegal trade of protected birds</t>
+        </is>
+      </c>
+      <c r="D645" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410929/indonesia-foils-illegal-trade-of-protected-birds</t>
+        </is>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" t="inlineStr">
+        <is>
+          <t>Friday, 03 April 2026</t>
+        </is>
+      </c>
+      <c r="B646" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C646" t="inlineStr">
+        <is>
+          <t>Gov't ensures aid for North Maluku, North Sulawesi quake victims</t>
+        </is>
+      </c>
+      <c r="D646" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/410925/govt-ensures-aid-for-north-maluku-north-sulawesi-quake-victims</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D586"/>
+  <autoFilter ref="A1:D646"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -13928,6 +15248,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D584" r:id="rId583"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D585" r:id="rId584"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D586" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D587" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D588" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D589" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D590" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D591" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D592" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D593" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D594" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D595" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D596" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D597" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D598" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D599" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D600" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D601" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D602" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D603" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D604" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D605" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D606" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D607" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D608" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D609" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D610" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D611" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D612" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D613" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D614" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D615" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D616" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D617" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D618" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D619" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D620" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D621" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D622" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D623" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D624" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D625" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D626" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D627" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D628" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D629" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D630" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D631" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D632" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D633" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D634" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D635" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D636" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D637" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D638" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D639" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D640" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D641" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D642" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D643" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D644" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D645" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D646" r:id="rId645"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-03
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$646</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$691</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D646"/>
+  <dimension ref="A1:D691"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -14660,8 +14660,998 @@
         </is>
       </c>
     </row>
+    <row r="647">
+      <c r="A647" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B647" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C647" t="inlineStr">
+        <is>
+          <t>Viral Netizen Tarik Tunai di ATM Dapat Uang Kertas Rp 50 Ribu Polos</t>
+        </is>
+      </c>
+      <c r="D647" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8428466/viral-netizen-tarik-tunai-di-atm-dapat-uang-kertas-rp-50-ribu-polos</t>
+        </is>
+      </c>
+    </row>
+    <row r="648">
+      <c r="A648" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B648" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C648" t="inlineStr">
+        <is>
+          <t>Picingkan Mata, Angka Berapa yang Terlihat?</t>
+        </is>
+      </c>
+      <c r="D648" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/asah-otak/d-8427999/picingkan-mata-angka-berapa-yang-terlihat</t>
+        </is>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B649" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C649" t="inlineStr">
+        <is>
+          <t>Video: Awas, Nutrisi Penting Hilang Saat Masak gara-gara Kesalahan Ini</t>
+        </is>
+      </c>
+      <c r="D649" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/detiktv/d-8428330/video-awas-nutrisi-penting-hilang-saat-masak-gara-gara-kesalahan-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B650" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C650" t="inlineStr">
+        <is>
+          <t>Benarkah Nasi Merah Lebih 'Diet-Friendly' ketimbang Nasi Putih? Ini Faktanya</t>
+        </is>
+      </c>
+      <c r="D650" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/diet/d-8427924/benarkah-nasi-merah-lebih-diet-friendly-ketimbang-nasi-putih-ini-faktanya</t>
+        </is>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B651" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C651" t="inlineStr">
+        <is>
+          <t>Video: Dahsyatnya Rudal Iran Bawa 400 Kg Hulu Ledak Guncang Israel</t>
+        </is>
+      </c>
+      <c r="D651" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8428424/video-dahsyatnya-rudal-iran-bawa-400-kg-hulu-ledak-guncang-israel</t>
+        </is>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B652" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C652" t="inlineStr">
+        <is>
+          <t>Pasukan Perdamaian Kembali Jadi Korban Serangan di Lebanon</t>
+        </is>
+      </c>
+      <c r="D652" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8428568/pasukan-perdamaian-kembali-jadi-korban-serangan-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B653" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C653" t="inlineStr">
+        <is>
+          <t>Trump Ancam Iran Lagi, Incar Infrastruktur Ini untuk Dihancurkan</t>
+        </is>
+      </c>
+      <c r="D653" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8427724/trump-ancam-iran-lagi-incar-infrastruktur-ini-untuk-dihancurkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B654" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C654" t="inlineStr">
+        <is>
+          <t>Serangan Israel Tewaskan 7 Orang di Beirut, Termasuk Komandan Hizbullah</t>
+        </is>
+      </c>
+      <c r="D654" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8426554/serangan-israel-tewaskan-7-orang-di-beirut-termasuk-komandan-hizbullah</t>
+        </is>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B655" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C655" t="inlineStr">
+        <is>
+          <t>Menanti Pembuktian Kebangkitan Arsenal Setelah Kalah di Carabao Cup</t>
+        </is>
+      </c>
+      <c r="D655" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8428547/menanti-pembuktian-kebangkitan-arsenal-setelah-kalah-di-carabao-cup</t>
+        </is>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B656" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C656" t="inlineStr">
+        <is>
+          <t>Cancelo Goda Bernardo Silva Gabung Barcelona</t>
+        </is>
+      </c>
+      <c r="D656" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-spanyol/d-8428546/cancelo-goda-bernardo-silva-gabung-barcelona</t>
+        </is>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B657" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C657" t="inlineStr">
+        <is>
+          <t>Analisis Pakar soal Kebijakan ASN WFH Tiap Jumat Bisa Hemat Konsumsi BBM</t>
+        </is>
+      </c>
+      <c r="D657" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8428218/analisis-pakar-soal-kebijakan-asn-wfh-tiap-jumat-bisa-hemat-konsumsi-bbm</t>
+        </is>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B658" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C658" t="inlineStr">
+        <is>
+          <t>Video Dubes Iran: Isu Perpecahan Mazhab Sunni-Syiah Bikinan Zionis</t>
+        </is>
+      </c>
+      <c r="D658" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260403-260403239/video-dubes-iran-isu-perpecahan-mazhab-sunni-syiah-bikinan-zionis</t>
+        </is>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B659" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C659" t="inlineStr">
+        <is>
+          <t>Video Timnas Indonesia Dibungkam Bulgaria di Final FIFA Series</t>
+        </is>
+      </c>
+      <c r="D659" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260330-260330132/video-timnas-indonesia-dibungkam-bulgaria-di-final-fifa-series</t>
+        </is>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B660" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C660" t="inlineStr">
+        <is>
+          <t>Bandung Hujan Angin hingga Puluhan Pohon Tumbang, 1 Orang Tewas</t>
+        </is>
+      </c>
+      <c r="D660" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8428565/bandung-hujan-angin-hingga-puluhan-pohon-tumbang-1-orang-tewas</t>
+        </is>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B661" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C661" t="inlineStr">
+        <is>
+          <t>Video: Dahsyatnya Rudal Iran Bawa 400 Kg Hulu Ledak Guncang Israel</t>
+        </is>
+      </c>
+      <c r="D661" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260403-260403253/video-dahsyatnya-rudal-iran-bawa-400-kg-hulu-ledak-guncang-israel-</t>
+        </is>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B662" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C662" t="inlineStr">
+        <is>
+          <t>KSAD AS Dipecat Hegseth di Tengah Perang Iran, Apa yang Terjadi?</t>
+        </is>
+      </c>
+      <c r="D662" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1921219/ksad-as-dipecat-hegseth-di-tengah-perang-iran-apa-yang-terjadi?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B663" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C663" t="inlineStr">
+        <is>
+          <t>Konflik Timur Tengah Menguji Ambisi Transisi Energi Indonesia</t>
+        </is>
+      </c>
+      <c r="D663" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/konflik-timur-tengah-menguji-ambisi-transisi-energi-indonesia?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>WIKA Kembali Turunkan Utang Senilai Rp 3,87 Triliun Sepanjang 2025</t>
+        </is>
+      </c>
+      <c r="D664" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/03/19474961/wika-kembali-turunkan-utang-senilai-rp-387-triliun-sepanjang-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>Satgas PRR Percepat Pemanfaatan Kayu Hanyutan sebagai Strategi Pemulihan Pascabencana di Wilayah Terdampak</t>
+        </is>
+      </c>
+      <c r="D665" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/03/16464471/satgas-prr-percepat-pemanfaatan-kayu-hanyutan-sebagai-strategi-pemulihan</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>Menaker Yassierli: Hubungan Industrial Harus Naik Kelas agar Pekerja Tak Tertinggal AI</t>
+        </is>
+      </c>
+      <c r="D666" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/03/13290221/menaker-yassierli-hubungan-industrial-harus-naik-kelas-agar-pekerja-tak</t>
+        </is>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B667" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C667" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D667" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B668" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C668" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D668" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B669" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C669" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D669" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B670" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C670" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D670" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B671" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C671" t="inlineStr">
+        <is>
+          <t>Penampakan Gudang Bantuan Kemanusiaan Iran Hancur Dihantam Serangan AS-Israel</t>
+        </is>
+      </c>
+      <c r="D671" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1921177/penampakan-gudang-bantuan-kemanusiaan-iran-hancur-dihantam-serangan-as-israel?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B672" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C672" t="inlineStr">
+        <is>
+          <t>Gizi Ibu Hamil: Menabung Nutrisi, Menyelamatkan Masa Depan Bangsa</t>
+        </is>
+      </c>
+      <c r="D672" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/rismayaniachmad/69ce93eac925c459ff1717d2/gizi-ibu-hamil-menabung-nutrisi-menyelamatkan-masa-depan-bangsa</t>
+        </is>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B673" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C673" t="inlineStr">
+        <is>
+          <t>Pameran Doraemon Terbesar Hadir di Tokyo, Ini Panduan Lengkapnya</t>
+        </is>
+      </c>
+      <c r="D673" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5730/pameran-doraemon-terbesar-hadir-di-tokyo-ini-panduan-lengkapnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B674" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C674" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D674" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B675" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C675" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D675" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B676" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C676" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Intip Bioskop Alfamart Pertama di Gading Serpong</t>
+        </is>
+      </c>
+      <c r="D676" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.kompas.com/read/2026/04/03/110300127/berita-foto--intip-bioskop-alfamart-pertama-di-gading-serpong</t>
+        </is>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B677" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C677" t="inlineStr">
+        <is>
+          <t>Lawmaker urges electrification to boost energy self-sufficiency</t>
+        </is>
+      </c>
+      <c r="D677" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411073/lawmaker-urges-electrification-to-boost-energy-self-sufficiency</t>
+        </is>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B678" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C678" t="inlineStr">
+        <is>
+          <t>Gradiant Wins Major Water Contract for UK Hyperscale Data Center</t>
+        </is>
+      </c>
+      <c r="D678" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411069/gradiant-wins-major-water-contract-for-uk-hyperscale-data-center</t>
+        </is>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B679" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C679" t="inlineStr">
+        <is>
+          <t>Minister calls to strengthen Kasepuhan Palace cultural education role</t>
+        </is>
+      </c>
+      <c r="D679" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411065/minister-calls-to-strengthen-kasepuhan-palace-cultural-education-role</t>
+        </is>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B680" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C680" t="inlineStr">
+        <is>
+          <t>Bulog targets 828,000 tons of SPHP rice distribution in 2026</t>
+        </is>
+      </c>
+      <c r="D680" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411061/bulog-targets-828000-tons-of-sphp-rice-distribution-in-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B681" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C681" t="inlineStr">
+        <is>
+          <t>Indonesian Army plans Central Papua Kodam to streamline command</t>
+        </is>
+      </c>
+      <c r="D681" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411057/indonesian-army-plans-central-papua-kodam-to-streamline-command</t>
+        </is>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B682" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C682" t="inlineStr">
+        <is>
+          <t>MPR calls on varsities to support Prabowo's energy transition program</t>
+        </is>
+      </c>
+      <c r="D682" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411053/mpr-calls-on-varsities-to-support-prabowos-energy-transition-program</t>
+        </is>
+      </c>
+    </row>
+    <row r="683">
+      <c r="A683" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B683" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C683" t="inlineStr">
+        <is>
+          <t>Jakarta sees job-seeking as main driver of post-Eid migration</t>
+        </is>
+      </c>
+      <c r="D683" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411049/jakarta-sees-job-seeking-as-main-driver-of-post-eid-migration</t>
+        </is>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B684" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C684" t="inlineStr">
+        <is>
+          <t>Indonesia sends 200 migrant workers to Japan under SSW scheme</t>
+        </is>
+      </c>
+      <c r="D684" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411045/indonesia-sends-200-migrant-workers-to-japan-under-ssw-scheme</t>
+        </is>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B685" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C685" t="inlineStr">
+        <is>
+          <t>BPBD responds swiftly as floods hit 3,176 households in Grobogan</t>
+        </is>
+      </c>
+      <c r="D685" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411041/bpbd-responds-swiftly-as-floods-hit-3176-households-in-grobogan</t>
+        </is>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B686" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C686" t="inlineStr">
+        <is>
+          <t>Sulawesi leads Indonesia in endemic bird species</t>
+        </is>
+      </c>
+      <c r="D686" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411037/sulawesi-leads-indonesia-in-endemic-bird-species</t>
+        </is>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B687" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C687" t="inlineStr">
+        <is>
+          <t>Jakarta lawmaker urges ban on Israeli passport holders</t>
+        </is>
+      </c>
+      <c r="D687" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411033/jakarta-lawmaker-urges-ban-on-israeli-passport-holders</t>
+        </is>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B688" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C688" t="inlineStr">
+        <is>
+          <t>Indonesia tightens coordination to curb illegal Hajj pilgrims</t>
+        </is>
+      </c>
+      <c r="D688" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411029/indonesia-tightens-coordination-to-curb-illegal-hajj-pilgrims</t>
+        </is>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B689" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C689" t="inlineStr">
+        <is>
+          <t>Indonesia plans 5,000 home renovations in East Nusa Tenggara</t>
+        </is>
+      </c>
+      <c r="D689" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411025/indonesia-plans-5000-home-renovations-in-east-nusa-tenggara</t>
+        </is>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B690" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C690" t="inlineStr">
+        <is>
+          <t>TransNusa Strengthens Domestic Network Connection with New Route Launch and Increased Scheduled Flight Frequency</t>
+        </is>
+      </c>
+      <c r="D690" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411021/transnusa-strengthens-domestic-network-connection-with-new-route-launch-and-increased-scheduled-flight-frequency</t>
+        </is>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" t="inlineStr">
+        <is>
+          <t>Saturday, 04 April 2026</t>
+        </is>
+      </c>
+      <c r="B691" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C691" t="inlineStr">
+        <is>
+          <t>True IDC Pushes "Security Economy", Breaking Ground on Mega Data Center in EEC with 77-Billion-Baht BOI Investment, Cementing Thailand's No. 1 Position</t>
+        </is>
+      </c>
+      <c r="D691" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411017/true-idc-pushes-security-economy-breaking-ground-on-mega-data-center-in-eec-with-77-billion-baht-boi-investment-cementing-thailands-no-1-position</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D646"/>
+  <autoFilter ref="A1:D691"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -15308,6 +16298,51 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D644" r:id="rId643"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D645" r:id="rId644"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D646" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D647" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D648" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D649" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D650" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D651" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D652" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D653" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D654" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D655" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D656" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D657" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D658" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D659" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D660" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D661" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D662" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D663" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D664" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D665" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D666" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D667" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D668" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D669" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D670" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D671" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D672" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D673" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D674" r:id="rId673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D675" r:id="rId674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D676" r:id="rId675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D677" r:id="rId676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D678" r:id="rId677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D679" r:id="rId678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D680" r:id="rId679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D681" r:id="rId680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D682" r:id="rId681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D683" r:id="rId682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D684" r:id="rId683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D685" r:id="rId684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D686" r:id="rId685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D687" r:id="rId686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D688" r:id="rId687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D689" r:id="rId688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D690" r:id="rId689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D691" r:id="rId690"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-04
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$691</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$751</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D691"/>
+  <dimension ref="A1:D751"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -15650,8 +15650,1328 @@
         </is>
       </c>
     </row>
+    <row r="692">
+      <c r="A692" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B692" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C692" t="inlineStr">
+        <is>
+          <t>Ada Berapa Segitiga dalam Gambar Bertumpuk Ini? Cuma IQ Super yang Bisa Temukan Semua</t>
+        </is>
+      </c>
+      <c r="D692" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/asah-otak/d-8428592/ada-berapa-segitiga-dalam-gambar-bertumpuk-ini-cuma-iq-super-yang-bisa-temukan-semua</t>
+        </is>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B693" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C693" t="inlineStr">
+        <is>
+          <t>Desakan RI ke PBB untuk Bersikap Buntut Prajurit TNI Jadi Korban di Lebanon</t>
+        </is>
+      </c>
+      <c r="D693" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8429533/desakan-ri-ke-pbb-untuk-bersikap-buntut-prajurit-tni-jadi-korban-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B694" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C694" t="inlineStr">
+        <is>
+          <t>City Vs Liverpool: Bantai Si Merah 4-0, Haaland Dkk ke Semifinal Piala FA</t>
+        </is>
+      </c>
+      <c r="D694" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8429424/city-vs-liverpool-bantai-si-merah-4-0-haaland-dkk-ke-semifinal-piala-fa</t>
+        </is>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B695" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C695" t="inlineStr">
+        <is>
+          <t>Mallorca Vs Real Madrid: Los Blancos Tumbang 1-2</t>
+        </is>
+      </c>
+      <c r="D695" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-spanyol/d-8429537/mallorca-vs-real-madrid-los-blancos-tumbang-1-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B696" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C696" t="inlineStr">
+        <is>
+          <t>Video: Kota Rosh Haayin di Israel Gelap Gulita Setelah Serangan Iran</t>
+        </is>
+      </c>
+      <c r="D696" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8429475/video-kota-rosh-haayin-di-israel-gelap-gulita-setelah-serangan-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B697" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C697" t="inlineStr">
+        <is>
+          <t>Polisi Bongkar Peredaran Obat Keras Ilegal di Tangerang, 2 Orang Ditangkap</t>
+        </is>
+      </c>
+      <c r="D697" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8429586/polisi-bongkar-peredaran-obat-keras-ilegal-di-tangerang-2-orang-ditangkap</t>
+        </is>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B698" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C698" t="inlineStr">
+        <is>
+          <t>Pondok Hijau Tangsel Masih Banjir, Warga Dievakuasi Pakai Perahu Karet</t>
+        </is>
+      </c>
+      <c r="D698" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8429554/pondok-hijau-tangsel-masih-banjir-warga-dievakuasi-pakai-perahu-karet</t>
+        </is>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B699" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C699" t="inlineStr">
+        <is>
+          <t>Banjir di Pamulang Tangsel, Polisi Evakuasi Warga Pakai Perahu Karet</t>
+        </is>
+      </c>
+      <c r="D699" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8429495/banjir-di-pamulang-tangsel-polisi-evakuasi-warga-pakai-perahu-karet</t>
+        </is>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B700" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C700" t="inlineStr">
+        <is>
+          <t>Sassuolo Vs Cagliari: Jay Idzes Sempat Blunder, I Neroverdi Menang 2-1</t>
+        </is>
+      </c>
+      <c r="D700" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-italia/d-8429485/sassuolo-vs-cagliari-jay-idzes-sempat-blunder-i-neroverdi-menang-2-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B701" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C701" t="inlineStr">
+        <is>
+          <t>Italia Gagal ke Piala Dunia, De Bruyne: Level di Eropa Makin Tinggi</t>
+        </is>
+      </c>
+      <c r="D701" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8429579/italia-gagal-ke-piala-dunia-de-bruyne-level-di-eropa-makin-tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B702" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C702" t="inlineStr">
+        <is>
+          <t>Mallorca Vs Real Madrid: Los Blancos Tumbang 1-2</t>
+        </is>
+      </c>
+      <c r="D702" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-spanyol/d-8429537/mallorca-vs-real-madrid-los-blancos-tumbang-1-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B703" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C703" t="inlineStr">
+        <is>
+          <t>Video Timnas Indonesia Dibungkam Bulgaria di Final FIFA Series</t>
+        </is>
+      </c>
+      <c r="D703" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260330-260330132/video-timnas-indonesia-dibungkam-bulgaria-di-final-fifa-series</t>
+        </is>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B704" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C704" t="inlineStr">
+        <is>
+          <t>Video: Bahlil Pastikan RI Punya Alternatif Impor Minyak-LPG Selain dari Timur Tengah</t>
+        </is>
+      </c>
+      <c r="D704" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260331-260331165/video-bahlil-pastikan-ri-punya-alternatif-impor-minyak-lpg-selain-dari-timur-tengah</t>
+        </is>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B705" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C705" t="inlineStr">
+        <is>
+          <t>Israel Hancurkan 17 Kamera Milik Penjaga Perdamaian PBB di Lebanon</t>
+        </is>
+      </c>
+      <c r="D705" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8429583/israel-hancurkan-17-kamera-milik-penjaga-perdamaian-pbb-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B706" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C706" t="inlineStr">
+        <is>
+          <t>Menyoal Cyberbullying Istri Bastoni, 'Dirujak' usai Kartu Merah Suami</t>
+        </is>
+      </c>
+      <c r="D706" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8428471/menyoal-cyberbullying-istri-bastoni-dirujak-usai-kartu-merah-suami</t>
+        </is>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B707" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C707" t="inlineStr">
+        <is>
+          <t>TNI Gugur di Lebanon, Indonesia Minta PBB Evaluasi Jaminan Keselamatan Pasukan Perdamaian</t>
+        </is>
+      </c>
+      <c r="D707" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1921360/tni-gugur-di-lebanon-indonesia-minta-pbb-evaluasi-jaminan-keselamatan-pasukan-perdamaian?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B708" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C708" t="inlineStr">
+        <is>
+          <t>Lagi, Prajurit TNI Jadi Korban Serangan di Lebanon</t>
+        </is>
+      </c>
+      <c r="D708" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/lagi-prajurit-tni-jadi-korban-serangan-di-lebanon?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B709" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C709" t="inlineStr">
+        <is>
+          <t>Kunjungi Aceh Tamiang, Kasatgas Tito Pastikan Percepatan Penanganan Pengungsi</t>
+        </is>
+      </c>
+      <c r="D709" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/04/20502991/kunjungi-aceh-tamiang-kasatgas-tito-pastikan-percepatan-penanganan-pengungsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B710" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C710" t="inlineStr">
+        <is>
+          <t>Kasatgas PRR Tito: Praja IPDN, Mari Kerja Keras Bersihkan Aceh Tamiang</t>
+        </is>
+      </c>
+      <c r="D710" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/04/18032001/kasatgas-prr-tito-praja-ipdn-mari-kerja-keras-bersihkan-aceh-tamiang</t>
+        </is>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B711" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C711" t="inlineStr">
+        <is>
+          <t>Kembali Terjunkan Praja IPDN ke Aceh Tamiang, Mendagri Tito: Sasar Pembersihan Sisa Lumpur di Permukiman Terdampak Bencana</t>
+        </is>
+      </c>
+      <c r="D711" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/04/14001331/kembali-terjunkan-praja-ipdn-ke-aceh-tamiang-mendagri-tito-sasar-pembersihan</t>
+        </is>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B712" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C712" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D712" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B713" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C713" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D713" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B714" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C714" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D714" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B715" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C715" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D715" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B716" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C716" t="inlineStr">
+        <is>
+          <t>Ajak Negara Asia-Eropa Bersatu Tinggalkan AS, Macron: Washington Inkonsisten</t>
+        </is>
+      </c>
+      <c r="D716" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1921302/ajak-negara-asia-eropa-bersatu-tinggalkan-as-macron-washington-inkonsisten?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B717" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C717" t="inlineStr">
+        <is>
+          <t>Cerpen: Cahaya di Langit Kediri</t>
+        </is>
+      </c>
+      <c r="D717" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/amirrrxitkj2044579/69cc4ee0ed6415137450efd2/cahaya-di-langit-kediri</t>
+        </is>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B718" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C718" t="inlineStr">
+        <is>
+          <t>Ribuan Kilometer Rel di Jepang Dihentikan Imbas Penurunan Populasi</t>
+        </is>
+      </c>
+      <c r="D718" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5755/ribuan-kilometer-rel-di-jepang-dihentikan-imbas-penurunan-populasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="719">
+      <c r="A719" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B719" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C719" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D719" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B720" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C720" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D720" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B721" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C721" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Intip Bioskop Alfamart Pertama di Gading Serpong</t>
+        </is>
+      </c>
+      <c r="D721" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.kompas.com/read/2026/04/03/110300127/berita-foto--intip-bioskop-alfamart-pertama-di-gading-serpong</t>
+        </is>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B722" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C722" t="inlineStr">
+        <is>
+          <t>Sultan HB X hingga Wakil Panglima TNI Sambut Jenazah Farizal</t>
+        </is>
+      </c>
+      <c r="D722" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096363/sultan-hb-x-hingga-wakil-panglima-tni-sambut-jenazah-farizal</t>
+        </is>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B723" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C723" t="inlineStr">
+        <is>
+          <t>Kasad: Penugasan Pasukan Perdamaian di Libanon Sudah Ada SOP</t>
+        </is>
+      </c>
+      <c r="D723" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096355/kasad-penugasan-pasukan-perdamaian-di-libanon-sudah-ada-sop</t>
+        </is>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B724" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C724" t="inlineStr">
+        <is>
+          <t>Ani Juwariyah, Difabel Tangguh yang Bertumbuh Bersama PNM</t>
+        </is>
+      </c>
+      <c r="D724" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096354/ani-juwariyah-difabel-tangguh-yang-bertumbuh-bersama-pnm</t>
+        </is>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B725" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C725" t="inlineStr">
+        <is>
+          <t>Jenazah Tiga Prajurit TNI Dilepas ke Daerah Masing-masing</t>
+        </is>
+      </c>
+      <c r="D725" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096347/jenazah-tiga-prajurit-tni-dilepas-ke-daerah-masing-masing</t>
+        </is>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B726" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C726" t="inlineStr">
+        <is>
+          <t>Tangis Keluarga Iringi Prosesi Persemayaman 3 Prajurit TNI</t>
+        </is>
+      </c>
+      <c r="D726" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096342/tangis-keluarga-iringi-prosesi-persemayaman-3-prajurit-tni</t>
+        </is>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B727" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C727" t="inlineStr">
+        <is>
+          <t>Jenazah Prajurit Gugur di Libanon Tiba di Soekarno-Hatta</t>
+        </is>
+      </c>
+      <c r="D727" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096338/jenazah-prajurit-gugur-di-libanon-tiba-di-soekarno-hatta</t>
+        </is>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B728" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C728" t="inlineStr">
+        <is>
+          <t>PGI Kecam Penyegelan Rumah Doa Jemaat POUK Tesalonika</t>
+        </is>
+      </c>
+      <c r="D728" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096329/pgi-kecam-penyegelan-rumah-doa-jemaat-pouk-tesalonika</t>
+        </is>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B729" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C729" t="inlineStr">
+        <is>
+          <t>Jokowi: Dunia Sedang Hadapi 3 Krisis Bisa Picu Efek Berantai</t>
+        </is>
+      </c>
+      <c r="D729" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096324/jokowi-dunia-sedang-hadapi-3-krisis-bisa-picu-efek-berantai</t>
+        </is>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B730" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C730" t="inlineStr">
+        <is>
+          <t>Beda Sikap Partai di DPR soal TGPF Kasus Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D730" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096319/beda-sikap-partai-di-dpr-soal-tgpf-kasus-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B731" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C731" t="inlineStr">
+        <is>
+          <t>Hingga Sabtu Siang, Sejumlah Genangan di Jakarta Surut</t>
+        </is>
+      </c>
+      <c r="D731" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096316/hingga-sabtu-siang-sejumlah-genangan-di-jakarta-surut</t>
+        </is>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B732" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C732" t="inlineStr">
+        <is>
+          <t>Pramono Ungkap Ada 72 Korban Keracunan MBG di Duren Sawit</t>
+        </is>
+      </c>
+      <c r="D732" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096311/pramono-ungkap-ada-72-korban-keracunan-mbg-di-duren-sawit</t>
+        </is>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B733" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C733" t="inlineStr">
+        <is>
+          <t>Panglima TNI Perintahkan Prajurit di Libanon Masuk Bunker</t>
+        </is>
+      </c>
+      <c r="D733" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096309/panglima-tni-perintahkan-prajurit-di-libanon-masuk-bunker</t>
+        </is>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B734" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C734" t="inlineStr">
+        <is>
+          <t>BGN Minta Maaf atas Keracunan MBG di Duren Sawit, Jaktim</t>
+        </is>
+      </c>
+      <c r="D734" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096307/bgn-minta-maaf-atas-keracunan-mbg-di-duren-sawit-jaktim</t>
+        </is>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B735" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C735" t="inlineStr">
+        <is>
+          <t>PDIP Desak PBB Menyeret Israel ke Mahkamah Internasional</t>
+        </is>
+      </c>
+      <c r="D735" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096299/pdip-desak-pbb-menyeret-israel-ke-mahkamah-internasional</t>
+        </is>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B736" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C736" t="inlineStr">
+        <is>
+          <t>Kasad Akan Pimpin Upacara Persemayaman Jenazah 3 TNI</t>
+        </is>
+      </c>
+      <c r="D736" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096295/kasad-akan-pimpin-upacara-persemayaman-jenazah-3-tni</t>
+        </is>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B737" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C737" t="inlineStr">
+        <is>
+          <t>Indonesia sends three fallen UN peacekeepers to hometowns for burial</t>
+        </is>
+      </c>
+      <c r="D737" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411141/indonesia-sends-three-fallen-un-peacekeepers-to-hometowns-for-burial</t>
+        </is>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B738" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C738" t="inlineStr">
+        <is>
+          <t>Indonesian lawmaker urges fuel price review as oil hits US$140</t>
+        </is>
+      </c>
+      <c r="D738" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411137/indonesian-lawmaker-urges-fuel-price-review-as-oil-hits-us140</t>
+        </is>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B739" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C739" t="inlineStr">
+        <is>
+          <t>President Prabowo pays tribute to three fallen TNI soldiers</t>
+        </is>
+      </c>
+      <c r="D739" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411133/president-prabowo-pays-tribute-to-three-fallen-tni-soldiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B740" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C740" t="inlineStr">
+        <is>
+          <t>Indonesian warship returns from Kakadu 2026 drill</t>
+        </is>
+      </c>
+      <c r="D740" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411129/indonesian-warship-returns-from-kakadu-2026-drill</t>
+        </is>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B741" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C741" t="inlineStr">
+        <is>
+          <t>Fallen Indonesian UN peacekeepers return home</t>
+        </is>
+      </c>
+      <c r="D741" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411125/fallen-indonesian-un-peacekeepers-return-home</t>
+        </is>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B742" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C742" t="inlineStr">
+        <is>
+          <t>Sustainable agriculture to achieve food security: deputy minister</t>
+        </is>
+      </c>
+      <c r="D742" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411121/sustainable-agriculture-to-achieve-food-security-deputy-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B743" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C743" t="inlineStr">
+        <is>
+          <t>Indonesia secures airport for return of fallen peacekeepers</t>
+        </is>
+      </c>
+      <c r="D743" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411117/indonesia-secures-airport-for-return-of-fallen-peacekeepers</t>
+        </is>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B744" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C744" t="inlineStr">
+        <is>
+          <t>Bulog prepares mitigation strategy ahead of El Niño drought risk</t>
+        </is>
+      </c>
+      <c r="D744" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411113/bulog-prepares-mitigation-strategy-ahead-of-el-nio-drought-risk</t>
+        </is>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B745" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C745" t="inlineStr">
+        <is>
+          <t>RI urges UNSC probe after peacekeepers injured in Lebanon blast</t>
+        </is>
+      </c>
+      <c r="D745" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411109/ri-urges-unsc-probe-after-peacekeepers-injured-in-lebanon-blast</t>
+        </is>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B746" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C746" t="inlineStr">
+        <is>
+          <t>Indonesia's minister urges unity, peace in Easter message</t>
+        </is>
+      </c>
+      <c r="D746" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411105/indonesias-minister-urges-unity-peace-in-easter-message</t>
+        </is>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B747" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C747" t="inlineStr">
+        <is>
+          <t>Indonesia ramps up efforts against illegal Hajj travel schemes</t>
+        </is>
+      </c>
+      <c r="D747" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411101/indonesia-ramps-up-efforts-against-illegal-hajj-travel-schemes</t>
+        </is>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B748" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C748" t="inlineStr">
+        <is>
+          <t>Indonesia's Mount Dukono erupts, ash rises 1.4 km</t>
+        </is>
+      </c>
+      <c r="D748" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411097/indonesias-mount-dukono-erupts-ash-rises-14-km</t>
+        </is>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B749" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C749" t="inlineStr">
+        <is>
+          <t>BGN covers treatment, suspends MBG kitchen after food poisoning</t>
+        </is>
+      </c>
+      <c r="D749" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411093/bgn-covers-treatment-suspends-mbg-kitchen-after-food-poisoning</t>
+        </is>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B750" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C750" t="inlineStr">
+        <is>
+          <t>Indonesia, Macau boost counterterrorism cooperation</t>
+        </is>
+      </c>
+      <c r="D750" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411089/indonesia-macau-boost-counterterrorism-cooperation</t>
+        </is>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" t="inlineStr">
+        <is>
+          <t>Sunday, 05 April 2026</t>
+        </is>
+      </c>
+      <c r="B751" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C751" t="inlineStr">
+        <is>
+          <t>Indonesia foils reptile smuggling attempt to Dubai</t>
+        </is>
+      </c>
+      <c r="D751" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411085/indonesia-foils-reptile-smuggling-attempt-to-dubai</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D691"/>
+  <autoFilter ref="A1:D751"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -16343,6 +17663,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D689" r:id="rId688"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D690" r:id="rId689"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D691" r:id="rId690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D692" r:id="rId691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D693" r:id="rId692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D694" r:id="rId693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D695" r:id="rId694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D696" r:id="rId695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D697" r:id="rId696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D698" r:id="rId697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D699" r:id="rId698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D700" r:id="rId699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D701" r:id="rId700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D702" r:id="rId701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D703" r:id="rId702"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D704" r:id="rId703"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D705" r:id="rId704"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D706" r:id="rId705"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D707" r:id="rId706"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D708" r:id="rId707"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D709" r:id="rId708"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D710" r:id="rId709"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D711" r:id="rId710"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D712" r:id="rId711"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D713" r:id="rId712"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D714" r:id="rId713"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D715" r:id="rId714"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D716" r:id="rId715"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D717" r:id="rId716"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D718" r:id="rId717"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D719" r:id="rId718"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D720" r:id="rId719"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D721" r:id="rId720"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D722" r:id="rId721"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D723" r:id="rId722"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D724" r:id="rId723"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D725" r:id="rId724"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D726" r:id="rId725"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D727" r:id="rId726"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D728" r:id="rId727"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D729" r:id="rId728"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D730" r:id="rId729"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D731" r:id="rId730"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D732" r:id="rId731"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D733" r:id="rId732"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D734" r:id="rId733"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D735" r:id="rId734"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D736" r:id="rId735"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D737" r:id="rId736"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D738" r:id="rId737"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D739" r:id="rId738"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D740" r:id="rId739"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D741" r:id="rId740"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D742" r:id="rId741"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D743" r:id="rId742"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D744" r:id="rId743"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D745" r:id="rId744"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D746" r:id="rId745"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D747" r:id="rId746"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D748" r:id="rId747"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D749" r:id="rId748"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D750" r:id="rId749"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D751" r:id="rId750"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-05
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$751</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$811</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D751"/>
+  <dimension ref="A1:D811"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -16970,8 +16970,1328 @@
         </is>
       </c>
     </row>
+    <row r="752">
+      <c r="A752" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B752" t="inlineStr">
+        <is>
+          <t>Crime</t>
+        </is>
+      </c>
+      <c r="C752" t="inlineStr">
+        <is>
+          <t>5 Fakta Pemilik Hajatan di Purwakarta Tewas di Tangan Preman</t>
+        </is>
+      </c>
+      <c r="D752" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8430525/5-fakta-pemilik-hajatan-di-purwakarta-tewas-di-tangan-preman</t>
+        </is>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B753" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C753" t="inlineStr">
+        <is>
+          <t>Beda Trump dan Iran soal Cerita Penyelamatan Pilot Jet Tempur AS</t>
+        </is>
+      </c>
+      <c r="D753" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8430566/beda-trump-dan-iran-soal-cerita-penyelamatan-pilot-jet-tempur-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B754" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C754" t="inlineStr">
+        <is>
+          <t>Harga Plastik Naik hingga 50%, Pedagang Pasar Menjerit!</t>
+        </is>
+      </c>
+      <c r="D754" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8430253/harga-plastik-naik-hingga-50-pedagang-pasar-menjerit</t>
+        </is>
+      </c>
+    </row>
+    <row r="755">
+      <c r="A755" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B755" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C755" t="inlineStr">
+        <is>
+          <t>Momen Happy Adinda Thomas Gender Reveal Anak Pertama, Suami Terharu</t>
+        </is>
+      </c>
+      <c r="D755" s="2" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8430173/momen-happy-adinda-thomas-gender-reveal-anak-pertama-suami-terharu</t>
+        </is>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B756" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C756" t="inlineStr">
+        <is>
+          <t>Alasan Ayah Selalu Bawa Mawar Biru ke Makam Vidi Aldiano</t>
+        </is>
+      </c>
+      <c r="D756" s="2" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8430042/alasan-ayah-selalu-bawa-mawar-biru-ke-makam-vidi-aldiano</t>
+        </is>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B757" t="inlineStr">
+        <is>
+          <t>Crime</t>
+        </is>
+      </c>
+      <c r="C757" t="inlineStr">
+        <is>
+          <t>Kakek di Langkat Bobol Rumah Saat Pemiliknya Liburan, Curi Uang Rp 110 Juta</t>
+        </is>
+      </c>
+      <c r="D757" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8430690/kakek-di-langkat-bobol-rumah-saat-pemiliknya-liburan-curi-uang-rp-110-juta</t>
+        </is>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B758" t="inlineStr">
+        <is>
+          <t>Crime</t>
+        </is>
+      </c>
+      <c r="C758" t="inlineStr">
+        <is>
+          <t>5 Fakta Pria Bekasi Disiram Air Keras Dilatari Sakit Hati</t>
+        </is>
+      </c>
+      <c r="D758" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8429670/5-fakta-pria-bekasi-disiram-air-keras-dilatari-sakit-hati</t>
+        </is>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B759" t="inlineStr">
+        <is>
+          <t>Crime</t>
+        </is>
+      </c>
+      <c r="C759" t="inlineStr">
+        <is>
+          <t>Terungkap Motif Pelaku Siram Air Keras ke Pria Bekasi: Sakit Hati dan Dendam</t>
+        </is>
+      </c>
+      <c r="D759" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8428740/terungkap-motif-pelaku-siram-air-keras-ke-pria-bekasi-sakit-hati-dan-dendam</t>
+        </is>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B760" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C760" t="inlineStr">
+        <is>
+          <t>Beda Trump dan Iran soal Cerita Penyelamatan Pilot Jet Tempur AS</t>
+        </is>
+      </c>
+      <c r="D760" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8430566/beda-trump-dan-iran-soal-cerita-penyelamatan-pilot-jet-tempur-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B761" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C761" t="inlineStr">
+        <is>
+          <t>Inter Vs Roma: 7 Gol Lahir, Si Ular Gigit Serigala Ibukota 5-2</t>
+        </is>
+      </c>
+      <c r="D761" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-italia/d-8430689/inter-vs-roma-7-gol-lahir-si-ular-gigit-serigala-ibukota-5-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B762" t="inlineStr">
+        <is>
+          <t>Crime</t>
+        </is>
+      </c>
+      <c r="C762" t="inlineStr">
+        <is>
+          <t>Suasana Haru di Pemakaman Pemilik Hajatan yang Tewas Dikeroyok Preman</t>
+        </is>
+      </c>
+      <c r="D762" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jabar/hukum-dan-kriminal/d-8430506/suasana-haru-di-pemakaman-pemilik-hajatan-yang-tewas-dikeroyok-preman</t>
+        </is>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B763" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C763" t="inlineStr">
+        <is>
+          <t>Video Iran Klaim 30 Universitas Jadi Sasaran Serangan AS-Israel</t>
+        </is>
+      </c>
+      <c r="D763" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260405-260405147/video-iran-klaim-30-universitas-jadi-sasaran-serangan-as-israel</t>
+        </is>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B764" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C764" t="inlineStr">
+        <is>
+          <t>Video: Panglima TNI Jamin Hak Keluarga Prajurit yang Gugur di Lebanon</t>
+        </is>
+      </c>
+      <c r="D764" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260405-260405034/video-panglima-tni-jamin-hak-keluarga-prajurit-yang-gugur-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B765" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C765" t="inlineStr">
+        <is>
+          <t>Video: Pesan Paskah Uskup Agung Jakarta soal Perang AS-Iran</t>
+        </is>
+      </c>
+      <c r="D765" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260405-260405036/video-pesan-paskah-uskup-agung-jakarta-soal-perang-as-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B766" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C766" t="inlineStr">
+        <is>
+          <t>Militer Nigeria Bunuh 65 Bandit yang Culik Penduduk Desa</t>
+        </is>
+      </c>
+      <c r="D766" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8430688/militer-nigeria-bunuh-65-bandit-yang-culik-penduduk-desa</t>
+        </is>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B767" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C767" t="inlineStr">
+        <is>
+          <t>Strategi “Gelap” Amerika-Israel: Lumpuhkan Fasilitas Kesehatan dan Produksi Vaksin Iran</t>
+        </is>
+      </c>
+      <c r="D767" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1921461/strategi-gelap-amerika-israel-lumpuhkan-fasilitas-kesehatan-dan-produksi-vaksin-iran?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B768" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C768" t="inlineStr">
+        <is>
+          <t>Taman Bendera Pusaka yang Kian Meriah</t>
+        </is>
+      </c>
+      <c r="D768" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/taman-bendera-pusaka-yang-kian-meriah?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B769" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C769" t="inlineStr">
+        <is>
+          <t>Kemnaker Buka Lagi Pembinaan K3 Gratis untuk 2.100 Peserta</t>
+        </is>
+      </c>
+      <c r="D769" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/05/20113951/kemnaker-buka-lagi-pembinaan-k3-gratis-untuk-2100-peserta</t>
+        </is>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B770" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C770" t="inlineStr">
+        <is>
+          <t>BPJS Ketenagakerjaan Hadirkan 3 Griya Pekerja di Batam, Solusi Hunian Layak dan Terjangkau</t>
+        </is>
+      </c>
+      <c r="D770" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/05/14421181/bpjs-ketenagakerjaan-hadirkan-3-griya-pekerja-di-batam-solusi-hunian-layak</t>
+        </is>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B771" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C771" t="inlineStr">
+        <is>
+          <t>Diskusi dengan Tim Kerja Pemantauan, DLH Jakarta Ingin RDF Plant Rorotan Dioperasikan Kembali</t>
+        </is>
+      </c>
+      <c r="D771" s="2" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/04/05/10224261/diskusi-dengan-tim-kerja-pemantauan-dlh-jakarta-ingin-rdf-plant-rorotan</t>
+        </is>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B772" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C772" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D772" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B773" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C773" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D773" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B774" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C774" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D774" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B775" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C775" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D775" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B776" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C776" t="inlineStr">
+        <is>
+          <t>Changan Lumin | Mencuri Poin Penting dari Para Pesaing | TEST DRIVE</t>
+        </is>
+      </c>
+      <c r="D776" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1921373/changan-lumin-mencuri-poin-penting-dari-para-pesaing-test-drive?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B777" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C777" t="inlineStr">
+        <is>
+          <t>[Puisi] Teras Sore</t>
+        </is>
+      </c>
+      <c r="D777" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/rismayaniachmad/69cfa8d7c925c4315c617612/puisi-teras-sore</t>
+        </is>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B778" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C778" t="inlineStr">
+        <is>
+          <t>Cara Urus Visa Intra-Company Transferee untuk Karyawan yang Transfer ke Jepang</t>
+        </is>
+      </c>
+      <c r="D778" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5760/cara-urus-visa-intra-company-transferee-untuk-karyawan-yang-transfer-ke-jepang</t>
+        </is>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B779" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C779" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D779" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B780" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C780" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D780" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B781" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C781" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Intip Bioskop Alfamart Pertama di Gading Serpong</t>
+        </is>
+      </c>
+      <c r="D781" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.kompas.com/read/2026/04/03/110300127/berita-foto--intip-bioskop-alfamart-pertama-di-gading-serpong</t>
+        </is>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B782" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C782" t="inlineStr">
+        <is>
+          <t>Penyebab Jemaat POUK Tesalonika Paskah di Kantor Kecamatan</t>
+        </is>
+      </c>
+      <c r="D782" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096455/penyebab-jemaat-pouk-tesalonika-paskah-di-kantor-kecamatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B783" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C783" t="inlineStr">
+        <is>
+          <t>Megawati: Semangat Paskah Jalan Pembebasan Bangsa Indonesia</t>
+        </is>
+      </c>
+      <c r="D783" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096452/megawati-semangat-paskah-jalan-pembebasan-bangsa-indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B784" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C784" t="inlineStr">
+        <is>
+          <t>Bupati Gresik Dampingi Gubernur Samarkand Ziarah ke Makam Maulana Malik Ibrahim</t>
+        </is>
+      </c>
+      <c r="D784" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096451/bupati-gresik-dampingi-gubernur-samarkand-ziarah-ke-makam-maulana-malik-ibrahim</t>
+        </is>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B785" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C785" t="inlineStr">
+        <is>
+          <t>3 TNI di Libanon Kembali Terluka, Sugiono: Diinvestigasi</t>
+        </is>
+      </c>
+      <c r="D785" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096449/3-tni-di-libanon-kembali-terluka-sugiono-diinvestigasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B786" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C786" t="inlineStr">
+        <is>
+          <t>Pemkot Semarang Hadirkan Diskon PBB untuk Warga</t>
+        </is>
+      </c>
+      <c r="D786" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096448/pemkot-semarang-hadirkan-diskon-pbb-untuk-warga</t>
+        </is>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B787" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C787" t="inlineStr">
+        <is>
+          <t>Paskah 2026, Kardinal Suharyo Bicara Ekologi Integral</t>
+        </is>
+      </c>
+      <c r="D787" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096447/paskah-2026-kardinal-suharyo-bicara-ekologi-integral</t>
+        </is>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B788" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C788" t="inlineStr">
+        <is>
+          <t>Mardiono Optimistis PPP Lolos Verifikasi Pemilu 2029</t>
+        </is>
+      </c>
+      <c r="D788" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096443/mardiono-optimistis-ppp-lolos-verifikasi-pemilu-2029</t>
+        </is>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B789" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C789" t="inlineStr">
+        <is>
+          <t>Pemerintah Desak PBB Evaluasi Keselamatan Penjaga Perdamaian</t>
+        </is>
+      </c>
+      <c r="D789" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096424/pemerintah-desak-pbb-evaluasi-keselamatan-penjaga-perdamaian</t>
+        </is>
+      </c>
+    </row>
+    <row r="790">
+      <c r="A790" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B790" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C790" t="inlineStr">
+        <is>
+          <t>Kardinal Suharyo Kutip Pesan Paus soal Pemimpin Suka Perang</t>
+        </is>
+      </c>
+      <c r="D790" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096423/kardinal-suharyo-kutip-pesan-paus-soal-pemimpin-suka-perang</t>
+        </is>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B791" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C791" t="inlineStr">
+        <is>
+          <t>SBY Minta PBB Setop Penugasan UNIFIL di Libanon</t>
+        </is>
+      </c>
+      <c r="D791" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096421/sby-minta-pbb-setop-penugasan-unifil-di-libanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B792" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C792" t="inlineStr">
+        <is>
+          <t>Pesan Kardinal Suharyo saat Paskah</t>
+        </is>
+      </c>
+      <c r="D792" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096417/pesan-kardinal-suharyo-saat-paskah</t>
+        </is>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B793" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C793" t="inlineStr">
+        <is>
+          <t>Kardinal Suharyo Pertanyakan Keseriusan Rezim Berantas KKN</t>
+        </is>
+      </c>
+      <c r="D793" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096416/kardinal-suharyo-pertanyakan-keseriusan-rezim-berantas-kkn</t>
+        </is>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B794" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C794" t="inlineStr">
+        <is>
+          <t>Komandan PMPP Besuk Korban Prajurit TNI Luka-luka di Libanon</t>
+        </is>
+      </c>
+      <c r="D794" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096410/komandan-pmpp-besuk-korban-prajurit-tni-luka-luka-di-libanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B795" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C795" t="inlineStr">
+        <is>
+          <t>Ketua DPR Minta Pemerintah Evaluasi Imunisasi Campak</t>
+        </is>
+      </c>
+      <c r="D795" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096408/ketua-dpr-minta-pemerintah-evaluasi-imunisasi-campak</t>
+        </is>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B796" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C796" t="inlineStr">
+        <is>
+          <t>Penjelasan TNI Soal Truk Militer Tabrak Motor di Kalideres</t>
+        </is>
+      </c>
+      <c r="D796" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096407/penjelasan-tni-soal-truk-militer-tabrak-motor-di-kalideres</t>
+        </is>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B797" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C797" t="inlineStr">
+        <is>
+          <t>Indonesia beat Kazakhstan 4-3 in Asian Games hockey qualifiers</t>
+        </is>
+      </c>
+      <c r="D797" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411237/indonesia-beat-kazakhstan-4-3-in-asian-games-hockey-qualifiers</t>
+        </is>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B798" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C798" t="inlineStr">
+        <is>
+          <t>Papua focuses on rice sufficiency to lift farmers' welfare</t>
+        </is>
+      </c>
+      <c r="D798" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411233/papua-focuses-on-rice-sufficiency-to-lift-farmers-welfare</t>
+        </is>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B799" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C799" t="inlineStr">
+        <is>
+          <t>BNPB prioritizes logistics for remote islands after North Maluku quake</t>
+        </is>
+      </c>
+      <c r="D799" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411229/bnpb-prioritizes-logistics-for-remote-islands-after-north-maluku-quake</t>
+        </is>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B800" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C800" t="inlineStr">
+        <is>
+          <t>Indonesia bags three gold medals at Bangkok World Archery Para Series</t>
+        </is>
+      </c>
+      <c r="D800" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411225/indonesia-bags-three-gold-medals-at-bangkok-world-archery-para-series</t>
+        </is>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B801" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C801" t="inlineStr">
+        <is>
+          <t>East Java, Uzbekistan explore religious tourism, cultural cooperation</t>
+        </is>
+      </c>
+      <c r="D801" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411221/east-java-uzbekistan-explore-religious-tourism-cultural-cooperation</t>
+        </is>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B802" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C802" t="inlineStr">
+        <is>
+          <t>Pindad prepares smokeless tech to tackle Bantargebang waste crisis</t>
+        </is>
+      </c>
+      <c r="D802" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411217/pindad-prepares-smokeless-tech-to-tackle-bantargebang-waste-crisis</t>
+        </is>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B803" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C803" t="inlineStr">
+        <is>
+          <t>Indonesia to export urea to 3 nations amid Strait of Hormuz closure</t>
+        </is>
+      </c>
+      <c r="D803" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411213/indonesia-to-export-urea-to-3-nations-amid-strait-of-hormuz-closure</t>
+        </is>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B804" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C804" t="inlineStr">
+        <is>
+          <t>Minister Sulaiman seeks to make Indonesia global food superpower</t>
+        </is>
+      </c>
+      <c r="D804" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411209/minister-sulaiman-seeks-to-make-indonesia-global-food-superpower</t>
+        </is>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B805" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C805" t="inlineStr">
+        <is>
+          <t>Indonesia prepares for El Nino, increases agricultural pumps: minister</t>
+        </is>
+      </c>
+      <c r="D805" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411205/indonesia-prepares-for-el-nino-increases-agricultural-pumps-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B806" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C806" t="inlineStr">
+        <is>
+          <t>Indonesia's rice reserves secure at 4.5 million tons: Minister</t>
+        </is>
+      </c>
+      <c r="D806" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411201/indonesias-rice-reserves-secure-at-45-million-tons-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B807" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C807" t="inlineStr">
+        <is>
+          <t>State guarantees all compensations for fallen Indonesian peacekeepers</t>
+        </is>
+      </c>
+      <c r="D807" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411197/state-guarantees-all-compensations-for-fallen-indonesian-peacekeepers</t>
+        </is>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B808" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C808" t="inlineStr">
+        <is>
+          <t>TNI ensures safety of Indonesian peacekeepers injured in Lebanon</t>
+        </is>
+      </c>
+      <c r="D808" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411193/tni-ensures-safety-of-indonesian-peacekeepers-injured-in-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B809" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C809" t="inlineStr">
+        <is>
+          <t>Governor highlights Cheng Beng as symbol of respect in Bangka Belitung</t>
+        </is>
+      </c>
+      <c r="D809" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411189/governor-highlights-cheng-beng-as-symbol-of-respect-in-bangka-belitung</t>
+        </is>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B810" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C810" t="inlineStr">
+        <is>
+          <t>Ministry seeks Rp24.8T additional budget to improve religious schools</t>
+        </is>
+      </c>
+      <c r="D810" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411185/ministry-seeks-rp248t-additional-budget-to-improve-religious-schools</t>
+        </is>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" t="inlineStr">
+        <is>
+          <t>Monday, 06 April 2026</t>
+        </is>
+      </c>
+      <c r="B811" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C811" t="inlineStr">
+        <is>
+          <t>Indonesia faces high costs in handling marine waste, says minister</t>
+        </is>
+      </c>
+      <c r="D811" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411181/indonesia-faces-high-costs-in-handling-marine-waste-says-minister</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D751"/>
+  <autoFilter ref="A1:D811"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -17723,6 +19043,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D749" r:id="rId748"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D750" r:id="rId749"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D751" r:id="rId750"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D752" r:id="rId751"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D753" r:id="rId752"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D754" r:id="rId753"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D755" r:id="rId754"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D756" r:id="rId755"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D757" r:id="rId756"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D758" r:id="rId757"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D759" r:id="rId758"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D760" r:id="rId759"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D761" r:id="rId760"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D762" r:id="rId761"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D763" r:id="rId762"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D764" r:id="rId763"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D765" r:id="rId764"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D766" r:id="rId765"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D767" r:id="rId766"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D768" r:id="rId767"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D769" r:id="rId768"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D770" r:id="rId769"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D771" r:id="rId770"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D772" r:id="rId771"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D773" r:id="rId772"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D774" r:id="rId773"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D775" r:id="rId774"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D776" r:id="rId775"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D777" r:id="rId776"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D778" r:id="rId777"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D779" r:id="rId778"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D780" r:id="rId779"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D781" r:id="rId780"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D782" r:id="rId781"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D783" r:id="rId782"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D784" r:id="rId783"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D785" r:id="rId784"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D786" r:id="rId785"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D787" r:id="rId786"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D788" r:id="rId787"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D789" r:id="rId788"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D790" r:id="rId789"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D791" r:id="rId790"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D792" r:id="rId791"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D793" r:id="rId792"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D794" r:id="rId793"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D795" r:id="rId794"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D796" r:id="rId795"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D797" r:id="rId796"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D798" r:id="rId797"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D799" r:id="rId798"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D800" r:id="rId799"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D801" r:id="rId800"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D802" r:id="rId801"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D803" r:id="rId802"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D804" r:id="rId803"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D805" r:id="rId804"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D806" r:id="rId805"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D807" r:id="rId806"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D808" r:id="rId807"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D809" r:id="rId808"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D810" r:id="rId809"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D811" r:id="rId810"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-06
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$811</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$871</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D811"/>
+  <dimension ref="A1:D871"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -18290,8 +18290,1328 @@
         </is>
       </c>
     </row>
+    <row r="812">
+      <c r="A812" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B812" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C812" t="inlineStr">
+        <is>
+          <t>RI Bakal Terapkan Nutri Level, Membantu atau Malah Bikin Parno?</t>
+        </is>
+      </c>
+      <c r="D812" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/polling/d-8432318/ri-bakal-terapkan-nutri-level-membantu-atau-malah-bikin-parno</t>
+        </is>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B813" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C813" t="inlineStr">
+        <is>
+          <t>Tiket Pesawat Boleh Naik hingga 13%, Asosiasi Maskapai Buka Suara</t>
+        </is>
+      </c>
+      <c r="D813" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8432302/tiket-pesawat-boleh-naik-hingga-13-asosiasi-maskapai-buka-suara</t>
+        </is>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B814" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C814" t="inlineStr">
+        <is>
+          <t>Angkasa Pura Minta Maaf soal Atap Terminal 3 Jebol Imbas Hujan Deras</t>
+        </is>
+      </c>
+      <c r="D814" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8432167/angkasa-pura-minta-maaf-soal-atap-terminal-3-jebol-imbas-hujan-deras</t>
+        </is>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B815" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C815" t="inlineStr">
+        <is>
+          <t>Video Purbaya Soal Pemotongan Gaji Menteri: Saya Tebak Kira-kira 25%</t>
+        </is>
+      </c>
+      <c r="D815" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/detiktv/d-8432136/video-purbaya-soal-pemotongan-gaji-menteri-saya-tebak-kira-kira-25</t>
+        </is>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B816" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C816" t="inlineStr">
+        <is>
+          <t>Saat Gibran Ikut Memikul Salib Paskah di Kupang</t>
+        </is>
+      </c>
+      <c r="D816" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.detik.com/travel-news/d-8431689/saat-gibran-ikut-memikul-salib-paskah-di-kupang</t>
+        </is>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B817" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C817" t="inlineStr">
+        <is>
+          <t>Napoli Vs Milan: Partenopei Sikat Rossoneri</t>
+        </is>
+      </c>
+      <c r="D817" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-italia/d-8432360/napoli-vs-milan-partenopei-sikat-rossoneri</t>
+        </is>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B818" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C818" t="inlineStr">
+        <is>
+          <t>Juventus Vs Genoa: Bianconeri Menang 2-0</t>
+        </is>
+      </c>
+      <c r="D818" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-italia/d-8432350/juventus-vs-genoa-bianconeri-menang-2-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B819" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C819" t="inlineStr">
+        <is>
+          <t>Head to Head Napoli Vs Milan: Potensi Duel Sengit di Naples</t>
+        </is>
+      </c>
+      <c r="D819" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-italia/d-8432201/head-to-head-napoli-vs-milan-potensi-duel-sengit-di-naples</t>
+        </is>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B820" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C820" t="inlineStr">
+        <is>
+          <t>Tiket Pesawat Boleh Naik hingga 13%, Asosiasi Maskapai Buka Suara</t>
+        </is>
+      </c>
+      <c r="D820" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8432302/tiket-pesawat-boleh-naik-hingga-13-asosiasi-maskapai-buka-suara</t>
+        </is>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B821" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C821" t="inlineStr">
+        <is>
+          <t>Trump Kecam NATO, Australia, Jepang hingga Korsel Tak Bantu Lawan Iran</t>
+        </is>
+      </c>
+      <c r="D821" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8432358/trump-kecam-nato-australia-jepang-hingga-korsel-tak-bantu-lawan-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B822" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C822" t="inlineStr">
+        <is>
+          <t>Tertinggal 9 Poin dari Persib, Persija Belum Nyerah Kejar Trofi Juara</t>
+        </is>
+      </c>
+      <c r="D822" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8432345/tertinggal-9-poin-dari-persib-persija-belum-nyerah-kejar-trofi-juara</t>
+        </is>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B823" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C823" t="inlineStr">
+        <is>
+          <t>Video: Drone Israel Tembak Warga Sipil Gaza, 10 Orang Tewas</t>
+        </is>
+      </c>
+      <c r="D823" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260407-260407003/video-drone-israel-tembak-warga-sipil-gaza-10-orang-tewas</t>
+        </is>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B824" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C824" t="inlineStr">
+        <is>
+          <t>Video Sejumlah Rumah Warga Rusak Terdampak Ledakan PT GWS Sidoarjo</t>
+        </is>
+      </c>
+      <c r="D824" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260406-260406075/video-sejumlah-rumah-warga-rusak-terdampak-ledakan-pt-gws-sidoarjo</t>
+        </is>
+      </c>
+    </row>
+    <row r="825">
+      <c r="A825" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B825" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C825" t="inlineStr">
+        <is>
+          <t>Video: DPR-DPD Deklarasi Kaukus Parlemen Perdamaian Dunia, Serukan Setop Perang</t>
+        </is>
+      </c>
+      <c r="D825" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260406-260406071/video-dpr-dpd-deklarasi-kaukus-parlemen-perdamaian-dunia-serukan-setop-perang</t>
+        </is>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B826" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C826" t="inlineStr">
+        <is>
+          <t>Video: Taklukan Genoa 2-0, Juventus Jaga Asa ke Liga Champions</t>
+        </is>
+      </c>
+      <c r="D826" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260407-260407004/video-taklukan-genoa-2-0-juventus-jaga-asa-ke-liga-champions</t>
+        </is>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B827" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C827" t="inlineStr">
+        <is>
+          <t>Purbaya Jamin Harga BBM Subsidi Tak Naik hingga Akhir 2026</t>
+        </is>
+      </c>
+      <c r="D827" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1921771/purbaya-jamin-harga-bbm-subsidi-tak-naik-hingga-akhir-2026?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B828" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C828" t="inlineStr">
+        <is>
+          <t>Kelas Kring Menjaga Nyala Harapan Pelaku UMKM Kopi</t>
+        </is>
+      </c>
+      <c r="D828" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/kelas-kring-menjaga-nyala-harapan-pelaku-umkm-kopi?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B829" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C829" t="inlineStr">
+        <is>
+          <t>Kemnaker Perkuat Integrasi MagangHub dengan Sertifikasi Kompetensi</t>
+        </is>
+      </c>
+      <c r="D829" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/06/21051511/kemnaker-perkuat-integrasi-maganghub-dengan-sertifikasi-kompetensi</t>
+        </is>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B830" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C830" t="inlineStr">
+        <is>
+          <t>WIKA Garap Harbour Road II, Tol Layang Ikonik dengan Teknologi Konstruksi Tinggi di Jakarta Utara</t>
+        </is>
+      </c>
+      <c r="D830" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/06/19573591/wika-garap-harbour-road-ii-tol-layang-ikonik-dengan-teknologi-konstruksi</t>
+        </is>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B831" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C831" t="inlineStr">
+        <is>
+          <t>Akselerasi Pemerintah Digital untuk Kemudahan Layanan Masyarakat</t>
+        </is>
+      </c>
+      <c r="D831" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/06/18280031/akselerasi-pemerintah-digital-untuk-kemudahan-layanan-masyarakat</t>
+        </is>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B832" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C832" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D832" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B833" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C833" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D833" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B834" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C834" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D834" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B835" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C835" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D835" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B836" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C836" t="inlineStr">
+        <is>
+          <t>Keunggulan Jet Tempur F-15E Milik AS, Berperan Defensif di Langit Iran</t>
+        </is>
+      </c>
+      <c r="D836" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1921736/keunggulan-jet-tempur-f-15e-milik-as-berperan-defensif-di-langit-iran?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B837" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C837" t="inlineStr">
+        <is>
+          <t>Ketika Dua Butir Beras Tak Tenggelam</t>
+        </is>
+      </c>
+      <c r="D837" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/dandungnurhono7545/69d0620134777c602f7da053/ketika-dua-butir-beras-tak-tenggelam</t>
+        </is>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B838" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C838" t="inlineStr">
+        <is>
+          <t>Industri Plus-Size Jepang Masih Bertahan di Tengah Stigma dan Perkembangan AI</t>
+        </is>
+      </c>
+      <c r="D838" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5764/industri-plus-size-jepang-masih-bertahan-di-tengah-stigma-dan-perkembangan-ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B839" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C839" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D839" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B840" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C840" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D840" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B841" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C841" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Intip Bioskop Alfamart Pertama di Gading Serpong</t>
+        </is>
+      </c>
+      <c r="D841" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.kompas.com/read/2026/04/03/110300127/berita-foto--intip-bioskop-alfamart-pertama-di-gading-serpong</t>
+        </is>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B842" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C842" t="inlineStr">
+        <is>
+          <t>Janji Wakil Presiden Gibran ke Guru PPPK di Kupang</t>
+        </is>
+      </c>
+      <c r="D842" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096656/janji-wakil-presiden-gibran-ke-guru-pppk-di-kupang</t>
+        </is>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B843" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C843" t="inlineStr">
+        <is>
+          <t>Siswa Sekolah Rakyat Doa Lintas Agama untuk Prajurit TNI Gugur di Lebanon</t>
+        </is>
+      </c>
+      <c r="D843" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096651/siswa-sekolah-rakyat-doa-lintas-agama-untuk-prajurit-tni-gugur-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B844" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C844" t="inlineStr">
+        <is>
+          <t>Maruarar: Target Bedah Rumah Naik Jadi 400 Ribu Unit</t>
+        </is>
+      </c>
+      <c r="D844" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096650/maruarar-target-bedah-rumah-naik-jadi-400-ribu-unit</t>
+        </is>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B845" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C845" t="inlineStr">
+        <is>
+          <t>Kemensos Kaji Pembelian Mobil Listrik untuk Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="D845" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096649/kemensos-kaji-pembelian-mobil-listrik-untuk-sekolah-rakyat</t>
+        </is>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B846" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C846" t="inlineStr">
+        <is>
+          <t>Arahan Prabowo, Maruarar Target 324 Rumah di Senen Juni</t>
+        </is>
+      </c>
+      <c r="D846" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096646/arahan-prabowo-maruarar-target-324-rumah-di-senen-juni</t>
+        </is>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B847" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C847" t="inlineStr">
+        <is>
+          <t>Barak PDIP Nilai Politik Luar Negeri Indonesia Bergeser</t>
+        </is>
+      </c>
+      <c r="D847" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096645/barak-pdip-nilai-politik-luar-negeri-indonesia-bergeser</t>
+        </is>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B848" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C848" t="inlineStr">
+        <is>
+          <t>Urgensi Standar Keamanan Transaksi Digital</t>
+        </is>
+      </c>
+      <c r="D848" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096638/urgensi-standar-keamanan-transaksi-digital</t>
+        </is>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B849" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C849" t="inlineStr">
+        <is>
+          <t>Apa Saja Langkah Penghematan di Kementerian Sosial</t>
+        </is>
+      </c>
+      <c r="D849" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096635/apa-saja-langkah-penghematan-di-kementerian-sosial</t>
+        </is>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B850" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C850" t="inlineStr">
+        <is>
+          <t>Pemerintah Dorong Kampus Terapkan WFH Satu Hari Sepekan</t>
+        </is>
+      </c>
+      <c r="D850" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096631/pemerintah-dorong-kampus-terapkan-wfh-satu-hari-sepekan</t>
+        </is>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B851" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C851" t="inlineStr">
+        <is>
+          <t>Prabowo Ingin Kampus Dilibatkan dalam Tata Ruang Kota</t>
+        </is>
+      </c>
+      <c r="D851" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096623/prabowo-ingin-kampus-dilibatkan-dalam-tata-ruang-kota</t>
+        </is>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B852" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C852" t="inlineStr">
+        <is>
+          <t>Ketua Banggar DPR Tak Setuju Pengurangan Subsidi BBM</t>
+        </is>
+      </c>
+      <c r="D852" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096618/ketua-banggar-dpr-tak-setuju-pengurangan-subsidi-bbm</t>
+        </is>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B853" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C853" t="inlineStr">
+        <is>
+          <t>DPR Agendakan Rapat Bahas Kasus Andrie Yunus-TNI Gugur</t>
+        </is>
+      </c>
+      <c r="D853" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096612/dpr-agendakan-rapat-bahas-kasus-andrie-yunus-tni-gugur</t>
+        </is>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B854" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C854" t="inlineStr">
+        <is>
+          <t>Sederet Langkah Penghematan di Kementerian Agama</t>
+        </is>
+      </c>
+      <c r="D854" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096607/sederet-langkah-penghematan-di-kementerian-agama</t>
+        </is>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B855" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C855" t="inlineStr">
+        <is>
+          <t>Respons Banggar DPR soal Usulan Dana MBG Dialihkan ke Guru</t>
+        </is>
+      </c>
+      <c r="D855" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096602/respons-banggar-dpr-soal-usulan-dana-mbg-dialihkan-ke-guru</t>
+        </is>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B856" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C856" t="inlineStr">
+        <is>
+          <t>Anggota DPR Yanuar Arif Wibowo Ingin Aset Negara Dinikmati Masyarakat</t>
+        </is>
+      </c>
+      <c r="D856" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096598/anggota-dpr-yanuar-arif-wibowo-ingin-aset-negara-dinikmati-masyarakat</t>
+        </is>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B857" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C857" t="inlineStr">
+        <is>
+          <t>Indonesia, Japan collaborate to bolster fisheries human resources</t>
+        </is>
+      </c>
+      <c r="D857" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411437/indonesia-japan-collaborate-to-bolster-fisheries-human-resources</t>
+        </is>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B858" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C858" t="inlineStr">
+        <is>
+          <t>OJK shuts down 953 illegal online lenders in Q1 2026</t>
+        </is>
+      </c>
+      <c r="D858" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411433/ojk-shuts-down-953-illegal-online-lenders-in-q1-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B859" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C859" t="inlineStr">
+        <is>
+          <t>Govt issues sanctions against 67 companies after Sumatra floods</t>
+        </is>
+      </c>
+      <c r="D859" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411429/govt-issues-sanctions-against-67-companies-after-sumatra-floods</t>
+        </is>
+      </c>
+    </row>
+    <row r="860">
+      <c r="A860" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B860" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C860" t="inlineStr">
+        <is>
+          <t>From cities to villages: harnessing the economic engine of Eid al-Fitr</t>
+        </is>
+      </c>
+      <c r="D860" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411425/from-cities-to-villages-harnessing-the-economic-engine-of-eid-al-fitr</t>
+        </is>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B861" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C861" t="inlineStr">
+        <is>
+          <t>Upgrading trust in Korea–Indonesia's strategic partnership</t>
+        </is>
+      </c>
+      <c r="D861" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411421/upgrading-trust-in-korea-indonesias-strategic-partnership</t>
+        </is>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B862" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C862" t="inlineStr">
+        <is>
+          <t>Govt targets renovation of 400 thousand people's houses in 2026</t>
+        </is>
+      </c>
+      <c r="D862" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411417/govt-targets-renovation-of-400-thousand-peoples-houses-in-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B863" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C863" t="inlineStr">
+        <is>
+          <t>Preventing fires, govt urges corporations to avoid land clearing</t>
+        </is>
+      </c>
+      <c r="D863" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411413/preventing-fires-govt-urges-corporations-to-avoid-land-clearing</t>
+        </is>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B864" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C864" t="inlineStr">
+        <is>
+          <t>OJK strengthens crypto ecosystem in response to transaction slowdown</t>
+        </is>
+      </c>
+      <c r="D864" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411409/ojk-strengthens-crypto-ecosystem-in-response-to-transaction-slowdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B865" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C865" t="inlineStr">
+        <is>
+          <t>Indonesia sets fuel surcharge ceiling to 38 percent amid rising costs</t>
+        </is>
+      </c>
+      <c r="D865" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411405/indonesia-sets-fuel-surcharge-ceiling-to-38-percent-amid-rising-costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B866" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>Waste management rate reaches 26 percent, up from 2024: Minister</t>
+        </is>
+      </c>
+      <c r="D866" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411401/waste-management-rate-reaches-26-percent-up-from-2024-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B867" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C867" t="inlineStr">
+        <is>
+          <t>Inflation in disaster-hit Sumatra eases as distribution recovers: govt</t>
+        </is>
+      </c>
+      <c r="D867" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411397/inflation-in-disaster-hit-sumatra-eases-as-distribution-recovers-govt</t>
+        </is>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B868" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C868" t="inlineStr">
+        <is>
+          <t>Extreme weather diverts several flights at Soekarno-Hatta Airport</t>
+        </is>
+      </c>
+      <c r="D868" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411393/extreme-weather-diverts-several-flights-at-soekarno-hatta-airport</t>
+        </is>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B869" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C869" t="inlineStr">
+        <is>
+          <t>Indonesia to roll out B50 biodiesel from July 1: Lahadalia</t>
+        </is>
+      </c>
+      <c r="D869" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411389/indonesia-to-roll-out-b50-biodiesel-from-july-1-lahadalia</t>
+        </is>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B870" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C870" t="inlineStr">
+        <is>
+          <t>Deputy minister calls for regions' commitment to eliminating TB</t>
+        </is>
+      </c>
+      <c r="D870" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411385/deputy-minister-calls-for-regions-commitment-to-eliminating-tb</t>
+        </is>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" t="inlineStr">
+        <is>
+          <t>Tuesday, 07 April 2026</t>
+        </is>
+      </c>
+      <c r="B871" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C871" t="inlineStr">
+        <is>
+          <t>Indonesia advances capital shift with 50 VP staff in Nusantara</t>
+        </is>
+      </c>
+      <c r="D871" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411381/indonesia-advances-capital-shift-with-50-vp-staff-in-nusantara</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D811"/>
+  <autoFilter ref="A1:D871"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -19103,6 +20423,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D809" r:id="rId808"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D810" r:id="rId809"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D811" r:id="rId810"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D812" r:id="rId811"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D813" r:id="rId812"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D814" r:id="rId813"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D815" r:id="rId814"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D816" r:id="rId815"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D817" r:id="rId816"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D818" r:id="rId817"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D819" r:id="rId818"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D820" r:id="rId819"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D821" r:id="rId820"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D822" r:id="rId821"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D823" r:id="rId822"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D824" r:id="rId823"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D825" r:id="rId824"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D826" r:id="rId825"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D827" r:id="rId826"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D828" r:id="rId827"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D829" r:id="rId828"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D830" r:id="rId829"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D831" r:id="rId830"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D832" r:id="rId831"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D833" r:id="rId832"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D834" r:id="rId833"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D835" r:id="rId834"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D836" r:id="rId835"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D837" r:id="rId836"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D838" r:id="rId837"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D839" r:id="rId838"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D840" r:id="rId839"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D841" r:id="rId840"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D842" r:id="rId841"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D843" r:id="rId842"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D844" r:id="rId843"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D845" r:id="rId844"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D846" r:id="rId845"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D847" r:id="rId846"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D848" r:id="rId847"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D849" r:id="rId848"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D850" r:id="rId849"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D851" r:id="rId850"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D852" r:id="rId851"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D853" r:id="rId852"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D854" r:id="rId853"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D855" r:id="rId854"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D856" r:id="rId855"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D857" r:id="rId856"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D858" r:id="rId857"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D859" r:id="rId858"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D860" r:id="rId859"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D861" r:id="rId860"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D862" r:id="rId861"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D863" r:id="rId862"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D864" r:id="rId863"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D865" r:id="rId864"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D866" r:id="rId865"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D867" r:id="rId866"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D868" r:id="rId867"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D869" r:id="rId868"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D870" r:id="rId869"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D871" r:id="rId870"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-07
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$871</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$931</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D871"/>
+  <dimension ref="A1:D931"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -19610,8 +19610,1328 @@
         </is>
       </c>
     </row>
+    <row r="872">
+      <c r="A872" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B872" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C872" t="inlineStr">
+        <is>
+          <t>Video: Marcella Zalianty Ketua PARFI '56 Tanggapi Banner Film Aku Harus Mati</t>
+        </is>
+      </c>
+      <c r="D872" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/detiktv/d-8433719/video-marcella-zalianty-ketua-parfi-56-tanggapi-banner-film-aku-harus-mati</t>
+        </is>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B873" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C873" t="inlineStr">
+        <is>
+          <t>Video: Rusia dan China Veto Resolusi Dewan Keamanan PBB soal Selat Hormuz</t>
+        </is>
+      </c>
+      <c r="D873" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8433989/video-rusia-dan-china-veto-resolusi-dewan-keamanan-pbb-soal-selat-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B874" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C874" t="inlineStr">
+        <is>
+          <t>Rusia dan China Veto Resolusi DK PBB soal Selat Hormuz</t>
+        </is>
+      </c>
+      <c r="D874" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8433969/rusia-dan-china-veto-resolusi-dk-pbb-soal-selat-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B875" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C875" t="inlineStr">
+        <is>
+          <t>AS-Israel Serang Pulau Kharg hingga Jembatan di Iran Jelang Deadline Trump</t>
+        </is>
+      </c>
+      <c r="D875" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8433834/as-israel-serang-pulau-kharg-hingga-jembatan-di-iran-jelang-deadline-trump</t>
+        </is>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B876" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C876" t="inlineStr">
+        <is>
+          <t>Dolar AS Ngamuk Tembus Rp 17.000/US$, Bank Indonesia Respons Begini</t>
+        </is>
+      </c>
+      <c r="D876" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/moneter/d-8433865/dolar-as-ngamuk-tembus-rp-17-000-us-bank-indonesia-respons-begini</t>
+        </is>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B877" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C877" t="inlineStr">
+        <is>
+          <t>Video: Serangan Jet Hantam Rumah di Irak, 3 Orang Tewas-5 Luka-luka</t>
+        </is>
+      </c>
+      <c r="D877" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8434025/video-serangan-jet-hantam-rumah-di-irak-3-orang-tewas-5-luka-luka</t>
+        </is>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B878" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C878" t="inlineStr">
+        <is>
+          <t>Video: Iran Ditekan AS, Aktivitas Kapal di Selat Hormuz Masih Terbatas</t>
+        </is>
+      </c>
+      <c r="D878" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8430802/video-iran-ditekan-as-aktivitas-kapal-di-selat-hormuz-masih-terbatas</t>
+        </is>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B879" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C879" t="inlineStr">
+        <is>
+          <t>Video: Trump Terang-terangan Ingin Minyak Iran</t>
+        </is>
+      </c>
+      <c r="D879" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8417351/video-trump-terang-terangan-ingin-minyak-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B880" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C880" t="inlineStr">
+        <is>
+          <t>Prabowo Kantongi Calon Pengganti 2 Dirjen PU yang Mundur</t>
+        </is>
+      </c>
+      <c r="D880" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8433938/prabowo-kantongi-calon-pengganti-2-dirjen-pu-yang-mundur</t>
+        </is>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B881" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C881" t="inlineStr">
+        <is>
+          <t>Sederet Makanan yang Bikin Ginjal Rusak, Nomor 6 Banyak Dikonsumsi Warga RI</t>
+        </is>
+      </c>
+      <c r="D881" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8433159/sederet-makanan-yang-bikin-ginjal-rusak-nomor-6-banyak-dikonsumsi-warga-ri</t>
+        </is>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B882" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C882" t="inlineStr">
+        <is>
+          <t>Menko Yusril Serahkan Putusan Kasasi Perkara Delpedro dkk ke MA</t>
+        </is>
+      </c>
+      <c r="D882" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8433910/menko-yusril-serahkan-putusan-kasasi-perkara-delpedro-dkk-ke-ma</t>
+        </is>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B883" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C883" t="inlineStr">
+        <is>
+          <t>Video: Respons AS Seusai Resolusi DK PBB soal Selat Hormuz Diveto China-Rusia</t>
+        </is>
+      </c>
+      <c r="D883" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260408-260408003/video-respons-as-seusai-resolusi-dk-pbb-soal-selat-hormuz-diveto-china-rusia</t>
+        </is>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B884" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C884" t="inlineStr">
+        <is>
+          <t>Video Paus Leo Kecam Ancaman Trump ke Rakyat Iran: Tak Dapat Diterima</t>
+        </is>
+      </c>
+      <c r="D884" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260408-260408004/video-paus-leo-kecam-ancaman-trump-ke-rakyat-iran-tak-dapat-diterima</t>
+        </is>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B885" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C885" t="inlineStr">
+        <is>
+          <t>Video: Gunung Semeru Erupsi, Masyarakat Diminta Waspada</t>
+        </is>
+      </c>
+      <c r="D885" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260407-260407140/video-gunung-semeru-erupsi-masyarakat-diminta-waspada</t>
+        </is>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B886" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C886" t="inlineStr">
+        <is>
+          <t>Pekan Kedua Final Four Proliga: JPE Evaluasi Internal</t>
+        </is>
+      </c>
+      <c r="D886" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sport-lain/d-8434020/pekan-kedua-final-four-proliga-jpe-evaluasi-internal</t>
+        </is>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B887" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C887" t="inlineStr">
+        <is>
+          <t>Dari Pikap hingga Truk Berat, Ini Daftar Merek di GIICOMVEC 2026</t>
+        </is>
+      </c>
+      <c r="D887" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1922051/dari-pikap-hingga-truk-berat-ini-daftar-merek-di-giicomvec-2026?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B888" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C888" t="inlineStr">
+        <is>
+          <t>Dago Elos Melawan Tak Bisa Dikalahkan</t>
+        </is>
+      </c>
+      <c r="D888" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/dago-elos-melawan-tak-bisa-dikalahkan?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B889" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C889" t="inlineStr">
+        <is>
+          <t>Lantik 12 Pejabat, Menaker: Jabatan Bukan Sekadar Posisi, Layanan Publik Harus Jadi Prioritas</t>
+        </is>
+      </c>
+      <c r="D889" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/07/19525121/lantik-12-pejabat-menaker-jabatan-bukan-sekadar-posisi-layanan-publik-harus</t>
+        </is>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B890" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C890" t="inlineStr">
+        <is>
+          <t>Ahli Lingkungan ITB: RDF Plant Solusi Paling Sesuai untuk Atasi Sampah Jakarta</t>
+        </is>
+      </c>
+      <c r="D890" s="2" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/04/07/19454751/ahli-lingkungan-itb-rdf-plant-solusi-paling-sesuai-untuk-atasi-sampah</t>
+        </is>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B891" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C891" t="inlineStr">
+        <is>
+          <t>Tingkatkan Kesejahteraan Lansia, Wakil Walkot Batam Salurkan Bansos</t>
+        </is>
+      </c>
+      <c r="D891" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/07/193352778/tingkatkan-kesejahteraan-lansia-wakil-walkot-batam-salurkan-bansos</t>
+        </is>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B892" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C892" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D892" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B893" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C893" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D893" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B894" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C894" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D894" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="895">
+      <c r="A895" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B895" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C895" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D895" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="896">
+      <c r="A896" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B896" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C896" t="inlineStr">
+        <is>
+          <t>Rusia Diam-diam Pasok Informasi Berharga untuk Iran, Apa Itu?</t>
+        </is>
+      </c>
+      <c r="D896" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1922019/rusia-diam-diam-pasok-informasi-berharga-untuk-iran-apa-itu?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="897">
+      <c r="A897" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B897" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C897" t="inlineStr">
+        <is>
+          <t>"The AI Doc", Keresahan tentang Perkembangan AI dan Etika AI</t>
+        </is>
+      </c>
+      <c r="D897" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/vrgultom/69d3e507ed641537b26a30e2/the-ai-doc-keresahan-tentang-perkembangan-ai-etika-ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="898">
+      <c r="A898" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B898" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C898" t="inlineStr">
+        <is>
+          <t>10 Taman Nasional Paling Ikonik di Jepang, Ada yang di Area Gunung Fuji</t>
+        </is>
+      </c>
+      <c r="D898" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5765/10-taman-nasional-paling-ikonik-di-jepang-ada-yang-di-area-gunung-fuji</t>
+        </is>
+      </c>
+    </row>
+    <row r="899">
+      <c r="A899" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B899" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C899" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D899" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="900">
+      <c r="A900" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B900" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C900" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D900" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="901">
+      <c r="A901" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B901" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C901" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Intip Bioskop Alfamart Pertama di Gading Serpong</t>
+        </is>
+      </c>
+      <c r="D901" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.kompas.com/read/2026/04/03/110300127/berita-foto--intip-bioskop-alfamart-pertama-di-gading-serpong</t>
+        </is>
+      </c>
+    </row>
+    <row r="902">
+      <c r="A902" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B902" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C902" t="inlineStr">
+        <is>
+          <t>Kementerian HAM Sisipkan Perlindungan Pembela HAM</t>
+        </is>
+      </c>
+      <c r="D902" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096905/kementerian-ham-sisipkan-perlindungan-pembela-ham</t>
+        </is>
+      </c>
+    </row>
+    <row r="903">
+      <c r="A903" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B903" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C903" t="inlineStr">
+        <is>
+          <t>Pemerintah Fokus Percepat Rehabilitasi Bencana Sumatera</t>
+        </is>
+      </c>
+      <c r="D903" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096903/pemerintah-fokus-percepat-rehabilitasi-bencana-sumatera</t>
+        </is>
+      </c>
+    </row>
+    <row r="904">
+      <c r="A904" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B904" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C904" t="inlineStr">
+        <is>
+          <t>BPJS Kesehatan Dorong Koperasi Jadi Fasilitas Kesehatan Desa</t>
+        </is>
+      </c>
+      <c r="D904" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096899/bpjs-kesehatan-dorong-koperasi-jadi-fasilitas-kesehatan-desa</t>
+        </is>
+      </c>
+    </row>
+    <row r="905">
+      <c r="A905" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B905" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C905" t="inlineStr">
+        <is>
+          <t>Menteri HAM Bantah Jawa Barat Intoleran, Singgung Satu Kasus</t>
+        </is>
+      </c>
+      <c r="D905" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096897/menteri-ham-bantah-jawa-barat-intoleran-singgung-satu-kasus</t>
+        </is>
+      </c>
+    </row>
+    <row r="906">
+      <c r="A906" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B906" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C906" t="inlineStr">
+        <is>
+          <t>AJI Desak Komdigi Cabut SK 127/2026, Bentuk Pembredelan</t>
+        </is>
+      </c>
+      <c r="D906" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096895/aji-desak-komdigi-cabut-sk-1272026-bentuk-pembredelan</t>
+        </is>
+      </c>
+    </row>
+    <row r="907">
+      <c r="A907" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B907" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C907" t="inlineStr">
+        <is>
+          <t>Puspom TNI Limpahkan Berkas Perkara Kasus Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D907" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096890/puspom-tni-limpahkan-berkas-perkara-kasus-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="908">
+      <c r="A908" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B908" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C908" t="inlineStr">
+        <is>
+          <t>Tanpa Kenaikan Pajak, PAD Jember Meningkat 36 Persen</t>
+        </is>
+      </c>
+      <c r="D908" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096889/tanpa-kenaikan-pajak-pad-jember-meningkat-36-persen</t>
+        </is>
+      </c>
+    </row>
+    <row r="909">
+      <c r="A909" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B909" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C909" t="inlineStr">
+        <is>
+          <t>Kota Semarang Siap Gelar Dialog Nasional, Bahas Makan Bergizi Gratis</t>
+        </is>
+      </c>
+      <c r="D909" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096879/kota-semarang-siap-gelar-dialog-nasional-bahas-makan-bergizi-gratis</t>
+        </is>
+      </c>
+    </row>
+    <row r="910">
+      <c r="A910" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B910" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C910" t="inlineStr">
+        <is>
+          <t>PT Kaltim Methanol Industri Raih Penghargaan PROPER Emas 2025</t>
+        </is>
+      </c>
+      <c r="D910" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096872/pt-kaltim-methanol-industri-raih-penghargaan-proper-emas-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="911">
+      <c r="A911" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B911" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C911" t="inlineStr">
+        <is>
+          <t>PTUN Jadwalkan Putusan Gugatan Terhadap Fadli Zon 21 April</t>
+        </is>
+      </c>
+      <c r="D911" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096870/ptun-jadwalkan-putusan-gugatan-terhadap-fadli-zon-21-april</t>
+        </is>
+      </c>
+    </row>
+    <row r="912">
+      <c r="A912" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B912" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C912" t="inlineStr">
+        <is>
+          <t>Kementerian HAM Usul Pembentukan RUU Kebebasan Umat Beragama</t>
+        </is>
+      </c>
+      <c r="D912" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096869/kementerian-ham-usul-pembentukan-ruu-kebebasan-umat-beragama</t>
+        </is>
+      </c>
+    </row>
+    <row r="913">
+      <c r="A913" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B913" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C913" t="inlineStr">
+        <is>
+          <t>Pigai: Hakim Penentu Apakah Sidang Andrie Yunus Terbuka</t>
+        </is>
+      </c>
+      <c r="D913" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096863/pigai-hakim-penentu-apakah-sidang-andrie-yunus-terbuka</t>
+        </is>
+      </c>
+    </row>
+    <row r="914">
+      <c r="A914" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B914" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C914" t="inlineStr">
+        <is>
+          <t>Pelajar yang Surati Prabowo Tolak MBG Mengalami Intimidasi</t>
+        </is>
+      </c>
+      <c r="D914" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096860/pelajar-yang-surati-prabowo-tolak-mbg-mengalami-intimidasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="915">
+      <c r="A915" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B915" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C915" t="inlineStr">
+        <is>
+          <t>Kumo Dorong Digitalisasi Layanan Kesehatan dan Klinik Gigi di APAC</t>
+        </is>
+      </c>
+      <c r="D915" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096857/kumo-dorong-digitalisasi-layanan-kesehatan-dan-klinik-gigi-di-apac</t>
+        </is>
+      </c>
+    </row>
+    <row r="916">
+      <c r="A916" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B916" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C916" t="inlineStr">
+        <is>
+          <t>Pemerintah Dorong Kompetensi Tenaga Kependidikan Merata</t>
+        </is>
+      </c>
+      <c r="D916" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2096855/pemerintah-dorong-kompetensi-tenaga-kependidikan-merata</t>
+        </is>
+      </c>
+    </row>
+    <row r="917">
+      <c r="A917" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B917" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C917" t="inlineStr">
+        <is>
+          <t>Indonesian govt says 2026 Hajj preparations nearly complete</t>
+        </is>
+      </c>
+      <c r="D917" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411583/indonesian-govt-says-2026-hajj-preparations-nearly-complete</t>
+        </is>
+      </c>
+    </row>
+    <row r="918">
+      <c r="A918" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B918" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C918" t="inlineStr">
+        <is>
+          <t>RI's finance minister says fuel subsidy policy follows president</t>
+        </is>
+      </c>
+      <c r="D918" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411580/ris-finance-minister-says-fuel-subsidy-policy-follows-president</t>
+        </is>
+      </c>
+    </row>
+    <row r="919">
+      <c r="A919" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B919" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C919" t="inlineStr">
+        <is>
+          <t>Arsari unit wins top green award, vows stronger action</t>
+        </is>
+      </c>
+      <c r="D919" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411576/arsari-unit-wins-top-green-award-vows-stronger-action</t>
+        </is>
+      </c>
+    </row>
+    <row r="920">
+      <c r="A920" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B920" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C920" t="inlineStr">
+        <is>
+          <t>World Health Day promotes science-based care for the elderly: Ministry</t>
+        </is>
+      </c>
+      <c r="D920" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411575/world-health-day-promotes-science-based-care-for-the-elderly-ministry</t>
+        </is>
+      </c>
+    </row>
+    <row r="921">
+      <c r="A921" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B921" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C921" t="inlineStr">
+        <is>
+          <t>Saudi Fund for Development Signs USD 15 Million Agreement with the Republic of Palau to Drive Local Economic Growth</t>
+        </is>
+      </c>
+      <c r="D921" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411571/saudi-fund-for-development-signs-usd-15-million-agreement-with-the-republic-of-palau-to-drive-local-economic-growth</t>
+        </is>
+      </c>
+    </row>
+    <row r="922">
+      <c r="A922" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B922" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C922" t="inlineStr">
+        <is>
+          <t>Maluku, Netherlands boost ties in education and commodities</t>
+        </is>
+      </c>
+      <c r="D922" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411567/maluku-netherlands-boost-ties-in-education-and-commodities</t>
+        </is>
+      </c>
+    </row>
+    <row r="923">
+      <c r="A923" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B923" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C923" t="inlineStr">
+        <is>
+          <t>Industry Ministry encourages SMEs to optimize digital technology</t>
+        </is>
+      </c>
+      <c r="D923" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411565/industry-ministry-encourages-smes-to-optimize-digital-technology</t>
+        </is>
+      </c>
+    </row>
+    <row r="924">
+      <c r="A924" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B924" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C924" t="inlineStr">
+        <is>
+          <t>Indonesia focuses on financing for UK-backed shipbuilding project</t>
+        </is>
+      </c>
+      <c r="D924" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411563/indonesia-focuses-on-financing-for-uk-backed-shipbuilding-project</t>
+        </is>
+      </c>
+    </row>
+    <row r="925">
+      <c r="A925" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B925" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C925" t="inlineStr">
+        <is>
+          <t>BI optimizes monetary instruments following rupiah's depreciation</t>
+        </is>
+      </c>
+      <c r="D925" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411562/bi-optimizes-monetary-instruments-following-rupiahs-depreciation</t>
+        </is>
+      </c>
+    </row>
+    <row r="926">
+      <c r="A926" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B926" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C926" t="inlineStr">
+        <is>
+          <t>Oil price tops US$100 to reduce growth by 0.1 percent: Bappenas</t>
+        </is>
+      </c>
+      <c r="D926" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411558/oil-price-tops-us100-to-reduce-growth-by-01-percent-bappenas</t>
+        </is>
+      </c>
+    </row>
+    <row r="927">
+      <c r="A927" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B927" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C927" t="inlineStr">
+        <is>
+          <t>Indonesia invites Uzbekistan to co-produce cultural history films</t>
+        </is>
+      </c>
+      <c r="D927" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411554/indonesia-invites-uzbekistan-to-co-produce-cultural-history-films</t>
+        </is>
+      </c>
+    </row>
+    <row r="928">
+      <c r="A928" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B928" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C928" t="inlineStr">
+        <is>
+          <t>Community infrastructure benefits low-income communities: Ministry</t>
+        </is>
+      </c>
+      <c r="D928" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411550/community-infrastructure-benefits-low-income-communities-ministry</t>
+        </is>
+      </c>
+    </row>
+    <row r="929">
+      <c r="A929" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B929" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C929" t="inlineStr">
+        <is>
+          <t>Indonesia's navy probes suspected unmanned sub found off Lombok</t>
+        </is>
+      </c>
+      <c r="D929" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411549/indonesias-navy-probes-suspected-unmanned-sub-found-off-lombok</t>
+        </is>
+      </c>
+    </row>
+    <row r="930">
+      <c r="A930" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B930" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C930" t="inlineStr">
+        <is>
+          <t>'Dana IndonesiaRaya' strengthens cultural ecosystem: MPR</t>
+        </is>
+      </c>
+      <c r="D930" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411546/dana-indonesiaraya-strengthens-cultural-ecosystem-mpr</t>
+        </is>
+      </c>
+    </row>
+    <row r="931">
+      <c r="A931" t="inlineStr">
+        <is>
+          <t>Wednesday, 08 April 2026</t>
+        </is>
+      </c>
+      <c r="B931" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C931" t="inlineStr">
+        <is>
+          <t>RI Govt aims to complete 100 Red-and-White fishermen villages by May</t>
+        </is>
+      </c>
+      <c r="D931" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411542/ri-govt-aims-to-complete-100-red-and-white-fishermen-villages-by-may</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D871"/>
+  <autoFilter ref="A1:D931"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -20483,6 +21803,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D869" r:id="rId868"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D870" r:id="rId869"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D871" r:id="rId870"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D872" r:id="rId871"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D873" r:id="rId872"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D874" r:id="rId873"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D875" r:id="rId874"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D876" r:id="rId875"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D877" r:id="rId876"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D878" r:id="rId877"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D879" r:id="rId878"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D880" r:id="rId879"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D881" r:id="rId880"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D882" r:id="rId881"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D883" r:id="rId882"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D884" r:id="rId883"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D885" r:id="rId884"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D886" r:id="rId885"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D887" r:id="rId886"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D888" r:id="rId887"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D889" r:id="rId888"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D890" r:id="rId889"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D891" r:id="rId890"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D892" r:id="rId891"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D893" r:id="rId892"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D894" r:id="rId893"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D895" r:id="rId894"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D896" r:id="rId895"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D897" r:id="rId896"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D898" r:id="rId897"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D899" r:id="rId898"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D900" r:id="rId899"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D901" r:id="rId900"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D902" r:id="rId901"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D903" r:id="rId902"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D904" r:id="rId903"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D905" r:id="rId904"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D906" r:id="rId905"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D907" r:id="rId906"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D908" r:id="rId907"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D909" r:id="rId908"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D910" r:id="rId909"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D911" r:id="rId910"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D912" r:id="rId911"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D913" r:id="rId912"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D914" r:id="rId913"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D915" r:id="rId914"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D916" r:id="rId915"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D917" r:id="rId916"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D918" r:id="rId917"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D919" r:id="rId918"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D920" r:id="rId919"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D921" r:id="rId920"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D922" r:id="rId921"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D923" r:id="rId922"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D924" r:id="rId923"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D925" r:id="rId924"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D926" r:id="rId925"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D927" r:id="rId926"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D928" r:id="rId927"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D929" r:id="rId928"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D930" r:id="rId929"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D931" r:id="rId930"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-08
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$931</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$976</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D931"/>
+  <dimension ref="A1:D976"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -20930,8 +20930,998 @@
         </is>
       </c>
     </row>
+    <row r="932">
+      <c r="A932" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B932" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C932" t="inlineStr">
+        <is>
+          <t>Rusia Tunggu AS di Meja Perundingan Usai Gencatan Senjata dengan Iran</t>
+        </is>
+      </c>
+      <c r="D932" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1922285/rusia-tunggu-as-di-meja-perundingan-usai-gencatan-senjata-dengan-iran?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="933">
+      <c r="A933" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B933" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C933" t="inlineStr">
+        <is>
+          <t>Izin PT Toba Pulp Lestari Dicabut, Langkah Awal Penyelamatan Ekologi di Sumut</t>
+        </is>
+      </c>
+      <c r="D933" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/izin-pt-toba-pulp-lestari-dicabut-langkah-awal-penyelamatan-ekologi-di-sumut?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="934">
+      <c r="A934" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B934" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C934" t="inlineStr">
+        <is>
+          <t>Gubernur Banten Dukung Larangan Vape demi Tangkal Narkoba Cair</t>
+        </is>
+      </c>
+      <c r="D934" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/08/211552578/gubernur-banten-dukung-larangan-vape-demi-tangkal-narkoba-cair</t>
+        </is>
+      </c>
+    </row>
+    <row r="935">
+      <c r="A935" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B935" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C935" t="inlineStr">
+        <is>
+          <t>Topang Kehidupan Penyintas Bencana, Satgas PRR Terus Dorong Penyaluran Aneka Bansos</t>
+        </is>
+      </c>
+      <c r="D935" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/08/17194341/topang-kehidupan-penyintas-bencana-satgas-prr-terus-dorong-penyaluran-aneka</t>
+        </is>
+      </c>
+    </row>
+    <row r="936">
+      <c r="A936" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B936" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C936" t="inlineStr">
+        <is>
+          <t>RDF Plant Dinilai Tepat Atasi Sampah Jakarta, Residu Diolah Jadi Bahan Bakar Industri</t>
+        </is>
+      </c>
+      <c r="D936" s="2" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/04/08/10411701/rdf-plant-dinilai-tepat-atasi-sampah-jakarta-residu-diolah-jadi-bahan</t>
+        </is>
+      </c>
+    </row>
+    <row r="937">
+      <c r="A937" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B937" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C937" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D937" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="938">
+      <c r="A938" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B938" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C938" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D938" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="939">
+      <c r="A939" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B939" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C939" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D939" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="940">
+      <c r="A940" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B940" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C940" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D940" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="941">
+      <c r="A941" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B941" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C941" t="inlineStr">
+        <is>
+          <t>Ratusan Makam Kucing di Perumahan Elit Jaksel</t>
+        </is>
+      </c>
+      <c r="D941" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1922267/ratusan-makam-kucing-di-perumahan-elit-jaksel?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="942">
+      <c r="A942" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B942" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C942" t="inlineStr">
+        <is>
+          <t>Sebuah Tempat pada Sebuah Cerita</t>
+        </is>
+      </c>
+      <c r="D942" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/ayahtuah/69d591d3c925c432a35c7222/sebuah-tempat-pada-sebuah-cerita</t>
+        </is>
+      </c>
+    </row>
+    <row r="943">
+      <c r="A943" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B943" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C943" t="inlineStr">
+        <is>
+          <t>Kenapa April Jadi Awal Baru di Jepang? Ini Penjelasan Tahun Ajaran hingga Dunia Kerja</t>
+        </is>
+      </c>
+      <c r="D943" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5784/kenapa-april-jadi-awal-baru-di-jepang-ini-penjelasan-tahun-ajaran-hingga-dunia-kerja</t>
+        </is>
+      </c>
+    </row>
+    <row r="944">
+      <c r="A944" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B944" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C944" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D944" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="945">
+      <c r="A945" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B945" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C945" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D945" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="946">
+      <c r="A946" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B946" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C946" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Intip Bioskop Alfamart Pertama di Gading Serpong</t>
+        </is>
+      </c>
+      <c r="D946" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.kompas.com/read/2026/04/03/110300127/berita-foto--intip-bioskop-alfamart-pertama-di-gading-serpong</t>
+        </is>
+      </c>
+    </row>
+    <row r="947">
+      <c r="A947" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B947" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C947" t="inlineStr">
+        <is>
+          <t>Respons Istana soal Usul Pembentukan TGPF Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D947" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097134/respons-istana-soal-usul-pembentukan-tgpf-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="948">
+      <c r="A948" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B948" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C948" t="inlineStr">
+        <is>
+          <t>Rumah Jokowi Jadi Replika "Tembok Ratapan" di Roblox</t>
+        </is>
+      </c>
+      <c r="D948" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097132/rumah-jokowi-jadi-replika-tembok-ratapan-di-roblox</t>
+        </is>
+      </c>
+    </row>
+    <row r="949">
+      <c r="A949" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B949" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C949" t="inlineStr">
+        <is>
+          <t>Andrie Yunus Ajukan Mosi Tidak Percaya ke Peradilan Militer</t>
+        </is>
+      </c>
+      <c r="D949" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097131/andrie-yunus-ajukan-mosi-tidak-percaya-ke-peradilan-militer</t>
+        </is>
+      </c>
+    </row>
+    <row r="950">
+      <c r="A950" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B950" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C950" t="inlineStr">
+        <is>
+          <t>Komnas HAM Surati TNI untuk Periksa 4 Penyerang Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D950" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097130/komnas-ham-surati-tni-untuk-periksa-4-penyerang-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="951">
+      <c r="A951" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B951" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C951" t="inlineStr">
+        <is>
+          <t>Prabowo Jawab Kritik soal Keras Kepala: Pejuang Iran juga</t>
+        </is>
+      </c>
+      <c r="D951" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097125/prabowo-jawab-kritik-soal-keras-kepala-pejuang-iran-juga</t>
+        </is>
+      </c>
+    </row>
+    <row r="952">
+      <c r="A952" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B952" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>BGN Mengklaim Motor MBG yang Dibeli di Bawah Harga Pasar</t>
+        </is>
+      </c>
+      <c r="D952" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097127/bgn-mengklaim-motor-mbg-yang-dibeli-di-bawah-harga-pasar</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B953" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>Menteri P2MI: Belum Ada Permintaan Evakuasi PMI Timur Tengah</t>
+        </is>
+      </c>
+      <c r="D953" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097119/menteri-p2mi-belum-ada-permintaan-evakuasi-pmi-timur-tengah</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B954" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>Andrie Yunus Menjalani Pemulihan Bola Mata</t>
+        </is>
+      </c>
+      <c r="D954" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097117/andrie-yunus-menjalani-pemulihan-bola-mata</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B955" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>Prabowo: Indonesia Termasuk Aman kalau Ada Perang Dunia III</t>
+        </is>
+      </c>
+      <c r="D955" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097111/prabowo-indonesia-termasuk-aman-kalau-ada-perang-dunia-iii</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B956" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>Korban Serangan Air Keras di Bangka Belitung Akan Dioperasi</t>
+        </is>
+      </c>
+      <c r="D956" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097109/korban-serangan-air-keras-di-bangka-belitung-akan-dioperasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B957" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>99,29 Persen SPBU Pulih, Pasokan BBM Lancar Jaya di Daerah Pascabencana Sumatra</t>
+        </is>
+      </c>
+      <c r="D957" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097107/9929-persen-spbu-pulih-pasokan-bbm-lancar-jaya-di-daerah-pascabencana-sumatra</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B958" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>Menteri Haji: Rute Penerbangan Jemaah Haji Masih Normal</t>
+        </is>
+      </c>
+      <c r="D958" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097101/menteri-haji-rute-penerbangan-jemaah-haji-masih-normal</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B959" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>DPRD Kabupaten Bogor SampaikanAspirasi Rakyat di Musrenbang RKPD</t>
+        </is>
+      </c>
+      <c r="D959" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097099/dprd-kabupaten-bogor-sampaikanaspirasi-rakyat-di-musrenbang-rkpd</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B960" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>Wali Kota Padang Fadly Amran Siap Selaraskan Program Pembangunan Kota dengan Provinsi</t>
+        </is>
+      </c>
+      <c r="D960" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097092/wali-kota-padang-fadly-amran-siap-selaraskan-program-pembangunan-kota-dengan-provinsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B961" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>BNI Bersama PBSI Perkuat Dukungan bagi Atlet Indonesia di BAC 2026</t>
+        </is>
+      </c>
+      <c r="D961" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097088/bni-bersama-pbsi-perkuat-dukungan-bagi-atlet-indonesia-di-bac-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B962" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>Minister denies reshuffle plan as salary cuts remain undecided</t>
+        </is>
+      </c>
+      <c r="D962" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411688/minister-denies-reshuffle-plan-as-salary-cuts-remain-undecided</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B963" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>Indonesia plans special financial hub to attract investors: Prabowo</t>
+        </is>
+      </c>
+      <c r="D963" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411684/indonesia-plans-special-financial-hub-to-attract-investors-prabowo</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B964" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>Indonesia's economic fundamentals steady despite global pressures</t>
+        </is>
+      </c>
+      <c r="D964" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411681/indonesias-economic-fundamentals-steady-despite-global-pressures</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B965" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>Indonesia seeks backing for 2029-30 UN Security Council bid</t>
+        </is>
+      </c>
+      <c r="D965" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411679/indonesia-seeks-backing-for-2029-30-un-security-council-bid</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B966" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>President Prabowo links overseas visits to oil supply push</t>
+        </is>
+      </c>
+      <c r="D966" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411677/president-prabowo-links-overseas-visits-to-oil-supply-push</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B967" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>Indonesia continues D-8 chairmanship agenda despite postponed summit</t>
+        </is>
+      </c>
+      <c r="D967" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411675/indonesia-continues-d-8-chairmanship-agenda-despite-postponed-summit</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B968" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>Indonesia to cut 2026 Hajj costs despite rising fuel prices</t>
+        </is>
+      </c>
+      <c r="D968" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411671/indonesia-to-cut-2026-hajj-costs-despite-rising-fuel-prices</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B969" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>Prabowo's core agenda includes continued transmigration: Ministry</t>
+        </is>
+      </c>
+      <c r="D969" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411667/prabowos-core-agenda-includes-continued-transmigration-ministry</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B970" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>CMES Indonesia International Machine Tool Exhibition 2026 Debuts July 2-4 in Jakarta</t>
+        </is>
+      </c>
+      <c r="D970" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411665/cmes-indonesia-international-machine-tool-exhibition-2026-debuts-july-2-4-in-jakarta</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B971" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>CMES Indonesia International Machine Tool Exhibition 2026 Debuts July 2-4 in Jakarta</t>
+        </is>
+      </c>
+      <c r="D971" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411663/cmes-indonesia-international-machine-tool-exhibition-2026-debuts-july-2-4-in-jakarta</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B972" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>Indonesia urges Meta, Google to complete 'PP Tunas' documents</t>
+        </is>
+      </c>
+      <c r="D972" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411661/indonesia-urges-meta-google-to-complete-pp-tunas-documents</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B973" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>Indonesian deputy minister urges students to embrace global mindset</t>
+        </is>
+      </c>
+      <c r="D973" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411659/indonesian-deputy-minister-urges-students-to-embrace-global-mindset</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B974" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>New Swisslog APeC structure delivers greater resources to Southeast Asian customers</t>
+        </is>
+      </c>
+      <c r="D974" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411655/new-swisslog-apec-structure-delivers-greater-resources-to-southeast-asian-customers</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B975" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>President Prabowo flags risks of AI-generated content</t>
+        </is>
+      </c>
+      <c r="D975" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411653/president-prabowo-flags-risks-of-ai-generated-content</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="inlineStr">
+        <is>
+          <t>Thursday, 09 April 2026</t>
+        </is>
+      </c>
+      <c r="B976" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>Indonesia taps campuses to boost skilled migrant workers</t>
+        </is>
+      </c>
+      <c r="D976" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411651/indonesia-taps-campuses-to-boost-skilled-migrant-workers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D931"/>
+  <autoFilter ref="A1:D976"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -21863,6 +22853,51 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D929" r:id="rId928"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D930" r:id="rId929"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D931" r:id="rId930"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D932" r:id="rId931"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D933" r:id="rId932"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D934" r:id="rId933"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D935" r:id="rId934"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D936" r:id="rId935"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D937" r:id="rId936"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D938" r:id="rId937"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D939" r:id="rId938"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D940" r:id="rId939"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D941" r:id="rId940"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D942" r:id="rId941"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D943" r:id="rId942"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D944" r:id="rId943"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D945" r:id="rId944"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D946" r:id="rId945"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D947" r:id="rId946"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D948" r:id="rId947"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D949" r:id="rId948"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D950" r:id="rId949"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D951" r:id="rId950"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D952" r:id="rId951"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D953" r:id="rId952"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D954" r:id="rId953"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D955" r:id="rId954"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D956" r:id="rId955"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D957" r:id="rId956"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D958" r:id="rId957"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D959" r:id="rId958"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D960" r:id="rId959"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D961" r:id="rId960"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D962" r:id="rId961"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D963" r:id="rId962"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D964" r:id="rId963"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D965" r:id="rId964"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D966" r:id="rId965"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D967" r:id="rId966"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D968" r:id="rId967"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D969" r:id="rId968"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D970" r:id="rId969"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D971" r:id="rId970"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D972" r:id="rId971"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D973" r:id="rId972"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D974" r:id="rId973"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D975" r:id="rId974"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D976" r:id="rId975"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-09
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$976</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1036</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D976"/>
+  <dimension ref="A1:D1036"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -21920,8 +21920,1328 @@
         </is>
       </c>
     </row>
+    <row r="977">
+      <c r="A977" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B977" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>Andy Robertson Tinggalkan Liverpool di Akhir Musim</t>
+        </is>
+      </c>
+      <c r="D977" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8437367/andy-robertson-tinggalkan-liverpool-di-akhir-musim</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B978" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>Diresmikan Prabowo, Kopdes di Kupang Masih Pakai Dana Pribadi</t>
+        </is>
+      </c>
+      <c r="D978" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/bali/nusra/d-8436876/diresmikan-prabowo-kopdes-di-kupang-masih-pakai-dana-pribadi</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B979" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>Video: Patuhi PP Tunas, Meta Ubah Batasan Usia Pengguna Jadi 16 Tahun</t>
+        </is>
+      </c>
+      <c r="D979" s="2" t="inlineStr">
+        <is>
+          <t>https://inet.detik.com/detiktv/d-8437285/video-patuhi-pp-tunas-meta-ubah-batasan-usia-pengguna-jadi-16-tahun</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B980" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>Video Penampakan Baby Whip Berisi 'Gas Tertawa' Ilegal Sitaan BPOM</t>
+        </is>
+      </c>
+      <c r="D980" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/detiktv/d-8437190/video-penampakan-baby-whip-berisi-gas-tertawa-ilegal-sitaan-bpom</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B981" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>Bisa Selesaikan dalam Sekali Lihat? Coba Uji Ketajaman Mata Lewat Permainan Ini</t>
+        </is>
+      </c>
+      <c r="D981" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/asah-otak/d-8437201/bisa-selesaikan-dalam-sekali-lihat-coba-uji-ketajaman-mata-lewat-permainan-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B982" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>Pekerja Asal Bali Ditahan di AS, Diduga Terlibat Kasus Kekerasan Seksual</t>
+        </is>
+      </c>
+      <c r="D982" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8437385/pekerja-asal-bali-ditahan-di-as-diduga-terlibat-kasus-kekerasan-seksual</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B983" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>Mahasiswa Untirta Perekam Dosen Diperiksa Polisi, Ternyata Ada Korban Lain</t>
+        </is>
+      </c>
+      <c r="D983" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8436001/mahasiswa-untirta-perekam-dosen-diperiksa-polisi-ternyata-ada-korban-lain</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B984" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>Polisi Periksa Mahasiswa di Serang yang Rekam Dosen di Toilet Pekan Ini</t>
+        </is>
+      </c>
+      <c r="D984" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8432389/polisi-periksa-mahasiswa-di-serang-yang-rekam-dosen-di-toilet-pekan-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B985" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>Kecam Israel, Rusia Desak Lebanon Jadi Bagian Gencatan Senjata AS-Iran</t>
+        </is>
+      </c>
+      <c r="D985" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8437289/kecam-israel-rusia-desak-lebanon-jadi-bagian-gencatan-senjata-as-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B986" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>Panjat Tebing Bawa Oleh-oleh 5 Tiket Asian Games 2026 dari Meishan</t>
+        </is>
+      </c>
+      <c r="D986" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sport-lain/d-8437376/panjat-tebing-bawa-oleh-oleh-5-tiket-asian-games-2026-dari-meishan</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B987" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>Menhub Wanti-wanti Kenaikan Tiket Pesawat: Nggak Boleh Lebih dari 13%!</t>
+        </is>
+      </c>
+      <c r="D987" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8437294/menhub-wanti-wanti-kenaikan-tiket-pesawat-nggak-boleh-lebih-dari-13</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B988" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>Video WHO: RS Lebanon Terancam Kehabisan Stok Medis gegara Serangan Israel</t>
+        </is>
+      </c>
+      <c r="D988" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260410-260410001/video-who-rs-lebanon-terancam-kehabisan-stok-medis-gegara-serangan-israel</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B989" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>Video: Menhub Buka Suara soal Peluang Aturan Ojol Masuk Revisi UU LLAJ</t>
+        </is>
+      </c>
+      <c r="D989" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260409-260409113/video-menhub-buka-suara-soal-peluang-aturan-ojol-masuk-revisi-uu-llaj</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B990" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>Video 147,55 Juta Orang Mudik saat Lebaran 2026</t>
+        </is>
+      </c>
+      <c r="D990" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260409-260409114/video-147-55-juta-orang-mudik-saat-lebaran-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B991" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>Hasil Lengkap Liga Europa: Aston Villa Sikat Bologna</t>
+        </is>
+      </c>
+      <c r="D991" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/uefa/d-8437375/hasil-lengkap-liga-europa-aston-villa-sikat-bologna</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B992" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>Momen Penyidik Kejati DKI Geledah Kementerian PU, Bawa Koper Besar</t>
+        </is>
+      </c>
+      <c r="D992" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1922553/momen-penyidik-kejati-dki-geledah-kementerian-pu-bawa-koper-besar?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B993" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>Kursi DPD Masih Diincar</t>
+        </is>
+      </c>
+      <c r="D993" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/kursi-dpd-masih-diincar?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B994" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>Kualitas SDM Ujung Tombak Kesuksesan Optimalisasi PHTC Presiden</t>
+        </is>
+      </c>
+      <c r="D994" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/09/19074931/kualitas-sdm-ujung-tombak-kesuksesan-optimalisasi-phtc-presiden</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B995" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>Mendagri Tito Ingatkan Pemda untuk Kreatif Tingkatkan PAD</t>
+        </is>
+      </c>
+      <c r="D995" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/09/16255931/mendagri-tito-ingatkan-pemda-untuk-kreatif-tingkatkan-pad</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B996" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>Buka Musrenbang Provinsi Sulut, Mendagri Ajak Pemda Tangkap Program Prioritas Nasional</t>
+        </is>
+      </c>
+      <c r="D996" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/09/16232901/buka-musrenbang-provinsi-sulut-mendagri-ajak-pemda-tangkap-program-prioritas</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B997" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D997" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B998" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D998" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D999" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D1000" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>Harga Minyak Melonjak, Permintaan Truk Listrik Meningkat</t>
+        </is>
+      </c>
+      <c r="D1001" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1922529/harga-minyak-melonjak-permintaan-truk-listrik-meningkat?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>Ketika Anak Mengajak Bermain Bareng, Tolak atau Iyain Aja Ya ?</t>
+        </is>
+      </c>
+      <c r="D1002" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/bapakdidin7237/69d210fbed64155a063b1c22/ketika-anak-mengajak-bermain-bareng-tolak-atau-iyain-aja-ya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>Aturan Berkendara di Jepang, Wajib Dipahami Sebelum Mengemudi</t>
+        </is>
+      </c>
+      <c r="D1003" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5774/aturan-berkendara-di-jepang-wajib-dipahami-sebelum-mengemudi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1004" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1005" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Penampakan Langka Bumi dan Bulan yang Dipotret Kru Artemis II NASA</t>
+        </is>
+      </c>
+      <c r="D1006" s="2" t="inlineStr">
+        <is>
+          <t>https://tekno.kompas.com/read/2026/04/09/18020027/berita-foto--penampakan-langka-bumi-dan-bulan-yang-dipotret-kru-artemis-ii-nasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>Kata Sekda Jawa Timur soal Efektivitas WFH pada Hari Rabu</t>
+        </is>
+      </c>
+      <c r="D1007" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097355/kata-sekda-jawa-timur-soal-efektivitas-wfh-pada-hari-rabu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>BNPP RI Perkuat Peran Da'i dalam Pembangunan Kawasan Perbatasan</t>
+        </is>
+      </c>
+      <c r="D1008" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097352/bnpp-ri-perkuat-peran-dai-dalam-pembangunan-kawasan-perbatasan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>BNPP RI Perkuat Kolaborasi Lintas Sektor untuk Kesejahteraan Masyarakat Pesisir</t>
+        </is>
+      </c>
+      <c r="D1009" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097341/bnpp-ri-perkuat-kolaborasi-lintas-sektor-untuk-kesejahteraan-masyarakat-pesisir</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Kementerian Wacanakan Sistem War Tiket untuk Berangkat Haji</t>
+        </is>
+      </c>
+      <c r="D1010" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097337/kementerian-wacanakan-sistem-war-tiket-untuk-berangkat-haji</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>Puskapol UI: Penundaan Revisi UU Pemilu Strategi Elite</t>
+        </is>
+      </c>
+      <c r="D1011" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097329/puskapol-ui-penundaan-revisi-uu-pemilu-strategi-elite</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Prabowo Targetkan Indonesia Tak Impor BBM dalam Tiga Tahun</t>
+        </is>
+      </c>
+      <c r="D1012" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097325/prabowo-targetkan-indonesia-tak-impor-bbm-dalam-tiga-tahun</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Penundaan Pembahasan Revisi UU Pemilu Rugikan Disabilitas</t>
+        </is>
+      </c>
+      <c r="D1013" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097320/penundaan-pembahasan-revisi-uu-pemilu-rugikan-disabilitas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>Pengadaan Motor MBG Tak Konsultasi dengan Komisi IX DPR</t>
+        </is>
+      </c>
+      <c r="D1014" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097319/pengadaan-motor-mbg-tak-konsultasi-dengan-komisi-ix-dpr</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>UI Terapkan Skema Kerja Fleksibel WFA-WFH untuk Hemat Energi</t>
+        </is>
+      </c>
+      <c r="D1015" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097318/ui-terapkan-skema-kerja-fleksibel-wfa-wfh-untuk-hemat-energi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>BGN Klaim Libatkan Kemenkeu dalam Pengadaan Barang untuk MBG</t>
+        </is>
+      </c>
+      <c r="D1016" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097316/bgn-klaim-libatkan-kemenkeu-dalam-pengadaan-barang-untuk-mbg</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>Korupsi Proyek Irigasi di Luwu, Kejari: Kerugian Bagi Masyarakat Petani</t>
+        </is>
+      </c>
+      <c r="D1017" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097313/korupsi-proyek-irigasi-di-luwu-kejari-kerugian-bagi-masyarakat-petani</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>Prabowo Dorong Garuda-Saudia Jajaki Joint Venture Haji</t>
+        </is>
+      </c>
+      <c r="D1018" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097311/prabowo-dorong-garuda-saudia-jajaki-joint-venture-haji</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>Penyebab Dedi Mulyadi Nonaktifkan Kepala Samsat</t>
+        </is>
+      </c>
+      <c r="D1019" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097310/penyebab-dedi-mulyadi-nonaktifkan-kepala-samsat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>Cara IPB University Cegah Kecurangan UTBK 2026</t>
+        </is>
+      </c>
+      <c r="D1020" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097305/cara-ipb-university-cegah-kecurangan-utbk-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>Pasar Rakyat Terdampak Banjir Sumatra Beroperasi 93,33 persen</t>
+        </is>
+      </c>
+      <c r="D1021" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097301/pasar-rakyat-terdampak-banjir-sumatra-beroperasi-9333-persen</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>Indonesia downplays World Bank growth cut to 4.7 percent</t>
+        </is>
+      </c>
+      <c r="D1022" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411829/indonesia-downplays-world-bank-growth-cut-to-47-percent</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Govt outlines strategy to expand digital infrastructure</t>
+        </is>
+      </c>
+      <c r="D1023" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411828/govt-outlines-strategy-to-expand-digital-infrastructure</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>Indonesia strongly condemns Israeli attacks in Lebanon</t>
+        </is>
+      </c>
+      <c r="D1024" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411824/indonesia-strongly-condemns-israeli-attacks-in-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>Frozen shrimp lead East Kalimantan exports in Q1</t>
+        </is>
+      </c>
+      <c r="D1025" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411823/frozen-shrimp-lead-east-kalimantan-exports-in-q1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>Indonesia secures naphtha supplies amid Middle East disruption</t>
+        </is>
+      </c>
+      <c r="D1026" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411820/indonesia-secures-naphtha-supplies-amid-middle-east-disruption</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>Indonesia's BPOM approves wider measles vaccine use amid outbreaks</t>
+        </is>
+      </c>
+      <c r="D1027" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411816/indonesias-bpom-approves-wider-measles-vaccine-use-amid-outbreaks</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>Indonesia targets domestic EV motorcycles, fuel bikes for export</t>
+        </is>
+      </c>
+      <c r="D1028" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411813/indonesia-targets-domestic-ev-motorcycles-fuel-bikes-for-export</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>Indonesia to expand internship program coverage: minister</t>
+        </is>
+      </c>
+      <c r="D1029" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411812/indonesia-to-expand-internship-program-coverage-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>Indonesian govt says disaster recovery in Sumatra still ongoing</t>
+        </is>
+      </c>
+      <c r="D1030" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411811/indonesian-govt-says-disaster-recovery-in-sumatra-still-ongoing</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>Danantara forms Denera to expand waste-to-energy push</t>
+        </is>
+      </c>
+      <c r="D1031" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411808/danantara-forms-denera-to-expand-waste-to-energy-push</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>Indonesia pushes cattle-palm integration to cut feed costs</t>
+        </is>
+      </c>
+      <c r="D1032" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411804/indonesia-pushes-cattle-palm-integration-to-cut-feed-costs</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>Meta complies with Indonesia's restrictions on access for children</t>
+        </is>
+      </c>
+      <c r="D1033" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411800/meta-complies-with-indonesias-restrictions-on-access-for-children</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>Indonesia warns Google after YouTube fails child safety standards</t>
+        </is>
+      </c>
+      <c r="D1034" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411799/indonesia-warns-google-after-youtube-fails-child-safety-standards</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>Prabowo calls Indonesia a "rising giant" amid global crisis</t>
+        </is>
+      </c>
+      <c r="D1035" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411797/prabowo-calls-indonesia-a-rising-giant-amid-global-crisis</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" t="inlineStr">
+        <is>
+          <t>Friday, 10 April 2026</t>
+        </is>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>RI's Air Force plans radar expansion to strengthen airspace monitoring</t>
+        </is>
+      </c>
+      <c r="D1036" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411793/ris-air-force-plans-radar-expansion-to-strengthen-airspace-monitoring</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D976"/>
+  <autoFilter ref="A1:D1036"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -22898,6 +24218,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D974" r:id="rId973"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D975" r:id="rId974"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D976" r:id="rId975"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D977" r:id="rId976"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D978" r:id="rId977"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D979" r:id="rId978"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D980" r:id="rId979"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D981" r:id="rId980"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D982" r:id="rId981"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D983" r:id="rId982"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D984" r:id="rId983"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D985" r:id="rId984"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D986" r:id="rId985"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D987" r:id="rId986"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D988" r:id="rId987"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D989" r:id="rId988"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D990" r:id="rId989"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D991" r:id="rId990"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D992" r:id="rId991"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D993" r:id="rId992"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D994" r:id="rId993"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D995" r:id="rId994"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D996" r:id="rId995"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D997" r:id="rId996"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D998" r:id="rId997"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D999" r:id="rId998"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1000" r:id="rId999"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1001" r:id="rId1000"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1002" r:id="rId1001"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1003" r:id="rId1002"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1004" r:id="rId1003"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1005" r:id="rId1004"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1006" r:id="rId1005"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1007" r:id="rId1006"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1008" r:id="rId1007"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1009" r:id="rId1008"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1010" r:id="rId1009"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1011" r:id="rId1010"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1012" r:id="rId1011"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1013" r:id="rId1012"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1014" r:id="rId1013"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1015" r:id="rId1014"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1016" r:id="rId1015"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1017" r:id="rId1016"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1018" r:id="rId1017"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1019" r:id="rId1018"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1020" r:id="rId1019"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1021" r:id="rId1020"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1022" r:id="rId1021"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1023" r:id="rId1022"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1024" r:id="rId1023"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1025" r:id="rId1024"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1026" r:id="rId1025"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1027" r:id="rId1026"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1028" r:id="rId1027"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1029" r:id="rId1028"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1030" r:id="rId1029"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1031" r:id="rId1030"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1032" r:id="rId1031"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1033" r:id="rId1032"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1034" r:id="rId1033"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1035" r:id="rId1034"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1036" r:id="rId1035"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-10
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1036</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1096</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1036"/>
+  <dimension ref="A1:D1096"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -23240,8 +23240,1328 @@
         </is>
       </c>
     </row>
+    <row r="1037">
+      <c r="A1037" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>Ahmad Sahroni Diperas KPK Gadungan Rp 300 Juta, Begini Kronologinya</t>
+        </is>
+      </c>
+      <c r="D1037" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/bali/hukum-dan-kriminal/d-8438529/ahmad-sahroni-diperas-kpk-gadungan-rp-300-juta-begini-kronologinya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>Pemerintah Tepis Isu Indonesia Bakal Chaos, Kasih Bukti BBM Nggak Naik</t>
+        </is>
+      </c>
+      <c r="D1038" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8438962/pemerintah-tepis-isu-indonesia-bakal-chaos-kasih-bukti-bbm-nggak-naik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>Geram ke Pengusaha Dablek, Prabowo Titah Jaksa Agung Pidanakan!</t>
+        </is>
+      </c>
+      <c r="D1039" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8438742/geram-ke-pengusaha-dablek-prabowo-titah-jaksa-agung-pidanakan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>Istana Minta Tak Cemas soal Kondisi Ekonomi: Dua Kali Lebaran, Stabil!</t>
+        </is>
+      </c>
+      <c r="D1040" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8438940/istana-minta-tak-cemas-soal-kondisi-ekonomi-dua-kali-lebaran-stabil</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>Tol Terpanjang RI Sepi Peminat, Investor Tak Tertarik</t>
+        </is>
+      </c>
+      <c r="D1041" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8438594/tol-terpanjang-ri-sepi-peminat-investor-tak-tertarik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>Kronologi Kapal China Berisi 3 ABK WNI di Perairan Pakistan-India Kena Rudal</t>
+        </is>
+      </c>
+      <c r="D1042" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8439080/kronologi-kapal-china-berisi-3-abk-wni-di-perairan-pakistan-india-kena-rudal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>Kapal China Berisi 3 ABK WNI Tertembak Rudal di Perairan Pakistan-India</t>
+        </is>
+      </c>
+      <c r="D1043" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8438967/kapal-china-berisi-3-abk-wni-tertembak-rudal-di-perairan-pakistan-india</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>9 ABK WNI Terjebak Hampir Setahun dalam Kapal di Mozambik Berhasil Dievakuasi</t>
+        </is>
+      </c>
+      <c r="D1044" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8123746/9-abk-wni-terjebak-hampir-setahun-dalam-kapal-di-mozambik-berhasil-dievakuasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>KPK OTT Bupati Tulungagung</t>
+        </is>
+      </c>
+      <c r="D1045" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8438942/kpk-ott-bupati-tulungagung</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>Rossi: Mustahil Motor Pelan Kalahkan Marc Marquez</t>
+        </is>
+      </c>
+      <c r="D1046" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/moto-gp/d-8439075/rossi-mustahil-motor-pelan-kalahkan-marc-marquez</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>Pemerintah Tepis Isu Indonesia Bakal Chaos, Kasih Bukti BBM Nggak Naik</t>
+        </is>
+      </c>
+      <c r="D1047" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8438962/pemerintah-tepis-isu-indonesia-bakal-chaos-kasih-bukti-bbm-nggak-naik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>Video: NASA dan Angkatan Laut AS Siap Jemput Astronaut Artemis II Usai Pendaratan</t>
+        </is>
+      </c>
+      <c r="D1048" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260411-260411003/video-nasa-dan-angkatan-laut-as-siap-jemput-astronaut-artemis-ii-usai-pendaratan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>Video: Kru Artemis II Segera Mendarat di Bumi, Bisa Ditonton di Sini!</t>
+        </is>
+      </c>
+      <c r="D1049" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260411-260411002/video-kru-artemis-ii-segera-mendarat-di-bumi-bisa-ditonton-di-sini</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>Video: OTT Tulungagung, KPK Amankan 16 Orang Termasuk Bupati Gatut Sunu</t>
+        </is>
+      </c>
+      <c r="D1050" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260411-260411001/video-ott-tulungagung-kpk-amankan-16-orang-termasuk-bupati-gatut-sunu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>Lebanon dan Israel Akan Bertemu di Washington Bahas Gencatan Senjata</t>
+        </is>
+      </c>
+      <c r="D1051" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8439074/lebanon-dan-israel-akan-bertemu-di-washington-bahas-gencatan-senjata</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>Bertolak ke Pakistan, Wapres AS Peringatkan Iran Tak Main-main dalam Negosiasi!</t>
+        </is>
+      </c>
+      <c r="D1052" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1922816/bertolak-ke-pakistan-wapres-as-peringatkan-iran-tak-main-main-dalam-negosiasi?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>Apa Saja Poin Kesepakatan Gencatan Senjata Iran dengan Amerika Serikat?</t>
+        </is>
+      </c>
+      <c r="D1053" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/apa-saja-poin-kesepakatan-gencatan-senjata-iran-dengan-amerika-serikat?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>Mendagri dan Menteri PKP Targetkan Renovasi 1.000 RTLH di Sitaro, Perkuat Perbatasan lewat Hunian Layak</t>
+        </is>
+      </c>
+      <c r="D1054" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/10/20455941/mendagri-dan-menteri-pkp-targetkan-renovasi-1000-rtlh-di-sitaro-perkuat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>Pastikan Program 3 Juta Rumah Berjalan, Mendagri Tinjau Perumahan Rakyat di Tomohon</t>
+        </is>
+      </c>
+      <c r="D1055" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/10/18392361/pastikan-program-3-juta-rumah-berjalan-mendagri-tinjau-perumahan-rakyat-di</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>Tinjau Dampak Banjir di Sitaro, Mendagri: Pemerintah Akan Tangani Rumah Terdampak</t>
+        </is>
+      </c>
+      <c r="D1056" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/10/17390161/tinjau-dampak-banjir-di-sitaro-mendagri-pemerintah-akan-tangani-rumah</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D1057" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D1058" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D1059" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D1060" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>Tak Diberi Uang, Preman Tanah Abang Pecahkan Mangkuk-mangkuk Pedagang Bakso</t>
+        </is>
+      </c>
+      <c r="D1061" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1922782/tak-diberi-uang-preman-tanah-abang-pecahkan-mangkuk-mangkuk-pedagang-bakso?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>Merajut di Tengah Notifikasi, Cara Sederhana Menyelamatkan Diri dari Lelah Digital</t>
+        </is>
+      </c>
+      <c r="D1062" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/belajarmenulis/69d876b2ed641571fa235552/merajut-di-tengah-notifikasi-cara-sederhana-menyelamatkan-diri-dari-lelah-digital</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>2 Tempat Melihat Sakura dari Atas Perahu di Tokyo, Chidorigafuchi Jadi Tujuan Wajib</t>
+        </is>
+      </c>
+      <c r="D1063" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5791/2-tempat-melihat-sakura-dari-atas-perahu-di-tokyo-chidorigafuchi-jadi-tujuan-wajib</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1064" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1065" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Penampakan Langka Bumi dan Bulan yang Dipotret Kru Artemis II NASA</t>
+        </is>
+      </c>
+      <c r="D1066" s="2" t="inlineStr">
+        <is>
+          <t>https://tekno.kompas.com/read/2026/04/09/18020027/berita-foto-penampakan-langka-bumi-dan-bulan-yang-dipotret-kru-artemis-ii-nasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>Jokowi Bantah JK Soal Kasus Ijazah Palsu Picu Konflik</t>
+        </is>
+      </c>
+      <c r="D1067" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097544/jokowi-bantah-jk-soal-kasus-ijazah-palsu-picu-konflik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>Kaltim Methanol Industri Gunakan CO2 Pupuk Kaltim untuk Produksi Metanol Rendah Emisi</t>
+        </is>
+      </c>
+      <c r="D1068" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097537/kaltim-methanol-industri-gunakan-co2-pupuk-kaltim-untuk-produksi-metanol-rendah-emisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>Kondisi WFH Perdana di Kampus Unpad dan UPI</t>
+        </is>
+      </c>
+      <c r="D1069" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097536/kondisi-wfh-perdana-di-kampus-unpad-dan-upi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>Mendagri dan Menteri PKP Targetkan Renovasi 1.000 RTLH di Sitaro</t>
+        </is>
+      </c>
+      <c r="D1070" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097533/mendagri-dan-menteri-pkp-targetkan-renovasi-1-000-rtlh-di-sitaro</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>Kaltim Methanol Industri Raih Penghargaan Green Leadership Tahun 2025</t>
+        </is>
+      </c>
+      <c r="D1071" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097532/kaltim-methanol-industri-raih-penghargaan-green-leadership-tahun-2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>JKN Memudahkan Pasien Jantung di Merauke Jalani Pengobatan Rutin</t>
+        </is>
+      </c>
+      <c r="D1072" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097528/jkn-memudahkan-pasien-jantung-di-merauke-jalani-pengobatan-rutin</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>Prabowo: Ada yang Pakai Kekuasaan Bantu Pencuri Uang Negara</t>
+        </is>
+      </c>
+      <c r="D1073" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097526/prabowo-ada-yang-pakai-kekuasaan-bantu-pencuri-uang-negara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>Prabowo Minta Jaksa Agung Menindak Pengusaha Dablek</t>
+        </is>
+      </c>
+      <c r="D1074" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097523/prabowo-minta-jaksa-agung-menindak-pengusaha-dablek</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>Jokowi Bantah Tudingan Bayar Rismon soal Perkara Ijazah</t>
+        </is>
+      </c>
+      <c r="D1075" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097519/jokowi-bantah-tudingan-bayar-rismon-soal-perkara-ijazah</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>Andi Arief: Masyarakat Tak Akan Memberontak pada Prabowo</t>
+        </is>
+      </c>
+      <c r="D1076" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097518/andi-arief-masyarakat-tak-akan-memberontak-pada-prabowo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>Prabowo Pidato di Depan Tumpukan Uang Sitaan Rp 11,4 triliun</t>
+        </is>
+      </c>
+      <c r="D1077" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097512/prabowo-pidato-di-depan-tumpukan-uang-sitaan-rp-114-triliun</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>Calon Peserta UTBK di ITB Meningkat, di Unpad Turun</t>
+        </is>
+      </c>
+      <c r="D1078" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097510/calon-peserta-utbk-di-itb-meningkat-di-unpad-turun</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>Ketum PBNU soal 3 TNI Tewas di Libanon: Risiko Terlibat Misi</t>
+        </is>
+      </c>
+      <c r="D1079" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097506/ketum-pbnu-soal-3-tni-tewas-di-libanon-risiko-terlibat-misi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>Komisi VIII DPR: Usulan Sistem War Tiket Haji Melawan UU</t>
+        </is>
+      </c>
+      <c r="D1080" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097500/komisi-viii-dpr-usulan-sistem-war-tiket-haji-melawan-uu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>Banjir Susulan Melanda Pidie Jaya, Kasatgas Tito Jelaskan Penyebabnya</t>
+        </is>
+      </c>
+      <c r="D1081" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097501/banjir-susulan-melanda-pidie-jaya-kasatgas-tito-jelaskan-penyebabnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>Indonesia targets 15,000 homes for renovation in border, remote areas</t>
+        </is>
+      </c>
+      <c r="D1082" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411929/indonesia-targets-15000-homes-for-renovation-in-border-remote-areas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>Indonesia's sacrifice in Lebanon and peacekeeping paradox</t>
+        </is>
+      </c>
+      <c r="D1083" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411927/indonesias-sacrifice-in-lebanon-and-peacekeeping-paradox</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>Indonesian govt backs Aceh polytechnic to train global nurses</t>
+        </is>
+      </c>
+      <c r="D1084" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411924/indonesian-govt-backs-aceh-polytechnic-to-train-global-nurses</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>Prabowo praises task force for reclaiming forest assets</t>
+        </is>
+      </c>
+      <c r="D1085" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411923/prabowo-praises-task-force-for-reclaiming-forest-assets</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>Indonesia must not lose to forest 'sucker' mafia: Attorney General</t>
+        </is>
+      </c>
+      <c r="D1086" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411919/indonesia-must-not-lose-to-forest-sucker-mafia-attorney-general</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>Indonesia rolls out measles shots for health workers</t>
+        </is>
+      </c>
+      <c r="D1087" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411915/indonesia-rolls-out-measles-shots-for-health-workers</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>Indonesia pushes export diversification via I-EAEU FTA</t>
+        </is>
+      </c>
+      <c r="D1088" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411913/indonesia-pushes-export-diversification-via-i-eaeu-fta</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>Prabowo stresses law enforcement to protect state assets</t>
+        </is>
+      </c>
+      <c r="D1089" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411909/prabowo-stresses-law-enforcement-to-protect-state-assets</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>Indonesian govt regains 5 million hectares of forest land</t>
+        </is>
+      </c>
+      <c r="D1090" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411908/indonesian-govt-regains-5-million-hectares-of-forest-land</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>Govt to use state asset recovery for schools, housing repair: Prabowo</t>
+        </is>
+      </c>
+      <c r="D1091" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411904/govt-to-use-state-asset-recovery-for-schools-housing-repair-prabowo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>Indonesia's Health Ministry reviews near baby mix-up in Bandung</t>
+        </is>
+      </c>
+      <c r="D1092" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411900/indonesias-health-ministry-reviews-near-baby-mix-up-in-bandung</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Indonesia, Russia strengthen economic cooperation through WGTII</t>
+        </is>
+      </c>
+      <c r="D1093" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411896/indonesia-russia-strengthen-economic-cooperation-through-wgtii</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Indonesia eyes Middle East to reduce steel export reliance</t>
+        </is>
+      </c>
+      <c r="D1094" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411893/indonesia-eyes-middle-east-to-reduce-steel-export-reliance</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Meta raises minimum age to access its services in Indonesia</t>
+        </is>
+      </c>
+      <c r="D1095" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411891/meta-raises-minimum-age-to-access-its-services-in-indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" t="inlineStr">
+        <is>
+          <t>Saturday, 11 April 2026</t>
+        </is>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>President Prabowo appoints new Ombudsman members</t>
+        </is>
+      </c>
+      <c r="D1096" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411889/president-prabowo-appoints-new-ombudsman-members</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1036"/>
+  <autoFilter ref="A1:D1096"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -24278,6 +25598,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1034" r:id="rId1033"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1035" r:id="rId1034"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1036" r:id="rId1035"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1037" r:id="rId1036"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1038" r:id="rId1037"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1039" r:id="rId1038"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1040" r:id="rId1039"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1041" r:id="rId1040"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1042" r:id="rId1041"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1043" r:id="rId1042"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1044" r:id="rId1043"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1045" r:id="rId1044"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1046" r:id="rId1045"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1047" r:id="rId1046"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1048" r:id="rId1047"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1049" r:id="rId1048"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1050" r:id="rId1049"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1051" r:id="rId1050"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1052" r:id="rId1051"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1053" r:id="rId1052"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1054" r:id="rId1053"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1055" r:id="rId1054"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1056" r:id="rId1055"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1057" r:id="rId1056"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1058" r:id="rId1057"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1059" r:id="rId1058"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1060" r:id="rId1059"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1061" r:id="rId1060"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1062" r:id="rId1061"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1063" r:id="rId1062"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1064" r:id="rId1063"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1065" r:id="rId1064"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1066" r:id="rId1065"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1067" r:id="rId1066"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1068" r:id="rId1067"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1069" r:id="rId1068"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1070" r:id="rId1069"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1071" r:id="rId1070"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1072" r:id="rId1071"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1073" r:id="rId1072"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1074" r:id="rId1073"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1075" r:id="rId1074"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1076" r:id="rId1075"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1077" r:id="rId1076"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1078" r:id="rId1077"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1079" r:id="rId1078"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1080" r:id="rId1079"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1081" r:id="rId1080"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1082" r:id="rId1081"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1083" r:id="rId1082"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1084" r:id="rId1083"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1085" r:id="rId1084"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1086" r:id="rId1085"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1087" r:id="rId1086"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1088" r:id="rId1087"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1089" r:id="rId1088"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1090" r:id="rId1089"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1091" r:id="rId1090"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1092" r:id="rId1091"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1093" r:id="rId1092"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1094" r:id="rId1093"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1095" r:id="rId1094"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1096" r:id="rId1095"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-11
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1096</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1141</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1096"/>
+  <dimension ref="A1:D1141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -24560,8 +24560,998 @@
         </is>
       </c>
     </row>
+    <row r="1097">
+      <c r="A1097" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>Mojtaba Khamenei Terluka Parah di Wajah dan Kaki, Masih Ikut Rapat dengan Petinggi Iran</t>
+        </is>
+      </c>
+      <c r="D1097" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1922965/mojtaba-khamenei-terluka-parah-di-wajah-dan-kaki-masih-ikut-rapat-dengan-petinggi-iran?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>Kalkulasi Mahalnya Harga Politik BBM</t>
+        </is>
+      </c>
+      <c r="D1098" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/kalkulasi-mahalnya-harga-politik-bbm?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>Satgas PRR Pastikan Pemutakhiran Data Penerima Huntara dan DTH Terus Dilakukan</t>
+        </is>
+      </c>
+      <c r="D1099" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/11/21303101/satgas-prr-pastikan-pemutakhiran-data-penerima-huntara-dan-dth-terus</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>Freeport-Serikat Pekerja Teken PKB Baru, Fokus pada Kesejahteraan dan Keselamatan</t>
+        </is>
+      </c>
+      <c r="D1100" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/11/15343861/freeport-serikat-pekerja-teken-pkb-baru-fokus-pada-kesejahteraan-dan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>NodesGroup Luncurkan Sistem Lacak Servis dan Layanan Pickup-Delivery</t>
+        </is>
+      </c>
+      <c r="D1101" s="2" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/04/11/115440526/nodesgroup-luncurkan-sistem-lacak-servis-dan-layanan-pickup-delivery</t>
+        </is>
+      </c>
+    </row>
+    <row r="1102">
+      <c r="A1102" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1102" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1102" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D1102" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1103">
+      <c r="A1103" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1103" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1103" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D1103" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1104">
+      <c r="A1104" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1104" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1104" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D1104" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1105">
+      <c r="A1105" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1105" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1105" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D1105" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1106">
+      <c r="A1106" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1106" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1106" t="inlineStr">
+        <is>
+          <t>Kim Jong Un Dukung China Wujudkan Dunia Multipolar, Singkirkan Dominasi AS?</t>
+        </is>
+      </c>
+      <c r="D1106" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1922909/kim-jong-un-dukung-china-wujudkan-dunia-multipolar-singkirkan-dominasi-as?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1107">
+      <c r="A1107" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1107" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1107" t="inlineStr">
+        <is>
+          <t>Cerpen: Selamat Ulang Tahun</t>
+        </is>
+      </c>
+      <c r="D1107" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/geokenarfairuzrachman1901/69d81758ed64150e63139c02/selamat-ulang-tahun</t>
+        </is>
+      </c>
+    </row>
+    <row r="1108">
+      <c r="A1108" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1108" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1108" t="inlineStr">
+        <is>
+          <t>Pengalaman Pertama Tukar Kartu Nama di Jepang, Ternyata Tak Sesederhana yang Dibayangkan</t>
+        </is>
+      </c>
+      <c r="D1108" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5800/pengalaman-pertama-tukar-kartu-nama-di-jepang-ternyata-tak-sesederhana-yang-dibayangkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1109">
+      <c r="A1109" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1109" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1109" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1109" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1110">
+      <c r="A1110" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1110" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1110" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1110" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1111">
+      <c r="A1111" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1111" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1111" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Penampakan Langka Bumi dan Bulan yang Dipotret Kru Artemis II NASA</t>
+        </is>
+      </c>
+      <c r="D1111" s="2" t="inlineStr">
+        <is>
+          <t>https://tekno.kompas.com/read/2026/04/09/18020027/berita-foto-penampakan-langka-bumi-dan-bulan-yang-dipotret-kru-artemis-ii-nasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1112">
+      <c r="A1112" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1112" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1112" t="inlineStr">
+        <is>
+          <t>Wali Kota Semarang Diminta Segera Realisasikan Program Perjalanan Keagamaan</t>
+        </is>
+      </c>
+      <c r="D1112" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097668/wali-kota-semarang-diminta-segera-realisasikan-program-perjalanan-keagamaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1113">
+      <c r="A1113" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1113" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1113" t="inlineStr">
+        <is>
+          <t>HUT ke-479 Kota Semarang, Pemkot Siapkan 17 Kado untuk Masyarakat</t>
+        </is>
+      </c>
+      <c r="D1113" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097665/hut-ke-479-kota-semarang-pemkot-siapkan-17-kado-untuk-masyarakat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1114">
+      <c r="A1114" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1114" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1114" t="inlineStr">
+        <is>
+          <t>Prabowo Prihatin Banyak Orang yang Lebih Suka Budaya Asing</t>
+        </is>
+      </c>
+      <c r="D1114" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097664/prabowo-prihatin-banyak-orang-yang-lebih-suka-budaya-asing</t>
+        </is>
+      </c>
+    </row>
+    <row r="1115">
+      <c r="A1115" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1115" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1115" t="inlineStr">
+        <is>
+          <t>DPR Minta Adanya Kajian untuk Penggolongan UKT bagi Anak ASN</t>
+        </is>
+      </c>
+      <c r="D1115" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097662/dpr-minta-adanya-kajian-untuk-penggolongan-ukt-bagi-anak-asn</t>
+        </is>
+      </c>
+    </row>
+    <row r="1116">
+      <c r="A1116" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1116" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1116" t="inlineStr">
+        <is>
+          <t>Prabowo Ingin Pencak Silat Jadi Cabang Olahraga Olimpiade</t>
+        </is>
+      </c>
+      <c r="D1116" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097659/prabowo-ingin-pencak-silat-jadi-cabang-olahraga-olimpiade</t>
+        </is>
+      </c>
+    </row>
+    <row r="1117">
+      <c r="A1117" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1117" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1117" t="inlineStr">
+        <is>
+          <t>Komnas HAM: Penyelesaian Rekomendasi Kasus Andrie Prioritas</t>
+        </is>
+      </c>
+      <c r="D1117" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097657/komnas-ham-penyelesaian-rekomendasi-kasus-andrie-prioritas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1118">
+      <c r="A1118" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1118" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1118" t="inlineStr">
+        <is>
+          <t>Dari One Piece hingga Solo Leveling, Ini 7 Manga dan Komik yang Menarik untuk Dibaca</t>
+        </is>
+      </c>
+      <c r="D1118" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097652/dari-one-piece-hingga-solo-leveling-ini-7-manga-dan-komik-yang-menarik-untuk-dibaca</t>
+        </is>
+      </c>
+    </row>
+    <row r="1119">
+      <c r="A1119" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1119" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1119" t="inlineStr">
+        <is>
+          <t>Mahasiswa Peduli Andrie Yunus Bakal Berkemah di Puspom TNI</t>
+        </is>
+      </c>
+      <c r="D1119" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097649/mahasiswa-peduli-andrie-yunus-bakal-berkemah-di-puspom-tni</t>
+        </is>
+      </c>
+    </row>
+    <row r="1120">
+      <c r="A1120" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1120" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1120" t="inlineStr">
+        <is>
+          <t>Kata Komnas HAM soal Usul Gibran Libatkan Hakim Ad Hoc di Kasus Andrie</t>
+        </is>
+      </c>
+      <c r="D1120" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097645/kata-komnas-ham-soal-usul-gibran-libatkan-hakim-ad-hoc-di-kasus-andrie</t>
+        </is>
+      </c>
+    </row>
+    <row r="1121">
+      <c r="A1121" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1121" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1121" t="inlineStr">
+        <is>
+          <t>Komnas HAM Gelar Diskusi dengan Kolektif Merpati, Bahas Apa?</t>
+        </is>
+      </c>
+      <c r="D1121" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097642/komnas-ham-gelar-diskusi-dengan-kolektif-merpati-bahas-apa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1122">
+      <c r="A1122" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1122" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1122" t="inlineStr">
+        <is>
+          <t>Prabowo Mengenang Saat di Akmil: Saya Agak Nakal Waktu Itu</t>
+        </is>
+      </c>
+      <c r="D1122" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097630/prabowo-mengenang-saat-di-akmil-saya-agak-nakal-waktu-itu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1123">
+      <c r="A1123" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1123" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1123" t="inlineStr">
+        <is>
+          <t>Seskab Teddy Soal Isu Indonesia Akan Chaos: Semua Terkendali</t>
+        </is>
+      </c>
+      <c r="D1123" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097629/seskab-teddy-soal-isu-indonesia-akan-chaos-semua-terkendali</t>
+        </is>
+      </c>
+    </row>
+    <row r="1124">
+      <c r="A1124" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1124" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1124" t="inlineStr">
+        <is>
+          <t>Wamenhaj Paparkan Mekanisme War Ticket Haji</t>
+        </is>
+      </c>
+      <c r="D1124" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097627/wamenhaj-paparkan-mekanisme-war-ticket-haji</t>
+        </is>
+      </c>
+    </row>
+    <row r="1125">
+      <c r="A1125" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1125" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1125" t="inlineStr">
+        <is>
+          <t>Prabowo Lepas Jabatan Ketua Umum PB IPSI</t>
+        </is>
+      </c>
+      <c r="D1125" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097624/prabowo-lepas-jabatan-ketua-umum-pb-ipsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1126">
+      <c r="A1126" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1126" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1126" t="inlineStr">
+        <is>
+          <t>Prabowo Dijadwalkan Berkunjung ke Rusia dalam Waktu Dekat</t>
+        </is>
+      </c>
+      <c r="D1126" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097621/prabowo-dijadwalkan-berkunjung-ke-rusia-dalam-waktu-dekat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1127">
+      <c r="A1127" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1127" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1127" t="inlineStr">
+        <is>
+          <t>Prabowo concludes multi-decade tenure as PB IPSI chairperson</t>
+        </is>
+      </c>
+      <c r="D1127" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411976/prabowo-concludes-multi-decade-tenure-as-pb-ipsi-chairperson</t>
+        </is>
+      </c>
+    </row>
+    <row r="1128">
+      <c r="A1128" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1128" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1128" t="inlineStr">
+        <is>
+          <t>Indonesia considers EV incentives with industry, regulators</t>
+        </is>
+      </c>
+      <c r="D1128" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411973/indonesia-considers-ev-incentives-with-industry-regulators</t>
+        </is>
+      </c>
+    </row>
+    <row r="1129">
+      <c r="A1129" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1129" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1129" t="inlineStr">
+        <is>
+          <t>RI opens opportunities for research collaboration with Qatar</t>
+        </is>
+      </c>
+      <c r="D1129" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411972/ri-opens-opportunities-for-research-collaboration-with-qatar</t>
+        </is>
+      </c>
+    </row>
+    <row r="1130">
+      <c r="A1130" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1130" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1130" t="inlineStr">
+        <is>
+          <t>Indonesia promotes human rights through EU dialogue</t>
+        </is>
+      </c>
+      <c r="D1130" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411971/indonesia-promotes-human-rights-through-eu-dialogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="1131">
+      <c r="A1131" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1131" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1131" t="inlineStr">
+        <is>
+          <t>Energy efficiency key to bolstering energy security : Council</t>
+        </is>
+      </c>
+      <c r="D1131" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411968/energy-efficiency-key-to-bolstering-energy-security-council</t>
+        </is>
+      </c>
+    </row>
+    <row r="1132">
+      <c r="A1132" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1132" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1132" t="inlineStr">
+        <is>
+          <t>Pencak silat martial arts reflects Indonesian character : Prabowo</t>
+        </is>
+      </c>
+      <c r="D1132" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411967/pencak-silat-martial-arts-reflects-indonesian-character-prabowo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1133">
+      <c r="A1133" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1133" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1133" t="inlineStr">
+        <is>
+          <t>BRIN researcher develops sourdough from local red rice</t>
+        </is>
+      </c>
+      <c r="D1133" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411964/brin-researcher-develops-sourdough-from-local-red-rice</t>
+        </is>
+      </c>
+    </row>
+    <row r="1134">
+      <c r="A1134" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1134" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1134" t="inlineStr">
+        <is>
+          <t>Prabowo wants pencak silat to be contested in Olympics</t>
+        </is>
+      </c>
+      <c r="D1134" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411961/prabowo-wants-pencak-silat-to-be-contested-in-olympics</t>
+        </is>
+      </c>
+    </row>
+    <row r="1135">
+      <c r="A1135" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1135" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1135" t="inlineStr">
+        <is>
+          <t>Tourism Ministry moves to bolster Bali's accommodation governance</t>
+        </is>
+      </c>
+      <c r="D1135" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411959/tourism-ministry-moves-to-bolster-balis-accommodation-governance</t>
+        </is>
+      </c>
+    </row>
+    <row r="1136">
+      <c r="A1136" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1136" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1136" t="inlineStr">
+        <is>
+          <t>Indonesia sees strong industry push for green steel transition</t>
+        </is>
+      </c>
+      <c r="D1136" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411957/indonesia-sees-strong-industry-push-for-green-steel-transition</t>
+        </is>
+      </c>
+    </row>
+    <row r="1137">
+      <c r="A1137" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1137" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1137" t="inlineStr">
+        <is>
+          <t>Need synergy to end violence against Down syndrome children: Ministry</t>
+        </is>
+      </c>
+      <c r="D1137" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411955/need-synergy-to-end-violence-against-down-syndrome-children-ministry</t>
+        </is>
+      </c>
+    </row>
+    <row r="1138">
+      <c r="A1138" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1138" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1138" t="inlineStr">
+        <is>
+          <t>Indonesia focuses on wellness tourism to boost arrivals: Ministry</t>
+        </is>
+      </c>
+      <c r="D1138" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411953/indonesia-focuses-on-wellness-tourism-to-boost-arrivals-ministry</t>
+        </is>
+      </c>
+    </row>
+    <row r="1139">
+      <c r="A1139" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1139" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1139" t="inlineStr">
+        <is>
+          <t>Indonesia rejects double standards in advancing global human rights</t>
+        </is>
+      </c>
+      <c r="D1139" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411952/indonesia-rejects-double-standards-in-advancing-global-human-rights</t>
+        </is>
+      </c>
+    </row>
+    <row r="1140">
+      <c r="A1140" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1140" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1140" t="inlineStr">
+        <is>
+          <t>Gov't accelerates recovery of disaster-affected MSMEs through MBG</t>
+        </is>
+      </c>
+      <c r="D1140" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411948/govt-accelerates-recovery-of-disaster-affected-msmes-through-mbg</t>
+        </is>
+      </c>
+    </row>
+    <row r="1141">
+      <c r="A1141" t="inlineStr">
+        <is>
+          <t>Sunday, 12 April 2026</t>
+        </is>
+      </c>
+      <c r="B1141" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1141" t="inlineStr">
+        <is>
+          <t>Indonesia boosts development in border areas, minister affirms</t>
+        </is>
+      </c>
+      <c r="D1141" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411944/indonesia-boosts-development-in-border-areas-minister-affirms</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1096"/>
+  <autoFilter ref="A1:D1141"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -25658,6 +26648,51 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1094" r:id="rId1093"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1095" r:id="rId1094"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1096" r:id="rId1095"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1097" r:id="rId1096"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1098" r:id="rId1097"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1099" r:id="rId1098"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1100" r:id="rId1099"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1101" r:id="rId1100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1102" r:id="rId1101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1103" r:id="rId1102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1104" r:id="rId1103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1105" r:id="rId1104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1106" r:id="rId1105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1107" r:id="rId1106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1108" r:id="rId1107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1109" r:id="rId1108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1110" r:id="rId1109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1111" r:id="rId1110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1112" r:id="rId1111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1113" r:id="rId1112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1114" r:id="rId1113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1115" r:id="rId1114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1116" r:id="rId1115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1117" r:id="rId1116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1118" r:id="rId1117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1119" r:id="rId1118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1120" r:id="rId1119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1121" r:id="rId1120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1122" r:id="rId1121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1123" r:id="rId1122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1124" r:id="rId1123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1125" r:id="rId1124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1126" r:id="rId1125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1127" r:id="rId1126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1128" r:id="rId1127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1129" r:id="rId1128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1130" r:id="rId1129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1131" r:id="rId1130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1132" r:id="rId1131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1133" r:id="rId1132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1134" r:id="rId1133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1135" r:id="rId1134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1136" r:id="rId1135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1137" r:id="rId1136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1138" r:id="rId1137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1139" r:id="rId1138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1140" r:id="rId1139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1141" r:id="rId1140"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-12
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1141</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1201</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1141"/>
+  <dimension ref="A1:D1201"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -25550,8 +25550,1328 @@
         </is>
       </c>
     </row>
+    <row r="1142">
+      <c r="A1142" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1142" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1142" t="inlineStr">
+        <is>
+          <t>Liburan Pilu, 30 Orang Tewas Desak-desakan di Benteng Laferriere</t>
+        </is>
+      </c>
+      <c r="D1142" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.detik.com/travel-news/d-8440966/liburan-pilu-30-orang-tewas-desak-desakan-di-benteng-laferriere</t>
+        </is>
+      </c>
+    </row>
+    <row r="1143">
+      <c r="A1143" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1143" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1143" t="inlineStr">
+        <is>
+          <t>Liburan Hemat Jakarta-Purwakarta Naik Kereta Rp 8.000, Sudah Coba atau Belum?</t>
+        </is>
+      </c>
+      <c r="D1143" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.detik.com/travel-news/d-8440945/liburan-hemat-jakarta-purwarta-naik-kereta-sudah-coba-atau-beum</t>
+        </is>
+      </c>
+    </row>
+    <row r="1144">
+      <c r="A1144" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1144" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1144" t="inlineStr">
+        <is>
+          <t>Penjualan Mobil Listrik Bulan Maret Turun, BYD Atto 1 Cuma Segini</t>
+        </is>
+      </c>
+      <c r="D1144" s="2" t="inlineStr">
+        <is>
+          <t>https://oto.detik.com/mobil-listrik/d-8440926/penjualan-mobil-listrik-bulan-maret-turun-byd-atto-1-cuma-segini</t>
+        </is>
+      </c>
+    </row>
+    <row r="1145">
+      <c r="A1145" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1145" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1145" t="inlineStr">
+        <is>
+          <t>Dubai Batasi Penerbangan, Maskapai-Maskapai India Meradang</t>
+        </is>
+      </c>
+      <c r="D1145" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.detik.com/travel-news/d-8440740/dubai-batasi-penerbangan-maskapai-maskapai-india-meradang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1146">
+      <c r="A1146" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1146" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1146" t="inlineStr">
+        <is>
+          <t>Butuh 'Otak Lemes' untuk Pecahkan Teka-teki Ini, Kanebo Kering Minggir Dulu</t>
+        </is>
+      </c>
+      <c r="D1146" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/asah-otak/d-8440187/butuh-otak-lemes-untuk-pecahkan-teka-teki-ini-kanebo-kering-minggir-dulu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1147">
+      <c r="A1147" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1147" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1147" t="inlineStr">
+        <is>
+          <t>Heboh Benda Bercahaya di Langit Malang Dikira Rudal, Ternyata Sampah Antariksa</t>
+        </is>
+      </c>
+      <c r="D1147" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8441324/heboh-benda-bercahaya-di-langit-malang-dikira-rudal-ternyata-sampah-antariksa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1148">
+      <c r="A1148" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1148" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1148" t="inlineStr">
+        <is>
+          <t>Usai Kena Tipu, Korban Bakal Laporkan Rey Pelaku Nikah Sesama Wanita ke Polisi</t>
+        </is>
+      </c>
+      <c r="D1148" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8441315/usai-kena-tipu-korban-bakal-laporkan-rey-pelaku-nikah-sesama-wanita-ke-polisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1149">
+      <c r="A1149" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1149" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1149" t="inlineStr">
+        <is>
+          <t>Apa itu El Nino? Ini Prediksi Tahun 2026 dan Langkah Antisipasi Dampaknya</t>
+        </is>
+      </c>
+      <c r="D1149" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8440560/apa-itu-el-nino-ini-prediksi-tahun-2026-dan-langkah-antisipasi-dampaknya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1150">
+      <c r="A1150" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1150" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1150" t="inlineStr">
+        <is>
+          <t>Hasil Piala AFF Futsal 2026: Kalah dari Thailand, Indonesia Gagal Juara</t>
+        </is>
+      </c>
+      <c r="D1150" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8441268/hasil-piala-aff-futsal-2026-kalah-dari-thailand-indonesia-gagal-juara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1151">
+      <c r="A1151" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1151" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1151" t="inlineStr">
+        <is>
+          <t>Nathan Tjoe-A-On Kembali Tampil Usai Kasus Paspoortgate</t>
+        </is>
+      </c>
+      <c r="D1151" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8441323/nathan-tjoe-a-on-kembali-tampil-usai-kasus-paspoortgate</t>
+        </is>
+      </c>
+    </row>
+    <row r="1152">
+      <c r="A1152" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1152" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1152" t="inlineStr">
+        <is>
+          <t>Chelsea Vs Man City: Hajar The Blues 3-0, The Citizens Terus Pepet Arsenal</t>
+        </is>
+      </c>
+      <c r="D1152" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8441303/chelsea-vs-man-city-hajar-the-blues-3-0-the-citizens-terus-pepet-arsenal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1153">
+      <c r="A1153" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1153" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1153" t="inlineStr">
+        <is>
+          <t>Video: Miris! Wanita di Poman Ditandu 9 Km ke Puskesmas gegara Jalan Rusak</t>
+        </is>
+      </c>
+      <c r="D1153" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260412-260412032/video-miris-wanita-di-poman-ditandu-9-km-ke-puskesmas-gegara-jalan-rusak</t>
+        </is>
+      </c>
+    </row>
+    <row r="1154">
+      <c r="A1154" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1154" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1154" t="inlineStr">
+        <is>
+          <t>Video: Penampakan Hajatan Meriah di Tengah Banjir Dayeuhkolot Bandung</t>
+        </is>
+      </c>
+      <c r="D1154" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260412-260412025/video-penampakan-hajatan-meriah-di-tengah-banjir-dayeuhkolot-bandung</t>
+        </is>
+      </c>
+    </row>
+    <row r="1155">
+      <c r="A1155" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1155" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1155" t="inlineStr">
+        <is>
+          <t>Video: Iran Mau Gencatan Senjata Setop Perang Semua Sisi, Termasuk Lebanon</t>
+        </is>
+      </c>
+      <c r="D1155" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260412-260412001/video-iran-mau-gencatan-senjata-setop-perang-semua-sisi-termasuk-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="1156">
+      <c r="A1156" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1156" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1156" t="inlineStr">
+        <is>
+          <t>Arsenal Masuki Masa Mengkhawatirkan</t>
+        </is>
+      </c>
+      <c r="D1156" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8441320/arsenal-masuki-masa-mengkhawatirkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1157">
+      <c r="A1157" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1157" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1157" t="inlineStr">
+        <is>
+          <t>PSI: Kami Berkomitmen Dukung Prabowo-Gibran Sampai Selesai 2029</t>
+        </is>
+      </c>
+      <c r="D1157" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1923077/psi-kami-berkomitmen-dukung-prabowo-gibran-sampai-selesai-2029?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1158">
+      <c r="A1158" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1158" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1158" t="inlineStr">
+        <is>
+          <t>Trump Perintahkan Blokade Selat Hormuz</t>
+        </is>
+      </c>
+      <c r="D1158" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/trump-perintahkan-blokade-selat-hormuz?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1159">
+      <c r="A1159" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1159" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1159" t="inlineStr">
+        <is>
+          <t>Satgas PRR Pastikan Pemutakhiran Data Penerima Huntara dan DTH Terus Dilakukan</t>
+        </is>
+      </c>
+      <c r="D1159" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/11/21303101/satgas-prr-pastikan-pemutakhiran-data-penerima-huntara-dan-dth-terus</t>
+        </is>
+      </c>
+    </row>
+    <row r="1160">
+      <c r="A1160" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1160" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1160" t="inlineStr">
+        <is>
+          <t>Freeport-Serikat Pekerja Teken PKB Baru, Fokus pada Kesejahteraan dan Keselamatan</t>
+        </is>
+      </c>
+      <c r="D1160" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/11/15343861/freeport-serikat-pekerja-teken-pkb-baru-fokus-pada-kesejahteraan-dan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1161">
+      <c r="A1161" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1161" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1161" t="inlineStr">
+        <is>
+          <t>NodesGroup Luncurkan Sistem Lacak Servis dan Layanan Pickup-Delivery</t>
+        </is>
+      </c>
+      <c r="D1161" s="2" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/04/11/115440526/nodesgroup-luncurkan-sistem-lacak-servis-dan-layanan-pickup-delivery</t>
+        </is>
+      </c>
+    </row>
+    <row r="1162">
+      <c r="A1162" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1162" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1162" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D1162" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1163">
+      <c r="A1163" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1163" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1163" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D1163" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1164">
+      <c r="A1164" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1164" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1164" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D1164" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1165">
+      <c r="A1165" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1165" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1165" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D1165" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1166">
+      <c r="A1166" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1166" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1166" t="inlineStr">
+        <is>
+          <t>Perundingan Iran dan AS Gagal, Tiga Isu Disorot jadi Penyebab, Apa Saja?</t>
+        </is>
+      </c>
+      <c r="D1166" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1923053/perundingan-iran-dan-as-gagal-tiga-isu-disorot-jadi-penyebab-apa-saja?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1167">
+      <c r="A1167" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1167" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1167" t="inlineStr">
+        <is>
+          <t>Telur Rebus</t>
+        </is>
+      </c>
+      <c r="D1167" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/syahrulchelsky/69db231bc925c4705970a332/telur-rebus</t>
+        </is>
+      </c>
+    </row>
+    <row r="1168">
+      <c r="A1168" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1168" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1168" t="inlineStr">
+        <is>
+          <t>Cara Perpanjang Visa Kegiatan Keagamaan di Jepang: Waktu, Proses, dan Hal Penting</t>
+        </is>
+      </c>
+      <c r="D1168" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5806/cara-perpanjang-visa-kegiatan-keagamaan-di-jepang-waktu-proses-dan-hal-penting</t>
+        </is>
+      </c>
+    </row>
+    <row r="1169">
+      <c r="A1169" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1169" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1169" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1169" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1170">
+      <c r="A1170" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1170" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1170" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1170" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1171">
+      <c r="A1171" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1171" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1171" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Penampakan Langka Bumi dan Bulan yang Dipotret Kru Artemis II NASA</t>
+        </is>
+      </c>
+      <c r="D1171" s="2" t="inlineStr">
+        <is>
+          <t>https://tekno.kompas.com/read/2026/04/09/18020027/berita-foto-penampakan-langka-bumi-dan-bulan-yang-dipotret-kru-artemis-ii-nasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1172">
+      <c r="A1172" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1172" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1172" t="inlineStr">
+        <is>
+          <t>Rincian 31 Paket Jasa EO yang Disewa BGN Rp 113 Miliar</t>
+        </is>
+      </c>
+      <c r="D1172" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097789/rincian-31-paket-jasa-eo-yang-disewa-bgn-rp-113-miliar</t>
+        </is>
+      </c>
+    </row>
+    <row r="1173">
+      <c r="A1173" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1173" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1173" t="inlineStr">
+        <is>
+          <t>BGN Hamburkan Rp 113 Miliar untuk Sewa Jasa Event Organizer</t>
+        </is>
+      </c>
+      <c r="D1173" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097781/bgn-hamburkan-rp-113-miliar-untuk-sewa-jasa-event-organizer</t>
+        </is>
+      </c>
+    </row>
+    <row r="1174">
+      <c r="A1174" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1174" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1174" t="inlineStr">
+        <is>
+          <t>Prabowo akan Bertemu Putin di Rusia</t>
+        </is>
+      </c>
+      <c r="D1174" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097779/prabowo-akan-bertemu-putin-di-rusia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1175">
+      <c r="A1175" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1175" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1175" t="inlineStr">
+        <is>
+          <t>Muslimat NU Mau Surati PBB Sikapi Dampak Perang di Timteng</t>
+        </is>
+      </c>
+      <c r="D1175" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097778/muslimat-nu-mau-surati-pbb-sikapi-dampak-perang-di-timteng</t>
+        </is>
+      </c>
+    </row>
+    <row r="1176">
+      <c r="A1176" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1176" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1176" t="inlineStr">
+        <is>
+          <t>Kondisi Andrie Yunus setelah 30 Hari Perawatan di RSCM</t>
+        </is>
+      </c>
+      <c r="D1176" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097771/kondisi-andrie-yunus-setelah-30-hari-perawatan-di-rscm</t>
+        </is>
+      </c>
+    </row>
+    <row r="1177">
+      <c r="A1177" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1177" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1177" t="inlineStr">
+        <is>
+          <t>Pemprov DKI Bakal Pasang Fitur Deteksi Foto AI di Jaki</t>
+        </is>
+      </c>
+      <c r="D1177" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097770/pemprov-dki-bakal-pasang-fitur-deteksi-foto-ai-di-jaki</t>
+        </is>
+      </c>
+    </row>
+    <row r="1178">
+      <c r="A1178" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1178" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1178" t="inlineStr">
+        <is>
+          <t>Respons Khofifah Soal 3 Kepala Daerah di Jatim Ditangkap KPK</t>
+        </is>
+      </c>
+      <c r="D1178" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097765/respons-khofifah-soal-3-kepala-daerah-di-jatim-ditangkap-kpk</t>
+        </is>
+      </c>
+    </row>
+    <row r="1179">
+      <c r="A1179" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1179" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1179" t="inlineStr">
+        <is>
+          <t>Sepeda Mewah yang Dipakai Ahmad Luthfi Tak Tercatat di LHKPN</t>
+        </is>
+      </c>
+      <c r="D1179" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097762/sepeda-mewah-yang-dipakai-ahmad-luthfi-tak-tercatat-di-lhkpn</t>
+        </is>
+      </c>
+    </row>
+    <row r="1180">
+      <c r="A1180" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1180" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1180" t="inlineStr">
+        <is>
+          <t>Pencurian Kendaraan dan Rumah Masih Dominan, Polisi Didorong Perkuat Pencegahan</t>
+        </is>
+      </c>
+      <c r="D1180" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097752/pencurian-kendaraan-dan-rumah-masih-dominan-polisi-didorong-perkuat-pencegahan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1181">
+      <c r="A1181" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1181" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1181" t="inlineStr">
+        <is>
+          <t>Keamanan Meningkat, Penilaian Kinerja Polri Naik dalam Tiga Bulan</t>
+        </is>
+      </c>
+      <c r="D1181" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097751/keamanan-meningkat-penilaian-kinerja-polri-naik-dalam-tiga-bulan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1182">
+      <c r="A1182" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1182" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1182" t="inlineStr">
+        <is>
+          <t>Peringati 30 Hari Kasus Andrie, Koalisi Desak Bentuk TGPF</t>
+        </is>
+      </c>
+      <c r="D1182" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097750/peringati-30-hari-kasus-andrie-koalisi-desak-bentuk-tgpf</t>
+        </is>
+      </c>
+    </row>
+    <row r="1183">
+      <c r="A1183" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1183" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1183" t="inlineStr">
+        <is>
+          <t>Koalisi Sipil Buat Mural Andrie Yunus di TKP Penyerangan</t>
+        </is>
+      </c>
+      <c r="D1183" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097748/koalisi-sipil-buat-mural-andrie-yunus-di-tkp-penyerangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1184">
+      <c r="A1184" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1184" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1184" t="inlineStr">
+        <is>
+          <t>Sugiono Gantikan Prabowo Jadi Ketua Umum Ikatan Pencak Silat</t>
+        </is>
+      </c>
+      <c r="D1184" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097743/sugiono-gantikan-prabowo-jadi-ketua-umum-ikatan-pencak-silat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1185">
+      <c r="A1185" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1185" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1185" t="inlineStr">
+        <is>
+          <t>Koalisi Sipil Gelar Peringatan 30 Hari Kasus Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D1185" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097740/koalisi-sipil-gelar-peringatan-30-hari-kasus-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="1186">
+      <c r="A1186" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1186" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1186" t="inlineStr">
+        <is>
+          <t>Badan Gizi Nasional Kembali Setop Sementara Ratusan SPPG</t>
+        </is>
+      </c>
+      <c r="D1186" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097725/badan-gizi-nasional-kembali-setop-sementara-ratusan-sppg</t>
+        </is>
+      </c>
+    </row>
+    <row r="1187">
+      <c r="A1187" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1187" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1187" t="inlineStr">
+        <is>
+          <t>Indonesia's BMKG says sky object likely rocket debris, not missile</t>
+        </is>
+      </c>
+      <c r="D1187" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412009/indonesias-bmkg-says-sky-object-likely-rocket-debris-not-missile</t>
+        </is>
+      </c>
+    </row>
+    <row r="1188">
+      <c r="A1188" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1188" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1188" t="inlineStr">
+        <is>
+          <t>Indonesian lawmaker urges better support for border immigration staff</t>
+        </is>
+      </c>
+      <c r="D1188" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412008/indonesian-lawmaker-urges-better-support-for-border-immigration-staff</t>
+        </is>
+      </c>
+    </row>
+    <row r="1189">
+      <c r="A1189" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1189" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1189" t="inlineStr">
+        <is>
+          <t>Minister pushes timely completion of Sekolah Rakyat phase 2</t>
+        </is>
+      </c>
+      <c r="D1189" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412004/minister-pushes-timely-completion-of-sekolah-rakyat-phase-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1190">
+      <c r="A1190" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1190" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1190" t="inlineStr">
+        <is>
+          <t>Indonesian women urged to support national development through family</t>
+        </is>
+      </c>
+      <c r="D1190" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412003/indonesian-women-urged-to-support-national-development-through-family</t>
+        </is>
+      </c>
+    </row>
+    <row r="1191">
+      <c r="A1191" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1191" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1191" t="inlineStr">
+        <is>
+          <t>KAI adopts B40 biodiesel, prepares for B50 transition</t>
+        </is>
+      </c>
+      <c r="D1191" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412000/kai-adopts-b40-biodiesel-prepares-for-b50-transition</t>
+        </is>
+      </c>
+    </row>
+    <row r="1192">
+      <c r="A1192" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1192" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1192" t="inlineStr">
+        <is>
+          <t>Jakarta backs invasive catfish crackdown for ecosystem safety</t>
+        </is>
+      </c>
+      <c r="D1192" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411996/jakarta-backs-invasive-catfish-crackdown-for-ecosystem-safety</t>
+        </is>
+      </c>
+    </row>
+    <row r="1193">
+      <c r="A1193" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1193" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1193" t="inlineStr">
+        <is>
+          <t>Indonesia food security holds firm amid global pressure</t>
+        </is>
+      </c>
+      <c r="D1193" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411995/indonesia-food-security-holds-firm-amid-global-pressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="1194">
+      <c r="A1194" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1194" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1194" t="inlineStr">
+        <is>
+          <t>Indonesia, Australia strengthen ties to combat online radicalization</t>
+        </is>
+      </c>
+      <c r="D1194" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411993/indonesia-australia-strengthen-ties-to-combat-online-radicalization</t>
+        </is>
+      </c>
+    </row>
+    <row r="1195">
+      <c r="A1195" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1195" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1195" t="inlineStr">
+        <is>
+          <t>Prabowo vows lifelong support for pencak silat development</t>
+        </is>
+      </c>
+      <c r="D1195" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411989/prabowo-vows-lifelong-support-for-pencak-silat-development</t>
+        </is>
+      </c>
+    </row>
+    <row r="1196">
+      <c r="A1196" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1196" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1196" t="inlineStr">
+        <is>
+          <t>Prabowo to meet Putin in Moscow over geopolitics, energy concerns</t>
+        </is>
+      </c>
+      <c r="D1196" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411988/prabowo-to-meet-putin-in-moscow-over-geopolitics-energy-concerns</t>
+        </is>
+      </c>
+    </row>
+    <row r="1197">
+      <c r="A1197" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1197" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1197" t="inlineStr">
+        <is>
+          <t>Ministry deploys 400 pumps, pledges more to shield crops from El Nino</t>
+        </is>
+      </c>
+      <c r="D1197" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411984/ministry-deploys-400-pumps-pledges-more-to-shield-crops-from-el-nino</t>
+        </is>
+      </c>
+    </row>
+    <row r="1198">
+      <c r="A1198" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1198" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1198" t="inlineStr">
+        <is>
+          <t>Minister urges regions to reactivate fire volunteers</t>
+        </is>
+      </c>
+      <c r="D1198" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411981/minister-urges-regions-to-reactivate-fire-volunteers</t>
+        </is>
+      </c>
+    </row>
+    <row r="1199">
+      <c r="A1199" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1199" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1199" t="inlineStr">
+        <is>
+          <t>OIKN taps local residents to rid new capital of malaria and dengue</t>
+        </is>
+      </c>
+      <c r="D1199" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411979/oikn-taps-local-residents-to-rid-new-capital-of-malaria-and-dengue</t>
+        </is>
+      </c>
+    </row>
+    <row r="1200">
+      <c r="A1200" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1200" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1200" t="inlineStr">
+        <is>
+          <t>Prabowo concludes multi-decade tenure as PB IPSI chairperson</t>
+        </is>
+      </c>
+      <c r="D1200" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411976/prabowo-concludes-multi-decade-tenure-as-pb-ipsi-chairperson</t>
+        </is>
+      </c>
+    </row>
+    <row r="1201">
+      <c r="A1201" t="inlineStr">
+        <is>
+          <t>Monday, 13 April 2026</t>
+        </is>
+      </c>
+      <c r="B1201" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1201" t="inlineStr">
+        <is>
+          <t>Indonesia considers EV incentives with industry, regulators</t>
+        </is>
+      </c>
+      <c r="D1201" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/411973/indonesia-considers-ev-incentives-with-industry-regulators</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1141"/>
+  <autoFilter ref="A1:D1201"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -26693,6 +28013,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1139" r:id="rId1138"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1140" r:id="rId1139"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1141" r:id="rId1140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1142" r:id="rId1141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1143" r:id="rId1142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1144" r:id="rId1143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1145" r:id="rId1144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1146" r:id="rId1145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1147" r:id="rId1146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1148" r:id="rId1147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1149" r:id="rId1148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1150" r:id="rId1149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1151" r:id="rId1150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1152" r:id="rId1151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1153" r:id="rId1152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1154" r:id="rId1153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1155" r:id="rId1154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1156" r:id="rId1155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1157" r:id="rId1156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1158" r:id="rId1157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1159" r:id="rId1158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1160" r:id="rId1159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1161" r:id="rId1160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1162" r:id="rId1161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1163" r:id="rId1162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1164" r:id="rId1163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1165" r:id="rId1164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1166" r:id="rId1165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1167" r:id="rId1166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1168" r:id="rId1167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1169" r:id="rId1168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1170" r:id="rId1169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1171" r:id="rId1170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1172" r:id="rId1171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1173" r:id="rId1172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1174" r:id="rId1173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1175" r:id="rId1174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1176" r:id="rId1175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1177" r:id="rId1176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1178" r:id="rId1177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1179" r:id="rId1178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1180" r:id="rId1179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1181" r:id="rId1180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1182" r:id="rId1181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1183" r:id="rId1182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1184" r:id="rId1183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1185" r:id="rId1184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1186" r:id="rId1185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1187" r:id="rId1186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1188" r:id="rId1187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1189" r:id="rId1188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1190" r:id="rId1189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1191" r:id="rId1190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1192" r:id="rId1191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1193" r:id="rId1192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1194" r:id="rId1193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1195" r:id="rId1194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1196" r:id="rId1195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1197" r:id="rId1196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1198" r:id="rId1197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1199" r:id="rId1198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1200" r:id="rId1199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1201" r:id="rId1200"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-13
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1201</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1261</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1201"/>
+  <dimension ref="A1:D1261"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -26870,8 +26870,1328 @@
         </is>
       </c>
     </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1202" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>Video: Prabowo Temui Putin, Bahas Kerja Sama Ekonomi hingga Energi</t>
+        </is>
+      </c>
+      <c r="D1202" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8442798/video-prabowo-temui-putin-bahas-kerja-sama-ekonomi-hingga-energi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1203" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>Video: Waspada Hipotermia! IDAI Jelaskan Risiko Bawa Anak Naik Gunung</t>
+        </is>
+      </c>
+      <c r="D1203" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/detiktv/d-8442815/video-waspada-hipotermia-idai-jelaskan-risiko-bawa-anak-naik-gunung</t>
+        </is>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1204" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>Veri AFI Blak-blakan Alami Ketakutan dan 'Diserang' Sederet Penyakit</t>
+        </is>
+      </c>
+      <c r="D1204" s="2" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8441761/veri-afi-blak-blakan-alami-ketakutan-dan-diserang-sederet-penyakit</t>
+        </is>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1205" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>Prabowo Terima Kasih ke Putin Bantu RI Masuk BRICS</t>
+        </is>
+      </c>
+      <c r="D1205" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8442621/prabowo-terima-kasih-ke-putin-bantu-ri-masuk-brics</t>
+        </is>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1206" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>Warga Sipil di Pusaran Operasi Percobaan Pembunuhan Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D1206" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/spotlight/d-8442581/warga-sipil-di-pusaran-operasi-percobaan-pembunuhan-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1207" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>Polisi Ungkap Penyebab Kematian Eks Dosen UIN Malang Yai Mim</t>
+        </is>
+      </c>
+      <c r="D1207" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8442945/polisi-ungkap-penyebab-kematian-eks-dosen-uin-malang-yai-mim</t>
+        </is>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1208" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>Eks Dosen UIN Malang Yai Mim Tersangka Pornografi Meninggal Dunia</t>
+        </is>
+      </c>
+      <c r="D1208" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8442769/eks-dosen-uin-malang-yai-mim-tersangka-pornografi-meninggal-dunia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1209" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>Polresta Malang Kota Luncurkan Microsite Mudik, Warga Bisa Cek Lalin-Akses CCTV</t>
+        </is>
+      </c>
+      <c r="D1209" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8408252/polresta-malang-kota-luncurkan-microsite-mudik-warga-bisa-cek-lalin-akses-cctv</t>
+        </is>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1210" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>MU Vs Leeds: Setan Merah Kalah 1-2 di Old Trafford</t>
+        </is>
+      </c>
+      <c r="D1210" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8442935/mu-vs-leeds-setan-merah-kalah-1-2-di-old-trafford</t>
+        </is>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1211" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>Perbasi Sambut Terobosan Ditjen Imigrasi Mudahkan Administrasi Atlet Asing</t>
+        </is>
+      </c>
+      <c r="D1211" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/basket/d-8442938/perbasi-sambut-terobosan-ditjen-imigrasi-mudahkan-administrasi-atlet-asing</t>
+        </is>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1212" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>Aksi Preman Palak Sopir Bajaj di Tanah Abang Berakhir di Balik Jeruji</t>
+        </is>
+      </c>
+      <c r="D1212" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8442837/aksi-preman-palak-sopir-bajaj-di-tanah-abang-berakhir-di-balik-jeruji</t>
+        </is>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1213" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>Video: Di Hadapan Putin, Prabowo Ngaku Mau Konsultasi Geopolitik</t>
+        </is>
+      </c>
+      <c r="D1213" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260414-260414003/video-di-hadapan-putin-prabowo-ngaku-mau-konsultasi-geopolitik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1214" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>Video: Bertemu Prabowo, Putin Ungkap Adanya Perlambatan Perdagangan RI-Rusia</t>
+        </is>
+      </c>
+      <c r="D1214" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260414-260414001/video-bertemu-prabowo-putin-ungkap-adanya-perlambatan-perdagangan-ri-rusia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1215" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>Video: Kuota 1000 Wisatawan Perhari Ditolak Pelaku Wisata di Labuan Bajo</t>
+        </is>
+      </c>
+      <c r="D1215" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260413-260413104/video-kuota-1000-wisatawan-perhari-ditolak-pelaku-wisata-di-labuan-bajo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1216" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>3 Bahan Alami 'Pembersih Ginjal', Bantu Hempaskan Racun di Tubuh</t>
+        </is>
+      </c>
+      <c r="D1216" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8442452/3-bahan-alami-pembersih-ginjal-bantu-hempaskan-racun-di-tubuh</t>
+        </is>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1217" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>Fenomena Joki Antran, Bisnis Baru di Balik Makanan Viral</t>
+        </is>
+      </c>
+      <c r="D1217" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1923344/fenomena-joki-antran-bisnis-baru-di-balik-makanan-viral?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1218" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>Apa Saja Poin Kesepakatan Gencatan Senjata Iran dengan Amerika Serikat?</t>
+        </is>
+      </c>
+      <c r="D1218" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/apa-saja-poin-kesepakatan-gencatan-senjata-iran-dengan-amerika-serikat?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1219" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>Mendagri Tegaskan Pemerintah Siap Perkuat Pengawasan dan Optimalisasi Dana Otsus</t>
+        </is>
+      </c>
+      <c r="D1219" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/13/21130441/mendagri-tegaskan-pemerintah-siap-perkuat-pengawasan-dan-optimalisasi-dana</t>
+        </is>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1220" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>Mendagri: Dana Otsus dan Dana Keistimewaan Harus Dirasakan oleh Masyarakat</t>
+        </is>
+      </c>
+      <c r="D1220" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/13/21031381/mendagri-dana-otsus-dan-dana-keistimewaan-harus-dirasakan-oleh-masyarakat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1221" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>Dukung Pelaksanaan Sensus Ekonomi 2026, Walkot Batam Tekankan Pentingnya Keakuratan Data</t>
+        </is>
+      </c>
+      <c r="D1221" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/13/115104978/dukung-pelaksanaan-sensus-ekonomi-2026-walkot-batam-tekankan-pentingnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1222" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D1222" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1223" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D1223" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1224" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D1224" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1225" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D1225" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1226" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>Dapat Ucapan Paskah Ortodoks, Putin Sanjung Prabowo di Istana Kremlin</t>
+        </is>
+      </c>
+      <c r="D1226" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1923314/dapat-ucapan-paskah-ortodoks-putin-sanjung-prabowo-di-istana-kremlin?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1227" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>Musim Pancaroba</t>
+        </is>
+      </c>
+      <c r="D1227" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/jora5074/69c85a8534777c40421d65a2/musim-pancaroba</t>
+        </is>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1228" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>Mengenal Yakult Ladies, Layanan Antar Minuman Sekaligus Lawan Kesepian di Jepang</t>
+        </is>
+      </c>
+      <c r="D1228" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5773/mengenal-yakult-ladies-layanan-antar-minuman-sekaligus-lawan-kesepian-di-jepang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1229" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1229" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1230" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1230" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1231" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Penampakan Langka Bumi dan Bulan yang Dipotret Kru Artemis II NASA</t>
+        </is>
+      </c>
+      <c r="D1231" s="2" t="inlineStr">
+        <is>
+          <t>https://tekno.kompas.com/read/2026/04/09/18020027/berita-foto-penampakan-langka-bumi-dan-bulan-yang-dipotret-kru-artemis-ii-nasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1232" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>BEM UI Kecam Kasus Dugaan Pelecehan Seksual Mahasiswa FH</t>
+        </is>
+      </c>
+      <c r="D1232" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098010/bem-ui-kecam-kasus-dugaan-pelecehan-seksual-mahasiswa-fh</t>
+        </is>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1233" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>BNPP Dorong Hunian Layak, Tingkatkan Kualitas Hidup Masyarakat</t>
+        </is>
+      </c>
+      <c r="D1233" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097999/bnpp-dorong-hunian-layak-tingkatkan-kualitas-hidup-masyarakat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1234" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>Dua Legislator Dorong TGPF Usut Kasus Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D1234" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097997/dua-legislator-dorong-tgpf-usut-kasus-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1235" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>Mendagri Ingatkan Daerah Patuhi WFH: Bukti Loyal ke Pusat</t>
+        </is>
+      </c>
+      <c r="D1235" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097991/mendagri-ingatkan-daerah-patuhi-wfh-bukti-loyal-ke-pusat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1236" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>WFH Tiap Rabu dengan Pengawasan Berlapis di Yogya</t>
+        </is>
+      </c>
+      <c r="D1236" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097990/wfh-tiap-rabu-dengan-pengawasan-berlapis-di-yogya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1237" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>DPR dan Pemerintah Sepakati Revisi UU PSDK ke Paripurna</t>
+        </is>
+      </c>
+      <c r="D1237" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097984/dpr-dan-pemerintah-sepakati-revisi-uu-psdk-ke-paripurna</t>
+        </is>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1238" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>Akademisi Desak Reposisi Proyek MBG agar Tepat Sasaran</t>
+        </is>
+      </c>
+      <c r="D1238" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097983/akademisi-desak-reposisi-proyek-mbg-agar-tepat-sasaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1239" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>Survei LSI: Publik Ingin Terlibat dalam Amandemen UUD</t>
+        </is>
+      </c>
+      <c r="D1239" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097979/survei-lsi-publik-ingin-terlibat-dalam-amandemen-uud</t>
+        </is>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1240" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>Dewi Priyanti, Kartini PNM yang Membawa Perubahan Nyata bagi Lingkungan</t>
+        </is>
+      </c>
+      <c r="D1240" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097969/dewi-priyanti-kartini-pnm-yang-membawa-perubahan-nyata-bagi-lingkungan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1241" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>Kemensos Siapkan Lulusan SekolahRakyat untuk Peluang Kerja di Jepang</t>
+        </is>
+      </c>
+      <c r="D1241" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097968/kemensos-siapkan-lulusan-sekolahrakyat-untuk-peluang-kerja-di-jepang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1242" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>Gus Ipul: Penerimaan Murid Baru Sekolah Rakyat Berdasarkan DTSEN</t>
+        </is>
+      </c>
+      <c r="D1242" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097965/gus-ipul-penerimaan-murid-baru-sekolah-rakyat-berdasarkan-dtsen</t>
+        </is>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1243" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>Banjir Susulan Putus Jalan dan Jembatan di Sumatra, Tito: Kita Harus Kerja Keras Lagi</t>
+        </is>
+      </c>
+      <c r="D1243" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097963/banjir-susulan-putus-jalan-dan-jembatan-di-sumatra-tito-kita-harus-kerja-keras-lagi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1244" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>Musrenbang 2026, Momentum PerkuatEkonomi dan Pembangunan Lampung</t>
+        </is>
+      </c>
+      <c r="D1244" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097962/musrenbang-2026-momentum-perkuatekonomi-dan-pembangunan-lampung</t>
+        </is>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1245" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>Banjir Bandang Kembali Mengancam Sumatra, BMKG Prediksi Hujan Lebat Dua Putaran di Aceh</t>
+        </is>
+      </c>
+      <c r="D1245" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097961/banjir-bandang-kembali-mengancam-sumatra-bmkg-prediksi-hujan-lebat-dua-putaran-di-aceh</t>
+        </is>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1246" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>Pemko Padang Minta Dukungan Kemenlu Angkat Isu Revitalisasi Batang Arau</t>
+        </is>
+      </c>
+      <c r="D1246" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2097954/pemko-padang-minta-dukungan-kemenlu-angkat-isu-revitalisasi-batang-arau</t>
+        </is>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1247" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>Govt to empower 18 million aid beneficiaries through village co-ops</t>
+        </is>
+      </c>
+      <c r="D1247" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412127/govt-to-empower-18-million-aid-beneficiaries-through-village-co-ops</t>
+        </is>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1248" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>Indonesia free from forced labor practices: minister</t>
+        </is>
+      </c>
+      <c r="D1248" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412125/indonesia-free-from-forced-labor-practices-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1249" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>Prabowo sends Easter, Cosmonautics Day greetings in Moscow talks</t>
+        </is>
+      </c>
+      <c r="D1249" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412123/prabowo-sends-easter-cosmonautics-day-greetings-in-moscow-talks</t>
+        </is>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1250" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>Prabowo consults Putin on global geopolitical uncertainty</t>
+        </is>
+      </c>
+      <c r="D1250" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412121/prabowo-consults-putin-on-global-geopolitical-uncertainty</t>
+        </is>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1251" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>Prabowo to oversee Indonesia-Russia monetary ties</t>
+        </is>
+      </c>
+      <c r="D1251" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412120/prabowo-to-oversee-indonesia-russia-monetary-ties</t>
+        </is>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1252" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>Govt eyes village co-ops to create 1.4 M jobs for aid beneficiaries</t>
+        </is>
+      </c>
+      <c r="D1252" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412119/govt-eyes-village-co-ops-to-create-14-m-jobs-for-aid-beneficiaries</t>
+        </is>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1253" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>Indonesia completes 4,741 village cooperatives, awaits rollout</t>
+        </is>
+      </c>
+      <c r="D1253" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412116/indonesia-completes-4741-village-cooperatives-awaits-rollout</t>
+        </is>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1254" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>Prabowo-Putin agree to increase economic, energy cooperation</t>
+        </is>
+      </c>
+      <c r="D1254" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412112/prabowo-putin-agree-to-increase-economic-energy-cooperation</t>
+        </is>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1255" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>Foreign investors remain committed to investing in Indonesia: minister</t>
+        </is>
+      </c>
+      <c r="D1255" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412111/foreign-investors-remain-committed-to-investing-in-indonesia-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="1256">
+      <c r="A1256" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1256" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1256" t="inlineStr">
+        <is>
+          <t>Lawmaker says Prabowo's visit to Rusia play role promoting peace</t>
+        </is>
+      </c>
+      <c r="D1256" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412108/lawmaker-says-prabowos-visit-to-rusia-play-role-promoting-peace</t>
+        </is>
+      </c>
+    </row>
+    <row r="1257">
+      <c r="A1257" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1257" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1257" t="inlineStr">
+        <is>
+          <t>Minister urges regions to end open dumping to curb landfill fires</t>
+        </is>
+      </c>
+      <c r="D1257" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412104/minister-urges-regions-to-end-open-dumping-to-curb-landfill-fires</t>
+        </is>
+      </c>
+    </row>
+    <row r="1258">
+      <c r="A1258" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1258" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1258" t="inlineStr">
+        <is>
+          <t>Indonesia maintains healthy debt ratio amidst global pressure</t>
+        </is>
+      </c>
+      <c r="D1258" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412100/indonesia-maintains-healthy-debt-ratio-amidst-global-pressure</t>
+        </is>
+      </c>
+    </row>
+    <row r="1259">
+      <c r="A1259" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1259" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1259" t="inlineStr">
+        <is>
+          <t>Megawati receives Qatari ambassador, exchanges cultural gifts</t>
+        </is>
+      </c>
+      <c r="D1259" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412096/megawati-receives-qatari-ambassador-exchanges-cultural-gifts</t>
+        </is>
+      </c>
+    </row>
+    <row r="1260">
+      <c r="A1260" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1260" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1260" t="inlineStr">
+        <is>
+          <t>Indonesia optimistic about achieving Rp497 T investment in Q1 2026</t>
+        </is>
+      </c>
+      <c r="D1260" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412092/indonesia-optimistic-about-achieving-rp497-t-investment-in-q1-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1261">
+      <c r="A1261" t="inlineStr">
+        <is>
+          <t>Tuesday, 14 April 2026</t>
+        </is>
+      </c>
+      <c r="B1261" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1261" t="inlineStr">
+        <is>
+          <t>Blaize and Nokia Advance Collaboration with Joint AI Solution Showcase at GITEX Asia</t>
+        </is>
+      </c>
+      <c r="D1261" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412089/blaize-and-nokia-advance-collaboration-with-joint-ai-solution-showcase-at-gitex-asia</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1201"/>
+  <autoFilter ref="A1:D1261"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -28073,6 +29393,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1199" r:id="rId1198"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1200" r:id="rId1199"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1201" r:id="rId1200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1202" r:id="rId1201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1203" r:id="rId1202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1204" r:id="rId1203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1205" r:id="rId1204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1206" r:id="rId1205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1207" r:id="rId1206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1208" r:id="rId1207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1209" r:id="rId1208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1210" r:id="rId1209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1211" r:id="rId1210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1212" r:id="rId1211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1213" r:id="rId1212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1214" r:id="rId1213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1215" r:id="rId1214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1216" r:id="rId1215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1217" r:id="rId1216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1218" r:id="rId1217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1219" r:id="rId1218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1220" r:id="rId1219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1221" r:id="rId1220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1222" r:id="rId1221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1223" r:id="rId1222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1224" r:id="rId1223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1225" r:id="rId1224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1226" r:id="rId1225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1227" r:id="rId1226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1228" r:id="rId1227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1229" r:id="rId1228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1230" r:id="rId1229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1231" r:id="rId1230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1232" r:id="rId1231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1233" r:id="rId1232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1234" r:id="rId1233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1235" r:id="rId1234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1236" r:id="rId1235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1237" r:id="rId1236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1238" r:id="rId1237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1239" r:id="rId1238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1240" r:id="rId1239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1241" r:id="rId1240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1242" r:id="rId1241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1243" r:id="rId1242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1244" r:id="rId1243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1245" r:id="rId1244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1246" r:id="rId1245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1247" r:id="rId1246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1248" r:id="rId1247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1249" r:id="rId1248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1250" r:id="rId1249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1251" r:id="rId1250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1252" r:id="rId1251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1253" r:id="rId1252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1254" r:id="rId1253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1255" r:id="rId1254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1256" r:id="rId1255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1257" r:id="rId1256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1258" r:id="rId1257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1259" r:id="rId1258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1260" r:id="rId1259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1261" r:id="rId1260"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-14
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1261</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1321</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1261"/>
+  <dimension ref="A1:D1321"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -28190,8 +28190,1328 @@
         </is>
       </c>
     </row>
+    <row r="1262">
+      <c r="A1262" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1262" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1262" t="inlineStr">
+        <is>
+          <t>Video Liverpool Vs PSG: Diam-diam Enrique Pernah Jadi 'Kopites'</t>
+        </is>
+      </c>
+      <c r="D1262" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/detiktv/d-8444539/video-liverpool-vs-psg-diam-diam-enrique-pernah-jadi-kopites</t>
+        </is>
+      </c>
+    </row>
+    <row r="1263">
+      <c r="A1263" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1263" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1263" t="inlineStr">
+        <is>
+          <t>Ini Hasil Evaluasi WFH ASN demi Hemat BBM Pekan Pertama</t>
+        </is>
+      </c>
+      <c r="D1263" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8444476/ini-hasil-evaluasi-wfh-asn-demi-hemat-bbm-pekan-pertama</t>
+        </is>
+      </c>
+    </row>
+    <row r="1264">
+      <c r="A1264" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1264" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1264" t="inlineStr">
+        <is>
+          <t>Video Pihak Korban: Grup Chat Mesum Mahasiswa FH UI Awalnya Grup Kos-kosan</t>
+        </is>
+      </c>
+      <c r="D1264" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8444444/video-pihak-korban-grup-chat-mesum-mahasiswa-fh-ui-awalnya-grup-kos-kosan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1265">
+      <c r="A1265" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1265" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1265" t="inlineStr">
+        <is>
+          <t>Thrash: Hiu di Tengah Badai</t>
+        </is>
+      </c>
+      <c r="D1265" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/pop/movie/d-8443355/thrash-hiu-di-tengah-badai</t>
+        </is>
+      </c>
+    </row>
+    <row r="1266">
+      <c r="A1266" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1266" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1266" t="inlineStr">
+        <is>
+          <t>Video Yamal: Buat Barca, Remontada Bukanlah Keajaiban!</t>
+        </is>
+      </c>
+      <c r="D1266" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/detiktv/d-8444384/video-yamal-buat-barca-remontada-bukanlah-keajaiban</t>
+        </is>
+      </c>
+    </row>
+    <row r="1267">
+      <c r="A1267" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1267" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1267" t="inlineStr">
+        <is>
+          <t>Bina Marga DKI Ganti Tiang Optik yang Roboh di Tamansari Jakbar</t>
+        </is>
+      </c>
+      <c r="D1267" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8444589/bina-marga-dki-ganti-tiang-optik-yang-roboh-di-tamansari-jakbar</t>
+        </is>
+      </c>
+    </row>
+    <row r="1268">
+      <c r="A1268" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1268" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1268" t="inlineStr">
+        <is>
+          <t>Cuaca Ekstrem Landa Bogor, Pohon Tumbang Rusak Rumah hingga Timpa Mobil</t>
+        </is>
+      </c>
+      <c r="D1268" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8444567/cuaca-ekstrem-landa-bogor-pohon-tumbang-rusak-rumah-hingga-timpa-mobil</t>
+        </is>
+      </c>
+    </row>
+    <row r="1269">
+      <c r="A1269" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1269" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1269" t="inlineStr">
+        <is>
+          <t>Terungkap, Total 14 SK Anggota Satpol PP Bogor yang Digadai Atasan</t>
+        </is>
+      </c>
+      <c r="D1269" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8444450/terungkap-total-14-sk-anggota-satpol-pp-bogor-yang-digadai-atasan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1270">
+      <c r="A1270" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1270" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1270" t="inlineStr">
+        <is>
+          <t>Atletico Vs Barca: Kalah 1-2, Griezmann cs Tetap ke Semifinal</t>
+        </is>
+      </c>
+      <c r="D1270" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/uefa/d-8444584/atletico-vs-barca-kalah-1-2-griezmann-cs-tetap-ke-semifinal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1271">
+      <c r="A1271" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1271" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1271" t="inlineStr">
+        <is>
+          <t>Kasus Gagal Ginjal 'Meledak' di Malaysia, Inikah Pemicunya?</t>
+        </is>
+      </c>
+      <c r="D1271" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8444018/kasus-gagal-ginjal-meledak-di-malaysia-inikah-pemicunya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1272">
+      <c r="A1272" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1272" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1272" t="inlineStr">
+        <is>
+          <t>Liverpool Vs PSG: Bungkam Si Merah 2-0, Dembele dkk ke Semifinal</t>
+        </is>
+      </c>
+      <c r="D1272" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/uefa/d-8444583/liverpool-vs-psg-bungkam-si-merah-2-0-dembele-dkk-ke-semifinal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1273">
+      <c r="A1273" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1273" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1273" t="inlineStr">
+        <is>
+          <t>Video China soal AS Blokade Selat Hormuz: Hanya Memperburuk Konfrontasi!</t>
+        </is>
+      </c>
+      <c r="D1273" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260415-260415003/video-china-soal-as-blokade-selat-hormuz-hanya-memperburuk-konfrontasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1274">
+      <c r="A1274" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1274" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1274" t="inlineStr">
+        <is>
+          <t>Video SBY Ingatkan Risiko Krisis Ekonomi Global Imbas Perang di Timur Tengah</t>
+        </is>
+      </c>
+      <c r="D1274" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260415-260415001/video-sby-ingatkan-risiko-krisis-ekonomi-global-imbas-perang-di-timur-tengah</t>
+        </is>
+      </c>
+    </row>
+    <row r="1275">
+      <c r="A1275" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1275" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1275" t="inlineStr">
+        <is>
+          <t>Video: Israel Rudal Mobil Polisi Gaza, 4 Tewas Termasuk Balita</t>
+        </is>
+      </c>
+      <c r="D1275" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260414-260414225/video-israel-rudal-mobil-polisi-gaza-4-tewas-termasuk-balita</t>
+        </is>
+      </c>
+    </row>
+    <row r="1276">
+      <c r="A1276" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1276" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1276" t="inlineStr">
+        <is>
+          <t>Dedikasi Tinggi Lulu Tobing Untuk Yang Lain Boleh Hilang Asal Kau Jangan</t>
+        </is>
+      </c>
+      <c r="D1276" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/pop/trending/d-8444448/dedikasi-tinggi-lulu-tobing-untuk-yang-lain-boleh-hilang-asal-kau-jangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1277">
+      <c r="A1277" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1277" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1277" t="inlineStr">
+        <is>
+          <t>Kapal Iran Masih Bebas! Blokade AS di Selat Hormuz Belum Jelas</t>
+        </is>
+      </c>
+      <c r="D1277" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1923639/kapal-iran-masih-bebas-blokade-as-di-selat-hormuz-belum-jelas?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1278">
+      <c r="A1278" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1278" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1278" t="inlineStr">
+        <is>
+          <t>Trump Menolak Damai dengan Paus Leo XIV</t>
+        </is>
+      </c>
+      <c r="D1278" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/trump-menolak-damai-dengan-paus-leo-xiv?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1279">
+      <c r="A1279" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1279" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1279" t="inlineStr">
+        <is>
+          <t>Lewat Simposium Internasional, Mayapada Healthcare Bawa Standar Global Operasi Lutut ke Indonesia</t>
+        </is>
+      </c>
+      <c r="D1279" s="2" t="inlineStr">
+        <is>
+          <t>https://health.kompas.com/read/26D14225902568/lewat-simposium-internasional-mayapada-healthcare-bawa-standar-global-operasi-lutut</t>
+        </is>
+      </c>
+    </row>
+    <row r="1280">
+      <c r="A1280" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1280" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1280" t="inlineStr">
+        <is>
+          <t>Bank Mandiri Gelar Donor Darah Massal, Targetkan Partisipasi 2.800 Pendonor</t>
+        </is>
+      </c>
+      <c r="D1280" s="2" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/04/14/191947726/bank-mandiri-gelar-donor-darah-massal-targetkan-partisipasi-2800-pendonor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1281">
+      <c r="A1281" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1281" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1281" t="inlineStr">
+        <is>
+          <t>Mendagri Tito Bahas Persiapan Program Perumahan di Wilayah Perbatasan</t>
+        </is>
+      </c>
+      <c r="D1281" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/14/18390111/mendagri-tito-bahas-persiapan-program-perumahan-di-wilayah-perbatasan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1282">
+      <c r="A1282" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1282" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1282" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D1282" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1283">
+      <c r="A1283" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1283" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1283" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D1283" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1284">
+      <c r="A1284" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1284" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1284" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D1284" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1285">
+      <c r="A1285" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1285" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1285" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D1285" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1286">
+      <c r="A1286" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1286" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1286" t="inlineStr">
+        <is>
+          <t>Kapal AS Ganggu Selat Hormuz, Anggota NATO: Iran Punya “Banyak Kartu” Berbahaya</t>
+        </is>
+      </c>
+      <c r="D1286" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1923601/kapal-as-ganggu-selat-hormuz-anggota-nato-iran-punya-banyak-kartu-berbahaya?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1287">
+      <c r="A1287" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1287" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1287" t="inlineStr">
+        <is>
+          <t>Mengenal Perbedaan Pupuk Organik dan Anorganik</t>
+        </is>
+      </c>
+      <c r="D1287" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/greg.nafanu/69db0e2d34777c30c822cf72/mengenal-perbedaan-pupuk-organik-dan-anorganik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1288">
+      <c r="A1288" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1288" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1288" t="inlineStr">
+        <is>
+          <t>Jepang Hentikan Visa Pekerja Restoran, Kuota 50.000 Orang Hampir Penuh</t>
+        </is>
+      </c>
+      <c r="D1288" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5821/jepang-hentikan-visa-pekerja-restoran-kuota-50-000-orang-hampir-penuh</t>
+        </is>
+      </c>
+    </row>
+    <row r="1289">
+      <c r="A1289" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1289" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1289" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1289" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1290">
+      <c r="A1290" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1290" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1290" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1290" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1291">
+      <c r="A1291" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1291" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1291" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Penampakan Langka Bumi dan Bulan yang Dipotret Kru Artemis II NASA</t>
+        </is>
+      </c>
+      <c r="D1291" s="2" t="inlineStr">
+        <is>
+          <t>https://tekno.kompas.com/read/2026/04/09/18020027/berita-foto-penampakan-langka-bumi-dan-bulan-yang-dipotret-kru-artemis-ii-nasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1292">
+      <c r="A1292" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1292" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1292" t="inlineStr">
+        <is>
+          <t>Pemerintah Terapkan Label Nutri-Level pada Minuman Manis</t>
+        </is>
+      </c>
+      <c r="D1292" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098239/pemerintah-terapkan-label-nutri-level-pada-minuman-manis</t>
+        </is>
+      </c>
+    </row>
+    <row r="1293">
+      <c r="A1293" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1293" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1293" t="inlineStr">
+        <is>
+          <t>Korban Dugaan Pelecehan di FH UI: 20 Mahasiswi dan 7 Dosen</t>
+        </is>
+      </c>
+      <c r="D1293" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098233/korban-dugaan-pelecehan-di-fh-ui-20-mahasiswi-dan-7-dosen</t>
+        </is>
+      </c>
+    </row>
+    <row r="1294">
+      <c r="A1294" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1294" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1294" t="inlineStr">
+        <is>
+          <t>5 Tuntutan Aliansi BEM UI soal Dugaan Pelecehan Seksual</t>
+        </is>
+      </c>
+      <c r="D1294" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098214/5-tuntutan-aliansi-bem-ui-soal-dugaan-pelecehan-seksual</t>
+        </is>
+      </c>
+    </row>
+    <row r="1295">
+      <c r="A1295" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1295" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1295" t="inlineStr">
+        <is>
+          <t>DPR Desak UI Beri Sanksi Tegas Pelaku Pelecehan Seksual</t>
+        </is>
+      </c>
+      <c r="D1295" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098208/dpr-desak-ui-beri-sanksi-tegas-pelaku-pelecehan-seksual</t>
+        </is>
+      </c>
+    </row>
+    <row r="1296">
+      <c r="A1296" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1296" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1296" t="inlineStr">
+        <is>
+          <t>Putin Undang Prabowo ke Rusia pada Mei dan Juli</t>
+        </is>
+      </c>
+      <c r="D1296" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098203/putin-undang-prabowo-ke-rusia-pada-mei-dan-juli</t>
+        </is>
+      </c>
+    </row>
+    <row r="1297">
+      <c r="A1297" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1297" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1297" t="inlineStr">
+        <is>
+          <t>UI: 16 Mahasiswa Pelaku Pelecehan Seksual Telah Diperiksa</t>
+        </is>
+      </c>
+      <c r="D1297" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098202/ui-16-mahasiswa-pelaku-pelecehan-seksual-telah-diperiksa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1298">
+      <c r="A1298" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1298" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1298" t="inlineStr">
+        <is>
+          <t>Aboe Bakar Minta Maaf Buntut Ucapan Ulama Terlibat Narkoba</t>
+        </is>
+      </c>
+      <c r="D1298" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098200/aboe-bakar-minta-maaf-buntut-ucapan-ulama-terlibat-narkoba</t>
+        </is>
+      </c>
+    </row>
+    <row r="1299">
+      <c r="A1299" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1299" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1299" t="inlineStr">
+        <is>
+          <t>Menteri Haji soal War Tiket: Kalau Prematur, Kita Tutup</t>
+        </is>
+      </c>
+      <c r="D1299" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098191/menteri-haji-soal-war-tiket-kalau-prematur-kita-tutup</t>
+        </is>
+      </c>
+    </row>
+    <row r="1300">
+      <c r="A1300" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1300" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1300" t="inlineStr">
+        <is>
+          <t>Megawati Didampingi Prananda Terima Kunjungan Dubes Qatar</t>
+        </is>
+      </c>
+      <c r="D1300" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098189/megawati-didampingi-prananda-terima-kunjungan-dubes-qatar</t>
+        </is>
+      </c>
+    </row>
+    <row r="1301">
+      <c r="A1301" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1301" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1301" t="inlineStr">
+        <is>
+          <t>Respons Tempo atas Protes NasDem perihal Sampul Majalah</t>
+        </is>
+      </c>
+      <c r="D1301" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098183/respons-tempo-atas-protes-nasdem-perihal-sampul-majalah</t>
+        </is>
+      </c>
+    </row>
+    <row r="1302">
+      <c r="A1302" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1302" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1302" t="inlineStr">
+        <is>
+          <t>Laput Diprotes NasDem, Tempo: Sudah Lewat Proses Jurnalistik</t>
+        </is>
+      </c>
+      <c r="D1302" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098182/laput-diprotes-nasdem-tempo-sudah-lewat-proses-jurnalistik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1303">
+      <c r="A1303" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1303" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1303" t="inlineStr">
+        <is>
+          <t>Pegadaian Raih Penghargaan Internasional di HongKong</t>
+        </is>
+      </c>
+      <c r="D1303" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098180/pegadaian-raih-penghargaan-internasional-di-hongkong</t>
+        </is>
+      </c>
+    </row>
+    <row r="1304">
+      <c r="A1304" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1304" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1304" t="inlineStr">
+        <is>
+          <t>Pasar Modal Indonesia Salurkan Bantuan Jembatan Cikotak</t>
+        </is>
+      </c>
+      <c r="D1304" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098176/pasar-modal-indonesia-salurkan-bantuan-jembatan-cikotak</t>
+        </is>
+      </c>
+    </row>
+    <row r="1305">
+      <c r="A1305" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1305" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1305" t="inlineStr">
+        <is>
+          <t>MDPC Tak Termasuk Perjanjian Akses Udara Militer AS</t>
+        </is>
+      </c>
+      <c r="D1305" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098174/mdpc-tak-termasuk-perjanjian-akses-udara-militer-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="1306">
+      <c r="A1306" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1306" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1306" t="inlineStr">
+        <is>
+          <t>Maxim Berikan Perlindungan BPJS Ketenagakerjaan Gratis untuk Pengemudi Disabilitas</t>
+        </is>
+      </c>
+      <c r="D1306" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098170/maxim-berikan-perlindungan-bpjs-ketenagakerjaan-gratis-untuk-pengemudi-disabilitas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1307">
+      <c r="A1307" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1307" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1307" t="inlineStr">
+        <is>
+          <t>Indonesia, Saudi Arabia boost creative economy cooperation</t>
+        </is>
+      </c>
+      <c r="D1307" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412283/indonesia-saudi-arabia-boost-creative-economy-cooperation</t>
+        </is>
+      </c>
+    </row>
+    <row r="1308">
+      <c r="A1308" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1308" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1308" t="inlineStr">
+        <is>
+          <t>Indonesia launches nutri-level policy to promote healthy living</t>
+        </is>
+      </c>
+      <c r="D1308" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412280/indonesia-launches-nutri-level-policy-to-promote-healthy-living</t>
+        </is>
+      </c>
+    </row>
+    <row r="1309">
+      <c r="A1309" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1309" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1309" t="inlineStr">
+        <is>
+          <t>Saudi sees cultural heritage as foundation of national identity</t>
+        </is>
+      </c>
+      <c r="D1309" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412277/saudi-sees-cultural-heritage-as-foundation-of-national-identity</t>
+        </is>
+      </c>
+    </row>
+    <row r="1310">
+      <c r="A1310" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1310" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1310" t="inlineStr">
+        <is>
+          <t>Indonesia eyes more sports schools to train young athletes</t>
+        </is>
+      </c>
+      <c r="D1310" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412276/indonesia-eyes-more-sports-schools-to-train-young-athletes</t>
+        </is>
+      </c>
+    </row>
+    <row r="1311">
+      <c r="A1311" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1311" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1311" t="inlineStr">
+        <is>
+          <t>Indonesia heeds global recognition on national economic resilience</t>
+        </is>
+      </c>
+      <c r="D1311" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412272/indonesia-heeds-global-recognition-on-national-economic-resilience</t>
+        </is>
+      </c>
+    </row>
+    <row r="1312">
+      <c r="A1312" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1312" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1312" t="inlineStr">
+        <is>
+          <t>Indonesia fast-tracks blue carbon pricing program</t>
+        </is>
+      </c>
+      <c r="D1312" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412268/indonesia-fast-tracks-blue-carbon-pricing-program</t>
+        </is>
+      </c>
+    </row>
+    <row r="1313">
+      <c r="A1313" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1313" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1313" t="inlineStr">
+        <is>
+          <t>Pertamina says it is capable of processing crude oil from Russia</t>
+        </is>
+      </c>
+      <c r="D1313" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412267/pertamina-says-it-is-capable-of-processing-crude-oil-from-russia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1314">
+      <c r="A1314" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1314" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1314" t="inlineStr">
+        <is>
+          <t>S Korea apologizes over Bali travel advisory controversy: Ministry</t>
+        </is>
+      </c>
+      <c r="D1314" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412264/s-korea-apologizes-over-bali-travel-advisory-controversy-ministry</t>
+        </is>
+      </c>
+    </row>
+    <row r="1315">
+      <c r="A1315" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1315" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1315" t="inlineStr">
+        <is>
+          <t>The salty sashimi of Banda Sea: A journey through inasua history</t>
+        </is>
+      </c>
+      <c r="D1315" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412261/the-salty-sashimi-of-banda-sea-a-journey-through-inasua-history</t>
+        </is>
+      </c>
+    </row>
+    <row r="1316">
+      <c r="A1316" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1316" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1316" t="inlineStr">
+        <is>
+          <t>Minister clarifies "hajj ticket war" is still just a discourse</t>
+        </is>
+      </c>
+      <c r="D1316" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412260/minister-clarifies-hajj-ticket-war-is-still-just-a-discourse</t>
+        </is>
+      </c>
+    </row>
+    <row r="1317">
+      <c r="A1317" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1317" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1317" t="inlineStr">
+        <is>
+          <t>Indonesia-US sign major defense cooperation pact, boost military ties</t>
+        </is>
+      </c>
+      <c r="D1317" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412256/indonesia-us-sign-major-defense-cooperation-pact-boost-military-ties</t>
+        </is>
+      </c>
+    </row>
+    <row r="1318">
+      <c r="A1318" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1318" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1318" t="inlineStr">
+        <is>
+          <t>Indonesia negotiates the purchase of crude oil and LPG from Russia</t>
+        </is>
+      </c>
+      <c r="D1318" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412253/indonesia-negotiates-the-purchase-of-crude-oil-and-lpg-from-russia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1319">
+      <c r="A1319" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1319" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1319" t="inlineStr">
+        <is>
+          <t>DayOne Announces RM28+ Billion Commitment and Talent Initiatives in Malaysia at Inaugural Tech &amp; AI Career Expo</t>
+        </is>
+      </c>
+      <c r="D1319" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412251/dayone-announces-rm28-billion-commitment-and-talent-initiatives-in-malaysia-at-inaugural-tech-ai-career-expo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1320">
+      <c r="A1320" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1320" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1320" t="inlineStr">
+        <is>
+          <t>Xinhua Silk Road: Xianyang Fu Tea delegation visits embassies of five countries in Beijing to promote Chinese tea culture</t>
+        </is>
+      </c>
+      <c r="D1320" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412247/xinhua-silk-road-xianyang-fu-tea-delegation-visits-embassies-of-five-countries-in-beijing-to-promote-chinese-tea-culture</t>
+        </is>
+      </c>
+    </row>
+    <row r="1321">
+      <c r="A1321" t="inlineStr">
+        <is>
+          <t>Wednesday, 15 April 2026</t>
+        </is>
+      </c>
+      <c r="B1321" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1321" t="inlineStr">
+        <is>
+          <t>This Beer Brand Didn't Film Commercials, It Printed Them</t>
+        </is>
+      </c>
+      <c r="D1321" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412244/this-beer-brand-didnt-film-commercials-it-printed-them</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1261"/>
+  <autoFilter ref="A1:D1321"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -29453,6 +30773,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1259" r:id="rId1258"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1260" r:id="rId1259"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1261" r:id="rId1260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1262" r:id="rId1261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1263" r:id="rId1262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1264" r:id="rId1263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1265" r:id="rId1264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1266" r:id="rId1265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1267" r:id="rId1266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1268" r:id="rId1267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1269" r:id="rId1268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1270" r:id="rId1269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1271" r:id="rId1270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1272" r:id="rId1271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1273" r:id="rId1272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1274" r:id="rId1273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1275" r:id="rId1274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1276" r:id="rId1275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1277" r:id="rId1276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1278" r:id="rId1277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1279" r:id="rId1278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1280" r:id="rId1279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1281" r:id="rId1280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1282" r:id="rId1281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1283" r:id="rId1282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1284" r:id="rId1283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1285" r:id="rId1284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1286" r:id="rId1285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1287" r:id="rId1286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1288" r:id="rId1287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1289" r:id="rId1288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1290" r:id="rId1289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1291" r:id="rId1290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1292" r:id="rId1291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1293" r:id="rId1292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1294" r:id="rId1293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1295" r:id="rId1294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1296" r:id="rId1295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1297" r:id="rId1296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1298" r:id="rId1297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1299" r:id="rId1298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1300" r:id="rId1299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1301" r:id="rId1300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1302" r:id="rId1301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1303" r:id="rId1302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1304" r:id="rId1303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1305" r:id="rId1304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1306" r:id="rId1305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1307" r:id="rId1306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1308" r:id="rId1307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1309" r:id="rId1308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1310" r:id="rId1309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1311" r:id="rId1310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1312" r:id="rId1311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1313" r:id="rId1312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1314" r:id="rId1313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1315" r:id="rId1314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1316" r:id="rId1315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1317" r:id="rId1316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1318" r:id="rId1317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1319" r:id="rId1318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1320" r:id="rId1319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1321" r:id="rId1320"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-15
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1321</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1381</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1321"/>
+  <dimension ref="A1:D1381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -29510,8 +29510,1328 @@
         </is>
       </c>
     </row>
+    <row r="1322">
+      <c r="A1322" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1322" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1322" t="inlineStr">
+        <is>
+          <t>Video Momen Polisi Gerebek Pabrik Whip-pink Ilegal Beromzet Miliaran</t>
+        </is>
+      </c>
+      <c r="D1322" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8446226/video-momen-polisi-gerebek-pabrik-whip-pink-ilegal-beromzet-miliaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="1323">
+      <c r="A1323" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1323" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1323" t="inlineStr">
+        <is>
+          <t>Purbaya Ungkap Investor AS Dengar Isu Tak Sedap soal RI</t>
+        </is>
+      </c>
+      <c r="D1323" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8446148/purbaya-ungkap-investor-as-dengar-isu-tak-sedap-soal-ri</t>
+        </is>
+      </c>
+    </row>
+    <row r="1324">
+      <c r="A1324" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1324" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1324" t="inlineStr">
+        <is>
+          <t>Video Wapres AS: Paus Leo Harus Hati-hati Kalau Bicara soal Agama</t>
+        </is>
+      </c>
+      <c r="D1324" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8445963/video-wapres-as-paus-leo-harus-hati-hati-kalau-bicara-soal-agama</t>
+        </is>
+      </c>
+    </row>
+    <row r="1325">
+      <c r="A1325" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1325" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1325" t="inlineStr">
+        <is>
+          <t>Video Terseret Dugaan Korupsi, Nadiem Curhat Tak Paham Budaya Birokrasi</t>
+        </is>
+      </c>
+      <c r="D1325" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8445938/video-terseret-dugaan-korupsi-nadiem-curhat-tak-paham-budaya-birokrasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1326">
+      <c r="A1326" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1326" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1326" t="inlineStr">
+        <is>
+          <t>Andrie Yunus dalam Pergerakan Perjuangan HAM</t>
+        </is>
+      </c>
+      <c r="D1326" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/spotlight/d-8445824/andrie-yunus-dalam-pergerakan-perjuangan-ham</t>
+        </is>
+      </c>
+    </row>
+    <row r="1327">
+      <c r="A1327" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1327" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1327" t="inlineStr">
+        <is>
+          <t>Video Mensos Pastikan 11 Juta Peserta PBI BPJS Nonaktif Tetap Bisa Berobat</t>
+        </is>
+      </c>
+      <c r="D1327" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8446352/video-mensos-pastikan-11-juta-peserta-pbi-bpjs-nonaktif-tetap-bisa-berobat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1328">
+      <c r="A1328" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1328" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1328" t="inlineStr">
+        <is>
+          <t>Video Sekjen PBNU Ucapkan Selamat Lebaran untuk Sekum Muhammadiyah</t>
+        </is>
+      </c>
+      <c r="D1328" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8408290/video-sekjen-pbnu-ucapkan-selamat-lebaran-untuk-sekum-muhammadiyah</t>
+        </is>
+      </c>
+    </row>
+    <row r="1329">
+      <c r="A1329" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1329" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1329" t="inlineStr">
+        <is>
+          <t>Video Pemerintah Mutakhirkan Data 11 Juta PBI JKN</t>
+        </is>
+      </c>
+      <c r="D1329" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8369500/video-pemerintah-mutakhirkan-data-11-juta-pbi-jkn</t>
+        </is>
+      </c>
+    </row>
+    <row r="1330">
+      <c r="A1330" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1330" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1330" t="inlineStr">
+        <is>
+          <t>Bayern Vs Madrid: Die Roten Menang 4-3, Lolos ke Semifinal</t>
+        </is>
+      </c>
+      <c r="D1330" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/uefa/d-8446339/bayern-vs-madrid-die-roten-menang-4-3-lolos-ke-semifinal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1331">
+      <c r="A1331" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1331" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1331" t="inlineStr">
+        <is>
+          <t>Ini Alasan Label 'Nutri-Level' Diprioritaskan untuk Minuman Kopsus-Boba Cs</t>
+        </is>
+      </c>
+      <c r="D1331" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8446080/ini-alasan-label-nutri-level-diprioritaskan-untuk-minuman-kopsus-boba-cs</t>
+        </is>
+      </c>
+    </row>
+    <row r="1332">
+      <c r="A1332" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1332" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1332" t="inlineStr">
+        <is>
+          <t>Arsenal Vs Sporting Imbang, Meriam London ke Semifinal Liga Champions</t>
+        </is>
+      </c>
+      <c r="D1332" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/uefa/d-8446338/arsenal-vs-sporting-imbang-meriam-london-ke-semifinal-liga-champions</t>
+        </is>
+      </c>
+    </row>
+    <row r="1333">
+      <c r="A1333" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1333" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1333" t="inlineStr">
+        <is>
+          <t>Video: Penampakan Macetnya Selat Hormuz Seusai Diblokade AS</t>
+        </is>
+      </c>
+      <c r="D1333" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260416-260416001/video-penampakan-macetnya-selat-hormuz-seusai-diblokade-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="1334">
+      <c r="A1334" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1334" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1334" t="inlineStr">
+        <is>
+          <t>Video Iran: Belum Ada Konfirmasi soal Perpanjangan Gencatan Senjata</t>
+        </is>
+      </c>
+      <c r="D1334" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260416-260416002/video-iran-belum-ada-konfirmasi-soal-perpanjangan-gencatan-senjata</t>
+        </is>
+      </c>
+    </row>
+    <row r="1335">
+      <c r="A1335" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1335" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1335" t="inlineStr">
+        <is>
+          <t>Video: Momen Polisi dan Warga Tangkap Begal di Probolinggo</t>
+        </is>
+      </c>
+      <c r="D1335" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260415-260415269/video-momen-polisi-dan-warga-tangkap-begal-di-probolinggo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1336">
+      <c r="A1336" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1336" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1336" t="inlineStr">
+        <is>
+          <t>Raffi Ahmad Sudah Bicara dengan Sri Wulansih, Jadi Beli Apartemen Jupe?</t>
+        </is>
+      </c>
+      <c r="D1336" s="2" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8445762/raffi-ahmad-sudah-bicara-dengan-sri-wulansih-jadi-beli-apartemen-jupe</t>
+        </is>
+      </c>
+    </row>
+    <row r="1337">
+      <c r="A1337" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1337" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1337" t="inlineStr">
+        <is>
+          <t>Banjir Solo-Sukoharjo Sebabkan 109 Warga Mengungsi, 715 KK Terdampak</t>
+        </is>
+      </c>
+      <c r="D1337" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1923876/banjir-solo-sukoharjo-sebabkan-109-warga-mengungsi-715-kk-terdampak?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1338">
+      <c r="A1338" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1338" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1338" t="inlineStr">
+        <is>
+          <t>Optimalisasi Platform Digital Memperkuat Pasar UMKM</t>
+        </is>
+      </c>
+      <c r="D1338" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/optimalisasi-platform-digital-memperkuat-pasar-umkm?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1339">
+      <c r="A1339" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1339" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1339" t="inlineStr">
+        <is>
+          <t>Transformasi Bank Brebes Berbuah Manis, Raih Penghargaan Bergengsi hingga Tingkatkan Kepercayaan Publik</t>
+        </is>
+      </c>
+      <c r="D1339" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/15/212532278/transformasi-bank-brebes-berbuah-manis-raih-penghargaan-bergengsi-hingga</t>
+        </is>
+      </c>
+    </row>
+    <row r="1340">
+      <c r="A1340" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1340" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1340" t="inlineStr">
+        <is>
+          <t>Mendagri Apresiasi Program Bedah Rumah Kementerian PKP di Papua</t>
+        </is>
+      </c>
+      <c r="D1340" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/15/20460021/mendagri-apresiasi-program-bedah-rumah-kementerian-pkp-di-papua</t>
+        </is>
+      </c>
+    </row>
+    <row r="1341">
+      <c r="A1341" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1341" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1341" t="inlineStr">
+        <is>
+          <t>Sinergi PAM JAYA dan TP PKK DKI Jakarta Bagikan 270 Toren Air Gratis di Jakut</t>
+        </is>
+      </c>
+      <c r="D1341" s="2" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/04/15/20362521/sinergi-pam-jaya-dan-tp-pkk-dki-jakarta-bagikan-270-toren-air-gratis-di</t>
+        </is>
+      </c>
+    </row>
+    <row r="1342">
+      <c r="A1342" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1342" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1342" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D1342" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1343">
+      <c r="A1343" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1343" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1343" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D1343" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1344">
+      <c r="A1344" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1344" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1344" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D1344" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1345">
+      <c r="A1345" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1345" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1345" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D1345" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1346">
+      <c r="A1346" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1346" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1346" t="inlineStr">
+        <is>
+          <t>Janji AS jika Iran Tak Akan Punya Senjata Nuklir</t>
+        </is>
+      </c>
+      <c r="D1346" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1923839/janji-as-jika-iran-tak-akan-punya-senjata-nuklir?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1347">
+      <c r="A1347" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1347" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1347" t="inlineStr">
+        <is>
+          <t>Menepi dari Keriuhan: Ziarah ke Gua Maria Ratu Besokor, Weleri</t>
+        </is>
+      </c>
+      <c r="D1347" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/bonaboni/69df4c5034777c6c142ac972/menepi-dari-keriuhan-ziarah-ke-gua-maria-ratu-besokor-weleri</t>
+        </is>
+      </c>
+    </row>
+    <row r="1348">
+      <c r="A1348" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1348" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1348" t="inlineStr">
+        <is>
+          <t>Viral Pajak Orang Single di Jepang, Ternyata Bukan Pajak Khusus Lajang</t>
+        </is>
+      </c>
+      <c r="D1348" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5825/viral-pajak-orang-single-di-jepang-ternyata-bukan-pajak-khusus-lajang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1349">
+      <c r="A1349" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1349" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1349" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1349" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1350">
+      <c r="A1350" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1350" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1350" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1350" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1351">
+      <c r="A1351" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1351" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1351" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Penampakan Langka Bumi dan Bulan yang Dipotret Kru Artemis II NASA</t>
+        </is>
+      </c>
+      <c r="D1351" s="2" t="inlineStr">
+        <is>
+          <t>https://tekno.kompas.com/read/2026/04/09/18020027/berita-foto-penampakan-langka-bumi-dan-bulan-yang-dipotret-kru-artemis-ii-nasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1352">
+      <c r="A1352" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1352" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1352" t="inlineStr">
+        <is>
+          <t>Doli: Pembahasan Awal Revisi UU Pemilu Tiba-tiba Ditunda</t>
+        </is>
+      </c>
+      <c r="D1352" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098459/doli-pembahasan-awal-revisi-uu-pemilu-tiba-tiba-ditunda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1353">
+      <c r="A1353" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1353" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1353" t="inlineStr">
+        <is>
+          <t>Pramono Anung Lantik Kepala Dishub Jadi Wali Kota Jaksel</t>
+        </is>
+      </c>
+      <c r="D1353" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098452/pramono-anung-lantik-kepala-dishub-jadi-wali-kota-jaksel</t>
+        </is>
+      </c>
+    </row>
+    <row r="1354">
+      <c r="A1354" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1354" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1354" t="inlineStr">
+        <is>
+          <t>Alasan Lemhanas Menggelar Retret DPRD di Akmil Magelang</t>
+        </is>
+      </c>
+      <c r="D1354" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098446/alasan-lemhanas-menggelar-retret-dprd-di-akmil-magelang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1355">
+      <c r="A1355" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1355" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1355" t="inlineStr">
+        <is>
+          <t>Wako Pekanbaru Integrasikan Bantuan Pangan dan Cek Kesehatan Gratis</t>
+        </is>
+      </c>
+      <c r="D1355" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098431/wako-pekanbaru-integrasikan-bantuan-pangan-dan-cek-kesehatan-gratis</t>
+        </is>
+      </c>
+    </row>
+    <row r="1356">
+      <c r="A1356" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1356" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1356" t="inlineStr">
+        <is>
+          <t>Ketua DPRD se-Indonesia Ikut Retret di Magelang</t>
+        </is>
+      </c>
+      <c r="D1356" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098430/ketua-dprd-se-indonesia-ikut-retret-di-magelang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1357">
+      <c r="A1357" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1357" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1357" t="inlineStr">
+        <is>
+          <t>KKJ: Keberatan Konten Jurnalistik Diajukan ke Dewan Pers</t>
+        </is>
+      </c>
+      <c r="D1357" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098417/kkj-keberatan-konten-jurnalistik-diajukan-ke-dewan-pers</t>
+        </is>
+      </c>
+    </row>
+    <row r="1358">
+      <c r="A1358" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1358" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1358" t="inlineStr">
+        <is>
+          <t>Wamen Dikti: Sanksi bagi Pelaku Pelecehan Tergantung Kampus</t>
+        </is>
+      </c>
+      <c r="D1358" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098412/wamen-dikti-sanksi-bagi-pelaku-pelecehan-tergantung-kampus</t>
+        </is>
+      </c>
+    </row>
+    <row r="1359">
+      <c r="A1359" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1359" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1359" t="inlineStr">
+        <is>
+          <t>Wilayah Indonesia Bertambah 127,3 Hektare di Pulau Sebatik</t>
+        </is>
+      </c>
+      <c r="D1359" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098410/wilayah-indonesia-bertambah-1273-hektare-di-pulau-sebatik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1360">
+      <c r="A1360" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1360" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1360" t="inlineStr">
+        <is>
+          <t>Pengadilan Militer Siapkan Jadwal Sidang Kasus Andrie Yunus</t>
+        </is>
+      </c>
+      <c r="D1360" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098402/pengadilan-militer-siapkan-jadwal-sidang-kasus-andrie-yunus</t>
+        </is>
+      </c>
+    </row>
+    <row r="1361">
+      <c r="A1361" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1361" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1361" t="inlineStr">
+        <is>
+          <t>HMT ITB Minta Maaf soal Viral Konten Lagu Erika</t>
+        </is>
+      </c>
+      <c r="D1361" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098399/hmt-itb-minta-maaf-soal-viral-konten-lagu-erika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1362">
+      <c r="A1362" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1362" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1362" t="inlineStr">
+        <is>
+          <t>Program MBG di Bogor Telan Rp 1 Triliun Per Bulan</t>
+        </is>
+      </c>
+      <c r="D1362" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098396/program-mbg-di-bogor-telan-rp-1-triliun-per-bulan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1363">
+      <c r="A1363" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1363" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1363" t="inlineStr">
+        <is>
+          <t>Bantah Tempo, Ketua NasDem Sumut: Ketua Umum Selalu Happy</t>
+        </is>
+      </c>
+      <c r="D1363" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098395/bantah-tempo-ketua-nasdem-sumut-ketua-umum-selalu-happy</t>
+        </is>
+      </c>
+    </row>
+    <row r="1364">
+      <c r="A1364" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1364" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1364" t="inlineStr">
+        <is>
+          <t>Pemerintah Cari Landasan Hukum Tambal Kenaikan Biaya Haji</t>
+        </is>
+      </c>
+      <c r="D1364" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098390/pemerintah-cari-landasan-hukum-tambal-kenaikan-biaya-haji</t>
+        </is>
+      </c>
+    </row>
+    <row r="1365">
+      <c r="A1365" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1365" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1365" t="inlineStr">
+        <is>
+          <t>Peringatan HUT Kota Semarang ke-479 Berfokus Pada Pelayanan Bagi Masyarakat</t>
+        </is>
+      </c>
+      <c r="D1365" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098389/peringatan-hut-kota-semarang-ke-479-berfokus-pada-pelayanan-bagi-masyarakat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1366">
+      <c r="A1366" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1366" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1366" t="inlineStr">
+        <is>
+          <t>Reaksi ITB Soal Konten Video Lagu Erika</t>
+        </is>
+      </c>
+      <c r="D1366" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098388/reaksi-itb-soal-konten-video-lagu-erika</t>
+        </is>
+      </c>
+    </row>
+    <row r="1367">
+      <c r="A1367" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1367" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1367" t="inlineStr">
+        <is>
+          <t>Indonesia eyes urea fertilizer exports to four countries</t>
+        </is>
+      </c>
+      <c r="D1367" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412420/indonesia-eyes-urea-fertilizer-exports-to-four-countries</t>
+        </is>
+      </c>
+    </row>
+    <row r="1368">
+      <c r="A1368" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1368" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1368" t="inlineStr">
+        <is>
+          <t>Indonesia to implement e-cigarette regulation in July</t>
+        </is>
+      </c>
+      <c r="D1368" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412416/indonesia-to-implement-e-cigarette-regulation-in-july</t>
+        </is>
+      </c>
+    </row>
+    <row r="1369">
+      <c r="A1369" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1369" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1369" t="inlineStr">
+        <is>
+          <t>Makassar, Finland explore infrastructure and education collaborations</t>
+        </is>
+      </c>
+      <c r="D1369" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412415/makassar-finland-explore-infrastructure-and-education-collaborations</t>
+        </is>
+      </c>
+    </row>
+    <row r="1370">
+      <c r="A1370" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1370" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1370" t="inlineStr">
+        <is>
+          <t>Govt sets 1,000 daily visitor cap as overtourism harms Komodo habitat</t>
+        </is>
+      </c>
+      <c r="D1370" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412412/govt-sets-1000-daily-visitor-cap-as-overtourism-harms-komodo-habitat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1371">
+      <c r="A1371" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1371" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1371" t="inlineStr">
+        <is>
+          <t>Indonesia rolls out five-pillar cement decarbonization strategy</t>
+        </is>
+      </c>
+      <c r="D1371" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412408/indonesia-rolls-out-five-pillar-cement-decarbonization-strategy</t>
+        </is>
+      </c>
+    </row>
+    <row r="1372">
+      <c r="A1372" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1372" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1372" t="inlineStr">
+        <is>
+          <t>World Bank, rating agencies back Prabowo's fiscal strategy: Minister</t>
+        </is>
+      </c>
+      <c r="D1372" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412404/world-bank-rating-agencies-back-prabowos-fiscal-strategy-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="1373">
+      <c r="A1373" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1373" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1373" t="inlineStr">
+        <is>
+          <t>Indonesia seeks Russia's expertise to boost digital governance reform</t>
+        </is>
+      </c>
+      <c r="D1373" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412401/indonesia-seeks-russias-expertise-to-boost-digital-governance-reform</t>
+        </is>
+      </c>
+    </row>
+    <row r="1374">
+      <c r="A1374" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1374" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1374" t="inlineStr">
+        <is>
+          <t>Isosolo dance welcomes international tourists in Yobeh Village</t>
+        </is>
+      </c>
+      <c r="D1374" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/photo/412400/isosolo-dance-welcomes-international-tourists-in-yobeh-village</t>
+        </is>
+      </c>
+    </row>
+    <row r="1375">
+      <c r="A1375" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1375" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1375" t="inlineStr">
+        <is>
+          <t>Indonesia's 3M homes plan to boost economy with massive ripple effect</t>
+        </is>
+      </c>
+      <c r="D1375" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412399/indonesias-3m-homes-plan-to-boost-economy-with-massive-ripple-effect</t>
+        </is>
+      </c>
+    </row>
+    <row r="1376">
+      <c r="A1376" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1376" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1376" t="inlineStr">
+        <is>
+          <t>VP Gibran discusses AI, welfare support for madrasa teachers</t>
+        </is>
+      </c>
+      <c r="D1376" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412395/vp-gibran-discusses-ai-welfare-support-for-madrasa-teachers</t>
+        </is>
+      </c>
+    </row>
+    <row r="1377">
+      <c r="A1377" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1377" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1377" t="inlineStr">
+        <is>
+          <t>Police uncover illegal N2O gas factory in Jakarta</t>
+        </is>
+      </c>
+      <c r="D1377" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412392/police-uncover-illegal-n2o-gas-factory-in-jakarta</t>
+        </is>
+      </c>
+    </row>
+    <row r="1378">
+      <c r="A1378" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1378" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1378" t="inlineStr">
+        <is>
+          <t>Indonesia, Japan back Harapan Kita as Asia's biggest cardiac hub</t>
+        </is>
+      </c>
+      <c r="D1378" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412388/indonesia-japan-back-harapan-kita-as-asias-biggest-cardiac-hub</t>
+        </is>
+      </c>
+    </row>
+    <row r="1379">
+      <c r="A1379" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1379" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1379" t="inlineStr">
+        <is>
+          <t>MPR speaker affirms RI's non-taking of sides in US-Iran conflict</t>
+        </is>
+      </c>
+      <c r="D1379" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412384/mpr-speaker-affirms-ris-non-taking-of-sides-in-us-iran-conflict</t>
+        </is>
+      </c>
+    </row>
+    <row r="1380">
+      <c r="A1380" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1380" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1380" t="inlineStr">
+        <is>
+          <t>Indonesia seizes three vessels over illegal fishing</t>
+        </is>
+      </c>
+      <c r="D1380" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412380/indonesia-seizes-three-vessels-over-illegal-fishing</t>
+        </is>
+      </c>
+    </row>
+    <row r="1381">
+      <c r="A1381" t="inlineStr">
+        <is>
+          <t>Thursday, 16 April 2026</t>
+        </is>
+      </c>
+      <c r="B1381" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1381" t="inlineStr">
+        <is>
+          <t>East Java targets Ijen Geopark UNESCO status renewal</t>
+        </is>
+      </c>
+      <c r="D1381" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412379/east-java-targets-ijen-geopark-unesco-status-renewal</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1321"/>
+  <autoFilter ref="A1:D1381"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -30833,6 +32153,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1319" r:id="rId1318"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1320" r:id="rId1319"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1321" r:id="rId1320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1322" r:id="rId1321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1323" r:id="rId1322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1324" r:id="rId1323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1325" r:id="rId1324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1326" r:id="rId1325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1327" r:id="rId1326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1328" r:id="rId1327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1329" r:id="rId1328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1330" r:id="rId1329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1331" r:id="rId1330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1332" r:id="rId1331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1333" r:id="rId1332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1334" r:id="rId1333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1335" r:id="rId1334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1336" r:id="rId1335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1337" r:id="rId1336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1338" r:id="rId1337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1339" r:id="rId1338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1340" r:id="rId1339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1341" r:id="rId1340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1342" r:id="rId1341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1343" r:id="rId1342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1344" r:id="rId1343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1345" r:id="rId1344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1346" r:id="rId1345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1347" r:id="rId1346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1348" r:id="rId1347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1349" r:id="rId1348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1350" r:id="rId1349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1351" r:id="rId1350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1352" r:id="rId1351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1353" r:id="rId1352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1354" r:id="rId1353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1355" r:id="rId1354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1356" r:id="rId1355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1357" r:id="rId1356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1358" r:id="rId1357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1359" r:id="rId1358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1360" r:id="rId1359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1361" r:id="rId1360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1362" r:id="rId1361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1363" r:id="rId1362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1364" r:id="rId1363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1365" r:id="rId1364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1366" r:id="rId1365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1367" r:id="rId1366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1368" r:id="rId1367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1369" r:id="rId1368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1370" r:id="rId1369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1371" r:id="rId1370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1372" r:id="rId1371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1373" r:id="rId1372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1374" r:id="rId1373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1375" r:id="rId1374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1376" r:id="rId1375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1377" r:id="rId1376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1378" r:id="rId1377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1379" r:id="rId1378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1380" r:id="rId1379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1381" r:id="rId1380"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-16
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1381</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1441</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1381"/>
+  <dimension ref="A1:D1441"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -30830,8 +30830,1328 @@
         </is>
       </c>
     </row>
+    <row r="1382">
+      <c r="A1382" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1382" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1382" t="inlineStr">
+        <is>
+          <t>Kondisi Ekonomi Indonesia Diklaim Tahan Banting!</t>
+        </is>
+      </c>
+      <c r="D1382" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8447879/kondisi-ekonomi-indonesia-diklaim-tahan-banting</t>
+        </is>
+      </c>
+    </row>
+    <row r="1383">
+      <c r="A1383" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1383" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1383" t="inlineStr">
+        <is>
+          <t>KPK Temukan Surat 'Sakti' Bupati Tulungagung untuk Peras Bawahan</t>
+        </is>
+      </c>
+      <c r="D1383" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jatim/hukum-dan-kriminal/d-8447579/kpk-temukan-surat-sakti-bupati-tulungagung-untuk-peras-bawahan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1384">
+      <c r="A1384" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1384" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1384" t="inlineStr">
+        <is>
+          <t>Piala AFF U-17 2026: Indonesia Dikalahkan Malaysia 0-1</t>
+        </is>
+      </c>
+      <c r="D1384" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8447861/piala-aff-u-17-2026-indonesia-dikalahkan-malaysia-0-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1385">
+      <c r="A1385" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1385" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1385" t="inlineStr">
+        <is>
+          <t>Serpihan Heli PK-CFX Ditemukan, Namun Kondisi 8 Korban Belum Bisa Dipastikan</t>
+        </is>
+      </c>
+      <c r="D1385" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/kalimantan/berita/d-8447804/serpihan-heli-pk-cfx-ditemukan-namun-kondisi-8-korban-belum-bisa-dipastikan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1386">
+      <c r="A1386" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1386" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1386" t="inlineStr">
+        <is>
+          <t>Rangkuman Kasus Guru Besar Unpad Diduga Minta Foto Bikini Mahasiswi</t>
+        </is>
+      </c>
+      <c r="D1386" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jabar/berita/d-8447171/rangkuman-kasus-guru-besar-unpad-diduga-minta-foto-bikini-mahasiswi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1387">
+      <c r="A1387" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1387" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1387" t="inlineStr">
+        <is>
+          <t>Momen Paus Leo Ucap 'Assalamualaikum' hingga Kunjungi Masjid Agung Aljazair</t>
+        </is>
+      </c>
+      <c r="D1387" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8448010/momen-paus-leo-ucap-assalamualaikum-hingga-kunjungi-masjid-agung-aljazair</t>
+        </is>
+      </c>
+    </row>
+    <row r="1388">
+      <c r="A1388" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1388" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1388" t="inlineStr">
+        <is>
+          <t>Tak Sudah-sudah Trump Senggol Paus Leo</t>
+        </is>
+      </c>
+      <c r="D1388" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8446362/tak-sudah-sudah-trump-senggol-paus-leo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1389">
+      <c r="A1389" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1389" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1389" t="inlineStr">
+        <is>
+          <t>Trump Kembali Senggol Paus Leo, Bilang Iran Tak Boleh Punya Bom Nuklir</t>
+        </is>
+      </c>
+      <c r="D1389" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8445399/trump-kembali-senggol-paus-leo-bilang-iran-tak-boleh-punya-bom-nuklir</t>
+        </is>
+      </c>
+    </row>
+    <row r="1390">
+      <c r="A1390" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1390" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1390" t="inlineStr">
+        <is>
+          <t>Hasil Liga Europa: Aston Villa Gilas Bologna, Duo Spanyol Tersingkir</t>
+        </is>
+      </c>
+      <c r="D1390" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/uefa/d-8448009/hasil-liga-europa-aston-villa-gilas-bologna-duo-spanyol-tersingkir</t>
+        </is>
+      </c>
+    </row>
+    <row r="1391">
+      <c r="A1391" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1391" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1391" t="inlineStr">
+        <is>
+          <t>Belajar dari Viktor Axelsen, Dokter Ingatkan Risiko Saraf Kejepit dalam Olahraga</t>
+        </is>
+      </c>
+      <c r="D1391" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/kebugaran/d-8447985/belajar-dari-viktor-axelsen-dokter-ingatkan-risiko-saraf-kejepit-dalam-olahraga</t>
+        </is>
+      </c>
+    </row>
+    <row r="1392">
+      <c r="A1392" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1392" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1392" t="inlineStr">
+        <is>
+          <t>Helikopter PK-CFX Jatuh di Sekadau, 7 Korban Ditemukan Meninggal</t>
+        </is>
+      </c>
+      <c r="D1392" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/kalimantan/berita/d-8447889/helikopter-pk-cfx-jatuh-di-sekadau-7-korban-ditemukan-meninggal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1393">
+      <c r="A1393" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1393" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1393" t="inlineStr">
+        <is>
+          <t>Video: Satu Wanita Tewas Akibat Longsor di Sukabumi</t>
+        </is>
+      </c>
+      <c r="D1393" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260417-260417004/video-satu-wanita-tewas-akibat-longsor-di-sukabumi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1394">
+      <c r="A1394" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1394" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1394" t="inlineStr">
+        <is>
+          <t>Video Kades di Lumajang Dikeroyok-Dibacok OTK, Polisi Buru Pelaku</t>
+        </is>
+      </c>
+      <c r="D1394" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260416-260416321/video-kades-di-lumajang-dikeroyok-dibacok-otk-polisi-buru-pelaku</t>
+        </is>
+      </c>
+    </row>
+    <row r="1395">
+      <c r="A1395" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1395" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1395" t="inlineStr">
+        <is>
+          <t>Video: Kejati Geledah Kantor ESDM Jatim Terkait Dugaan Pungli</t>
+        </is>
+      </c>
+      <c r="D1395" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260416-260416320/video-kejati-geledah-kantor-esdm-jatim-terkait-dugaan-pungli</t>
+        </is>
+      </c>
+    </row>
+    <row r="1396">
+      <c r="A1396" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1396" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1396" t="inlineStr">
+        <is>
+          <t>Kisah Abdullah bin Al-Mubarak: Tidak Berhaji namun Menerima Predikat Haji Mabrur</t>
+        </is>
+      </c>
+      <c r="D1396" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/kisah/d-8447760/kisah-abdullah-bin-al-mubarak-tidak-berhaji-namun-menerima-predikat-haji-mabrur</t>
+        </is>
+      </c>
+    </row>
+    <row r="1397">
+      <c r="A1397" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1397" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1397" t="inlineStr">
+        <is>
+          <t>Iran Resmi Setop Ekspor Bahan Baku Plastik dan Pupuk akibat Serangan Israel</t>
+        </is>
+      </c>
+      <c r="D1397" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1924149/iran-resmi-setop-ekspor-bahan-baku-plastik-dan-pupuk-akibat-serangan-israel?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1398">
+      <c r="A1398" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1398" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1398" t="inlineStr">
+        <is>
+          <t>Kehormatan dan Aib</t>
+        </is>
+      </c>
+      <c r="D1398" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/cerpen-jumat-kehormatan-dan-aib?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1399">
+      <c r="A1399" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1399" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1399" t="inlineStr">
+        <is>
+          <t>KP2MI Pastikan Penanganan Kendala Pengiriman Barang Milik PMI Asal Medan Berjalan Transparan dan Akuntabel</t>
+        </is>
+      </c>
+      <c r="D1399" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/16/20204731/kp2mi-pastikan-penanganan-kendala-pengiriman-barang-milik-pmi-asal-medan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1400">
+      <c r="A1400" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1400" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1400" t="inlineStr">
+        <is>
+          <t>Produksi Sampah 550 Ton Per Hari, Ini Strategi Hulu-Hilir Pemkab Lamongan Ubah Sampah Jadi Berkah</t>
+        </is>
+      </c>
+      <c r="D1400" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/16/194104878/produksi-sampah-550-ton-per-hari-ini-strategi-hulu-hilir-pemkab-lamongan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1401">
+      <c r="A1401" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1401" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1401" t="inlineStr">
+        <is>
+          <t>Kumpulkan Industri Hulu-Hilir Plastik, Menperin Komitmen Jaga Stabilitas Pasokan Nasional</t>
+        </is>
+      </c>
+      <c r="D1401" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/16/19214881/kumpulkan-industri-hulu-hilir-plastik-menperin-komitmen-jaga-stabilitas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1402">
+      <c r="A1402" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1402" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1402" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D1402" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1403">
+      <c r="A1403" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1403" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1403" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D1403" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1404">
+      <c r="A1404" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1404" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1404" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D1404" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1405">
+      <c r="A1405" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1405" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1405" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D1405" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1406">
+      <c r="A1406" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1406" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1406" t="inlineStr">
+        <is>
+          <t>Trump Pede Bahagiakan Xi Jinping bila Selat Hormuz Terbuka Permanen</t>
+        </is>
+      </c>
+      <c r="D1406" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1924114/trump-pede-bahagiakan-xi-jinping-bila-selat-hormuz-terbuka-permanen?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1407">
+      <c r="A1407" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1407" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1407" t="inlineStr">
+        <is>
+          <t>Menggugat Meritokrasi: Bukan Sekadar Urusan Rajin dan Malas</t>
+        </is>
+      </c>
+      <c r="D1407" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/ajuskoto/69da1704ed641578762d06d4/menggugat-meritokrasi-bukan-sekedar-urusan-rajin-dan-malas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1408">
+      <c r="A1408" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1408" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1408" t="inlineStr">
+        <is>
+          <t>Film Detective Conan: Fallen Angel of the Highway Pecahkan Rekor, Raih 3,5 Miliar Yen dalam Tiga Hari!</t>
+        </is>
+      </c>
+      <c r="D1408" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5834/film-detective-conan-fallen-angel-of-the-highway-pecahkan-rekor-raih-3-5-miliar-yen-dalam-tiga-hari-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1409">
+      <c r="A1409" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1409" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1409" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1409" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1410">
+      <c r="A1410" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1410" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1410" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1410" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1411">
+      <c r="A1411" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1411" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1411" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Penampakan Langka Bumi dan Bulan yang Dipotret Kru Artemis II NASA</t>
+        </is>
+      </c>
+      <c r="D1411" s="2" t="inlineStr">
+        <is>
+          <t>https://tekno.kompas.com/read/2026/04/09/18020027/berita-foto-penampakan-langka-bumi-dan-bulan-yang-dipotret-kru-artemis-ii-nasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1412">
+      <c r="A1412" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1412" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1412" t="inlineStr">
+        <is>
+          <t>KSAD Temui Prabowo, Laporkan Pembangunan Jembatan</t>
+        </is>
+      </c>
+      <c r="D1412" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098695/ksad-temui-prabowo-laporkan-pembangunan-jembatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1413">
+      <c r="A1413" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1413" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1413" t="inlineStr">
+        <is>
+          <t>Ketua Ombudsman Tersangka, Begini Saran Komisi II DPR</t>
+        </is>
+      </c>
+      <c r="D1413" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098694/ketua-ombudsman-tersangka-begini-saran-komisi-ii-dpr</t>
+        </is>
+      </c>
+    </row>
+    <row r="1414">
+      <c r="A1414" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1414" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1414" t="inlineStr">
+        <is>
+          <t>Demokrat soal RUU Pemilu: Waktunya Masih Panjang</t>
+        </is>
+      </c>
+      <c r="D1414" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098689/demokrat-soal-ruu-pemilu-waktunya-masih-panjang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1415">
+      <c r="A1415" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1415" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1415" t="inlineStr">
+        <is>
+          <t>Prabowo Menerima Dasco di Istana Kepresidenan</t>
+        </is>
+      </c>
+      <c r="D1415" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098681/prabowo-menerima-dasco-di-istana-kepresidenan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1416">
+      <c r="A1416" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1416" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1416" t="inlineStr">
+        <is>
+          <t>Pemprov Sumbar Bentuk Tim Percepatan Pemulihan Sawah 3,902 Hektare</t>
+        </is>
+      </c>
+      <c r="D1416" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098680/pemprov-sumbar-bentuk-tim-percepatan-pemulihan-sawah-3902-hektare</t>
+        </is>
+      </c>
+    </row>
+    <row r="1417">
+      <c r="A1417" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1417" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1417" t="inlineStr">
+        <is>
+          <t>Kendaraan Listrik Tak Lagi Bebas Pajak, Pemprov DKI Berikan Keringanan</t>
+        </is>
+      </c>
+      <c r="D1417" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098679/kendaraan-listrik-tak-lagi-bebas-pajak-pemprov-dki-berikan-keringanan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1418">
+      <c r="A1418" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1418" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1418" t="inlineStr">
+        <is>
+          <t>Gubernur Lemhanas Beberkan Tujuan Retret Ketua DPRD</t>
+        </is>
+      </c>
+      <c r="D1418" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098678/gubernur-lemhanas-beberkan-tujuan-retret-ketua-dprd</t>
+        </is>
+      </c>
+    </row>
+    <row r="1419">
+      <c r="A1419" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1419" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1419" t="inlineStr">
+        <is>
+          <t>Pemprov Sumbar Bentuk Tim Percepatan Pemulihan Sawah 3,902 hektare</t>
+        </is>
+      </c>
+      <c r="D1419" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098676/pemprov-sumbar-bentuk-tim-percepatan-pemulihan-sawah-3902-hektare</t>
+        </is>
+      </c>
+    </row>
+    <row r="1420">
+      <c r="A1420" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1420" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1420" t="inlineStr">
+        <is>
+          <t>Bahlil Umumkan BBM Subsidi Tak Naik Sampai 2027</t>
+        </is>
+      </c>
+      <c r="D1420" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098670/bahlil-umumkan-bbm-subsidi-tak-naik-sampai-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="1421">
+      <c r="A1421" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1421" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1421" t="inlineStr">
+        <is>
+          <t>Sugiono Beri Wejangan ke Siswa Taruna Nusantara di Istana</t>
+        </is>
+      </c>
+      <c r="D1421" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098669/sugiono-beri-wejangan-ke-siswa-taruna-nusantara-di-istana</t>
+        </is>
+      </c>
+    </row>
+    <row r="1422">
+      <c r="A1422" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1422" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1422" t="inlineStr">
+        <is>
+          <t>Bahlil: Politik Bebas Aktif, Ekonomi Juga Bebas Aktif</t>
+        </is>
+      </c>
+      <c r="D1422" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098666/bahlil-politik-bebas-aktif-ekonomi-juga-bebas-aktif</t>
+        </is>
+      </c>
+    </row>
+    <row r="1423">
+      <c r="A1423" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1423" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1423" t="inlineStr">
+        <is>
+          <t>Wali Kota Agustina: Karnaval Paskah 2026 Semarang Kolaborasi Lintas Sektor</t>
+        </is>
+      </c>
+      <c r="D1423" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098665/wali-kota-agustina-karnaval-paskah-2026-semarang-kolaborasi-lintas-sektor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1424">
+      <c r="A1424" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1424" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1424" t="inlineStr">
+        <is>
+          <t>Harga Plastik Naik, Bahan Pokok di Cilegon Tetap Stabil</t>
+        </is>
+      </c>
+      <c r="D1424" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098663/harga-plastik-naik-bahan-pokok-di-cilegon-tetap-stabil</t>
+        </is>
+      </c>
+    </row>
+    <row r="1425">
+      <c r="A1425" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1425" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1425" t="inlineStr">
+        <is>
+          <t>Sekjen Golkar: DPR Harus Segera Bahas Revisi UU Pemilu</t>
+        </is>
+      </c>
+      <c r="D1425" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098660/sekjen-golkar-dpr-harus-segera-bahas-revisi-uu-pemilu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1426">
+      <c r="A1426" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1426" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1426" t="inlineStr">
+        <is>
+          <t>Istri Wali Kota Cilegon Turun Langsung Salurkan Bantuan Dinsos</t>
+        </is>
+      </c>
+      <c r="D1426" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098657/istri-wali-kota-cilegon-turun-langsung-salurkan-bantuan-dinsos</t>
+        </is>
+      </c>
+    </row>
+    <row r="1427">
+      <c r="A1427" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1427" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1427" t="inlineStr">
+        <is>
+          <t>Deputy Minister praises climate village in Central Java's Magelang</t>
+        </is>
+      </c>
+      <c r="D1427" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412633/deputy-minister-praises-climate-village-in-central-javas-magelang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1428">
+      <c r="A1428" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1428" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1428" t="inlineStr">
+        <is>
+          <t>Indonesia says AS, Russia visits reflect free and active policy</t>
+        </is>
+      </c>
+      <c r="D1428" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412631/indonesia-says-as-russia-visits-reflect-free-and-active-policy</t>
+        </is>
+      </c>
+    </row>
+    <row r="1429">
+      <c r="A1429" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1429" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1429" t="inlineStr">
+        <is>
+          <t>Indonesia carries energy cooperation based on national interests</t>
+        </is>
+      </c>
+      <c r="D1429" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412628/indonesia-carries-energy-cooperation-based-on-national-interests</t>
+        </is>
+      </c>
+    </row>
+    <row r="1430">
+      <c r="A1430" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1430" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1430" t="inlineStr">
+        <is>
+          <t>Indonesia eyes Russian oil while balancing US partnership: Minister</t>
+        </is>
+      </c>
+      <c r="D1430" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412625/indonesia-eyes-russian-oil-while-balancing-us-partnership-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="1431">
+      <c r="A1431" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1431" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1431" t="inlineStr">
+        <is>
+          <t>Basarnas finds debris of missing PK-CFX helicopter in West Kalimantan</t>
+        </is>
+      </c>
+      <c r="D1431" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412621/basarnas-finds-debris-of-missing-pk-cfx-helicopter-in-west-kalimantan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1432">
+      <c r="A1432" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1432" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1432" t="inlineStr">
+        <is>
+          <t>Indonesian textile competitive in domestic, international market: govt</t>
+        </is>
+      </c>
+      <c r="D1432" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412619/indonesian-textile-competitive-in-domestic-international-market-govt</t>
+        </is>
+      </c>
+    </row>
+    <row r="1433">
+      <c r="A1433" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1433" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1433" t="inlineStr">
+        <is>
+          <t>Purbaya reassures S&amp;P Indonesia's debt ratio safe, deficit may fall</t>
+        </is>
+      </c>
+      <c r="D1433" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412615/purbaya-reassures-sp-indonesias-debt-ratio-safe-deficit-may-fall</t>
+        </is>
+      </c>
+    </row>
+    <row r="1434">
+      <c r="A1434" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1434" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1434" t="inlineStr">
+        <is>
+          <t>Indonesia near final deal to import Russian crude oil: Minister</t>
+        </is>
+      </c>
+      <c r="D1434" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412611/indonesia-near-final-deal-to-import-russian-crude-oil-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="1435">
+      <c r="A1435" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1435" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1435" t="inlineStr">
+        <is>
+          <t>Indian Ambassador meets Dy Minister Sudaryono for urea import prospect</t>
+        </is>
+      </c>
+      <c r="D1435" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412608/indian-ambassador-meets-dy-minister-sudaryono-for-urea-import-prospect</t>
+        </is>
+      </c>
+    </row>
+    <row r="1436">
+      <c r="A1436" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1436" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1436" t="inlineStr">
+        <is>
+          <t>Indonesia certifies 13,576 MBG kitchens, eyes completion by August</t>
+        </is>
+      </c>
+      <c r="D1436" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412607/indonesia-certifies-13576-mbg-kitchens-eyes-completion-by-august</t>
+        </is>
+      </c>
+    </row>
+    <row r="1437">
+      <c r="A1437" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1437" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1437" t="inlineStr">
+        <is>
+          <t>Indonesia offers full scholarships, jobs for Sekolah Rakyat graduates</t>
+        </is>
+      </c>
+      <c r="D1437" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412604/indonesia-offers-full-scholarships-jobs-for-sekolah-rakyat-graduates</t>
+        </is>
+      </c>
+    </row>
+    <row r="1438">
+      <c r="A1438" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1438" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1438" t="inlineStr">
+        <is>
+          <t>Indonesia encourages US and Iran to continue dialogue</t>
+        </is>
+      </c>
+      <c r="D1438" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412603/indonesia-encourages-us-and-iran-to-continue-dialogue</t>
+        </is>
+      </c>
+    </row>
+    <row r="1439">
+      <c r="A1439" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1439" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1439" t="inlineStr">
+        <is>
+          <t>Human rights minister urges probe into Central Papua fatal shooting</t>
+        </is>
+      </c>
+      <c r="D1439" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412599/human-rights-minister-urges-probe-into-central-papua-fatal-shooting</t>
+        </is>
+      </c>
+    </row>
+    <row r="1440">
+      <c r="A1440" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1440" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1440" t="inlineStr">
+        <is>
+          <t>BRIN targets strategic research to boost Indonesia's cosmetic industry</t>
+        </is>
+      </c>
+      <c r="D1440" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412595/brin-targets-strategic-research-to-boost-indonesias-cosmetic-industry</t>
+        </is>
+      </c>
+    </row>
+    <row r="1441">
+      <c r="A1441" t="inlineStr">
+        <is>
+          <t>Friday, 17 April 2026</t>
+        </is>
+      </c>
+      <c r="B1441" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1441" t="inlineStr">
+        <is>
+          <t>Prabowo's Russia-France deals boost Indonesia's global bargaining</t>
+        </is>
+      </c>
+      <c r="D1441" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412592/prabowos-russia-france-deals-boost-indonesias-global-bargaining</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1381"/>
+  <autoFilter ref="A1:D1441"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -32213,6 +33533,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1379" r:id="rId1378"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1380" r:id="rId1379"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1381" r:id="rId1380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1382" r:id="rId1381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1383" r:id="rId1382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1384" r:id="rId1383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1385" r:id="rId1384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1386" r:id="rId1385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1387" r:id="rId1386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1388" r:id="rId1387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1389" r:id="rId1388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1390" r:id="rId1389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1391" r:id="rId1390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1392" r:id="rId1391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1393" r:id="rId1392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1394" r:id="rId1393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1395" r:id="rId1394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1396" r:id="rId1395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1397" r:id="rId1396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1398" r:id="rId1397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1399" r:id="rId1398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1400" r:id="rId1399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1401" r:id="rId1400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1402" r:id="rId1401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1403" r:id="rId1402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1404" r:id="rId1403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1405" r:id="rId1404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1406" r:id="rId1405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1407" r:id="rId1406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1408" r:id="rId1407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1409" r:id="rId1408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1410" r:id="rId1409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1411" r:id="rId1410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1412" r:id="rId1411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1413" r:id="rId1412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1414" r:id="rId1413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1415" r:id="rId1414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1416" r:id="rId1415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1417" r:id="rId1416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1418" r:id="rId1417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1419" r:id="rId1418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1420" r:id="rId1419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1421" r:id="rId1420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1422" r:id="rId1421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1423" r:id="rId1422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1424" r:id="rId1423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1425" r:id="rId1424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1426" r:id="rId1425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1427" r:id="rId1426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1428" r:id="rId1427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1429" r:id="rId1428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1430" r:id="rId1429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1431" r:id="rId1430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1432" r:id="rId1431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1433" r:id="rId1432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1434" r:id="rId1433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1435" r:id="rId1434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1436" r:id="rId1435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1437" r:id="rId1436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1438" r:id="rId1437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1439" r:id="rId1438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1440" r:id="rId1439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1441" r:id="rId1440"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-17
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1441</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1501</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1441"/>
+  <dimension ref="A1:D1501"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -32150,8 +32150,1328 @@
         </is>
       </c>
     </row>
+    <row r="1442">
+      <c r="A1442" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1442" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1442" t="inlineStr">
+        <is>
+          <t>Video Warga Lebanon Berbondong-bondong Pulang ke Rumah Usai Gencatan Senjata</t>
+        </is>
+      </c>
+      <c r="D1442" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8449665/video-warga-lebanon-berbondong-bondong-pulang-ke-rumah-usai-gencatan-senjata</t>
+        </is>
+      </c>
+    </row>
+    <row r="1443">
+      <c r="A1443" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1443" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1443" t="inlineStr">
+        <is>
+          <t>Video Iran Buka Selat Hormuz Selama Gencatan Senjata di Lebanon</t>
+        </is>
+      </c>
+      <c r="D1443" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8449659/video-iran-buka-selat-hormuz-selama-gencatan-senjata-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="1444">
+      <c r="A1444" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1444" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1444" t="inlineStr">
+        <is>
+          <t>Menteri PU Ngaku Stres-Sakit Perut Saat Kementerian Digeledah Kejati DKI</t>
+        </is>
+      </c>
+      <c r="D1444" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/infrastruktur/d-8449399/menteri-pu-ngaku-stres-sakit-perut-saat-kementerian-digeledah-kejati-dki</t>
+        </is>
+      </c>
+    </row>
+    <row r="1445">
+      <c r="A1445" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1445" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1445" t="inlineStr">
+        <is>
+          <t>Harga Minyak Indonesia Naik Jadi US$ 102,26/ Barel!</t>
+        </is>
+      </c>
+      <c r="D1445" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8449347/harga-minyak-indonesia-naik-jadi-us-102-26-barel</t>
+        </is>
+      </c>
+    </row>
+    <row r="1446">
+      <c r="A1446" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1446" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1446" t="inlineStr">
+        <is>
+          <t>Gas 3 Kg Nggak Naik!</t>
+        </is>
+      </c>
+      <c r="D1446" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8449318/gas-3-kg-nggak-naik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1447">
+      <c r="A1447" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1447" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1447" t="inlineStr">
+        <is>
+          <t>Infografis: RI Resmi Luncurkan Nutri Level, Begini Aturannya</t>
+        </is>
+      </c>
+      <c r="D1447" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/infografis/d-8449666/infografis-ri-resmi-luncurkan-nutri-level-begini-aturannya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1448">
+      <c r="A1448" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1448" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1448" t="inlineStr">
+        <is>
+          <t>Infografis: Kandungan Gizi Lele Vs Salmon, Apa Saja yang Beda?</t>
+        </is>
+      </c>
+      <c r="D1448" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/infografis/d-8440181/infografis-kandungan-gizi-lele-vs-salmon-apa-saja-yang-beda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1449">
+      <c r="A1449" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1449" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1449" t="inlineStr">
+        <is>
+          <t>Infografis: Komparasi Gizi Tahu Vs Tempe, Mana Lebih Unggul?</t>
+        </is>
+      </c>
+      <c r="D1449" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/infografis/d-8439046/infografis-komparasi-gizi-tahu-vs-tempe-mana-lebih-unggul</t>
+        </is>
+      </c>
+    </row>
+    <row r="1450">
+      <c r="A1450" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1450" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1450" t="inlineStr">
+        <is>
+          <t>Sarapan Pisang atau Jeruk? Ini Perbedaan Efek Energinya di Tubuh</t>
+        </is>
+      </c>
+      <c r="D1450" s="2" t="inlineStr">
+        <is>
+          <t>https://food.detik.com/info-sehat/d-8449661/sarapan-pisang-atau-jeruk-ini-perbedaan-efek-energinya-di-tubuh</t>
+        </is>
+      </c>
+    </row>
+    <row r="1451">
+      <c r="A1451" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1451" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1451" t="inlineStr">
+        <is>
+          <t>Tradisi Mengantar Jemaah Haji di Indonesia, Ini Sejarah dan Maknanya</t>
+        </is>
+      </c>
+      <c r="D1451" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8449352/tradisi-mengantar-jemaah-haji-di-indonesia-ini-sejarah-dan-maknanya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1452">
+      <c r="A1452" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1452" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1452" t="inlineStr">
+        <is>
+          <t>Trump Klaim AS Bantu Iran Bersihkan Ranjau Laut Usai Selat Hormuz Dibuka</t>
+        </is>
+      </c>
+      <c r="D1452" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8449543/trump-klaim-as-bantu-iran-bersihkan-ranjau-laut-usai-selat-hormuz-dibuka</t>
+        </is>
+      </c>
+    </row>
+    <row r="1453">
+      <c r="A1453" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1453" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1453" t="inlineStr">
+        <is>
+          <t>Video Menkomdigi Puji detikcom Gelar Apresiasi Konektivitas Digital 2026</t>
+        </is>
+      </c>
+      <c r="D1453" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260417-260417197/video-menkomdigi-puji-detikcom-gelar-apresiasi-konektivitas-digital-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1454">
+      <c r="A1454" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1454" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1454" t="inlineStr">
+        <is>
+          <t>Video: Daftar Pemenang Apresiasi Konektivitas Digital terhadap Mitra detikcom</t>
+        </is>
+      </c>
+      <c r="D1454" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260417-260417189/video-daftar-pemenang-apresiasi-konektivitas-digital-terhadap-mitra-detikcom</t>
+        </is>
+      </c>
+    </row>
+    <row r="1455">
+      <c r="A1455" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1455" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1455" t="inlineStr">
+        <is>
+          <t>Video Momen Meutya Hafid Nyanyi Bareng Nassar di Apresiasi Konektivitas Digital</t>
+        </is>
+      </c>
+      <c r="D1455" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260417-260417191/video-momen-meutya-hafid-nyanyi-bareng-nassar-di-apresiasi-konektivitas-digital</t>
+        </is>
+      </c>
+    </row>
+    <row r="1456">
+      <c r="A1456" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1456" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1456" t="inlineStr">
+        <is>
+          <t>Hore! Kapten Juventus Dapat Kontrak Baru</t>
+        </is>
+      </c>
+      <c r="D1456" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-italia/d-8449652/hore-kapten-juventus-dapat-kontrak-baru</t>
+        </is>
+      </c>
+    </row>
+    <row r="1457">
+      <c r="A1457" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1457" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1457" t="inlineStr">
+        <is>
+          <t>Mobil Listrik Tidak Lagi Otomatis Bebas Pajak, Ini Aturan Barunya</t>
+        </is>
+      </c>
+      <c r="D1457" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1924413/mobil-listrik-tidak-lagi-otomatis-bebas-pajak-ini-aturan-barunya?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1458">
+      <c r="A1458" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1458" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1458" t="inlineStr">
+        <is>
+          <t>Bagaimana Duduk Perkara Penggelapan Dana Gereja Rp 28 Miliar di Sumut?</t>
+        </is>
+      </c>
+      <c r="D1458" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/bagaimana-duduk-perkara-penggelapan-dana-gereja-rp-28-miliar-di-sumut?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1459">
+      <c r="A1459" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1459" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1459" t="inlineStr">
+        <is>
+          <t>Dukung Industri Dalam Negeri, KAI Hadirkan Layanan Gerbong Datar dari Banyuwangi ke Sumatera Selatan</t>
+        </is>
+      </c>
+      <c r="D1459" s="2" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/04/17/195857126/dukung-industri-dalam-negeri-kai-hadirkan-layanan-gerbong-datar-dari</t>
+        </is>
+      </c>
+    </row>
+    <row r="1460">
+      <c r="A1460" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1460" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1460" t="inlineStr">
+        <is>
+          <t>Ratusan Pustu Terdampak Bencana Kembali Beroperasi, Layanan Kesehatan Semakin Dekat</t>
+        </is>
+      </c>
+      <c r="D1460" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/17/19442391/ratusan-pustu-terdampak-bencana-kembali-beroperasi-layanan-kesehatan-semakin</t>
+        </is>
+      </c>
+    </row>
+    <row r="1461">
+      <c r="A1461" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1461" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1461" t="inlineStr">
+        <is>
+          <t>Ringankan Beban TPST Bantargebang, DLH Jakarta Optimalisasi RDF Plant Rorotan</t>
+        </is>
+      </c>
+      <c r="D1461" s="2" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/04/17/15452981/ringankan-beban-tpst-bantargebang-dlh-jakarta-optimalisasi-rdf-plant</t>
+        </is>
+      </c>
+    </row>
+    <row r="1462">
+      <c r="A1462" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1462" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1462" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D1462" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1463">
+      <c r="A1463" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1463" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1463" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D1463" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1464">
+      <c r="A1464" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1464" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1464" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D1464" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1465">
+      <c r="A1465" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1465" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1465" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D1465" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1466">
+      <c r="A1466" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1466" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1466" t="inlineStr">
+        <is>
+          <t>Gencatan Senjata Iran-AS: Umat Yahudi di Teheran Kenang Khamenei, Trump Masih Tebar Ancaman</t>
+        </is>
+      </c>
+      <c r="D1466" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1924391/gencatan-senjata-iran-as-umat-yahudi-di-teheran-kenang-khamenei-trump-masih-tebar-ancaman?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1467">
+      <c r="A1467" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1467" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1467" t="inlineStr">
+        <is>
+          <t>Mulai dari Nol: Titik Balik dalam Perjalanan Hidupku</t>
+        </is>
+      </c>
+      <c r="D1467" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/yycorjesu/69e1a3cec925c44d6c421bc3/mulai-dari-nol-titik-balik-dalam-perjalanan-hidupku</t>
+        </is>
+      </c>
+    </row>
+    <row r="1468">
+      <c r="A1468" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1468" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1468" t="inlineStr">
+        <is>
+          <t>Ternyata Begini Proses Mekarnya Sakura dan Kaitannya dengan Makanan Musiman</t>
+        </is>
+      </c>
+      <c r="D1468" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5841/ternyata-begini-proses-mekarnya-sakura-dan-kaitannya-dengan-makanan-musiman</t>
+        </is>
+      </c>
+    </row>
+    <row r="1469">
+      <c r="A1469" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1469" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1469" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1469" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1470">
+      <c r="A1470" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1470" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1470" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1470" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1471">
+      <c r="A1471" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1471" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1471" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Penampakan Langka Bumi dan Bulan yang Dipotret Kru Artemis II NASA</t>
+        </is>
+      </c>
+      <c r="D1471" s="2" t="inlineStr">
+        <is>
+          <t>https://tekno.kompas.com/read/2026/04/09/18020027/berita-foto-penampakan-langka-bumi-dan-bulan-yang-dipotret-kru-artemis-ii-nasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1472">
+      <c r="A1472" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1472" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1472" t="inlineStr">
+        <is>
+          <t>BUMD Leaders Forum, Pemprov DKI Jakarta Dorong Peran BUMD DKI Sebagai Pilar Ekonomi</t>
+        </is>
+      </c>
+      <c r="D1472" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098908/bumd-leaders-forum-pemprov-dki-jakarta-dorong-peran-bumd-dki-sebagai-pilar-ekonomi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1473">
+      <c r="A1473" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1473" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1473" t="inlineStr">
+        <is>
+          <t>Gubernur Pramono Anung Dorong BUMD Jakarta Berani Ekspansi</t>
+        </is>
+      </c>
+      <c r="D1473" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098904/gubernur-pramono-anung-dorong-bumd-jakarta-berani-ekspansi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1474">
+      <c r="A1474" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1474" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1474" t="inlineStr">
+        <is>
+          <t>Pemprov DKI Jakarta Lanjutkan Insentif PBB-P2 Tahun 2026, Ringankan Beban Wajib Pajak</t>
+        </is>
+      </c>
+      <c r="D1474" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098901/pemprov-dki-jakarta-lanjutkan-insentif-pbb-p2-tahun-2026-ringankan-beban-wajib-pajak</t>
+        </is>
+      </c>
+    </row>
+    <row r="1475">
+      <c r="A1475" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1475" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1475" t="inlineStr">
+        <is>
+          <t>BEM UI Tolak SK Rektor Soal Tarif Sewa Ruangan di Kampus</t>
+        </is>
+      </c>
+      <c r="D1475" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098888/bem-ui-tolak-sk-rektor-soal-tarif-sewa-ruangan-di-kampus</t>
+        </is>
+      </c>
+    </row>
+    <row r="1476">
+      <c r="A1476" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1476" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1476" t="inlineStr">
+        <is>
+          <t>LPSK Akan Lindungi Korban Dugaan Kekerasan Seksual di UI</t>
+        </is>
+      </c>
+      <c r="D1476" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098882/lpsk-akan-lindungi-korban-dugaan-kekerasan-seksual-di-ui</t>
+        </is>
+      </c>
+    </row>
+    <row r="1477">
+      <c r="A1477" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1477" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1477" t="inlineStr">
+        <is>
+          <t>Banyak Memiliki Keunggulan, BPD Didorong Naik Kelas</t>
+        </is>
+      </c>
+      <c r="D1477" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098881/banyak-memiliki-keunggulan-bpd-didorong-naik-kelas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1478">
+      <c r="A1478" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1478" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1478" t="inlineStr">
+        <is>
+          <t>Pusat UTBK di Bandung Waspadai Potensi Kehadiran Joki Ujian</t>
+        </is>
+      </c>
+      <c r="D1478" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098878/pusat-utbk-di-bandung-waspadai-potensi-kehadiran-joki-ujian</t>
+        </is>
+      </c>
+    </row>
+    <row r="1479">
+      <c r="A1479" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1479" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1479" t="inlineStr">
+        <is>
+          <t>Surat Andrie Yunus untuk Presiden Prabowo</t>
+        </is>
+      </c>
+      <c r="D1479" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098870/surat-andrie-yunus-untuk-presiden-prabowo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1480">
+      <c r="A1480" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1480" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1480" t="inlineStr">
+        <is>
+          <t>BGN: Semir dan Sikat Sepatu Bagian Fasilitas SPPI</t>
+        </is>
+      </c>
+      <c r="D1480" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098867/bgn-semir-dan-sikat-sepatu-bagian-fasilitas-sppi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1481">
+      <c r="A1481" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1481" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1481" t="inlineStr">
+        <is>
+          <t>Temuan ICW: Guru Laporkan Banyak Masalah Akibat MBG</t>
+        </is>
+      </c>
+      <c r="D1481" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098866/temuan-icw-guru-laporkan-banyak-masalah-akibat-mbg</t>
+        </is>
+      </c>
+    </row>
+    <row r="1482">
+      <c r="A1482" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1482" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1482" t="inlineStr">
+        <is>
+          <t>Pengganti Hery Susanto Diserahkan ke Internal Ombudsman RI</t>
+        </is>
+      </c>
+      <c r="D1482" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098863/pengganti-hery-susanto-diserahkan-ke-internal-ombudsman-ri</t>
+        </is>
+      </c>
+    </row>
+    <row r="1483">
+      <c r="A1483" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1483" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1483" t="inlineStr">
+        <is>
+          <t>KontraS Kritik Alasan TNI Soal Motif Pelaku Serang Andrie</t>
+        </is>
+      </c>
+      <c r="D1483" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098859/kontras-kritik-alasan-tni-soal-motif-pelaku-serang-andrie</t>
+        </is>
+      </c>
+    </row>
+    <row r="1484">
+      <c r="A1484" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1484" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1484" t="inlineStr">
+        <is>
+          <t>BPJS Kesehatan Pastikan Pengurusan Kepesertaan Gratis 100 Persen</t>
+        </is>
+      </c>
+      <c r="D1484" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098852/bpjs-kesehatan-pastikan-pengurusan-kepesertaan-gratis-100-persen</t>
+        </is>
+      </c>
+    </row>
+    <row r="1485">
+      <c r="A1485" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1485" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1485" t="inlineStr">
+        <is>
+          <t>Militer AS Langgar Wilayah RI, Kemlu: Sudah Ada Tindakan</t>
+        </is>
+      </c>
+      <c r="D1485" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098848/militer-as-langgar-wilayah-ri-kemlu-sudah-ada-tindakan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1486">
+      <c r="A1486" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1486" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1486" t="inlineStr">
+        <is>
+          <t>Tumbuh Bersama PNM Mekaar, Mardiana Berhasil Kembangkan Usahanya</t>
+        </is>
+      </c>
+      <c r="D1486" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098845/tumbuh-bersama-pnm-mekaar-mardiana-berhasil-kembangkan-usahanya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1487">
+      <c r="A1487" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1487" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1487" t="inlineStr">
+        <is>
+          <t>BGN to operate 900 free meals kitchens in remote areas</t>
+        </is>
+      </c>
+      <c r="D1487" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412759/bgn-to-operate-900-free-meals-kitchens-in-remote-areas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1488">
+      <c r="A1488" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1488" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1488" t="inlineStr">
+        <is>
+          <t>Free meals program aims to change people's mindsets on nutrition: BGN</t>
+        </is>
+      </c>
+      <c r="D1488" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412757/free-meals-program-aims-to-change-peoples-mindsets-on-nutrition-bgn</t>
+        </is>
+      </c>
+    </row>
+    <row r="1489">
+      <c r="A1489" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1489" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1489" t="inlineStr">
+        <is>
+          <t>Ministry pushes creative content to promote regional tourism</t>
+        </is>
+      </c>
+      <c r="D1489" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412753/ministry-pushes-creative-content-to-promote-regional-tourism</t>
+        </is>
+      </c>
+    </row>
+    <row r="1490">
+      <c r="A1490" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1490" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1490" t="inlineStr">
+        <is>
+          <t>Indonesia touts Bandung Principles as solution to global conflicts</t>
+        </is>
+      </c>
+      <c r="D1490" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412749/indonesia-touts-bandung-principles-as-solution-to-global-conflicts</t>
+        </is>
+      </c>
+    </row>
+    <row r="1491">
+      <c r="A1491" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1491" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1491" t="inlineStr">
+        <is>
+          <t>Indonesia, Japan seek deeper defense ties in ministerial talks</t>
+        </is>
+      </c>
+      <c r="D1491" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412747/indonesia-japan-seek-deeper-defense-ties-in-ministerial-talks</t>
+        </is>
+      </c>
+    </row>
+    <row r="1492">
+      <c r="A1492" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1492" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1492" t="inlineStr">
+        <is>
+          <t>President Prabowo urges forgiveness, unity after Nyepi observance</t>
+        </is>
+      </c>
+      <c r="D1492" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412744/president-prabowo-urges-forgiveness-unity-after-nyepi-observance</t>
+        </is>
+      </c>
+    </row>
+    <row r="1493">
+      <c r="A1493" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1493" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1493" t="inlineStr">
+        <is>
+          <t>Indonesia eyes AI to boost lab-based preventive care</t>
+        </is>
+      </c>
+      <c r="D1493" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412740/indonesia-eyes-ai-to-boost-lab-based-preventive-care</t>
+        </is>
+      </c>
+    </row>
+    <row r="1494">
+      <c r="A1494" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1494" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1494" t="inlineStr">
+        <is>
+          <t>Indonesia targets June completion for 97 Sekolah Rakyat sites</t>
+        </is>
+      </c>
+      <c r="D1494" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412737/indonesia-targets-june-completion-for-97-sekolah-rakyat-sites</t>
+        </is>
+      </c>
+    </row>
+    <row r="1495">
+      <c r="A1495" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1495" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1495" t="inlineStr">
+        <is>
+          <t>Multi-Color Corporation Announces Confirmation of Plan of Reorganization</t>
+        </is>
+      </c>
+      <c r="D1495" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412735/multi-color-corporation-announces-confirmation-of-plan-of-reorganization</t>
+        </is>
+      </c>
+    </row>
+    <row r="1496">
+      <c r="A1496" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1496" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1496" t="inlineStr">
+        <is>
+          <t>Ministries collaborate to bolster sports development in universities</t>
+        </is>
+      </c>
+      <c r="D1496" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412733/ministries-collaborate-to-bolster-sports-development-in-universities</t>
+        </is>
+      </c>
+    </row>
+    <row r="1497">
+      <c r="A1497" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1497" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1497" t="inlineStr">
+        <is>
+          <t>Export activities stay strong amid global turmoil: Indonesia Eximbank</t>
+        </is>
+      </c>
+      <c r="D1497" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412731/export-activities-stay-strong-amid-global-turmoil-indonesia-eximbank</t>
+        </is>
+      </c>
+    </row>
+    <row r="1498">
+      <c r="A1498" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1498" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1498" t="inlineStr">
+        <is>
+          <t>Baznas earmarks 10 percent of Qurbani meat to disaster-hit regions</t>
+        </is>
+      </c>
+      <c r="D1498" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412727/baznas-earmarks-10-percent-of-qurbani-meat-to-disaster-hit-regions</t>
+        </is>
+      </c>
+    </row>
+    <row r="1499">
+      <c r="A1499" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1499" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1499" t="inlineStr">
+        <is>
+          <t>Jakarta targets 50 percent emissions cut by 2030 via electric vehicles</t>
+        </is>
+      </c>
+      <c r="D1499" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412725/jakarta-targets-50-percent-emissions-cut-by-2030-via-electric-vehicles</t>
+        </is>
+      </c>
+    </row>
+    <row r="1500">
+      <c r="A1500" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1500" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1500" t="inlineStr">
+        <is>
+          <t>Minister says waste sorting habit reaches 60 pct in Denpasar</t>
+        </is>
+      </c>
+      <c r="D1500" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412724/minister-says-waste-sorting-habit-reaches-60-pct-in-denpasar</t>
+        </is>
+      </c>
+    </row>
+    <row r="1501">
+      <c r="A1501" t="inlineStr">
+        <is>
+          <t>Saturday, 18 April 2026</t>
+        </is>
+      </c>
+      <c r="B1501" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1501" t="inlineStr">
+        <is>
+          <t>MBG program needed by 65 percent of Indonesians, BGN says</t>
+        </is>
+      </c>
+      <c r="D1501" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412723/mbg-program-needed-by-65-percent-of-indonesians-bgn-says</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1441"/>
+  <autoFilter ref="A1:D1501"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -33593,6 +34913,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1439" r:id="rId1438"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1440" r:id="rId1439"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1441" r:id="rId1440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1442" r:id="rId1441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1443" r:id="rId1442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1444" r:id="rId1443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1445" r:id="rId1444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1446" r:id="rId1445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1447" r:id="rId1446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1448" r:id="rId1447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1449" r:id="rId1448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1450" r:id="rId1449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1451" r:id="rId1450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1452" r:id="rId1451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1453" r:id="rId1452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1454" r:id="rId1453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1455" r:id="rId1454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1456" r:id="rId1455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1457" r:id="rId1456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1458" r:id="rId1457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1459" r:id="rId1458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1460" r:id="rId1459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1461" r:id="rId1460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1462" r:id="rId1461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1463" r:id="rId1462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1464" r:id="rId1463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1465" r:id="rId1464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1466" r:id="rId1465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1467" r:id="rId1466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1468" r:id="rId1467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1469" r:id="rId1468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1470" r:id="rId1469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1471" r:id="rId1470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1472" r:id="rId1471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1473" r:id="rId1472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1474" r:id="rId1473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1475" r:id="rId1474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1476" r:id="rId1475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1477" r:id="rId1476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1478" r:id="rId1477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1479" r:id="rId1478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1480" r:id="rId1479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1481" r:id="rId1480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1482" r:id="rId1481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1483" r:id="rId1482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1484" r:id="rId1483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1485" r:id="rId1484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1486" r:id="rId1485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1487" r:id="rId1486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1488" r:id="rId1487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1489" r:id="rId1488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1490" r:id="rId1489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1491" r:id="rId1490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1492" r:id="rId1491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1493" r:id="rId1492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1494" r:id="rId1493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1495" r:id="rId1494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1496" r:id="rId1495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1497" r:id="rId1496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1498" r:id="rId1497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1499" r:id="rId1498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1500" r:id="rId1499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1501" r:id="rId1500"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-18
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1501</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1561</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1501"/>
+  <dimension ref="A1:D1561"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -33470,8 +33470,1328 @@
         </is>
       </c>
     </row>
+    <row r="1502">
+      <c r="A1502" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1502" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1502" t="inlineStr">
+        <is>
+          <t>Perkara Uranium yang Bikin Iran dan AS Berbantah-bantahan</t>
+        </is>
+      </c>
+      <c r="D1502" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8450613/perkara-uranium-yang-bikin-iran-dan-as-berbantah-bantahan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1503">
+      <c r="A1503" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1503" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1503" t="inlineStr">
+        <is>
+          <t>Siasat Eks Suami Bunuh Mantan Istri di Tangsel hingga Kelabui Saksi</t>
+        </is>
+      </c>
+      <c r="D1503" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8450569/siasat-eks-suami-bunuh-mantan-istri-di-tangsel-hingga-kelabui-saksi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1504">
+      <c r="A1504" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1504" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1504" t="inlineStr">
+        <is>
+          <t>Video JK: Kasih Tahu Semua 'Termul' Itu, Jokowi Jadi Presiden karena Saya!</t>
+        </is>
+      </c>
+      <c r="D1504" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8450529/video-jk-kasih-tahu-semua-termul-itu-jokowi-jadi-presiden-karena-saya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1505">
+      <c r="A1505" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1505" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1505" t="inlineStr">
+        <is>
+          <t>Video: Baru Beberapa Jam Dibuka, Selat Hormuz Kembali Ditutup Iran!</t>
+        </is>
+      </c>
+      <c r="D1505" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8450516/video-baru-beberapa-jam-dibuka-selat-hormuz-kembali-ditutup-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="1506">
+      <c r="A1506" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1506" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1506" t="inlineStr">
+        <is>
+          <t>Korban Pelecehan Sering Cemas dan Takut, Ini yang Sebenarnya Terjadi di Otak</t>
+        </is>
+      </c>
+      <c r="D1506" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8450330/korban-pelecehan-sering-cemas-dan-takut-ini-yang-sebenarnya-terjadi-di-otak</t>
+        </is>
+      </c>
+    </row>
+    <row r="1507">
+      <c r="A1507" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1507" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1507" t="inlineStr">
+        <is>
+          <t>Gempa M 5,9 Guncang Nias Utara</t>
+        </is>
+      </c>
+      <c r="D1507" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8450767/gempa-m-5-9-guncang-nias-utara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1508">
+      <c r="A1508" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1508" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1508" t="inlineStr">
+        <is>
+          <t>Waspada Banjir Rob di Pesisir RI Sampai 28 April, Ini Daftar Wilayahnya</t>
+        </is>
+      </c>
+      <c r="D1508" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8449926/waspada-banjir-rob-di-pesisir-ri-sampai-28-april-ini-daftar-wilayahnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1509">
+      <c r="A1509" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1509" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1509" t="inlineStr">
+        <is>
+          <t>Sudah Masuk Musim Kemarau Tapi Masih Hujan, Ini Penjelasannya</t>
+        </is>
+      </c>
+      <c r="D1509" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8449825/sudah-masuk-musim-kemarau-tapi-masih-hujan-ini-penjelasannya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1510">
+      <c r="A1510" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1510" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1510" t="inlineStr">
+        <is>
+          <t>2 Pencuri Brankas Isi 1 Kg Emas di Pinrang Sulsel Ditangkap</t>
+        </is>
+      </c>
+      <c r="D1510" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8450766/2-pencuri-brankas-isi-1-kg-emas-di-pinrang-sulsel-ditangkap</t>
+        </is>
+      </c>
+    </row>
+    <row r="1511">
+      <c r="A1511" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1511" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1511" t="inlineStr">
+        <is>
+          <t>Roma VS Atalanta Tuntas 1-1</t>
+        </is>
+      </c>
+      <c r="D1511" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-italia/d-8450764/roma-vs-atalanta-tuntas-1-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1512">
+      <c r="A1512" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1512" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1512" t="inlineStr">
+        <is>
+          <t>Clash of Legends: Barcelona Legends Gebuk DRX World Legends 3-0</t>
+        </is>
+      </c>
+      <c r="D1512" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-indonesia/d-8450625/clash-of-legends-barcelona-legends-gebuk-drx-world-legends-3-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="1513">
+      <c r="A1513" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1513" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1513" t="inlineStr">
+        <is>
+          <t>Video JK: Kasih Tahu Semua 'Termul' Itu, Jokowi Jadi Presiden karena Saya!</t>
+        </is>
+      </c>
+      <c r="D1513" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260418-260418038/video-jk-kasih-tahu-semua-termul-itu-jokowi-jadi-presiden-karena-saya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1514">
+      <c r="A1514" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1514" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1514" t="inlineStr">
+        <is>
+          <t>Video: Fans Naruto Merapat! Asian Kungfu Generation Ramaikan GBK</t>
+        </is>
+      </c>
+      <c r="D1514" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260418-260418042/video-fans-naruto-merapat-asian-kungfu-generation-ramaikan-gbk</t>
+        </is>
+      </c>
+    </row>
+    <row r="1515">
+      <c r="A1515" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1515" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1515" t="inlineStr">
+        <is>
+          <t>Video K-Talk: Euforia BTS-ARMY Bersatu Lagi Lewat Konser di Goyang Stadium</t>
+        </is>
+      </c>
+      <c r="D1515" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260418-260418031/video-k-talk-euforia-bts-army-bersatu-lagi-lewat-konser-di-goyang-stadium</t>
+        </is>
+      </c>
+    </row>
+    <row r="1516">
+      <c r="A1516" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1516" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1516" t="inlineStr">
+        <is>
+          <t>Chelsea Vs Man Utd: King MU Pecundangi London Biru 1-0</t>
+        </is>
+      </c>
+      <c r="D1516" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8450763/chelsea-vs-man-utd-king-mu-pecundangi-london-biru-1-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="1517">
+      <c r="A1517" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1517" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1517" t="inlineStr">
+        <is>
+          <t>Update Harga BBM Pertamina, Pertamax Turbo Naik</t>
+        </is>
+      </c>
+      <c r="D1517" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1924579/update-harga-bbm-pertamina-pertamax-turbo-naik?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1518">
+      <c r="A1518" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1518" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1518" t="inlineStr">
+        <is>
+          <t>Bocoran Program Para Cawapres untuk Debat Ketiga</t>
+        </is>
+      </c>
+      <c r="D1518" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/bocoran-program-para-cawapres-untuk-debat-ketiga?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1519">
+      <c r="A1519" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1519" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1519" t="inlineStr">
+        <is>
+          <t>BPJPH Benchmarking ke BPOM, Perkuat Standardisasi Laboratorium Halal Nasional</t>
+        </is>
+      </c>
+      <c r="D1519" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/18/17074481/bpjph-benchmarking-ke-bpom-perkuat-standardisasi-laboratorium-halal-nasional</t>
+        </is>
+      </c>
+    </row>
+    <row r="1520">
+      <c r="A1520" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1520" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1520" t="inlineStr">
+        <is>
+          <t>Bupati Jembrana Rintis Bus Gratis Pemedek, Berangkat Perdana 18 April 2026</t>
+        </is>
+      </c>
+      <c r="D1520" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/18/170656878/bupati-jembrana-rintis-bus-gratis-pemedek-berangkat-perdana-18-april-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1521">
+      <c r="A1521" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1521" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1521" t="inlineStr">
+        <is>
+          <t>Perkuat Keamanan Perbatasan, BNPP Percepat Penataan Eks OBP Simantipal dan Sebatik</t>
+        </is>
+      </c>
+      <c r="D1521" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/18/13413191/perkuat-keamanan-perbatasan-bnpp-percepat-penataan-eks-obp-simantipal-dan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1522">
+      <c r="A1522" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1522" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1522" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D1522" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1523">
+      <c r="A1523" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1523" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1523" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D1523" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1524">
+      <c r="A1524" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1524" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1524" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D1524" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1525">
+      <c r="A1525" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1525" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1525" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D1525" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1526">
+      <c r="A1526" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1526" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1526" t="inlineStr">
+        <is>
+          <t>Bantah Klaim Trump, Teheran Ogah Uraniumnya Dibawa Keluar Dari Iran</t>
+        </is>
+      </c>
+      <c r="D1526" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1924515/bantah-klaim-trump-teheran-ogah-uraniumnya-dibawa-keluar-dari-iran?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1527">
+      <c r="A1527" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1527" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1527" t="inlineStr">
+        <is>
+          <t>Orkes di Lantai Delapan Belas</t>
+        </is>
+      </c>
+      <c r="D1527" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/amirrrxitkj2044579/69d991c1c925c4329c1855e2/orkes-di-lantai-delapan-belas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1528">
+      <c r="A1528" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1528" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1528" t="inlineStr">
+        <is>
+          <t>Belajar Bahasa Jepang, 3 Peribahasa Sakura dan Artinya untuk Pemula</t>
+        </is>
+      </c>
+      <c r="D1528" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5845/belajar-bahasa-jepang-3-peribahasa-sakura-dan-artinya-untuk-pemula</t>
+        </is>
+      </c>
+    </row>
+    <row r="1529">
+      <c r="A1529" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1529" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1529" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1529" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1530">
+      <c r="A1530" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1530" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1530" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1530" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1531">
+      <c r="A1531" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1531" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1531" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Penampakan Langka Bumi dan Bulan yang Dipotret Kru Artemis II NASA</t>
+        </is>
+      </c>
+      <c r="D1531" s="2" t="inlineStr">
+        <is>
+          <t>https://tekno.kompas.com/read/2026/04/09/18020027/berita-foto-penampakan-langka-bumi-dan-bulan-yang-dipotret-kru-artemis-ii-nasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1532">
+      <c r="A1532" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1532" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1532" t="inlineStr">
+        <is>
+          <t>Rekrutmen Manajer Koperasi Merah Putih Tak Boleh Ada Titipan</t>
+        </is>
+      </c>
+      <c r="D1532" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099037/rekrutmen-manajer-koperasi-merah-putih-tak-boleh-ada-titipan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1533">
+      <c r="A1533" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1533" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1533" t="inlineStr">
+        <is>
+          <t>PDIP Dukung KPK soal Transparansi Dana Pendidikan Parpol</t>
+        </is>
+      </c>
+      <c r="D1533" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099034/pdip-dukung-kpk-soal-transparansi-dana-pendidikan-parpol</t>
+        </is>
+      </c>
+    </row>
+    <row r="1534">
+      <c r="A1534" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1534" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1534" t="inlineStr">
+        <is>
+          <t>Bupati Malang Angkat Anak Jadi Kadis, PDIP Minta Kritisi</t>
+        </is>
+      </c>
+      <c r="D1534" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099025/bupati-malang-angkat-anak-jadi-kadis-pdip-minta-kritisi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1535">
+      <c r="A1535" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1535" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1535" t="inlineStr">
+        <is>
+          <t>PDIP Dorong RUU Pemilu Segera Dibahas</t>
+        </is>
+      </c>
+      <c r="D1535" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099023/pdip-dorong-ruu-pemilu-segera-dibahas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1536">
+      <c r="A1536" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1536" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1536" t="inlineStr">
+        <is>
+          <t>Prabowo Sidak Gudang Bulog di Magelang</t>
+        </is>
+      </c>
+      <c r="D1536" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099021/prabowo-sidak-gudang-bulog-di-magelang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1537">
+      <c r="A1537" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1537" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1537" t="inlineStr">
+        <is>
+          <t>Jusuf Kalla Puji Megawati: Orang Paling Demokratis</t>
+        </is>
+      </c>
+      <c r="D1537" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099019/jusuf-kalla-puji-megawati-orang-paling-demokratis</t>
+        </is>
+      </c>
+    </row>
+    <row r="1538">
+      <c r="A1538" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1538" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1538" t="inlineStr">
+        <is>
+          <t>Minta Jokowi Tunjukkan Ijazah Asli, JK: Kasih Nasihat</t>
+        </is>
+      </c>
+      <c r="D1538" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099016/minta-jokowi-tunjukkan-ijazah-asli-jk-kasih-nasihat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1539">
+      <c r="A1539" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1539" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1539" t="inlineStr">
+        <is>
+          <t>Hasto Cerita Kebenaran Kritik Publik ke Pemerintahan Jokowi</t>
+        </is>
+      </c>
+      <c r="D1539" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099011/hasto-cerita-kebenaran-kritik-publik-ke-pemerintahan-jokowi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1540">
+      <c r="A1540" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1540" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1540" t="inlineStr">
+        <is>
+          <t>Cerita Jusuf Kalla Pertanyakan Keputusan Mega Usung Jokowi</t>
+        </is>
+      </c>
+      <c r="D1540" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099010/cerita-jusuf-kalla-pertanyakan-keputusan-mega-usung-jokowi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1541">
+      <c r="A1541" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1541" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1541" t="inlineStr">
+        <is>
+          <t>Polemik Internal Partai, Kader Daerah PPP Siapkan Langkah Hukum</t>
+        </is>
+      </c>
+      <c r="D1541" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098999/polemik-internal-partai-kader-daerah-ppp-siapkan-langkah-hukum</t>
+        </is>
+      </c>
+    </row>
+    <row r="1542">
+      <c r="A1542" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1542" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1542" t="inlineStr">
+        <is>
+          <t>Megawati Usulkan KAA Jilid II</t>
+        </is>
+      </c>
+      <c r="D1542" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098997/megawati-usulkan-kaa-jilid-ii</t>
+        </is>
+      </c>
+    </row>
+    <row r="1543">
+      <c r="A1543" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1543" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1543" t="inlineStr">
+        <is>
+          <t>Prabowo Soroti Perbedaan Partai hingga Suku di Retret DPRD</t>
+        </is>
+      </c>
+      <c r="D1543" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098985/prabowo-soroti-perbedaan-partai-hingga-suku-di-retret-dprd</t>
+        </is>
+      </c>
+    </row>
+    <row r="1544">
+      <c r="A1544" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1544" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1544" t="inlineStr">
+        <is>
+          <t>Prabowo di Retret DPRD: Saya Ingin Bicara dari Hati ke Hati</t>
+        </is>
+      </c>
+      <c r="D1544" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098982/prabowo-di-retret-dprd-saya-ingin-bicara-dari-hati-ke-hati</t>
+        </is>
+      </c>
+    </row>
+    <row r="1545">
+      <c r="A1545" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1545" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1545" t="inlineStr">
+        <is>
+          <t>Anggota DPR Minta Peradilan Andrie Yunus Dilakukan Terbuka</t>
+        </is>
+      </c>
+      <c r="D1545" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098980/anggota-dpr-minta-peradilan-andrie-yunus-dilakukan-terbuka</t>
+        </is>
+      </c>
+    </row>
+    <row r="1546">
+      <c r="A1546" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1546" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1546" t="inlineStr">
+        <is>
+          <t>PDIP: Kolonialisme Belum Berakhir</t>
+        </is>
+      </c>
+      <c r="D1546" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2098970/pdip-kolonialisme-belum-berakhir</t>
+        </is>
+      </c>
+    </row>
+    <row r="1547">
+      <c r="A1547" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1547" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1547" t="inlineStr">
+        <is>
+          <t>Govt removes 4.1 million illegal content items to secure digital space</t>
+        </is>
+      </c>
+      <c r="D1547" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412799/govt-removes-41-million-illegal-content-items-to-secure-digital-space</t>
+        </is>
+      </c>
+    </row>
+    <row r="1548">
+      <c r="A1548" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1548" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1548" t="inlineStr">
+        <is>
+          <t>Megawati proposes Bandung Conference 2.0 to counter global tensions</t>
+        </is>
+      </c>
+      <c r="D1548" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412797/megawati-proposes-bandung-conference-20-to-counter-global-tensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="1549">
+      <c r="A1549" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1549" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1549" t="inlineStr">
+        <is>
+          <t>Indonesia welcomes Lebanon-Israel ceasefire, calls for permanent peace</t>
+        </is>
+      </c>
+      <c r="D1549" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412795/indonesia-welcomes-lebanon-israel-ceasefire-calls-for-permanent-peace</t>
+        </is>
+      </c>
+    </row>
+    <row r="1550">
+      <c r="A1550" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1550" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1550" t="inlineStr">
+        <is>
+          <t>All eight victims of West Kalimantan helicopter crash identified</t>
+        </is>
+      </c>
+      <c r="D1550" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412791/all-eight-victims-of-west-kalimantan-helicopter-crash-identified</t>
+        </is>
+      </c>
+    </row>
+    <row r="1551">
+      <c r="A1551" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1551" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1551" t="inlineStr">
+        <is>
+          <t>Minister highlights architecture's vital role in disaster mitigation</t>
+        </is>
+      </c>
+      <c r="D1551" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412787/minister-highlights-architectures-vital-role-in-disaster-mitigation</t>
+        </is>
+      </c>
+    </row>
+    <row r="1552">
+      <c r="A1552" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1552" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1552" t="inlineStr">
+        <is>
+          <t>Minister encourages downstreaming and food research on campus</t>
+        </is>
+      </c>
+      <c r="D1552" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412784/minister-encourages-downstreaming-and-food-research-on-campus</t>
+        </is>
+      </c>
+    </row>
+    <row r="1553">
+      <c r="A1553" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1553" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1553" t="inlineStr">
+        <is>
+          <t>Minister urges inclusive, protective services for Hajj pilgrims</t>
+        </is>
+      </c>
+      <c r="D1553" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412781/minister-urges-inclusive-protective-services-for-hajj-pilgrims</t>
+        </is>
+      </c>
+    </row>
+    <row r="1554">
+      <c r="A1554" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1554" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1554" t="inlineStr">
+        <is>
+          <t>Minister urges SPPGs to prioritize nutrition in free meals program</t>
+        </is>
+      </c>
+      <c r="D1554" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412777/minister-urges-sppgs-to-prioritize-nutrition-in-free-meals-program</t>
+        </is>
+      </c>
+    </row>
+    <row r="1555">
+      <c r="A1555" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1555" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1555" t="inlineStr">
+        <is>
+          <t>Govt bolsters higher ed partnerships to spur economic transformation</t>
+        </is>
+      </c>
+      <c r="D1555" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412775/govt-bolsters-higher-ed-partnerships-to-spur-economic-transformation</t>
+        </is>
+      </c>
+    </row>
+    <row r="1556">
+      <c r="A1556" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1556" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1556" t="inlineStr">
+        <is>
+          <t>Prabowo urges regional lawmakers to be 'patriots' for national goals</t>
+        </is>
+      </c>
+      <c r="D1556" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412772/prabowo-urges-regional-lawmakers-to-be-patriots-for-national-goals</t>
+        </is>
+      </c>
+    </row>
+    <row r="1557">
+      <c r="A1557" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1557" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1557" t="inlineStr">
+        <is>
+          <t>Higher Education Ministry, BRIN to strengthen research roadmap</t>
+        </is>
+      </c>
+      <c r="D1557" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412771/higher-education-ministry-brin-to-strengthen-research-roadmap</t>
+        </is>
+      </c>
+    </row>
+    <row r="1558">
+      <c r="A1558" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1558" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1558" t="inlineStr">
+        <is>
+          <t>Immigration arrests British national intimidating residents in Bali</t>
+        </is>
+      </c>
+      <c r="D1558" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412768/immigration-arrests-british-national-intimidating-residents-in-bali</t>
+        </is>
+      </c>
+    </row>
+    <row r="1559">
+      <c r="A1559" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1559" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1559" t="inlineStr">
+        <is>
+          <t>Ministries push for collaboration on tech-based waste management</t>
+        </is>
+      </c>
+      <c r="D1559" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412767/ministries-push-for-collaboration-on-tech-based-waste-management</t>
+        </is>
+      </c>
+    </row>
+    <row r="1560">
+      <c r="A1560" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1560" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1560" t="inlineStr">
+        <is>
+          <t>Indonesia, Austria seek to expand education, research ties</t>
+        </is>
+      </c>
+      <c r="D1560" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412765/indonesia-austria-seek-to-expand-education-research-ties</t>
+        </is>
+      </c>
+    </row>
+    <row r="1561">
+      <c r="A1561" t="inlineStr">
+        <is>
+          <t>Sunday, 19 April 2026</t>
+        </is>
+      </c>
+      <c r="B1561" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1561" t="inlineStr">
+        <is>
+          <t>Bapanas ensures soybean supply sufficient for tofu, tempeh producers</t>
+        </is>
+      </c>
+      <c r="D1561" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412761/bapanas-ensures-soybean-supply-sufficient-for-tofu-tempeh-producers</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1501"/>
+  <autoFilter ref="A1:D1561"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -34973,6 +36293,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1499" r:id="rId1498"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1500" r:id="rId1499"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1501" r:id="rId1500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1502" r:id="rId1501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1503" r:id="rId1502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1504" r:id="rId1503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1505" r:id="rId1504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1506" r:id="rId1505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1507" r:id="rId1506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1508" r:id="rId1507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1509" r:id="rId1508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1510" r:id="rId1509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1511" r:id="rId1510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1512" r:id="rId1511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1513" r:id="rId1512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1514" r:id="rId1513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1515" r:id="rId1514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1516" r:id="rId1515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1517" r:id="rId1516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1518" r:id="rId1517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1519" r:id="rId1518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1520" r:id="rId1519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1521" r:id="rId1520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1522" r:id="rId1521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1523" r:id="rId1522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1524" r:id="rId1523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1525" r:id="rId1524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1526" r:id="rId1525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1527" r:id="rId1526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1528" r:id="rId1527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1529" r:id="rId1528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1530" r:id="rId1529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1531" r:id="rId1530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1532" r:id="rId1531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1533" r:id="rId1532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1534" r:id="rId1533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1535" r:id="rId1534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1536" r:id="rId1535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1537" r:id="rId1536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1538" r:id="rId1537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1539" r:id="rId1538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1540" r:id="rId1539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1541" r:id="rId1540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1542" r:id="rId1541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1543" r:id="rId1542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1544" r:id="rId1543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1545" r:id="rId1544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1546" r:id="rId1545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1547" r:id="rId1546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1548" r:id="rId1547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1549" r:id="rId1548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1550" r:id="rId1549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1551" r:id="rId1550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1552" r:id="rId1551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1553" r:id="rId1552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1554" r:id="rId1553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1555" r:id="rId1554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1556" r:id="rId1555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1557" r:id="rId1556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1558" r:id="rId1557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1559" r:id="rId1558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1560" r:id="rId1559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1561" r:id="rId1560"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-19
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1561</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1621</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1561"/>
+  <dimension ref="A1:D1621"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -34790,8 +34790,1328 @@
         </is>
       </c>
     </row>
+    <row r="1562">
+      <c r="A1562" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1562" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1562" t="inlineStr">
+        <is>
+          <t>Tes Ketajaman Otak dan Saraf Mata! Hitungnya Sih Gampang, Soalnya Belum Tentu Kelihatan</t>
+        </is>
+      </c>
+      <c r="D1562" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/asah-otak/d-8451251/tes-ketajaman-otak-dan-saraf-mata-hitungnya-sih-gampang-soalnya-belum-tentu-kelihatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1563">
+      <c r="A1563" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1563" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1563" t="inlineStr">
+        <is>
+          <t>Video: Arah Tumbuh Bulu Mata Kebalik, Normal atau Kelainan?</t>
+        </is>
+      </c>
+      <c r="D1563" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/detiktv/d-8451659/video-arah-tumbuh-bulu-mata-kebalik-normal-atau-kelainan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1564">
+      <c r="A1564" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1564" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1564" t="inlineStr">
+        <is>
+          <t>Sayur dan Buah Ini Mengandung Mikroplastik Tinggi, Riset Ungkap Temuannya</t>
+        </is>
+      </c>
+      <c r="D1564" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8451627/sayur-dan-buah-ini-mengandung-mikroplastik-tinggi-riset-ungkap-temuannya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1565">
+      <c r="A1565" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1565" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1565" t="inlineStr">
+        <is>
+          <t>Potret Makanan UPF Bikin Paha Manusia Mirip Daging Berlemak, Seserius Ini Efeknya</t>
+        </is>
+      </c>
+      <c r="D1565" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8451543/potret-makanan-upf-bikin-paha-manusia-mirip-daging-berlemak-seserius-ini-efeknya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1566">
+      <c r="A1566" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1566" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1566" t="inlineStr">
+        <is>
+          <t>Lengkap! Ini Daftar Harga Gas 12 Kg Terbaru</t>
+        </is>
+      </c>
+      <c r="D1566" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8451389/lengkap-ini-daftar-harga-gas-12-kg-terbaru</t>
+        </is>
+      </c>
+    </row>
+    <row r="1567">
+      <c r="A1567" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1567" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1567" t="inlineStr">
+        <is>
+          <t>Video: Tubuh "Lupa" Gravitasi, Astronaut Artemis II Harus Belajar Jalan Lagi</t>
+        </is>
+      </c>
+      <c r="D1567" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260420-260420001/video-tubuh-lupa-gravitasi-astronaut-artemis-ii-harus-belajar-jalan-lagi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1568">
+      <c r="A1568" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1568" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1568" t="inlineStr">
+        <is>
+          <t>Man City Bungkam Arsenal 2-1, Persaingan Gelar EPL Memanas!</t>
+        </is>
+      </c>
+      <c r="D1568" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8451881/man-city-bungkam-arsenal-2-1-persaingan-gelar-epl-memanas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1569">
+      <c r="A1569" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1569" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1569" t="inlineStr">
+        <is>
+          <t>Juventus Vs Bologna: Bianconeri Menang 2-0</t>
+        </is>
+      </c>
+      <c r="D1569" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-italia/d-8451894/juventus-vs-bologna-bianconeri-menang-2-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="1570">
+      <c r="A1570" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1570" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1570" t="inlineStr">
+        <is>
+          <t>Al Wasl Vs Al Nassr: Menang 4-0, Ronaldo Cs ke Semifinal ACL 2</t>
+        </is>
+      </c>
+      <c r="D1570" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8451855/al-wasl-vs-al-nassr-menang-4-0-ronaldo-cs-ke-semifinal-acl-2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1571">
+      <c r="A1571" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1571" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1571" t="inlineStr">
+        <is>
+          <t>Video: Melihat Progres Pembangunan Sekolah Rakyat di Kedung Cowek Surabaya</t>
+        </is>
+      </c>
+      <c r="D1571" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260419-260419074/video-melihat-progres-pembangunan-sekolah-rakyat-di-kedung-cowek-surabaya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1572">
+      <c r="A1572" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1572" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1572" t="inlineStr">
+        <is>
+          <t>Video: Penembakan Massal-Penyanderaan Terjadi di Ukraina, 6 Tewas</t>
+        </is>
+      </c>
+      <c r="D1572" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260419-260419014/video-penembakan-massal-penyanderaan-terjadi-di-ukraina-6-tewas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1573">
+      <c r="A1573" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1573" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1573" t="inlineStr">
+        <is>
+          <t>Video Top 5: Label Nutri-Level Dirilis hingga D4vd Ditangkap soal Pembunuhan</t>
+        </is>
+      </c>
+      <c r="D1573" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260419-260419002/video-top-5-label-nutri-level-dirilis-hingga-d4vd-ditangkap-soal-pembunuhan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1574">
+      <c r="A1574" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1574" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1574" t="inlineStr">
+        <is>
+          <t>Pakistan Perketat Keamanan di Islamabad Jelang Perundingan AS dan Iran</t>
+        </is>
+      </c>
+      <c r="D1574" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8451893/pakistan-perketat-keamanan-di-islamabad-jelang-perundingan-as-dan-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="1575">
+      <c r="A1575" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1575" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1575" t="inlineStr">
+        <is>
+          <t>Video Fasilitas Nabawi: Ribuan Mushaf Indah di Setiap Sudut Masjid</t>
+        </is>
+      </c>
+      <c r="D1575" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260419-260419119/video-fasilitas-nabawi-ribuan-mushaf-indah-di-setiap-sudut-masjid</t>
+        </is>
+      </c>
+    </row>
+    <row r="1576">
+      <c r="A1576" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1576" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1576" t="inlineStr">
+        <is>
+          <t>Warga Sulut Tewas Diduga Keracunan Usai Makan Kepiting, 4 Lainnya Dirawat</t>
+        </is>
+      </c>
+      <c r="D1576" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8451891/warga-sulut-tewas-diduga-keracunan-usai-makan-kepiting-4-lainnya-dirawat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1577">
+      <c r="A1577" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1577" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1577" t="inlineStr">
+        <is>
+          <t>Jajanan Indonesia Terbaik Versi TasteAtlas 2026</t>
+        </is>
+      </c>
+      <c r="D1577" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1924717/jajanan-indonesia-terbaik-versi-tasteatlas-2026?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1578">
+      <c r="A1578" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1578" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1578" t="inlineStr">
+        <is>
+          <t>Monumen Garuda, Mengenang Pengorbanan TNI di Kamboja</t>
+        </is>
+      </c>
+      <c r="D1578" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/monumen-garuda-mengenang-pengorbanan-tni-di-kamboja?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1579">
+      <c r="A1579" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1579" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1579" t="inlineStr">
+        <is>
+          <t>Genjot Serapan Tenaga Kerja, Menaker Targetkan 70.000 Peserta Pelatihan Vokasi Nasional 2026</t>
+        </is>
+      </c>
+      <c r="D1579" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/19/20352151/genjot-serapan-tenaga-kerja-menaker-targetkan-70000-peserta-pelatihan-vokasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1580">
+      <c r="A1580" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1580" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1580" t="inlineStr">
+        <is>
+          <t>Sukses Digelar, wondr Kemala Run 2026 Dongkrak Ekonomi Bali dengan Libatkan UMKM</t>
+        </is>
+      </c>
+      <c r="D1580" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/19/12121461/sukses-digelar-wondr-kemala-run-2026-dongkrak-ekonomi-bali-dengan-libatkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1581">
+      <c r="A1581" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1581" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1581" t="inlineStr">
+        <is>
+          <t>Ketua Harian Dekranas Dorong Penguatan Pemasaran dan Kreativitas Tenun di Belu</t>
+        </is>
+      </c>
+      <c r="D1581" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/19/10501571/ketua-harian-dekranas-dorong-penguatan-pemasaran-dan-kreativitas-tenun-di</t>
+        </is>
+      </c>
+    </row>
+    <row r="1582">
+      <c r="A1582" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1582" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1582" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D1582" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1583">
+      <c r="A1583" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1583" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1583" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D1583" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1584">
+      <c r="A1584" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1584" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1584" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D1584" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1585">
+      <c r="A1585" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1585" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1585" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D1585" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1586">
+      <c r="A1586" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1586" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1586" t="inlineStr">
+        <is>
+          <t>Kenaikan BBM Nonsubsidi Disebut Bisa Picu Efek ke Sektor Pangan</t>
+        </is>
+      </c>
+      <c r="D1586" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1924687/kenaikan-bbm-nonsubsidi-disebut-bisa-picu-efek-ke-sektor-pangan?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1587">
+      <c r="A1587" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1587" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1587" t="inlineStr">
+        <is>
+          <t>Menyaksikan Layar Perak, Ludruk, dan Ketoprak Berbagi Panggung di "Misbar" Karto Dasil</t>
+        </is>
+      </c>
+      <c r="D1587" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/kaekaha.4277/69e0769eed6415120f61f492/menyaksikan-layar-perak-dan-kesenian-tradisional-berebut-panggung-misbar-karto-dasil-di-kaki-gunung-lawu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1588">
+      <c r="A1588" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1588" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1588" t="inlineStr">
+        <is>
+          <t>Mencoba Okonomiyaki di Yokohama Sky Building, Lumer dengan 5 Jenis Keju</t>
+        </is>
+      </c>
+      <c r="D1588" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5848/mencoba-okonomiyaki-di-yokohama-sky-building-lumer-dengan-5-jenis-keju</t>
+        </is>
+      </c>
+    </row>
+    <row r="1589">
+      <c r="A1589" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1589" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1589" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1589" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1590">
+      <c r="A1590" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1590" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1590" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1590" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1591">
+      <c r="A1591" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1591" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1591" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Penampakan Langka Bumi dan Bulan yang Dipotret Kru Artemis II NASA</t>
+        </is>
+      </c>
+      <c r="D1591" s="2" t="inlineStr">
+        <is>
+          <t>https://tekno.kompas.com/read/2026/04/09/18020027/berita-foto-penampakan-langka-bumi-dan-bulan-yang-dipotret-kru-artemis-ii-nasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1592">
+      <c r="A1592" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1592" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1592" t="inlineStr">
+        <is>
+          <t>Melatih Masa Depan Digital Anak Muda Jailolo</t>
+        </is>
+      </c>
+      <c r="D1592" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099163/melatih-masa-depan-digital-anak-muda-jailolo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1593">
+      <c r="A1593" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1593" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1593" t="inlineStr">
+        <is>
+          <t>Pemkot Semarang Matangkan Persiapan MTQ Nasional 2026</t>
+        </is>
+      </c>
+      <c r="D1593" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099156/pemkot-semarang-matangkan-persiapan-mtq-nasional-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1594">
+      <c r="A1594" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1594" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1594" t="inlineStr">
+        <is>
+          <t>Mensos Tinjau Kesiapan Sekolah Rakyat di LAN</t>
+        </is>
+      </c>
+      <c r="D1594" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099151/mensos-tinjau-kesiapan-sekolah-rakyat-di-lan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1595">
+      <c r="A1595" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1595" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1595" t="inlineStr">
+        <is>
+          <t>Mensos Tinjau Kesiapan STIP Jakarta untuk Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="D1595" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099148/mensos-tinjau-kesiapan-stip-jakarta-untuk-sekolah-rakyat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1596">
+      <c r="A1596" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1596" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1596" t="inlineStr">
+        <is>
+          <t>Projo Mendebat Pernyataan Jusuf Kalla soal Jokowi</t>
+        </is>
+      </c>
+      <c r="D1596" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099145/projo-mendebat-pernyataan-jusuf-kalla-soal-jokowi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1597">
+      <c r="A1597" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1597" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1597" t="inlineStr">
+        <is>
+          <t>Golkar Imbau Kader Tak Terpancing Kasus Penusukan Nus Kei</t>
+        </is>
+      </c>
+      <c r="D1597" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099142/golkar-imbau-kader-tak-terpancing-kasus-penusukan-nus-kei</t>
+        </is>
+      </c>
+    </row>
+    <row r="1598">
+      <c r="A1598" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1598" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1598" t="inlineStr">
+        <is>
+          <t>Wali Kota Semarang Pastikan Kirab Budaya KH Sholeh Darat Tetap Berjalan</t>
+        </is>
+      </c>
+      <c r="D1598" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099141/wali-kota-semarang-pastikan-kirab-budaya-kh-sholeh-darat-tetap-berjalan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1599">
+      <c r="A1599" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1599" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1599" t="inlineStr">
+        <is>
+          <t>Penjelasan TNI AL soal Kapal Perang AS di Selat Malaka</t>
+        </is>
+      </c>
+      <c r="D1599" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099138/penjelasan-tni-al-soal-kapal-perang-as-di-selat-malaka</t>
+        </is>
+      </c>
+    </row>
+    <row r="1600">
+      <c r="A1600" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1600" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1600" t="inlineStr">
+        <is>
+          <t>Retret DPRD Rampung, Lemhannas Harap Pusat-Daerah Selaras</t>
+        </is>
+      </c>
+      <c r="D1600" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099131/retret-dprd-rampung-lemhannas-harap-pusat-daerah-selaras</t>
+        </is>
+      </c>
+    </row>
+    <row r="1601">
+      <c r="A1601" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1601" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1601" t="inlineStr">
+        <is>
+          <t>Wali Kota Semarang Targetkan Perwal BOP RT Rampung dalam Tiga Minggu</t>
+        </is>
+      </c>
+      <c r="D1601" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099124/wali-kota-semarang-targetkan-perwal-bop-rt-rampung-dalam-tiga-minggu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1602">
+      <c r="A1602" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1602" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1602" t="inlineStr">
+        <is>
+          <t>TNI AL Benarkan Ada Kapal Perang AS di Selat Malaka</t>
+        </is>
+      </c>
+      <c r="D1602" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099111/tni-al-benarkan-ada-kapal-perang-as-di-selat-malaka</t>
+        </is>
+      </c>
+    </row>
+    <row r="1603">
+      <c r="A1603" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1603" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1603" t="inlineStr">
+        <is>
+          <t>Harga BBM Naik, Anggota DPR: Pemerintah Beri Harapan Palsu</t>
+        </is>
+      </c>
+      <c r="D1603" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099105/harga-bbm-naik-anggota-dpr-pemerintah-beri-harapan-palsu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1604">
+      <c r="A1604" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1604" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1604" t="inlineStr">
+        <is>
+          <t>Pendatang yang Masuk Jakarta Setelah Lebaran Capai 7.911 Jiwa</t>
+        </is>
+      </c>
+      <c r="D1604" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099104/pendatang-yang-masuk-jakarta-setelah-lebaran-capai-7-911-jiwa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1605">
+      <c r="A1605" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1605" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1605" t="inlineStr">
+        <is>
+          <t>PSI Menilai Pernyataan Jusuf Kalla tentang Jokowi Terlalu Emosional</t>
+        </is>
+      </c>
+      <c r="D1605" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099102/psi-menilai-pernyataan-jusuf-kalla-tentang-jokowi-terlalu-emosional</t>
+        </is>
+      </c>
+    </row>
+    <row r="1606">
+      <c r="A1606" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1606" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1606" t="inlineStr">
+        <is>
+          <t>Nelayan Temukan Benda Menyerupai Rudal di Laut Sulawesi</t>
+        </is>
+      </c>
+      <c r="D1606" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099099/nelayan-temukan-benda-menyerupai-rudal-di-laut-sulawesi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1607">
+      <c r="A1607" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1607" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1607" t="inlineStr">
+        <is>
+          <t>Free meals program serves 62 million, creates over 1 million jobs</t>
+        </is>
+      </c>
+      <c r="D1607" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412856/free-meals-program-serves-62-million-creates-over-1-million-jobs</t>
+        </is>
+      </c>
+    </row>
+    <row r="1608">
+      <c r="A1608" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1608" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1608" t="inlineStr">
+        <is>
+          <t>Indonesia raises non-subsidized LPG prices up to 18 percent</t>
+        </is>
+      </c>
+      <c r="D1608" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412853/indonesia-raises-non-subsidized-lpg-prices-up-to-18-percent</t>
+        </is>
+      </c>
+    </row>
+    <row r="1609">
+      <c r="A1609" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1609" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1609" t="inlineStr">
+        <is>
+          <t>Deputy minister urges waste sorting as open dumping ban nears</t>
+        </is>
+      </c>
+      <c r="D1609" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412849/deputy-minister-urges-waste-sorting-as-open-dumping-ban-nears</t>
+        </is>
+      </c>
+    </row>
+    <row r="1610">
+      <c r="A1610" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1610" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1610" t="inlineStr">
+        <is>
+          <t>Indonesia to stop diesel imports, shift to palm oil fuel</t>
+        </is>
+      </c>
+      <c r="D1610" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412845/indonesia-to-stop-diesel-imports-shift-to-palm-oil-fuel</t>
+        </is>
+      </c>
+    </row>
+    <row r="1611">
+      <c r="A1611" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1611" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1611" t="inlineStr">
+        <is>
+          <t>Leadership retreat to help align central-region policies: Lemhannas</t>
+        </is>
+      </c>
+      <c r="D1611" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412844/leadership-retreat-to-help-align-central-region-policies-lemhannas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1612">
+      <c r="A1612" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1612" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1612" t="inlineStr">
+        <is>
+          <t>Bandung Spirit still a moral compass in uncertain world: Minister</t>
+        </is>
+      </c>
+      <c r="D1612" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412840/bandung-spirit-still-a-moral-compass-in-uncertain-world-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="1613">
+      <c r="A1613" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1613" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1613" t="inlineStr">
+        <is>
+          <t>Social solidarity key in achieving demographic bonus: Ministry</t>
+        </is>
+      </c>
+      <c r="D1613" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412836/social-solidarity-key-in-achieving-demographic-bonus-ministry</t>
+        </is>
+      </c>
+    </row>
+    <row r="1614">
+      <c r="A1614" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1614" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1614" t="inlineStr">
+        <is>
+          <t>Some 1,000 dancers set record with 34-province dance medley</t>
+        </is>
+      </c>
+      <c r="D1614" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412832/some-1000-dancers-set-record-with-34-province-dance-medley</t>
+        </is>
+      </c>
+    </row>
+    <row r="1615">
+      <c r="A1615" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1615" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1615" t="inlineStr">
+        <is>
+          <t>Indonesia condemns Israel at IPU Forum over Gaza and Lebanon strikes</t>
+        </is>
+      </c>
+      <c r="D1615" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412828/indonesia-condemns-israel-at-ipu-forum-over-gaza-and-lebanon-strikes</t>
+        </is>
+      </c>
+    </row>
+    <row r="1616">
+      <c r="A1616" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1616" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1616" t="inlineStr">
+        <is>
+          <t>Two Pertamina tankers remain stuck amid renewed Hormuz curbs</t>
+        </is>
+      </c>
+      <c r="D1616" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412827/two-pertamina-tankers-remain-stuck-amid-renewed-hormuz-curbs</t>
+        </is>
+      </c>
+    </row>
+    <row r="1617">
+      <c r="A1617" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1617" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1617" t="inlineStr">
+        <is>
+          <t>Indonesia exports 300 tonnes of kratom monthly amid rising demand</t>
+        </is>
+      </c>
+      <c r="D1617" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412823/indonesia-exports-300-tonnes-of-kratom-monthly-amid-rising-demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="1618">
+      <c r="A1618" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1618" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1618" t="inlineStr">
+        <is>
+          <t>Indonesia eyes 3.67 percent national GDP boost through AI adoption</t>
+        </is>
+      </c>
+      <c r="D1618" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412820/indonesia-eyes-367-percent-national-gdp-boost-through-ai-adoption</t>
+        </is>
+      </c>
+    </row>
+    <row r="1619">
+      <c r="A1619" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1619" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1619" t="inlineStr">
+        <is>
+          <t>Indonesia accelerates disaster recovery across Sumatra</t>
+        </is>
+      </c>
+      <c r="D1619" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412817/indonesia-accelerates-disaster-recovery-across-sumatra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1620">
+      <c r="A1620" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1620" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1620" t="inlineStr">
+        <is>
+          <t>Minister urges cultural preservation, highlights keris heritage</t>
+        </is>
+      </c>
+      <c r="D1620" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412816/minister-urges-cultural-preservation-highlights-keris-heritage</t>
+        </is>
+      </c>
+    </row>
+    <row r="1621">
+      <c r="A1621" t="inlineStr">
+        <is>
+          <t>Monday, 20 April 2026</t>
+        </is>
+      </c>
+      <c r="B1621" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1621" t="inlineStr">
+        <is>
+          <t>Indonesia's rice reserves hit record as President makes spot check</t>
+        </is>
+      </c>
+      <c r="D1621" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/412813/indonesias-rice-reserves-hit-record-as-president-makes-spot-check</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1561"/>
+  <autoFilter ref="A1:D1621"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -36353,6 +37673,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1559" r:id="rId1558"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1560" r:id="rId1559"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1561" r:id="rId1560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1562" r:id="rId1561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1563" r:id="rId1562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1564" r:id="rId1563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1565" r:id="rId1564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1566" r:id="rId1565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1567" r:id="rId1566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1568" r:id="rId1567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1569" r:id="rId1568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1570" r:id="rId1569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1571" r:id="rId1570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1572" r:id="rId1571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1573" r:id="rId1572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1574" r:id="rId1573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1575" r:id="rId1574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1576" r:id="rId1575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1577" r:id="rId1576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1578" r:id="rId1577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1579" r:id="rId1578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1580" r:id="rId1579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1581" r:id="rId1580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1582" r:id="rId1581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1583" r:id="rId1582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1584" r:id="rId1583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1585" r:id="rId1584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1586" r:id="rId1585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1587" r:id="rId1586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1588" r:id="rId1587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1589" r:id="rId1588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1590" r:id="rId1589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1591" r:id="rId1590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1592" r:id="rId1591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1593" r:id="rId1592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1594" r:id="rId1593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1595" r:id="rId1594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1596" r:id="rId1595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1597" r:id="rId1596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1598" r:id="rId1597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1599" r:id="rId1598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1600" r:id="rId1599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1601" r:id="rId1600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1602" r:id="rId1601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1603" r:id="rId1602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1604" r:id="rId1603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1605" r:id="rId1604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1606" r:id="rId1605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1607" r:id="rId1606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1608" r:id="rId1607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1609" r:id="rId1608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1610" r:id="rId1609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1611" r:id="rId1610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1612" r:id="rId1611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1613" r:id="rId1612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1614" r:id="rId1613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1615" r:id="rId1614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1616" r:id="rId1615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1617" r:id="rId1616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1618" r:id="rId1617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1619" r:id="rId1618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1620" r:id="rId1619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1621" r:id="rId1620"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-20
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1621</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1681</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1621"/>
+  <dimension ref="A1:D1681"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -36110,8 +36110,1328 @@
         </is>
       </c>
     </row>
+    <row r="1622">
+      <c r="A1622" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1622" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1622" t="inlineStr">
+        <is>
+          <t>Kloter Pertama Haji 2026 Berangkat 22 April, Cek Jadwal Lengkapnya</t>
+        </is>
+      </c>
+      <c r="D1622" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8452605/kloter-pertama-haji-2026-berangkat-22-april-cek-jadwal-lengkapnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1623">
+      <c r="A1623" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1623" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1623" t="inlineStr">
+        <is>
+          <t>Gelang Haji 2026 Berisi Data Penting, Ini Detail yang Harus Kamu Tahu</t>
+        </is>
+      </c>
+      <c r="D1623" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jatim/berita/d-8453031/gelang-haji-2026-berisi-data-penting-ini-detail-yang-harus-kamu-tahu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1624">
+      <c r="A1624" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1624" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1624" t="inlineStr">
+        <is>
+          <t>Berapa Uang yang Perlu Dibawa Saat Haji? Ini Estimasi Idealnya</t>
+        </is>
+      </c>
+      <c r="D1624" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jatim/berita/d-8453041/berapa-uang-yang-perlu-dibawa-saat-haji-ini-estimasi-idealnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1625">
+      <c r="A1625" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1625" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1625" t="inlineStr">
+        <is>
+          <t>Besok Masuk Asrama, Ini Larangan Calon Jemaah Haji 2026 SelamaÂ Karantina</t>
+        </is>
+      </c>
+      <c r="D1625" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jatim/berita/d-8453002/besok-masuk-asrama-ini-larangan-calon-jemaah-haji-2026-selama-karantina</t>
+        </is>
+      </c>
+    </row>
+    <row r="1626">
+      <c r="A1626" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1626" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1626" t="inlineStr">
+        <is>
+          <t>Akomodasi Haji Madinah Siap 100%, Klinik Kesehatan Ada Tiap Sektor</t>
+        </is>
+      </c>
+      <c r="D1626" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8453453/akomodasi-haji-madinah-siap-100-klinik-kesehatan-ada-tiap-sektor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1627">
+      <c r="A1627" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1627" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1627" t="inlineStr">
+        <is>
+          <t>Kloter Pertama Haji 2026 Berangkat 22 April, Cek Jadwal Lengkapnya</t>
+        </is>
+      </c>
+      <c r="D1627" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8452605/kloter-pertama-haji-2026-berangkat-22-april-cek-jadwal-lengkapnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1628">
+      <c r="A1628" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1628" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1628" t="inlineStr">
+        <is>
+          <t>Video Tsunami 80 Cm Terjadi di Pelabuhan Kuji Usai Gempa M 7,4</t>
+        </is>
+      </c>
+      <c r="D1628" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8453537/video-tsunami-80-cm-terjadi-di-pelabuhan-kuji-usai-gempa-m-7-4</t>
+        </is>
+      </c>
+    </row>
+    <row r="1629">
+      <c r="A1629" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1629" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1629" t="inlineStr">
+        <is>
+          <t>Bahlil Sentil Orang Mampu Masih Beli BBM Subsidi: Apa Tidak Malu?</t>
+        </is>
+      </c>
+      <c r="D1629" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8453487/bahlil-sentil-orang-mampu-masih-beli-bbm-subsidi-apa-tidak-malu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1630">
+      <c r="A1630" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1630" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1630" t="inlineStr">
+        <is>
+          <t>Video Tempe Resmi Masuk Menu Utama Jemaah Haji</t>
+        </is>
+      </c>
+      <c r="D1630" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/video/d-8453446/video-tempe-resmi-masuk-menu-utama-jemaah-haji</t>
+        </is>
+      </c>
+    </row>
+    <row r="1631">
+      <c r="A1631" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1631" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1631" t="inlineStr">
+        <is>
+          <t>Video Bahlil Umumkan Penemuan Cadangan Gas 5 Triliun Kaki Kubik di Kutai</t>
+        </is>
+      </c>
+      <c r="D1631" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/detiktv/d-8453123/video-bahlil-umumkan-penemuan-cadangan-gas-5-triliun-kaki-kubik-di-kutai</t>
+        </is>
+      </c>
+    </row>
+    <row r="1632">
+      <c r="A1632" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1632" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1632" t="inlineStr">
+        <is>
+          <t>Tersengat Motor Listrik Badan Gizi Nasional</t>
+        </is>
+      </c>
+      <c r="D1632" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/investigasi/d-8453342/tersengat-motor-listrik-badan-gizi-nasional</t>
+        </is>
+      </c>
+    </row>
+    <row r="1633">
+      <c r="A1633" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1633" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1633" t="inlineStr">
+        <is>
+          <t>Rusak Puluhan Tahun, Andra Soni Ambil Alih Renovasi Jalan di Saketi Pandeglang</t>
+        </is>
+      </c>
+      <c r="D1633" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8453606/rusak-puluhan-tahun-andra-soni-ambil-alih-renovasi-jalan-di-saketi-pandeglang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1634">
+      <c r="A1634" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1634" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1634" t="inlineStr">
+        <is>
+          <t>Andra Soni Minta Kantor Pemprov Banten Hemat Energi</t>
+        </is>
+      </c>
+      <c r="D1634" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8448340/andra-soni-minta-kantor-pemprov-banten-hemat-energi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1635">
+      <c r="A1635" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1635" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1635" t="inlineStr">
+        <is>
+          <t>Andra Perkuat Pengawasan Usai Temuan Sisik Trenggiling Diselundupkan via Banten</t>
+        </is>
+      </c>
+      <c r="D1635" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8438179/andra-perkuat-pengawasan-usai-temuan-sisik-trenggiling-diselundupkan-via-banten</t>
+        </is>
+      </c>
+    </row>
+    <row r="1636">
+      <c r="A1636" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1636" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1636" t="inlineStr">
+        <is>
+          <t>Tok! DPR Setujui RUU PPRT Dibawa ke Paripurna</t>
+        </is>
+      </c>
+      <c r="D1636" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8453493/tok-dpr-setujui-ruu-pprt-dibawa-ke-paripurna</t>
+        </is>
+      </c>
+    </row>
+    <row r="1637">
+      <c r="A1637" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1637" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1637" t="inlineStr">
+        <is>
+          <t>KKB Baku Tembak dengan TNI di Puncak Papua, 22 Warga Sipil Jadi Korban</t>
+        </is>
+      </c>
+      <c r="D1637" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1924979/kkb-baku-tembak-dengan-tni-di-puncak-papua-22-warga-sipil-jadi-korban?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1638">
+      <c r="A1638" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1638" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1638" t="inlineStr">
+        <is>
+          <t>Iran Buka Selat Hormuz Sepenuhnya, AS Tetap Memblokade</t>
+        </is>
+      </c>
+      <c r="D1638" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/as-tetap-memblokade-meski-iran-telah-membuka-selat-hormuz-sepenuhnya?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1639">
+      <c r="A1639" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1639" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1639" t="inlineStr">
+        <is>
+          <t>KAI Tambah Fasilitas Ramah Perempuan, dari Kursi Khusus hingga 120 Ruang Laktasi</t>
+        </is>
+      </c>
+      <c r="D1639" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/20/19500091/kai-tambah-fasilitas-ramah-perempuan-dari-kursi-khusus-hingga-120-ruang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1640">
+      <c r="A1640" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1640" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1640" t="inlineStr">
+        <is>
+          <t>Manasik Haji jejak imani Hadirkan Persiapan Menyeluruh Raih Haji Mabrur</t>
+        </is>
+      </c>
+      <c r="D1640" s="2" t="inlineStr">
+        <is>
+          <t>https://travel.kompas.com/read/2026/04/20/192542827/manasik-haji-jejak-imani-hadirkan-persiapan-menyeluruh-raih-haji-mabrur</t>
+        </is>
+      </c>
+    </row>
+    <row r="1641">
+      <c r="A1641" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1641" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1641" t="inlineStr">
+        <is>
+          <t>Apresiasi Ibu di Hari Kartini, PAM JAYA Bagikan Toren Air Gratis</t>
+        </is>
+      </c>
+      <c r="D1641" s="2" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/04/20/18490061/apresiasi-ibu-di-hari-kartini-pam-jaya-bagikan-toren-air-gratis-</t>
+        </is>
+      </c>
+    </row>
+    <row r="1642">
+      <c r="A1642" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1642" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1642" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D1642" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1643">
+      <c r="A1643" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1643" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1643" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D1643" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1644">
+      <c r="A1644" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1644" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1644" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D1644" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1645">
+      <c r="A1645" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1645" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1645" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D1645" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1646">
+      <c r="A1646" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1646" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1646" t="inlineStr">
+        <is>
+          <t>Apa yang Dipelajari China dari Memantau Trump Berperang di Iran?</t>
+        </is>
+      </c>
+      <c r="D1646" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1924955/apa-yang-dipelajari-china-dari-memantau-trump-berperang-di-iran?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1647">
+      <c r="A1647" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1647" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1647" t="inlineStr">
+        <is>
+          <t>Refleksi Hari Ulang Tahun Mama</t>
+        </is>
+      </c>
+      <c r="D1647" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/listhiahr/69e4d17eed64154fd522b812/refleksi-hari-ulang-tahun-mama</t>
+        </is>
+      </c>
+    </row>
+    <row r="1648">
+      <c r="A1648" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1648" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1648" t="inlineStr">
+        <is>
+          <t>Gempa M 7,5 Guncang Jepang, Peringatan Tsunami Dikeluarkan</t>
+        </is>
+      </c>
+      <c r="D1648" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5852/gempa-m-7-5-guncang-jepang-peringatan-tsunami-dikeluarkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1649">
+      <c r="A1649" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1649" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1649" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1649" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1650">
+      <c r="A1650" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1650" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1650" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1650" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1651">
+      <c r="A1651" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1651" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1651" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Penampakan Langka Bumi dan Bulan yang Dipotret Kru Artemis II NASA</t>
+        </is>
+      </c>
+      <c r="D1651" s="2" t="inlineStr">
+        <is>
+          <t>https://tekno.kompas.com/read/2026/04/09/18020027/berita-foto-penampakan-langka-bumi-dan-bulan-yang-dipotret-kru-artemis-ii-nasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1652">
+      <c r="A1652" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1652" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1652" t="inlineStr">
+        <is>
+          <t>RUU PPRT Akan Disahkan di Rapat Paripurna Besok</t>
+        </is>
+      </c>
+      <c r="D1652" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099365/ruu-pprt-akan-disahkan-di-rapat-paripurna-besok</t>
+        </is>
+      </c>
+    </row>
+    <row r="1653">
+      <c r="A1653" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1653" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1653" t="inlineStr">
+        <is>
+          <t>Megawati Teringat Visi Besar Soekarno Saat Memperingati KAA</t>
+        </is>
+      </c>
+      <c r="D1653" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099363/megawati-teringat-visi-besar-soekarno-saat-memperingati-kaa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1654">
+      <c r="A1654" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1654" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1654" t="inlineStr">
+        <is>
+          <t>Sanksi Pelaku Kekerasan Seksual di UI Kewenangan Rektor</t>
+        </is>
+      </c>
+      <c r="D1654" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099360/sanksi-pelaku-kekerasan-seksual-di-ui-kewenangan-rektor</t>
+        </is>
+      </c>
+    </row>
+    <row r="1655">
+      <c r="A1655" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1655" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1655" t="inlineStr">
+        <is>
+          <t>Proyek Tanggul Laut Dibangun Bertahap dari Pantura Jawa</t>
+        </is>
+      </c>
+      <c r="D1655" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099357/proyek-tanggul-laut-dibangun-bertahap-dari-pantura-jawa</t>
+        </is>
+      </c>
+    </row>
+    <row r="1656">
+      <c r="A1656" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1656" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1656" t="inlineStr">
+        <is>
+          <t>Menkes: Daya Tular Campak Lebih Cepat dari Covid-19</t>
+        </is>
+      </c>
+      <c r="D1656" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099353/menkes-daya-tular-campak-lebih-cepat-dari-covid-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="1657">
+      <c r="A1657" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1657" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1657" t="inlineStr">
+        <is>
+          <t>IPB University Beri Pendampingan Korban Pelecehan Seksual</t>
+        </is>
+      </c>
+      <c r="D1657" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099351/ipb-university-beri-pendampingan-korban-pelecehan-seksual</t>
+        </is>
+      </c>
+    </row>
+    <row r="1658">
+      <c r="A1658" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1658" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1658" t="inlineStr">
+        <is>
+          <t>Pemprov Lampung Dorong RSUD BNH Jadi Green Hospital</t>
+        </is>
+      </c>
+      <c r="D1658" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099345/pemprov-lampung-dorong-rsud-bnh-jadi-green-hospital</t>
+        </is>
+      </c>
+    </row>
+    <row r="1659">
+      <c r="A1659" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1659" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1659" t="inlineStr">
+        <is>
+          <t>Ingatkan Visi Bung Karno, Megawati:Lemhannas Wahana Penggemblengan Pemimpin Progresif</t>
+        </is>
+      </c>
+      <c r="D1659" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099344/ingatkan-visi-bung-karno-megawatilemhannas-wahana-penggemblengan-pemimpin-progresif</t>
+        </is>
+      </c>
+    </row>
+    <row r="1660">
+      <c r="A1660" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1660" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1660" t="inlineStr">
+        <is>
+          <t>29 Ribu Jemaah Haji Asal Jawa Tengah Masuk Asrama Donohudan</t>
+        </is>
+      </c>
+      <c r="D1660" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099343/29-ribu-jemaah-haji-asal-jawa-tengah-masuk-asrama-donohudan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1661">
+      <c r="A1661" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1661" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1661" t="inlineStr">
+        <is>
+          <t>DPR Targetkan RUU PPRT Disahkan Selasa 21 April 2026</t>
+        </is>
+      </c>
+      <c r="D1661" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099340/dpr-targetkan-ruu-pprt-disahkan-selasa-21-april-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1662">
+      <c r="A1662" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1662" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1662" t="inlineStr">
+        <is>
+          <t>Pemprov Lampung Resmikan Indag Coffee Shop Lampung, Dorong Ekonomi Kreatif Daerah</t>
+        </is>
+      </c>
+      <c r="D1662" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099338/pemprov-lampung-resmikan-indag-coffee-shop-lampung-dorong-ekonomi-kreatif-daerah</t>
+        </is>
+      </c>
+    </row>
+    <row r="1663">
+      <c r="A1663" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1663" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1663" t="inlineStr">
+        <is>
+          <t>BPOM Belum Menguji Sampel MBG Akibat Keterbatasan Anggaran</t>
+        </is>
+      </c>
+      <c r="D1663" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099329/bpom-belum-menguji-sampel-mbg-akibat-keterbatasan-anggaran</t>
+        </is>
+      </c>
+    </row>
+    <row r="1664">
+      <c r="A1664" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1664" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1664" t="inlineStr">
+        <is>
+          <t>Kemendagri Usul Denda untuk E-KTP Hilang</t>
+        </is>
+      </c>
+      <c r="D1664" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099328/kemendagri-usul-denda-untuk-e-ktp-hilang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1665">
+      <c r="A1665" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1665" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1665" t="inlineStr">
+        <is>
+          <t>Bahlil: Golkar Beri Pendampingan Hukum Kasus Nus Kei</t>
+        </is>
+      </c>
+      <c r="D1665" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099327/bahlil-golkar-beri-pendampingan-hukum-kasus-nus-kei</t>
+        </is>
+      </c>
+    </row>
+    <row r="1666">
+      <c r="A1666" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1666" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1666" t="inlineStr">
+        <is>
+          <t>Prabowo Ingin Guru Besar Dilibatkan di Proyek Tanggul Laut</t>
+        </is>
+      </c>
+      <c r="D1666" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099321/prabowo-ingin-guru-besar-dilibatkan-di-proyek-tanggul-laut</t>
+        </is>
+      </c>
+    </row>
+    <row r="1667">
+      <c r="A1667" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1667" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1667" t="inlineStr">
+        <is>
+          <t>Asia-Pacific urged to uphold cooperation amid tensions</t>
+        </is>
+      </c>
+      <c r="D1667" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413057/asia-pacific-urged-to-uphold-cooperation-amid-tensions</t>
+        </is>
+      </c>
+    </row>
+    <row r="1668">
+      <c r="A1668" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1668" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1668" t="inlineStr">
+        <is>
+          <t>RI ready to become partner in establishing global AI governance: govt</t>
+        </is>
+      </c>
+      <c r="D1668" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413053/ri-ready-to-become-partner-in-establishing-global-ai-governance-govt</t>
+        </is>
+      </c>
+    </row>
+    <row r="1669">
+      <c r="A1669" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1669" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1669" t="inlineStr">
+        <is>
+          <t>Vice President calls Nabire Port as strategic regional economic hub</t>
+        </is>
+      </c>
+      <c r="D1669" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413052/vice-president-calls-nabire-port-as-strategic-regional-economic-hub</t>
+        </is>
+      </c>
+    </row>
+    <row r="1670">
+      <c r="A1670" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1670" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1670" t="inlineStr">
+        <is>
+          <t>IMF calls Indonesia a 'bright spot' in global economy: Purbaya</t>
+        </is>
+      </c>
+      <c r="D1670" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413049/imf-calls-indonesia-a-bright-spot-in-global-economy-purbaya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1671">
+      <c r="A1671" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1671" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1671" t="inlineStr">
+        <is>
+          <t>Indonesia relies on structural economic reforms to face energy crisis</t>
+        </is>
+      </c>
+      <c r="D1671" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413048/indonesia-relies-on-structural-economic-reforms-to-face-energy-crisis</t>
+        </is>
+      </c>
+    </row>
+    <row r="1672">
+      <c r="A1672" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1672" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1672" t="inlineStr">
+        <is>
+          <t>Indonesia ramps up communication to boost measles vaccination</t>
+        </is>
+      </c>
+      <c r="D1672" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413044/indonesia-ramps-up-communication-to-boost-measles-vaccination</t>
+        </is>
+      </c>
+    </row>
+    <row r="1673">
+      <c r="A1673" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1673" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1673" t="inlineStr">
+        <is>
+          <t>President Prabowo orders fast tracking of giant sea wall project</t>
+        </is>
+      </c>
+      <c r="D1673" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413040/president-prabowo-orders-fast-tracking-of-giant-sea-wall-project</t>
+        </is>
+      </c>
+    </row>
+    <row r="1674">
+      <c r="A1674" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1674" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1674" t="inlineStr">
+        <is>
+          <t>Indonesia detains three Pakistanis over migrant smuggling</t>
+        </is>
+      </c>
+      <c r="D1674" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413037/indonesia-detains-three-pakistanis-over-migrant-smuggling</t>
+        </is>
+      </c>
+    </row>
+    <row r="1675">
+      <c r="A1675" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1675" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1675" t="inlineStr">
+        <is>
+          <t>Subsidized LPG price to stay, supply above minimum: RI Govt</t>
+        </is>
+      </c>
+      <c r="D1675" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413033/subsidized-lpgprice-to-stay-supply-above-minimum-ri-govt</t>
+        </is>
+      </c>
+    </row>
+    <row r="1676">
+      <c r="A1676" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1676" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1676" t="inlineStr">
+        <is>
+          <t>Indonesia finds major gas reserves in East Kalimantan</t>
+        </is>
+      </c>
+      <c r="D1676" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413032/indonesia-finds-major-gas-reserves-in-east-kalimantan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1677">
+      <c r="A1677" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1677" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1677" t="inlineStr">
+        <is>
+          <t>Indonesia's home minister urges regions to brace for global shocks</t>
+        </is>
+      </c>
+      <c r="D1677" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413028/indonesias-home-ministerurges-regions-to-brace-for-global-shocks</t>
+        </is>
+      </c>
+    </row>
+    <row r="1678">
+      <c r="A1678" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1678" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1678" t="inlineStr">
+        <is>
+          <t>Indonesia's military denies role in Papua child death</t>
+        </is>
+      </c>
+      <c r="D1678" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413027/indonesias-military-denies-role-in-papua-child-death</t>
+        </is>
+      </c>
+    </row>
+    <row r="1679">
+      <c r="A1679" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1679" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1679" t="inlineStr">
+        <is>
+          <t>Indonesia's home minister warns of risks from rapid urbanisation</t>
+        </is>
+      </c>
+      <c r="D1679" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413023/indonesias-home-minister-warns-of-risks-from-rapid-urbanisation</t>
+        </is>
+      </c>
+    </row>
+    <row r="1680">
+      <c r="A1680" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1680" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1680" t="inlineStr">
+        <is>
+          <t>Indonesia expands inclusive school admissions system</t>
+        </is>
+      </c>
+      <c r="D1680" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413019/indonesia-expands-inclusive-school-admissions-system</t>
+        </is>
+      </c>
+    </row>
+    <row r="1681">
+      <c r="A1681" t="inlineStr">
+        <is>
+          <t>Tuesday, 21 April 2026</t>
+        </is>
+      </c>
+      <c r="B1681" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1681" t="inlineStr">
+        <is>
+          <t>Indonesia pushes inclusive education for all students</t>
+        </is>
+      </c>
+      <c r="D1681" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413017/indonesia-pushes-inclusive-education-for-all-students</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1621"/>
+  <autoFilter ref="A1:D1681"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -37733,6 +39053,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1619" r:id="rId1618"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1620" r:id="rId1619"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1621" r:id="rId1620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1622" r:id="rId1621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1623" r:id="rId1622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1624" r:id="rId1623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1625" r:id="rId1624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1626" r:id="rId1625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1627" r:id="rId1626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1628" r:id="rId1627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1629" r:id="rId1628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1630" r:id="rId1629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1631" r:id="rId1630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1632" r:id="rId1631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1633" r:id="rId1632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1634" r:id="rId1633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1635" r:id="rId1634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1636" r:id="rId1635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1637" r:id="rId1636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1638" r:id="rId1637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1639" r:id="rId1638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1640" r:id="rId1639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1641" r:id="rId1640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1642" r:id="rId1641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1643" r:id="rId1642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1644" r:id="rId1643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1645" r:id="rId1644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1646" r:id="rId1645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1647" r:id="rId1646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1648" r:id="rId1647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1649" r:id="rId1648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1650" r:id="rId1649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1651" r:id="rId1650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1652" r:id="rId1651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1653" r:id="rId1652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1654" r:id="rId1653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1655" r:id="rId1654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1656" r:id="rId1655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1657" r:id="rId1656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1658" r:id="rId1657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1659" r:id="rId1658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1660" r:id="rId1659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1661" r:id="rId1660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1662" r:id="rId1661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1663" r:id="rId1662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1664" r:id="rId1663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1665" r:id="rId1664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1666" r:id="rId1665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1667" r:id="rId1666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1668" r:id="rId1667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1669" r:id="rId1668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1670" r:id="rId1669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1671" r:id="rId1670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1672" r:id="rId1671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1673" r:id="rId1672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1674" r:id="rId1673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1675" r:id="rId1674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1676" r:id="rId1675"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1677" r:id="rId1676"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1678" r:id="rId1677"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1679" r:id="rId1678"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1680" r:id="rId1679"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1681" r:id="rId1680"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-21
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1681</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1741</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1681"/>
+  <dimension ref="A1:D1741"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -37430,8 +37430,1328 @@
         </is>
       </c>
     </row>
+    <row r="1682">
+      <c r="A1682" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1682" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1682" t="inlineStr">
+        <is>
+          <t>Kloter Pertama Haji 2026 Berangkat 22 April, Cek Jadwal Lengkapnya</t>
+        </is>
+      </c>
+      <c r="D1682" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8452605/kloter-pertama-haji-2026-berangkat-22-april-cek-jadwal-lengkapnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1683">
+      <c r="A1683" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1683" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1683" t="inlineStr">
+        <is>
+          <t>Kloter 1 Calon Haji Asal Jateng Terbang ke Arab Saudi Rabu Dini Hari</t>
+        </is>
+      </c>
+      <c r="D1683" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jateng/berita/d-8455296/kloter-1-calon-haji-asal-jateng-terbang-ke-arab-saudi-rabu-dini-hari</t>
+        </is>
+      </c>
+    </row>
+    <row r="1684">
+      <c r="A1684" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1684" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1684" t="inlineStr">
+        <is>
+          <t>Calon Haji Kloter Pertama Dilepas dari Embarkasi Yogyakarta</t>
+        </is>
+      </c>
+      <c r="D1684" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jogja/berita/d-8455242/calon-haji-kloter-pertama-dilepas-dari-embarkasi-yogyakarta</t>
+        </is>
+      </c>
+    </row>
+    <row r="1685">
+      <c r="A1685" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1685" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1685" t="inlineStr">
+        <is>
+          <t>Kartu Nusuk Hilang Saat Haji? Ini yang Harus Dilakukan</t>
+        </is>
+      </c>
+      <c r="D1685" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jatim/berita/d-8454318/kartu-nusuk-hilang-saat-haji-ini-yang-harus-dilakukan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1686">
+      <c r="A1686" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1686" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1686" t="inlineStr">
+        <is>
+          <t>Bocah 13 Tahun dari Magelang Jadi Calon Haji Gantikan Mendiang Ayah</t>
+        </is>
+      </c>
+      <c r="D1686" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jateng/berita/d-8455153/bocah-13-tahun-dari-magelang-jadi-calon-haji-gantikan-mendiang-ayah</t>
+        </is>
+      </c>
+    </row>
+    <row r="1687">
+      <c r="A1687" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1687" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1687" t="inlineStr">
+        <is>
+          <t>Kloter Pertama Haji 2026 Berangkat 22 April, Cek Jadwal Lengkapnya</t>
+        </is>
+      </c>
+      <c r="D1687" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8452605/kloter-pertama-haji-2026-berangkat-22-april-cek-jadwal-lengkapnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1688">
+      <c r="A1688" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1688" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1688" t="inlineStr">
+        <is>
+          <t>Ancaman Hukuman Rapper D4vd Usai Dakwaan Bunuh-Mutilasi Celeste Rivas Hernandez</t>
+        </is>
+      </c>
+      <c r="D1688" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/pop/trending/d-8454829/ancaman-hukuman-rapper-d4vd-usai-dakwaan-bunuh-mutilasi-celeste-rivas-hernandez</t>
+        </is>
+      </c>
+    </row>
+    <row r="1689">
+      <c r="A1689" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1689" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1689" t="inlineStr">
+        <is>
+          <t>Video Kepala BGN soal Pengadaan Motor Trail MBG: Untuk Laki-laki</t>
+        </is>
+      </c>
+      <c r="D1689" s="2" t="inlineStr">
+        <is>
+          <t>https://oto.detik.com/detiktv/d-8455010/video-kepala-bgn-soal-pengadaan-motor-trail-mbg-untuk-laki-laki</t>
+        </is>
+      </c>
+    </row>
+    <row r="1690">
+      <c r="A1690" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1690" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1690" t="inlineStr">
+        <is>
+          <t>Video Room Tour Hotel Jemaah Haji di Madinah</t>
+        </is>
+      </c>
+      <c r="D1690" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/video/d-8454313/video-room-tour-hotel-jemaah-haji-di-madinah</t>
+        </is>
+      </c>
+    </row>
+    <row r="1691">
+      <c r="A1691" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1691" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1691" t="inlineStr">
+        <is>
+          <t>Video DPR Tak Ingin Buru-buru Bahas RUU Pemilu, Takut Digugat ke MK</t>
+        </is>
+      </c>
+      <c r="D1691" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8454986/video-dpr-tak-ingin-buru-buru-bahas-ruu-pemilu-takut-digugat-ke-mk</t>
+        </is>
+      </c>
+    </row>
+    <row r="1692">
+      <c r="A1692" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1692" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1692" t="inlineStr">
+        <is>
+          <t>Video Tangis Bahagia Emak-emak ART Usai RUU PPRT Resmi Jadi UU</t>
+        </is>
+      </c>
+      <c r="D1692" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/detiktv/d-8454926/video-tangis-bahagia-emak-emak-art-usai-ruu-pprt-resmi-jadi-uu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1693">
+      <c r="A1693" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1693" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1693" t="inlineStr">
+        <is>
+          <t>Bawa Sampel Tanah dari Pertambangan di Gorontalo, 4 WN China Dideportasi</t>
+        </is>
+      </c>
+      <c r="D1693" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8455360/bawa-sampel-tanah-dari-pertambangan-di-gorontalo-4-wn-china-dideportasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1694">
+      <c r="A1694" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1694" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1694" t="inlineStr">
+        <is>
+          <t>Imigrasi Soetta Cegah 13 WNI Hendak Berangkat Haji Pakai Visa Kerja</t>
+        </is>
+      </c>
+      <c r="D1694" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8455250/imigrasi-soetta-cegah-13-wni-hendak-berangkat-haji-pakai-visa-kerja</t>
+        </is>
+      </c>
+    </row>
+    <row r="1695">
+      <c r="A1695" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1695" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1695" t="inlineStr">
+        <is>
+          <t>Imigrasi Tunda Keberangkatan 13 Calon Jemaah Pengguna Visa Non-haji</t>
+        </is>
+      </c>
+      <c r="D1695" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8453327/imigrasi-tunda-keberangkatan-13-calon-jemaah-pengguna-visa-non-haji</t>
+        </is>
+      </c>
+    </row>
+    <row r="1696">
+      <c r="A1696" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1696" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1696" t="inlineStr">
+        <is>
+          <t>Imigrasi Soetta Cegah 13 WNI Hendak Berangkat Haji Pakai Visa Kerja</t>
+        </is>
+      </c>
+      <c r="D1696" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8455250/imigrasi-soetta-cegah-13-wni-hendak-berangkat-haji-pakai-visa-kerja</t>
+        </is>
+      </c>
+    </row>
+    <row r="1697">
+      <c r="A1697" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1697" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1697" t="inlineStr">
+        <is>
+          <t>Trump Yakin AS Ada di Posisi Kuat, Klaim Iran Tak Punya Pilihan</t>
+        </is>
+      </c>
+      <c r="D1697" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1925225/trump-yakin-as-ada-di-posisi-kuat-klaim-iran-tak-punya-pilihan?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1698">
+      <c r="A1698" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1698" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1698" t="inlineStr">
+        <is>
+          <t>Perupa Subandi Giyanto Suguhkan Sunggingan “Nunggak Semi” di BBY</t>
+        </is>
+      </c>
+      <c r="D1698" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/perupa-subandi-giyanto-suguhkan-sunggingan-nunggak-semi-di-bby?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1699">
+      <c r="A1699" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1699" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1699" t="inlineStr">
+        <is>
+          <t>Indonesia Perkuat Daya Saing dan Ketahanan Ekonomi lewat Aksesi OECD</t>
+        </is>
+      </c>
+      <c r="D1699" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/21/21221851/indonesia-perkuat-daya-saing-dan-ketahanan-ekonomi-lewat-aksesi-oecd</t>
+        </is>
+      </c>
+    </row>
+    <row r="1700">
+      <c r="A1700" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1700" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1700" t="inlineStr">
+        <is>
+          <t>BPJPH Terima Hibah Lahan Pemprov Jateng untuk Pembangunan Gedung UPT Layanan Jaminan Produk Halal</t>
+        </is>
+      </c>
+      <c r="D1700" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/21/21061601/bpjph-terima-hibah-lahan-pemprov-jateng-untuk-pembangunan-gedung-upt-layanan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1701">
+      <c r="A1701" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1701" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1701" t="inlineStr">
+        <is>
+          <t>Pemkab Cilacap dan Polresta Teken MoU Perkuat Perlindungan Perempuan dan Anak</t>
+        </is>
+      </c>
+      <c r="D1701" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/21/205444378/pemkab-cilacap-dan-polresta-teken-mou-perkuat-perlindungan-perempuan-dan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1702">
+      <c r="A1702" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1702" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1702" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D1702" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1703">
+      <c r="A1703" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1703" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1703" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D1703" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1704">
+      <c r="A1704" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1704" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1704" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D1704" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1705">
+      <c r="A1705" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1705" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1705" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D1705" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1706">
+      <c r="A1706" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1706" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1706" t="inlineStr">
+        <is>
+          <t>Ambisi NASA Jelajahi Bulan, Pamerkan Roket Raksasa untuk Misi Artemis III</t>
+        </is>
+      </c>
+      <c r="D1706" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1925168/ambisi-nasa-jelajahi-bulan-pamerkan-roket-raksasa-untuk-misi-artemis-iii?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1707">
+      <c r="A1707" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1707" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1707" t="inlineStr">
+        <is>
+          <t>Perempuan yang Menulis dengan Bara</t>
+        </is>
+      </c>
+      <c r="D1707" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/syahrulchelsky/69e6d587ed641510ef251ad2/perempuan-yang-menulis-dengan-bara</t>
+        </is>
+      </c>
+    </row>
+    <row r="1708">
+      <c r="A1708" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1708" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1708" t="inlineStr">
+        <is>
+          <t>6 Orang Terluka Usai Gempa M 7,7 Guncang Jepang, Peringatan Megaquake Dikeluarkan</t>
+        </is>
+      </c>
+      <c r="D1708" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5858/6-orang-terluka-usai-gempa-m-7-7-guncang-jepang-peringatan-megaquake-dikeluarkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1709">
+      <c r="A1709" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1709" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1709" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1709" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1710">
+      <c r="A1710" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1710" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1710" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1710" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1711">
+      <c r="A1711" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1711" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1711" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Puing-puing Helikopter PK-CFX di Sekadau, Mesin Akhirnya Dievakuasi</t>
+        </is>
+      </c>
+      <c r="D1711" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/21/072900978/berita-foto--puing-puing-helikopter-pk-cfx-di-sekadau-mesin-akhirnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1712">
+      <c r="A1712" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1712" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1712" t="inlineStr">
+        <is>
+          <t>Prabowo Targetkan Pembangunan PLTS 17 Gigawatt Tahun Ini</t>
+        </is>
+      </c>
+      <c r="D1712" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099583/prabowo-targetkan-pembangunan-plts-17-gigawatt-tahun-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="1713">
+      <c r="A1713" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1713" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1713" t="inlineStr">
+        <is>
+          <t>Prabowo Menerima Telepon PM Australia, Bahas Pupuk Urea</t>
+        </is>
+      </c>
+      <c r="D1713" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099581/prabowo-menerima-telepon-pm-australia-bahas-pupuk-urea</t>
+        </is>
+      </c>
+    </row>
+    <row r="1714">
+      <c r="A1714" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1714" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1714" t="inlineStr">
+        <is>
+          <t>Tuntutan Massa yang Demo Gubernur di DPRD Kalimantan Timur</t>
+        </is>
+      </c>
+      <c r="D1714" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099580/tuntutan-massa-yang-demo-gubernur-di-dprd-kalimantan-timur</t>
+        </is>
+      </c>
+    </row>
+    <row r="1715">
+      <c r="A1715" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1715" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1715" t="inlineStr">
+        <is>
+          <t>Balita hingga Ibu Hamil Keracunan MBG di Demak</t>
+        </is>
+      </c>
+      <c r="D1715" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099566/balita-hingga-ibu-hamil-keracunan-mbg-di-demak</t>
+        </is>
+      </c>
+    </row>
+    <row r="1716">
+      <c r="A1716" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1716" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1716" t="inlineStr">
+        <is>
+          <t>Bantah Punya Dapur MBG, Uya Kuya Laporkan 10 Akun Medsos</t>
+        </is>
+      </c>
+      <c r="D1716" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099565/bantah-punya-dapur-mbg-uya-kuya-laporkan-10-akun-medsos</t>
+        </is>
+      </c>
+    </row>
+    <row r="1717">
+      <c r="A1717" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1717" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1717" t="inlineStr">
+        <is>
+          <t>BEM KM IPB Mengundurkan Diri dari Aliansi BEM SI</t>
+        </is>
+      </c>
+      <c r="D1717" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099562/bem-km-ipb-mengundurkan-diri-dari-aliansi-bem-si</t>
+        </is>
+      </c>
+    </row>
+    <row r="1718">
+      <c r="A1718" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1718" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1718" t="inlineStr">
+        <is>
+          <t>Prabowo Bahas Ekonomi dengan Luhut di Istana Merdeka</t>
+        </is>
+      </c>
+      <c r="D1718" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099561/prabowo-bahas-ekonomi-dengan-luhut-di-istana-merdeka</t>
+        </is>
+      </c>
+    </row>
+    <row r="1719">
+      <c r="A1719" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1719" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1719" t="inlineStr">
+        <is>
+          <t>Joki UTBK yang Tertangkap di Unesa Palsukan Ijazah Peserta</t>
+        </is>
+      </c>
+      <c r="D1719" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099559/joki-utbk-yang-tertangkap-di-unesa-palsukan-ijazah-peserta</t>
+        </is>
+      </c>
+    </row>
+    <row r="1720">
+      <c r="A1720" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1720" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1720" t="inlineStr">
+        <is>
+          <t>Kronologi Peserta UTBK Kedapatan Bawa Alat Bantu di Telinga</t>
+        </is>
+      </c>
+      <c r="D1720" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099551/kronologi-peserta-utbk-kedapatan-bawa-alat-bantu-di-telinga</t>
+        </is>
+      </c>
+    </row>
+    <row r="1721">
+      <c r="A1721" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1721" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1721" t="inlineStr">
+        <is>
+          <t>Peringatan Hari Kartini, Pemkot Semarang Jadikan Momentum Perkuat Pemberdayaan Perempuan</t>
+        </is>
+      </c>
+      <c r="D1721" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099528/peringatan-hari-kartini-pemkot-semarang-jadikan-momentum-perkuat-pemberdayaan-perempuan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1722">
+      <c r="A1722" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1722" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1722" t="inlineStr">
+        <is>
+          <t>Ketua DPR: Evaluasi Penempatan TNI di Wilayah Konflik</t>
+        </is>
+      </c>
+      <c r="D1722" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099524/ketua-dpr-evaluasi-penempatan-tni-di-wilayah-konflik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1723">
+      <c r="A1723" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1723" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1723" t="inlineStr">
+        <is>
+          <t>Tren Penggunaan Tanda Tangan Digital di Indonesia Tahun 2026</t>
+        </is>
+      </c>
+      <c r="D1723" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099522/tren-penggunaan-tanda-tangan-digital-di-indonesia-tahun-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1724">
+      <c r="A1724" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1724" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1724" t="inlineStr">
+        <is>
+          <t>Kata Dasco soal DPR Tak Kunjung Bahas Revisi UU Pemilu</t>
+        </is>
+      </c>
+      <c r="D1724" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099520/kata-dasco-soal-dpr-tak-kunjung-bahas-revisi-uu-pemilu</t>
+        </is>
+      </c>
+    </row>
+    <row r="1725">
+      <c r="A1725" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1725" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1725" t="inlineStr">
+        <is>
+          <t>Pemerintah Provinsi Lampung Dukung Akses Global bagi Generasi Muda</t>
+        </is>
+      </c>
+      <c r="D1725" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099519/pemerintah-provinsi-lampung-dukung-akses-global-bagi-generasi-muda</t>
+        </is>
+      </c>
+    </row>
+    <row r="1726">
+      <c r="A1726" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1726" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1726" t="inlineStr">
+        <is>
+          <t>Pemkab Bogor Fokus Pulihkan Akses Pascabencana</t>
+        </is>
+      </c>
+      <c r="D1726" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099516/pemkab-bogor-fokus-pulihkan-akses-pascabencana</t>
+        </is>
+      </c>
+    </row>
+    <row r="1727">
+      <c r="A1727" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1727" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1727" t="inlineStr">
+        <is>
+          <t>Manpower Minister asked companies not to withhold workers' diplomas</t>
+        </is>
+      </c>
+      <c r="D1727" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413200/manpower-minister-asked-companies-not-to-withhold-workers-diplomas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1728">
+      <c r="A1728" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1728" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1728" t="inlineStr">
+        <is>
+          <t>President Prabowo calls for accelerated 100 GW solar power push</t>
+        </is>
+      </c>
+      <c r="D1728" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413197/president-prabowo-calls-for-accelerated-100-gw-solar-power-push</t>
+        </is>
+      </c>
+    </row>
+    <row r="1729">
+      <c r="A1729" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1729" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1729" t="inlineStr">
+        <is>
+          <t>Prabowo, Albanese discuss export of 250,000 tons of urea to Australia</t>
+        </is>
+      </c>
+      <c r="D1729" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413196/prabowo-albanese-discuss-export-of-250000-tons-of-urea-to-australia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1730">
+      <c r="A1730" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1730" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1730" t="inlineStr">
+        <is>
+          <t>Seven HKTDC Lifestyle Fairs Power Sourcing and Showcase Hong Kong’s Creative Industries</t>
+        </is>
+      </c>
+      <c r="D1730" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413193/seven-hktdc-lifestyle-fairs-power-sourcing-and-showcase-hong-kongs-creative-industries</t>
+        </is>
+      </c>
+    </row>
+    <row r="1731">
+      <c r="A1731" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1731" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1731" t="inlineStr">
+        <is>
+          <t>Makassar embarkation introduces two new services for Hajj pilgrims</t>
+        </is>
+      </c>
+      <c r="D1731" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413192/makassar-embarkation-introduces-two-new-services-for-hajj-pilgrims</t>
+        </is>
+      </c>
+    </row>
+    <row r="1732">
+      <c r="A1732" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1732" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1732" t="inlineStr">
+        <is>
+          <t>KP2MI called on female migrant workers become Kartinis of global era</t>
+        </is>
+      </c>
+      <c r="D1732" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413188/kp2mi-called-on-female-migrant-workers-become-kartinis-of-global-era</t>
+        </is>
+      </c>
+    </row>
+    <row r="1733">
+      <c r="A1733" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1733" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1733" t="inlineStr">
+        <is>
+          <t>Prabowo meets Luhut to discuss economic resilience amid global tension</t>
+        </is>
+      </c>
+      <c r="D1733" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413185/prabowo-meets-luhut-to-discuss-economic-resilience-amid-global-tension</t>
+        </is>
+      </c>
+    </row>
+    <row r="1734">
+      <c r="A1734" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1734" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1734" t="inlineStr">
+        <is>
+          <t>Gov't urges collaboration to cut maternal death to pursue 2045 target</t>
+        </is>
+      </c>
+      <c r="D1734" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413181/govt-urges-collaboration-to-cut-maternal-death-to-pursue-2045-target</t>
+        </is>
+      </c>
+    </row>
+    <row r="1735">
+      <c r="A1735" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1735" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1735" t="inlineStr">
+        <is>
+          <t>Indonesia enters OECD review stage in July, Kadin welcomes move</t>
+        </is>
+      </c>
+      <c r="D1735" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413177/indonesia-enters-oecd-review-stage-in-july-kadin-welcomes-move</t>
+        </is>
+      </c>
+    </row>
+    <row r="1736">
+      <c r="A1736" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1736" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1736" t="inlineStr">
+        <is>
+          <t>DPD urges government to draft roadmap to end Papua conflict</t>
+        </is>
+      </c>
+      <c r="D1736" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413175/dpd-urges-government-to-draft-roadmap-to-end-papua-conflict</t>
+        </is>
+      </c>
+    </row>
+    <row r="1737">
+      <c r="A1737" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1737" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1737" t="inlineStr">
+        <is>
+          <t>PPRT Law serves as legal basis for domestic workers protection: govt</t>
+        </is>
+      </c>
+      <c r="D1737" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413172/pprt-law-serves-as-legal-basis-for-domestic-workers-protection-govt</t>
+        </is>
+      </c>
+    </row>
+    <row r="1738">
+      <c r="A1738" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1738" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1738" t="inlineStr">
+        <is>
+          <t>LMKN launches new music royalty scheme for 2026</t>
+        </is>
+      </c>
+      <c r="D1738" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413171/lmkn-launches-new-music-royalty-scheme-for-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1739">
+      <c r="A1739" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1739" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1739" t="inlineStr">
+        <is>
+          <t>BRIN pushes principal researcher rank for Indonesian academics abroad</t>
+        </is>
+      </c>
+      <c r="D1739" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413168/brin-pushes-principal-researcher-rank-for-indonesian-academics-abroad</t>
+        </is>
+      </c>
+    </row>
+    <row r="1740">
+      <c r="A1740" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1740" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1740" t="inlineStr">
+        <is>
+          <t>President never asks for state budget funding for BoP contribution</t>
+        </is>
+      </c>
+      <c r="D1740" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413167/president-never-asks-for-state-budget-funding-for-bop-contribution</t>
+        </is>
+      </c>
+    </row>
+    <row r="1741">
+      <c r="A1741" t="inlineStr">
+        <is>
+          <t>Wednesday, 22 April 2026</t>
+        </is>
+      </c>
+      <c r="B1741" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1741" t="inlineStr">
+        <is>
+          <t>Indonesia considers safety of UN peacekeepers as non-negotiable</t>
+        </is>
+      </c>
+      <c r="D1741" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413163/indonesia-considers-safety-of-un-peacekeepers-as-non-negotiable</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1681"/>
+  <autoFilter ref="A1:D1741"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -39113,6 +40433,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1679" r:id="rId1678"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1680" r:id="rId1679"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1681" r:id="rId1680"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1682" r:id="rId1681"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1683" r:id="rId1682"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1684" r:id="rId1683"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1685" r:id="rId1684"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1686" r:id="rId1685"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1687" r:id="rId1686"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1688" r:id="rId1687"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1689" r:id="rId1688"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1690" r:id="rId1689"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1691" r:id="rId1690"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1692" r:id="rId1691"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1693" r:id="rId1692"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1694" r:id="rId1693"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1695" r:id="rId1694"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1696" r:id="rId1695"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1697" r:id="rId1696"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1698" r:id="rId1697"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1699" r:id="rId1698"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1700" r:id="rId1699"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1701" r:id="rId1700"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1702" r:id="rId1701"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1703" r:id="rId1702"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1704" r:id="rId1703"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1705" r:id="rId1704"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1706" r:id="rId1705"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1707" r:id="rId1706"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1708" r:id="rId1707"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1709" r:id="rId1708"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1710" r:id="rId1709"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1711" r:id="rId1710"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1712" r:id="rId1711"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1713" r:id="rId1712"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1714" r:id="rId1713"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1715" r:id="rId1714"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1716" r:id="rId1715"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1717" r:id="rId1716"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1718" r:id="rId1717"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1719" r:id="rId1718"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1720" r:id="rId1719"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1721" r:id="rId1720"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1722" r:id="rId1721"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1723" r:id="rId1722"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1724" r:id="rId1723"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1725" r:id="rId1724"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1726" r:id="rId1725"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1727" r:id="rId1726"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1728" r:id="rId1727"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1729" r:id="rId1728"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1730" r:id="rId1729"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1731" r:id="rId1730"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1732" r:id="rId1731"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1733" r:id="rId1732"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1734" r:id="rId1733"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1735" r:id="rId1734"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1736" r:id="rId1735"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1737" r:id="rId1736"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1738" r:id="rId1737"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1739" r:id="rId1738"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1740" r:id="rId1739"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1741" r:id="rId1740"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-22
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1741</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1801</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1741"/>
+  <dimension ref="A1:D1801"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -38750,8 +38750,1328 @@
         </is>
       </c>
     </row>
+    <row r="1742">
+      <c r="A1742" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1742" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1742" t="inlineStr">
+        <is>
+          <t>Dubes RI Abdul Aziz Ahmad Pastikan Pelayanan Jemaah Haji di Madinah Lancar</t>
+        </is>
+      </c>
+      <c r="D1742" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8456549/dubes-ri-abdul-aziz-ahmad-pastikan-pelayanan-jemaah-haji-di-madinah-lancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="1743">
+      <c r="A1743" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1743" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1743" t="inlineStr">
+        <is>
+          <t>Apa Itu Murur dan Tanazul dalam Ibadah Haji?</t>
+        </is>
+      </c>
+      <c r="D1743" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jatim/berita/d-8456566/apa-itu-murur-dan-tanazul-dalam-ibadah-haji</t>
+        </is>
+      </c>
+    </row>
+    <row r="1744">
+      <c r="A1744" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1744" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1744" t="inlineStr">
+        <is>
+          <t>Durasi Haji 2026 Berapa Lama? Ini Penjelasan Lengkapnya</t>
+        </is>
+      </c>
+      <c r="D1744" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jatim/berita/d-8456553/durasi-haji-2026-berapa-lama-ini-penjelasan-lengkapnya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1745">
+      <c r="A1745" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1745" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1745" t="inlineStr">
+        <is>
+          <t>Video Petugas Pastikan Jemaah Lansia Nyaman Tiba di Tanah Suci</t>
+        </is>
+      </c>
+      <c r="D1745" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260422-260422103/video-petugas-pastikan-jemaah-lansia-nyaman-tiba-di-tanah-suci</t>
+        </is>
+      </c>
+    </row>
+    <row r="1746">
+      <c r="A1746" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1746" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1746" t="inlineStr">
+        <is>
+          <t>Kisah Nenek Patimang, Janda Sebatang Kara Pergi Haji dari Sisa Rumput Laut</t>
+        </is>
+      </c>
+      <c r="D1746" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8456711/kisah-nenek-patimang-janda-sebatang-kara-pergi-haji-dari-sisa-rumput-laut</t>
+        </is>
+      </c>
+    </row>
+    <row r="1747">
+      <c r="A1747" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1747" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1747" t="inlineStr">
+        <is>
+          <t>Dubes RI Abdul Aziz Ahmad Pastikan Pelayanan Jemaah Haji di Madinah Lancar</t>
+        </is>
+      </c>
+      <c r="D1747" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8456549/dubes-ri-abdul-aziz-ahmad-pastikan-pelayanan-jemaah-haji-di-madinah-lancar</t>
+        </is>
+      </c>
+    </row>
+    <row r="1748">
+      <c r="A1748" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1748" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1748" t="inlineStr">
+        <is>
+          <t>Chelsea Pecat Liam Rosenior!</t>
+        </is>
+      </c>
+      <c r="D1748" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-inggris/d-8457082/chelsea-pecat-liam-rosenior</t>
+        </is>
+      </c>
+    </row>
+    <row r="1749">
+      <c r="A1749" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1749" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1749" t="inlineStr">
+        <is>
+          <t>Perang Timur Tengah Tak Kunjung Usai, RI Bidik Minyak dari Nigeria-Gabon</t>
+        </is>
+      </c>
+      <c r="D1749" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8457049/perang-timur-tengah-tak-kunjung-usai-ri-bidik-minyak-dari-nigeria-gabon</t>
+        </is>
+      </c>
+    </row>
+    <row r="1750">
+      <c r="A1750" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1750" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1750" t="inlineStr">
+        <is>
+          <t>Video: Resmi Patuhi PP Tunas, YouTube Akan Hapus Iklan yang Targetkan Anak-anak</t>
+        </is>
+      </c>
+      <c r="D1750" s="2" t="inlineStr">
+        <is>
+          <t>https://inet.detik.com/detiktv/d-8457011/video-resmi-patuhi-pp-tunas-youtube-akan-hapus-iklan-yang-targetkan-anak-anak</t>
+        </is>
+      </c>
+    </row>
+    <row r="1751">
+      <c r="A1751" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1751" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1751" t="inlineStr">
+        <is>
+          <t>RI Punya Uranium &amp; Torium, Pembangkit Listrik Tenaga Nuklir Diputuskan 2027</t>
+        </is>
+      </c>
+      <c r="D1751" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8457003/ri-punya-uranium-torium-pembangkit-listrik-tenaga-nuklir-diputuskan-2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="1752">
+      <c r="A1752" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1752" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1752" t="inlineStr">
+        <is>
+          <t>Video: Tawa Kecil Kepala BPOM Anggarannya Disebut Lebih Kecil dari Pengadaan Kaos Kaki</t>
+        </is>
+      </c>
+      <c r="D1752" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/detiktv/d-8456790/video-tawa-kecil-kepala-bpom-anggarannya-disebut-lebih-kecil-dari-pengadaan-kaos-kaki</t>
+        </is>
+      </c>
+    </row>
+    <row r="1753">
+      <c r="A1753" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1753" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1753" t="inlineStr">
+        <is>
+          <t>Iran Pastikan Selat Hormuz Tak Mungkin Dibuka Selama AS Blokade Pelabuhan</t>
+        </is>
+      </c>
+      <c r="D1753" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8457107/iran-pastikan-selat-hormuz-tak-mungkin-dibuka-selama-as-blokade-pelabuhan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1754">
+      <c r="A1754" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1754" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1754" t="inlineStr">
+        <is>
+          <t>Trump Sebut Negosiasi dengan Iran Kemungkinan Digelar dalam 3 Hari ke Depan</t>
+        </is>
+      </c>
+      <c r="D1754" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8457055/trump-sebut-negosiasi-dengan-iran-kemungkinan-digelar-dalam-3-hari-ke-depan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1755">
+      <c r="A1755" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1755" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1755" t="inlineStr">
+        <is>
+          <t>Jauh Panggang dari Api, Damai AS dan Iran Kapan Terjadi</t>
+        </is>
+      </c>
+      <c r="D1755" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8456989/jauh-panggang-dari-api-damai-as-dan-iran-kapan-terjadi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1756">
+      <c r="A1756" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1756" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1756" t="inlineStr">
+        <is>
+          <t>Perang Timur Tengah Tak Kunjung Usai, RI Bidik Minyak dari Nigeria-Gabon</t>
+        </is>
+      </c>
+      <c r="D1756" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8457049/perang-timur-tengah-tak-kunjung-usai-ri-bidik-minyak-dari-nigeria-gabon</t>
+        </is>
+      </c>
+    </row>
+    <row r="1757">
+      <c r="A1757" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1757" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1757" t="inlineStr">
+        <is>
+          <t>RI Kecam Israel Pasang Spanduk Propaganda di Reruntuhan RS Indonesia di Gaza</t>
+        </is>
+      </c>
+      <c r="D1757" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1925448/ri-kecam-israel-pasang-spanduk-propaganda-di-reruntuhan-rs-indonesia-di-gaza?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1758">
+      <c r="A1758" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1758" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1758" t="inlineStr">
+        <is>
+          <t>Kenali Batas Diri, Guru Rentan ”Burnout”</t>
+        </is>
+      </c>
+      <c r="D1758" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/guru-rentan-burnout?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1759">
+      <c r="A1759" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1759" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1759" t="inlineStr">
+        <is>
+          <t>Temui Jokowi, KPPU Dorong Amandemen UU Persaingan Usaha dan Penguatan Kelembagaan</t>
+        </is>
+      </c>
+      <c r="D1759" s="2" t="inlineStr">
+        <is>
+          <t>https://money.kompas.com/read/2026/04/22/214600326/temui-jokowi-kppu-dorong-amandemen-uu-persaingan-usaha-dan-penguatan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1760">
+      <c r="A1760" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1760" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1760" t="inlineStr">
+        <is>
+          <t>Bawa Resep Kepemimpinan Jateng ke Sumatera, Ahmad Luthfi: Kepala Daerah adalah “Manajer Marketing”</t>
+        </is>
+      </c>
+      <c r="D1760" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/22/210941178/bawa-resep-kepemimpinan-jateng-ke-sumatera-ahmad-luthfi-kepala-daerah</t>
+        </is>
+      </c>
+    </row>
+    <row r="1761">
+      <c r="A1761" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1761" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1761" t="inlineStr">
+        <is>
+          <t>6 Budaya Semarang Raih Status WBTB Nasional, Walkot Agustina: Kado Jelang HUT Ke-479</t>
+        </is>
+      </c>
+      <c r="D1761" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/22/204707778/6-budaya-semarang-raih-status-wbtb-nasional-walkot-agustina-kado-jelang-hut</t>
+        </is>
+      </c>
+    </row>
+    <row r="1762">
+      <c r="A1762" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1762" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1762" t="inlineStr">
+        <is>
+          <t>TIRTA DAN EMILIANA</t>
+        </is>
+      </c>
+      <c r="D1762" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/membangun-tata-kelola-air-dan-sanitasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1763">
+      <c r="A1763" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1763" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1763" t="inlineStr">
+        <is>
+          <t>Menghijaukan Tanah Pasundan</t>
+        </is>
+      </c>
+      <c r="D1763" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/menghijaukan-tanah-pasundan-demi-masa-depan/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1764">
+      <c r="A1764" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1764" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1764" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D1764" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1765">
+      <c r="A1765" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1765" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1765" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D1765" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1766">
+      <c r="A1766" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1766" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1766" t="inlineStr">
+        <is>
+          <t>Sudah Bayar Rp 840 Juta, Akses Rumah di Tangerang Ditutup Tembok oleh Kelompok Diduga Ormas</t>
+        </is>
+      </c>
+      <c r="D1766" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1925414/sudah-bayar-rp-840-juta-akses-rumah-di-tangerang-ditutup-tembok-oleh-kelompok-diduga-ormas?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1767">
+      <c r="A1767" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1767" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1767" t="inlineStr">
+        <is>
+          <t>Penantian Alas</t>
+        </is>
+      </c>
+      <c r="D1767" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/masrortegan5996/69e8844c34777c38bc294b12/penantian-alas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1768">
+      <c r="A1768" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1768" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1768" t="inlineStr">
+        <is>
+          <t>Prefektur Dekat Tokyo Ini Akan Berikan Imbalan Rp 1 Juta bagi Pelapor Perusahaan yang Pekerjakan WNA Ilegal</t>
+        </is>
+      </c>
+      <c r="D1768" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5867/prefektur-dekat-tokyo-ini-akan-berikan-imbalan-rp-1-juta-bagi-pelapor-perusahaan-yang-pekerjakan-wna-ilegal</t>
+        </is>
+      </c>
+    </row>
+    <row r="1769">
+      <c r="A1769" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1769" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1769" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1769" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1770">
+      <c r="A1770" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1770" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1770" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1770" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1771">
+      <c r="A1771" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1771" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1771" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Demo Ricuh di Kaltim, Tuntutan Peserta Aksi Tak Digubris</t>
+        </is>
+      </c>
+      <c r="D1771" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/22/072805878/berita-foto-demo-ricuh-di-kaltim-tuntutan-peserta-aksi-tak-digubris</t>
+        </is>
+      </c>
+    </row>
+    <row r="1772">
+      <c r="A1772" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1772" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1772" t="inlineStr">
+        <is>
+          <t>Menteri Haji: Prabowo Ingin Keselamatan Jemaah Terjamin</t>
+        </is>
+      </c>
+      <c r="D1772" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099832/menteri-haji-prabowo-ingin-keselamatan-jemaah-terjamin</t>
+        </is>
+      </c>
+    </row>
+    <row r="1773">
+      <c r="A1773" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1773" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1773" t="inlineStr">
+        <is>
+          <t>Komisi VIII DPR Meninjau Skema Embarkasi Haji Berbasis Hotel di Yogya</t>
+        </is>
+      </c>
+      <c r="D1773" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099830/komisi-viii-dpr-meninjau-skema-embarkasi-haji-berbasis-hotel-di-yogya</t>
+        </is>
+      </c>
+    </row>
+    <row r="1774">
+      <c r="A1774" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1774" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1774" t="inlineStr">
+        <is>
+          <t>Setara Rilis IKT 2025, Salatiga Jadi Kota Paling Toleran</t>
+        </is>
+      </c>
+      <c r="D1774" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099827/setara-rilis-ikt-2025-salatiga-jadi-kota-paling-toleran</t>
+        </is>
+      </c>
+    </row>
+    <row r="1775">
+      <c r="A1775" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1775" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1775" t="inlineStr">
+        <is>
+          <t>HUT ke-479 Kota Semarang: Pemkot Luncurkan Program Penukaran Botol Plastik dengan Lumpia</t>
+        </is>
+      </c>
+      <c r="D1775" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099823/hut-ke-479-kota-semarang-pemkot-luncurkan-program-penukaran-botol-plastik-dengan-lumpia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1776">
+      <c r="A1776" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1776" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1776" t="inlineStr">
+        <is>
+          <t>Tanggap Darurat, Pemkot Semarang Langsung Dampingi Anak Korban Penganiayaan</t>
+        </is>
+      </c>
+      <c r="D1776" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099763/tanggap-darurat-pemkot-semarang-langsung-dampingi-anak-korban-penganiayaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1777">
+      <c r="A1777" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1777" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1777" t="inlineStr">
+        <is>
+          <t>Kisah Sepasang Lansia Berangkat Haji Setelah Mengantre 7 Tahun</t>
+        </is>
+      </c>
+      <c r="D1777" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099797/kisah-sepasang-lansia-berangkat-haji-setelah-mengantre-7-tahun</t>
+        </is>
+      </c>
+    </row>
+    <row r="1778">
+      <c r="A1778" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1778" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1778" t="inlineStr">
+        <is>
+          <t>Anak Penganut Ajaran Leluhur Sunda Alami Perundungan</t>
+        </is>
+      </c>
+      <c r="D1778" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099795/anak-penganut-ajaran-leluhur-sunda-alami-perundungan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1779">
+      <c r="A1779" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1779" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1779" t="inlineStr">
+        <is>
+          <t>UTBK Diwarnai Kecurangan, Anggota DPR: Pengawasan Perlu Diperketat</t>
+        </is>
+      </c>
+      <c r="D1779" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099787/utbk-diwarnai-kecurangan-anggota-dpr-pengawasan-perlu-diperketat</t>
+        </is>
+      </c>
+    </row>
+    <row r="1780">
+      <c r="A1780" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1780" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1780" t="inlineStr">
+        <is>
+          <t>Pertama dalam Sejarah: Solidaritas lewat TKD untuk Pemulihan Banjir Sumatra</t>
+        </is>
+      </c>
+      <c r="D1780" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099786/pertama-dalam-sejarah-solidaritas-lewat-tkd-untuk-pemulihan-banjir-sumatra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1781">
+      <c r="A1781" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1781" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1781" t="inlineStr">
+        <is>
+          <t>Menteri PPPA: UU PPRT Belum Detail</t>
+        </is>
+      </c>
+      <c r="D1781" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099782/menteri-pppa-uu-pprt-belum-detail</t>
+        </is>
+      </c>
+    </row>
+    <row r="1782">
+      <c r="A1782" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1782" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1782" t="inlineStr">
+        <is>
+          <t>Menlu soal Kapal Perang AS di Selat Malaka: Patroli Kawasan</t>
+        </is>
+      </c>
+      <c r="D1782" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099778/menlu-soal-kapal-perang-as-di-selat-malaka-patroli-kawasan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1783">
+      <c r="A1783" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1783" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1783" t="inlineStr">
+        <is>
+          <t>Cerita Nenek Masuah, Jemaah Haji dengan Demensia Minta Pulang</t>
+        </is>
+      </c>
+      <c r="D1783" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099775/cerita-nenek-masuah-jemaah-haji-dengan-demensia-minta-pulang</t>
+        </is>
+      </c>
+    </row>
+    <row r="1784">
+      <c r="A1784" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1784" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1784" t="inlineStr">
+        <is>
+          <t>Pemkab Jember Sabet Tiga Penghargaan dalam Sepekan</t>
+        </is>
+      </c>
+      <c r="D1784" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099769/pemkab-jember-sabet-tiga-penghargaan-dalam-sepekan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1785">
+      <c r="A1785" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1785" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1785" t="inlineStr">
+        <is>
+          <t>Bupati Gresik Tegaskan CSR Harus Berdampak Nyata</t>
+        </is>
+      </c>
+      <c r="D1785" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099767/bupati-gresik-tegaskan-csr-harus-berdampak-nyata</t>
+        </is>
+      </c>
+    </row>
+    <row r="1786">
+      <c r="A1786" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1786" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1786" t="inlineStr">
+        <is>
+          <t>Soal Pembelian Alutsista dari Prancis, Menlu Singgung Transfer Teknologi</t>
+        </is>
+      </c>
+      <c r="D1786" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2099765/soal-pembelian-alutsista-dari-prancis-menlu-singgung-transfer-teknologi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1787">
+      <c r="A1787" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1787" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1787" t="inlineStr">
+        <is>
+          <t>Govt urges mental readiness for 2026 hajj pilgrims</t>
+        </is>
+      </c>
+      <c r="D1787" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413331/govt-urges-mental-readiness-for-2026-hajj-pilgrims</t>
+        </is>
+      </c>
+    </row>
+    <row r="1788">
+      <c r="A1788" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1788" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1788" t="inlineStr">
+        <is>
+          <t>Indonesia eyes leadership in global halal economy</t>
+        </is>
+      </c>
+      <c r="D1788" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413329/indonesia-eyes-leadership-in-global-halal-economy</t>
+        </is>
+      </c>
+    </row>
+    <row r="1789">
+      <c r="A1789" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1789" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1789" t="inlineStr">
+        <is>
+          <t>RI slams Israel over military banner at Gaza's Indonesian Hospital</t>
+        </is>
+      </c>
+      <c r="D1789" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413325/ri-slams-israel-over-military-banner-at-gazas-indonesian-hospital</t>
+        </is>
+      </c>
+    </row>
+    <row r="1790">
+      <c r="A1790" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1790" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1790" t="inlineStr">
+        <is>
+          <t>BNI completes $1.65 million refund in embezzlement case</t>
+        </is>
+      </c>
+      <c r="D1790" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413323/bni-completes-165-million-refund-in-embezzlement-case</t>
+        </is>
+      </c>
+    </row>
+    <row r="1791">
+      <c r="A1791" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1791" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1791" t="inlineStr">
+        <is>
+          <t>RI targets June groundbreaking for five waste-to-energy projects</t>
+        </is>
+      </c>
+      <c r="D1791" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413320/ri-targets-june-groundbreaking-for-five-waste-to-energy-projects</t>
+        </is>
+      </c>
+    </row>
+    <row r="1792">
+      <c r="A1792" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1792" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1792" t="inlineStr">
+        <is>
+          <t>Indonesia removes EV tax exemptions due to fiscal considerations: govt</t>
+        </is>
+      </c>
+      <c r="D1792" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413317/indonesia-removes-ev-tax-exemptions-due-to-fiscal-considerations-govt</t>
+        </is>
+      </c>
+    </row>
+    <row r="1793">
+      <c r="A1793" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1793" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1793" t="inlineStr">
+        <is>
+          <t>Four countries ask for Indonesia's urea, over 750,000 tons sought</t>
+        </is>
+      </c>
+      <c r="D1793" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413313/four-countries-ask-for-indonesias-urea-over-750000-tons-sought</t>
+        </is>
+      </c>
+    </row>
+    <row r="1794">
+      <c r="A1794" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1794" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1794" t="inlineStr">
+        <is>
+          <t>Banking resilience strong to mitigate impact of war: BI</t>
+        </is>
+      </c>
+      <c r="D1794" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413311/banking-resilience-strong-to-mitigate-impact-of-war-bi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1795">
+      <c r="A1795" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1795" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1795" t="inlineStr">
+        <is>
+          <t>Indonesia in 'survival mode' amid global uncertainty: finance minister</t>
+        </is>
+      </c>
+      <c r="D1795" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413307/indonesia-in-survival-mode-amid-global-uncertainty-finance-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="1796">
+      <c r="A1796" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1796" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1796" t="inlineStr">
+        <is>
+          <t>Govt strengthens role of 'early adopter' to boost EV market</t>
+        </is>
+      </c>
+      <c r="D1796" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413303/govt-strengthens-role-of-early-adopter-to-boost-ev-market</t>
+        </is>
+      </c>
+    </row>
+    <row r="1797">
+      <c r="A1797" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1797" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1797" t="inlineStr">
+        <is>
+          <t>Japanese tourists can soon use QRIS for inbound transaction: BI</t>
+        </is>
+      </c>
+      <c r="D1797" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413300/japanese-tourists-can-soon-use-qris-for-inbound-transaction-bi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1798">
+      <c r="A1798" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1798" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1798" t="inlineStr">
+        <is>
+          <t>Govt prepares weather modification, water measures ahead of El Nino</t>
+        </is>
+      </c>
+      <c r="D1798" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413297/govt-prepares-weather-modification-water-measures-ahead-of-el-nino</t>
+        </is>
+      </c>
+    </row>
+    <row r="1799">
+      <c r="A1799" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1799" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1799" t="inlineStr">
+        <is>
+          <t>BGN calls for tighter supply chain oversight for free meal program</t>
+        </is>
+      </c>
+      <c r="D1799" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413296/bgn-calls-for-tighter-supply-chain-oversight-for-free-meal-program</t>
+        </is>
+      </c>
+    </row>
+    <row r="1800">
+      <c r="A1800" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1800" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1800" t="inlineStr">
+        <is>
+          <t>Citizens without proper visa cannot perform Hajj, minister says</t>
+        </is>
+      </c>
+      <c r="D1800" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413293/citizens-without-proper-visa-cannot-perform-hajj-minister-says</t>
+        </is>
+      </c>
+    </row>
+    <row r="1801">
+      <c r="A1801" t="inlineStr">
+        <is>
+          <t>Thursday, 23 April 2026</t>
+        </is>
+      </c>
+      <c r="B1801" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1801" t="inlineStr">
+        <is>
+          <t>Indonesia to maintain inflation rate at 2,51 percent: BI</t>
+        </is>
+      </c>
+      <c r="D1801" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413292/indonesia-to-maintain-inflation-rate-at-251-percent-bi</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1741"/>
+  <autoFilter ref="A1:D1801"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -40493,6 +41813,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1739" r:id="rId1738"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1740" r:id="rId1739"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1741" r:id="rId1740"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1742" r:id="rId1741"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1743" r:id="rId1742"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1744" r:id="rId1743"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1745" r:id="rId1744"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1746" r:id="rId1745"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1747" r:id="rId1746"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1748" r:id="rId1747"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1749" r:id="rId1748"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1750" r:id="rId1749"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1751" r:id="rId1750"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1752" r:id="rId1751"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1753" r:id="rId1752"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1754" r:id="rId1753"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1755" r:id="rId1754"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1756" r:id="rId1755"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1757" r:id="rId1756"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1758" r:id="rId1757"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1759" r:id="rId1758"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1760" r:id="rId1759"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1761" r:id="rId1760"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1762" r:id="rId1761"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1763" r:id="rId1762"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1764" r:id="rId1763"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1765" r:id="rId1764"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1766" r:id="rId1765"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1767" r:id="rId1766"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1768" r:id="rId1767"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1769" r:id="rId1768"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1770" r:id="rId1769"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1771" r:id="rId1770"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1772" r:id="rId1771"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1773" r:id="rId1772"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1774" r:id="rId1773"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1775" r:id="rId1774"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1776" r:id="rId1775"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1777" r:id="rId1776"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1778" r:id="rId1777"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1779" r:id="rId1778"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1780" r:id="rId1779"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1781" r:id="rId1780"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1782" r:id="rId1781"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1783" r:id="rId1782"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1784" r:id="rId1783"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1785" r:id="rId1784"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1786" r:id="rId1785"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1787" r:id="rId1786"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1788" r:id="rId1787"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1789" r:id="rId1788"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1790" r:id="rId1789"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1791" r:id="rId1790"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1792" r:id="rId1791"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1793" r:id="rId1792"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1794" r:id="rId1793"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1795" r:id="rId1794"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1796" r:id="rId1795"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1797" r:id="rId1796"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1798" r:id="rId1797"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1799" r:id="rId1798"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1800" r:id="rId1799"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1801" r:id="rId1800"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-23
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1801</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$1861</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1801"/>
+  <dimension ref="A1:D1861"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -40070,8 +40070,1328 @@
         </is>
       </c>
     </row>
+    <row r="1802">
+      <c r="A1802" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1802" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1802" t="inlineStr">
+        <is>
+          <t>Dua Kali Tertunda, Ashanty: Insyaallah Berangkat Haji Mei Tahun Ini</t>
+        </is>
+      </c>
+      <c r="D1802" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8457674/dua-kali-tertunda-ashanty-insyaallah-berangkat-haji-mei-tahun-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="1803">
+      <c r="A1803" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1803" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1803" t="inlineStr">
+        <is>
+          <t>Jadwal JCH Berangkat Malam, Bandara Syamsudin Noor Optimalkan Personel</t>
+        </is>
+      </c>
+      <c r="D1803" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/kalimantan/berita/d-8458827/jadwal-jch-berangkat-malam-bandara-syamsudin-noor-optimalkan-personel</t>
+        </is>
+      </c>
+    </row>
+    <row r="1804">
+      <c r="A1804" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1804" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1804" t="inlineStr">
+        <is>
+          <t>Bendara Juanda Layani Mecca Route Haji 2026, Jemaah Tak Repot Antre</t>
+        </is>
+      </c>
+      <c r="D1804" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jatim/berita/d-8458753/bendara-juanda-layani-mecca-route-haji-2026-jemaah-tak-repot-antre</t>
+        </is>
+      </c>
+    </row>
+    <row r="1805">
+      <c r="A1805" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1805" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1805" t="inlineStr">
+        <is>
+          <t>359 Jemaah Kloter 1 Embarkasi Banjarmasin Lepas Landas ke Tanah Suci</t>
+        </is>
+      </c>
+      <c r="D1805" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/kalimantan/berita/d-8458805/359-jemaah-kloter-1-embarkasi-banjarmasin-lepas-landas-ke-tanah-suci</t>
+        </is>
+      </c>
+    </row>
+    <row r="1806">
+      <c r="A1806" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1806" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1806" t="inlineStr">
+        <is>
+          <t>Video: 2 Calon Haji Embarkasi Padang Batal Berangkat Hari Ini karena Sakit</t>
+        </is>
+      </c>
+      <c r="D1806" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260423-260423127/video-2-calon-haji-embarkasi-padang-batal-berangkat-hari-ini-karena-sakit</t>
+        </is>
+      </c>
+    </row>
+    <row r="1807">
+      <c r="A1807" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1807" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1807" t="inlineStr">
+        <is>
+          <t>Dua Kali Tertunda, Ashanty: Insyaallah Berangkat Haji Mei Tahun Ini</t>
+        </is>
+      </c>
+      <c r="D1807" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8457674/dua-kali-tertunda-ashanty-insyaallah-berangkat-haji-mei-tahun-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="1808">
+      <c r="A1808" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1808" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C1808" t="inlineStr">
+        <is>
+          <t>Video Arsenal Disalip Man City, The Gunners Cuma 'Jagain Trofi' Lagi?</t>
+        </is>
+      </c>
+      <c r="D1808" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/detiktv/d-8458687/video-arsenal-disalip-man-city-the-gunners-cuma-jagain-trofi-lagi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1809">
+      <c r="A1809" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1809" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1809" t="inlineStr">
+        <is>
+          <t>Beredar Kabar APBN Cuma Tahan 3 Bulan, Kemenkeu Pastikan Hoaks!</t>
+        </is>
+      </c>
+      <c r="D1809" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8458735/beredar-kabar-apbn-cuma-tahan-3-bulan-kemenkeu-pastikan-hoaks</t>
+        </is>
+      </c>
+    </row>
+    <row r="1810">
+      <c r="A1810" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1810" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1810" t="inlineStr">
+        <is>
+          <t>Mentan Bongkar Beras Premium Abal-abal: Harga Rp 8.000/Kg, Dijual Rp 17.000/Kg</t>
+        </is>
+      </c>
+      <c r="D1810" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8458714/mentan-bongkar-beras-premium-abal-abal-harga-rp-8-000-kg-dijual-rp-17-000-kg</t>
+        </is>
+      </c>
+    </row>
+    <row r="1811">
+      <c r="A1811" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1811" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1811" t="inlineStr">
+        <is>
+          <t>Potret Song Joong Ki dan Istri Jadi Narator Konser Klasik</t>
+        </is>
+      </c>
+      <c r="D1811" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/pop/foto/d-8458119/potret-song-joong-ki-dan-istri-jadi-narator-konser-klasik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1812">
+      <c r="A1812" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1812" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C1812" t="inlineStr">
+        <is>
+          <t>JP Morgan Sebut RI Negara Tangguh Hadapi Krisis Energi Dunia</t>
+        </is>
+      </c>
+      <c r="D1812" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/energi/d-8458675/jp-morgan-sebut-ri-negara-tangguh-hadapi-krisis-energi-dunia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1813">
+      <c r="A1813" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1813" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1813" t="inlineStr">
+        <is>
+          <t>Kakek di Sumut Bunuh Selingkuhan Usai Ditolak Hubungan Badan</t>
+        </is>
+      </c>
+      <c r="D1813" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8458828/kakek-di-sumut-bunuh-selingkuhan-usai-ditolak-hubungan-badan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1814">
+      <c r="A1814" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1814" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1814" t="inlineStr">
+        <is>
+          <t>Pacu Ekonomi, Mendagri Dorong Sumut Optimalkan APBD &amp; Kendalikan Inflasi</t>
+        </is>
+      </c>
+      <c r="D1814" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8457797/pacu-ekonomi-mendagri-dorong-sumut-optimalkan-apbd-kendalikan-inflasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1815">
+      <c r="A1815" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1815" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1815" t="inlineStr">
+        <is>
+          <t>Kasus Naik Penyidikan, 2 Pembunuh Nus Kei Terancam Hukuman Mati</t>
+        </is>
+      </c>
+      <c r="D1815" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8457219/kasus-naik-penyidikan-2-pembunuh-nus-kei-terancam-hukuman-mati</t>
+        </is>
+      </c>
+    </row>
+    <row r="1816">
+      <c r="A1816" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1816" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1816" t="inlineStr">
+        <is>
+          <t>Alasan di Balik KPK Usul Masa Jabatan Ketum Parpol 2 Periode</t>
+        </is>
+      </c>
+      <c r="D1816" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8458711/alasan-di-balik-kpk-usul-masa-jabatan-ketum-parpol-2-periode</t>
+        </is>
+      </c>
+    </row>
+    <row r="1817">
+      <c r="A1817" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1817" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1817" t="inlineStr">
+        <is>
+          <t>Dua Menteri Peru Mundur Gara-gara Pembelian 24 Jet F-16 AS Ditunda</t>
+        </is>
+      </c>
+      <c r="D1817" s="2" t="inlineStr">
+        <is>
+          <t>https://video.kompas.com/watch/1925692/dua-menteri-peru-mundur-gara-gara-pembelian-24-jet-f-16-as-ditunda?source=KOMPASCOM&amp;position=wp_terkini__player_1</t>
+        </is>
+      </c>
+    </row>
+    <row r="1818">
+      <c r="A1818" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1818" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1818" t="inlineStr">
+        <is>
+          <t>Blunder Komunikasi Politik Bayangi Satu Tahun Pemerintahan Prabowo-Gibran</t>
+        </is>
+      </c>
+      <c r="D1818" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.id/artikel/blunder-komunikasi-politik-bayangi-satu-tahun-pemerintahan-prabowo-gibran?utm_source=external_kompascom&amp;utm_medium=headline&amp;utm_campaign=tpd_-_popular_traffic</t>
+        </is>
+      </c>
+    </row>
+    <row r="1819">
+      <c r="A1819" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1819" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1819" t="inlineStr">
+        <is>
+          <t>Hunian Layak Tersedia, Senyum Penyintas di Bener Meriah Kembali Hadir</t>
+        </is>
+      </c>
+      <c r="D1819" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/23/21234801/hunian-layak-tersedia-senyum-penyintas-di-bener-meriah-kembali-hadir</t>
+        </is>
+      </c>
+    </row>
+    <row r="1820">
+      <c r="A1820" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1820" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1820" t="inlineStr">
+        <is>
+          <t>Jateng–Aceh Teken Kerja Sama Senilai Rp 1,06 Triliun, Dorong Kolaborasi OPD hingga BUMD</t>
+        </is>
+      </c>
+      <c r="D1820" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/23/210641678/jatengaceh-teken-kerja-sama-senilai-rp-106-triliun-dorong-kolaborasi-opd</t>
+        </is>
+      </c>
+    </row>
+    <row r="1821">
+      <c r="A1821" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1821" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1821" t="inlineStr">
+        <is>
+          <t>FK Universitas Ciputra Buka PPDS Obgyn dan Bedah, Dorong Pemerataan Dokter Spesialis ke Indonesia Timur</t>
+        </is>
+      </c>
+      <c r="D1821" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompas.com/edu/read/2026/04/23/195557171/fk-universitas-ciputra-buka-ppds-obgyn-dan-bedah-dorong-pemerataan-dokter</t>
+        </is>
+      </c>
+    </row>
+    <row r="1822">
+      <c r="A1822" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1822" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C1822" t="inlineStr">
+        <is>
+          <t>Jaga Ekonomi Tetap Tangguh</t>
+        </is>
+      </c>
+      <c r="D1822" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/jaga-ekonomi-tetap-tangguh/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1823">
+      <c r="A1823" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1823" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1823" t="inlineStr">
+        <is>
+          <t>Indonesia Bebas Kemiskinan Ekstrem</t>
+        </is>
+      </c>
+      <c r="D1823" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/indonesia-bebas-kemiskinan-ekstrem/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1824">
+      <c r="A1824" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1824" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1824" t="inlineStr">
+        <is>
+          <t>Mangrove</t>
+        </is>
+      </c>
+      <c r="D1824" s="2" t="inlineStr">
+        <is>
+          <t>https://vip.kompas.com/M4CR</t>
+        </is>
+      </c>
+    </row>
+    <row r="1825">
+      <c r="A1825" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1825" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1825" t="inlineStr">
+        <is>
+          <t>Merajut Nadi Sumatera</t>
+        </is>
+      </c>
+      <c r="D1825" s="2" t="inlineStr">
+        <is>
+          <t>https://vik.kompas.com/merajut-nadi-sumatera-jalan-tol-hingga-gerbang-dunia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="1826">
+      <c r="A1826" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1826" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1826" t="inlineStr">
+        <is>
+          <t>Situs Berusia Ribuan Tahun di Timur Tengah Terancam Hilang Akibat Konflik</t>
+        </is>
+      </c>
+      <c r="D1826" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kgnow.com/watch/1925651/situs-berusia-ribuan-tahun-di-timur-tengah-terancam-hilang-akibat-konflik?source=KOMPASCOM&amp;position=wp_terkini__player_2</t>
+        </is>
+      </c>
+    </row>
+    <row r="1827">
+      <c r="A1827" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1827" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1827" t="inlineStr">
+        <is>
+          <t>Di Bawah Langit Desa, Kesederhanaan Menjadi Mewah</t>
+        </is>
+      </c>
+      <c r="D1827" s="2" t="inlineStr">
+        <is>
+          <t>https://www.kompasiana.com/goestanchannel1762/69e9724b34777c47c3147532/di-bawah-langit-desa-kesederhanaan-menjadi-mewah</t>
+        </is>
+      </c>
+    </row>
+    <row r="1828">
+      <c r="A1828" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1828" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1828" t="inlineStr">
+        <is>
+          <t>Museum Maritim di Jepang Ini Buka Kembali Usai Renovasi Besar, Tampilkan Miniatur Kapal Perang Yamato</t>
+        </is>
+      </c>
+      <c r="D1828" s="2" t="inlineStr">
+        <is>
+          <t>https://ohayojepang.kompas.com/read/5870/museum-maritim-di-jepang-ini-buka-kembali-usai-renovasi-besar-tampilkan-miniatur-kapal-perang-yamato</t>
+        </is>
+      </c>
+    </row>
+    <row r="1829">
+      <c r="A1829" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1829" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1829" t="inlineStr">
+        <is>
+          <t>Damai Studio, Oase Literasi di Surabaya, Lahir dari Ketidaksengajaan</t>
+        </is>
+      </c>
+      <c r="D1829" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/01/13/183644778/damai-studio-oase-literasi-di-surabaya-lahir-dari-ketidaksengajaan</t>
+        </is>
+      </c>
+    </row>
+    <row r="1830">
+      <c r="A1830" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1830" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1830" t="inlineStr">
+        <is>
+          <t>Meraba Masa Depan dengan AI sebagai Copilot</t>
+        </is>
+      </c>
+      <c r="D1830" s="2" t="inlineStr">
+        <is>
+          <t>https://jeo.kompas.com/meraba-masa-depan-dengan-ai-sebagai-copilot</t>
+        </is>
+      </c>
+    </row>
+    <row r="1831">
+      <c r="A1831" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1831" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1831" t="inlineStr">
+        <is>
+          <t>BERITA FOTO: Demo Ricuh di Kaltim, Tuntutan Peserta Aksi Tak Digubris</t>
+        </is>
+      </c>
+      <c r="D1831" s="2" t="inlineStr">
+        <is>
+          <t>https://regional.kompas.com/read/2026/04/22/072805878/berita-foto-demo-ricuh-di-kaltim-tuntutan-peserta-aksi-tak-digubris</t>
+        </is>
+      </c>
+    </row>
+    <row r="1832">
+      <c r="A1832" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1832" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1832" t="inlineStr">
+        <is>
+          <t>Mendagri Minta Pemda Bebaskan Pajak Kendaraan Listrik</t>
+        </is>
+      </c>
+      <c r="D1832" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100076/mendagri-minta-pemda-bebaskan-pajak-kendaraan-listrik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1833">
+      <c r="A1833" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1833" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1833" t="inlineStr">
+        <is>
+          <t>NasDem Usul Ambang Batas Parlemen di Atas 5 Persen</t>
+        </is>
+      </c>
+      <c r="D1833" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100071/nasdem-usul-ambang-batas-parlemen-di-atas-5-persen</t>
+        </is>
+      </c>
+    </row>
+    <row r="1834">
+      <c r="A1834" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1834" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1834" t="inlineStr">
+        <is>
+          <t>Langkah Dedi Mulyadi Satukan Gedung Sate-Gasibu Tuai Kritik</t>
+        </is>
+      </c>
+      <c r="D1834" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100070/langkah-dedi-mulyadi-satukan-gedung-sate-gasibu-tuai-kritik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1835">
+      <c r="A1835" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1835" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1835" t="inlineStr">
+        <is>
+          <t>Koalisi Sipil Desak Pemerintah Tunda Pembahasan PP Tugas TNI</t>
+        </is>
+      </c>
+      <c r="D1835" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100068/koalisi-sipil-desak-pemerintah-tunda-pembahasan-pp-tugas-tni</t>
+        </is>
+      </c>
+    </row>
+    <row r="1836">
+      <c r="A1836" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1836" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1836" t="inlineStr">
+        <is>
+          <t>15 Negara Siap Ramaikan Semarang Night Carnival 2026</t>
+        </is>
+      </c>
+      <c r="D1836" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100066/15-negara-siap-ramaikan-semarang-night-carnival-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1837">
+      <c r="A1837" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1837" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1837" t="inlineStr">
+        <is>
+          <t>BNI Rehabilitasi 50 Hektare Mangrove di Banyuwangi</t>
+        </is>
+      </c>
+      <c r="D1837" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100064/bni-rehabilitasi-50-hektare-mangrove-di-banyuwangi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1838">
+      <c r="A1838" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1838" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1838" t="inlineStr">
+        <is>
+          <t>5 Aplikasi Investasi Reksa Dana Terbaik Berdasarkan Profil Risiko</t>
+        </is>
+      </c>
+      <c r="D1838" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100063/5-aplikasi-investasi-reksa-dana-terbaik-berdasarkan-profil-risiko</t>
+        </is>
+      </c>
+    </row>
+    <row r="1839">
+      <c r="A1839" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1839" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1839" t="inlineStr">
+        <is>
+          <t>Komisioner Komnas HAM Kritik Putusan PTUN soal Perkara Fadli</t>
+        </is>
+      </c>
+      <c r="D1839" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100056/komisioner-komnas-ham-kritik-putusan-ptun-soal-perkara-fadli</t>
+        </is>
+      </c>
+    </row>
+    <row r="1840">
+      <c r="A1840" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1840" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1840" t="inlineStr">
+        <is>
+          <t>KPK Usul Capres-Cawapres Harus Kader Partai, PKB: Menarik</t>
+        </is>
+      </c>
+      <c r="D1840" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100053/kpk-usul-capres-cawapres-harus-kader-partai-pkb-menarik</t>
+        </is>
+      </c>
+    </row>
+    <row r="1841">
+      <c r="A1841" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1841" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1841" t="inlineStr">
+        <is>
+          <t>Jalan Panjang di Balik Solidaritas Lewat TKD untuk Pemulihan Banjir Sumatra</t>
+        </is>
+      </c>
+      <c r="D1841" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100052/jalan-panjang-di-balik-solidaritas-lewat-tkd-untuk-pemulihan-banjir-sumatra</t>
+        </is>
+      </c>
+    </row>
+    <row r="1842">
+      <c r="A1842" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1842" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1842" t="inlineStr">
+        <is>
+          <t>Raja Emas Indonesia, Tempat Aman untuk Semua Transaksi Emas</t>
+        </is>
+      </c>
+      <c r="D1842" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100051/raja-emas-indonesia-tempat-aman-untuk-semua-transaksi-emas</t>
+        </is>
+      </c>
+    </row>
+    <row r="1843">
+      <c r="A1843" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1843" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1843" t="inlineStr">
+        <is>
+          <t>PKB: Pembatasan Masa Jabatan Ketum Tak Jamin Atasi Korupsi</t>
+        </is>
+      </c>
+      <c r="D1843" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100045/pkb-pembatasan-masa-jabatan-ketum-tak-jamin-atasi-korupsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="1844">
+      <c r="A1844" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1844" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1844" t="inlineStr">
+        <is>
+          <t>Bank Jakarta Raih Indonesia 50 Best CEO Awards dan Indonesia Best COO Awards 2026</t>
+        </is>
+      </c>
+      <c r="D1844" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100037/bank-jakarta-raih-indonesia-50-best-ceo-awards-dan-indonesia-best-coo-awards-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="1845">
+      <c r="A1845" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1845" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1845" t="inlineStr">
+        <is>
+          <t>Menhum: Royalti Karya Jurnalistik Harus Masuk UU Hak Cipta</t>
+        </is>
+      </c>
+      <c r="D1845" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100035/menhum-royalti-karya-jurnalistik-harus-masuk-uu-hak-cipta</t>
+        </is>
+      </c>
+    </row>
+    <row r="1846">
+      <c r="A1846" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1846" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C1846" t="inlineStr">
+        <is>
+          <t>Bupati Blora Tekankan Peran GenRe dalam Pemetaan Potensi Remaja</t>
+        </is>
+      </c>
+      <c r="D1846" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100034/bupati-blora-tekankan-peran-genre-dalam-pemetaan-potensi-remaja</t>
+        </is>
+      </c>
+    </row>
+    <row r="1847">
+      <c r="A1847" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1847" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C1847" t="inlineStr">
+        <is>
+          <t>Indonesia pushes for South China Sea CoC this year</t>
+        </is>
+      </c>
+      <c r="D1847" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413449/indonesia-pushes-for-south-china-sea-coc-this-year</t>
+        </is>
+      </c>
+    </row>
+    <row r="1848">
+      <c r="A1848" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1848" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C1848" t="inlineStr">
+        <is>
+          <t>‘Concrete in Life 2025/26’ Winners Announced – Spectacular Photographs From Around the World</t>
+        </is>
+      </c>
+      <c r="D1848" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413448/concrete-in-life-2025-26-winners-announced-spectacular-photographs-from-around-the-world</t>
+        </is>
+      </c>
+    </row>
+    <row r="1849">
+      <c r="A1849" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1849" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C1849" t="inlineStr">
+        <is>
+          <t>Two tourists airlifted to safety after being trapped on Bali cliff</t>
+        </is>
+      </c>
+      <c r="D1849" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413444/two-tourists-airlifted-to-safety-after-being-trapped-on-bali-cliff</t>
+        </is>
+      </c>
+    </row>
+    <row r="1850">
+      <c r="A1850" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1850" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C1850" t="inlineStr">
+        <is>
+          <t>Indonesia seeks more teachers for Sekolah Rakyat expansion</t>
+        </is>
+      </c>
+      <c r="D1850" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413443/indonesia-seeks-more-teachers-for-sekolah-rakyat-expansion</t>
+        </is>
+      </c>
+    </row>
+    <row r="1851">
+      <c r="A1851" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1851" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C1851" t="inlineStr">
+        <is>
+          <t>Indonesia anti-graft body urges two-term limits for party chiefs</t>
+        </is>
+      </c>
+      <c r="D1851" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413441/indonesia-anti-graft-body-urges-two-term-limits-for-party-chiefs</t>
+        </is>
+      </c>
+    </row>
+    <row r="1852">
+      <c r="A1852" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1852" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1852" t="inlineStr">
+        <is>
+          <t>Govt ensures full support for Hajj pilgrims: Cabinet Secretary</t>
+        </is>
+      </c>
+      <c r="D1852" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413439/govt-ensures-full-support-for-hajj-pilgrims-cabinet-secretary</t>
+        </is>
+      </c>
+    </row>
+    <row r="1853">
+      <c r="A1853" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1853" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C1853" t="inlineStr">
+        <is>
+          <t>Defense Minister urges troops to maintain community harmony</t>
+        </is>
+      </c>
+      <c r="D1853" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413437/defense-minister-urges-troops-to-maintain-community-harmony</t>
+        </is>
+      </c>
+    </row>
+    <row r="1854">
+      <c r="A1854" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1854" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1854" t="inlineStr">
+        <is>
+          <t>Pupuk Indonesia ready to export urea to Australia amid global demand</t>
+        </is>
+      </c>
+      <c r="D1854" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413435/pupuk-indonesia-ready-to-export-urea-to-australia-amid-global-demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="1855">
+      <c r="A1855" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1855" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C1855" t="inlineStr">
+        <is>
+          <t>Indonesia expands free meals to tackle stunting risk: minister</t>
+        </is>
+      </c>
+      <c r="D1855" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413433/indonesia-expands-free-meals-to-tackle-stunting-risk-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="1856">
+      <c r="A1856" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1856" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C1856" t="inlineStr">
+        <is>
+          <t>Whale Cloud and AGIBOT Announce Strategic Partnership to Accelerate Global Expansion of Embodied AI</t>
+        </is>
+      </c>
+      <c r="D1856" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413431/whale-cloud-and-agibot-announce-strategic-partnership-to-accelerate-global-expansion-of-embodied-ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="1857">
+      <c r="A1857" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1857" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C1857" t="inlineStr">
+        <is>
+          <t>Indonesian Police foil attempted smuggling of 68 migrants to Malaysia</t>
+        </is>
+      </c>
+      <c r="D1857" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413427/indonesian-police-foil-attempted-smuggling-of-68-migrants-to-malaysia</t>
+        </is>
+      </c>
+    </row>
+    <row r="1858">
+      <c r="A1858" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1858" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C1858" t="inlineStr">
+        <is>
+          <t>Indonesia's BRIN develops railway technologies to boost transport</t>
+        </is>
+      </c>
+      <c r="D1858" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413425/indonesias-brin-develops-railway-technologies-to-boost-transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="1859">
+      <c r="A1859" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1859" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C1859" t="inlineStr">
+        <is>
+          <t>Danantara waiting for Hajj Village land tender results</t>
+        </is>
+      </c>
+      <c r="D1859" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413423/danantara-waiting-for-hajj-village-land-tender-results</t>
+        </is>
+      </c>
+    </row>
+    <row r="1860">
+      <c r="A1860" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1860" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C1860" t="inlineStr">
+        <is>
+          <t>Indonesia to reopen Mount Semeru climbing routes on April 24</t>
+        </is>
+      </c>
+      <c r="D1860" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413421/indonesia-to-reopen-mount-semeru-climbing-routes-on-april-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="1861">
+      <c r="A1861" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B1861" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C1861" t="inlineStr">
+        <is>
+          <t>EZVIZ joins the United Nations Global Compact, starting a new chapter of its unwavering journey</t>
+        </is>
+      </c>
+      <c r="D1861" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413417/ezviz-joins-the-united-nations-global-compact-starting-a-new-chapter-of-its-unwavering-journey</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D1801"/>
+  <autoFilter ref="A1:D1861"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -41873,6 +43193,66 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1799" r:id="rId1798"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1800" r:id="rId1799"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1801" r:id="rId1800"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1802" r:id="rId1801"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1803" r:id="rId1802"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1804" r:id="rId1803"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1805" r:id="rId1804"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1806" r:id="rId1805"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1807" r:id="rId1806"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1808" r:id="rId1807"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1809" r:id="rId1808"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1810" r:id="rId1809"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1811" r:id="rId1810"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1812" r:id="rId1811"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1813" r:id="rId1812"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1814" r:id="rId1813"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1815" r:id="rId1814"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1816" r:id="rId1815"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1817" r:id="rId1816"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1818" r:id="rId1817"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1819" r:id="rId1818"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1820" r:id="rId1819"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1821" r:id="rId1820"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1822" r:id="rId1821"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1823" r:id="rId1822"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1824" r:id="rId1823"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1825" r:id="rId1824"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1826" r:id="rId1825"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1827" r:id="rId1826"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1828" r:id="rId1827"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1829" r:id="rId1828"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1830" r:id="rId1829"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1831" r:id="rId1830"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1832" r:id="rId1831"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1833" r:id="rId1832"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1834" r:id="rId1833"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1835" r:id="rId1834"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1836" r:id="rId1835"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1837" r:id="rId1836"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1838" r:id="rId1837"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1839" r:id="rId1838"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1840" r:id="rId1839"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1841" r:id="rId1840"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1842" r:id="rId1841"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1843" r:id="rId1842"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1844" r:id="rId1843"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1845" r:id="rId1844"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1846" r:id="rId1845"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1847" r:id="rId1846"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1848" r:id="rId1847"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1849" r:id="rId1848"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1850" r:id="rId1849"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1851" r:id="rId1850"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1852" r:id="rId1851"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1853" r:id="rId1852"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1854" r:id="rId1853"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1855" r:id="rId1854"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1856" r:id="rId1855"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1857" r:id="rId1856"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1858" r:id="rId1857"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1859" r:id="rId1858"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1860" r:id="rId1859"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D1861" r:id="rId1860"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-24
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$2018</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$2092</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2018"/>
+  <dimension ref="A1:D2092"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -44844,8 +44844,1636 @@
         </is>
       </c>
     </row>
+    <row r="2019">
+      <c r="A2019" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2019" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2019" t="inlineStr">
+        <is>
+          <t>Dua Kali Tertunda, Ashanty: Insyaallah Berangkat Haji Mei Tahun Ini</t>
+        </is>
+      </c>
+      <c r="D2019" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8457674/dua-kali-tertunda-ashanty-insyaallah-berangkat-haji-mei-tahun-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="2020">
+      <c r="A2020" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2020" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2020" t="inlineStr">
+        <is>
+          <t>Hingga Hari Kedua Haji 2026, 6.737 Jemaah dari 17 Kloter Sudah di Madinah</t>
+        </is>
+      </c>
+      <c r="D2020" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8459013/hingga-hari-kedua-haji-2026-6-737-jemaah-dari-17-kloter-sudah-di-madinah</t>
+        </is>
+      </c>
+    </row>
+    <row r="2021">
+      <c r="A2021" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2021" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2021" t="inlineStr">
+        <is>
+          <t>8 Doa untuk Jemaah Haji dari Berangkat hingga Pulang, Lengkap Arab dan Artinya</t>
+        </is>
+      </c>
+      <c r="D2021" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/doa-dan-hadits/d-8458664/8-doa-untuk-jemaah-haji-dari-berangkat-hingga-pulang-lengkap-arab-dan-artinya</t>
+        </is>
+      </c>
+    </row>
+    <row r="2022">
+      <c r="A2022" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2022" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2022" t="inlineStr">
+        <is>
+          <t>Tata Cara Sholat di Pesawat untuk Jemaah Haji</t>
+        </is>
+      </c>
+      <c r="D2022" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/infografis/d-8457904/tata-cara-sholat-di-pesawat-untuk-jemaah-haji</t>
+        </is>
+      </c>
+    </row>
+    <row r="2023">
+      <c r="A2023" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2023" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2023" t="inlineStr">
+        <is>
+          <t>Video Life Hack Haji 2026: Gak Perlu Angkut Koper Sendiri!</t>
+        </is>
+      </c>
+      <c r="D2023" s="2" t="inlineStr">
+        <is>
+          <t>https://20.detik.com/detikupdate/20260424-260424011/video-life-hack-haji-2026-gak-perlu-angkut-koper-sendiri</t>
+        </is>
+      </c>
+    </row>
+    <row r="2024">
+      <c r="A2024" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2024" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C2024" t="inlineStr">
+        <is>
+          <t>Video: Menakar Peluang Tempe Jadi 'Superfood' Masa Depan</t>
+        </is>
+      </c>
+      <c r="D2024" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/detiktv/d-8459018/video-menakar-peluang-tempe-jadi-superfood-masa-depan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2025">
+      <c r="A2025" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2025" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C2025" t="inlineStr">
+        <is>
+          <t>Detik-detik Pelaku Teror Bakar Mobil Kades Hoho Pakai Molotov</t>
+        </is>
+      </c>
+      <c r="D2025" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/jateng/berita/d-8458967/detik-detik-pelaku-teror-bakar-mobil-kades-hoho-pakai-molotov</t>
+        </is>
+      </c>
+    </row>
+    <row r="2026">
+      <c r="A2026" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2026" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2026" t="inlineStr">
+        <is>
+          <t>Perpanjang STNK Wajib Ada KTP Pemilik Lama Bikin Sulit, Warga Banyak yang Ngeluh</t>
+        </is>
+      </c>
+      <c r="D2026" s="2" t="inlineStr">
+        <is>
+          <t>https://oto.detik.com/berita/d-8458875/perpanjang-stnk-wajib-ada-ktp-pemilik-lama-bikin-sulit-warga-banyak-yang-ngeluh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2027">
+      <c r="A2027" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2027" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C2027" t="inlineStr">
+        <is>
+          <t>Rencana Denada Ajak Ressa Rizky ke Singapura Temui Aisha</t>
+        </is>
+      </c>
+      <c r="D2027" s="2" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8457351/rencana-denada-ajak-ressa-rizky-ke-singapura-temui-aisha</t>
+        </is>
+      </c>
+    </row>
+    <row r="2028">
+      <c r="A2028" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2028" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C2028" t="inlineStr">
+        <is>
+          <t>Ahmad Dhani Bicara soal Rencana Ngunduh Mantu di Pernikahan El-Syifa</t>
+        </is>
+      </c>
+      <c r="D2028" s="2" t="inlineStr">
+        <is>
+          <t>https://hot.detik.com/celeb/d-8457754/ahmad-dhani-bicara-soal-rencana-ngunduh-mantu-di-pernikahan-el-syifa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2029">
+      <c r="A2029" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2029" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2029" t="inlineStr">
+        <is>
+          <t>AS Sita Kapal Tanker Diduga Selundupkan Minyak Iran</t>
+        </is>
+      </c>
+      <c r="D2029" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8459056/as-sita-kapal-tanker-diduga-selundupkan-minyak-iran</t>
+        </is>
+      </c>
+    </row>
+    <row r="2030">
+      <c r="A2030" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2030" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2030" t="inlineStr">
+        <is>
+          <t>Kapal Induk Ketiga AS Tiba di Kawasan Timur Tengah</t>
+        </is>
+      </c>
+      <c r="D2030" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8458970/kapal-induk-ketiga-as-tiba-di-kawasan-timur-tengah</t>
+        </is>
+      </c>
+    </row>
+    <row r="2031">
+      <c r="A2031" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2031" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2031" t="inlineStr">
+        <is>
+          <t>Isu Liar Trump Coba-coba Kode Nuklir</t>
+        </is>
+      </c>
+      <c r="D2031" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/internasional/d-8458859/isu-liar-trump-coba-coba-kode-nuklir</t>
+        </is>
+      </c>
+    </row>
+    <row r="2032">
+      <c r="A2032" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2032" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C2032" t="inlineStr">
+        <is>
+          <t>Utusan Trump Minta Iran Diganti Italia di Piala Dunia 2026, Apa Respon FIFA?</t>
+        </is>
+      </c>
+      <c r="D2032" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/bola-dunia/d-8458672/utusan-trump-minta-iran-diganti-italia-di-piala-dunia-2026-apa-respon-fifa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2033">
+      <c r="A2033" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2033" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2033" t="inlineStr">
+        <is>
+          <t>Semarang Kian Inklusif, Masuk Tiga Besar Kota Toleran Nasional</t>
+        </is>
+      </c>
+      <c r="D2033" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100119/semarang-kian-inklusif-masuk-tiga-besar-kota-toleran-nasional</t>
+        </is>
+      </c>
+    </row>
+    <row r="2034">
+      <c r="A2034" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2034" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2034" t="inlineStr">
+        <is>
+          <t>Mantan Panglima TNI Berkumpul di Gedung Kemenhan</t>
+        </is>
+      </c>
+      <c r="D2034" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100118/mantan-panglima-tni-berkumpul-di-gedung-kemenhan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2035">
+      <c r="A2035" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2035" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2035" t="inlineStr">
+        <is>
+          <t>PAN Minta KPK Tak Ikut Campur soal Masa Jabatan Ketum Partai</t>
+        </is>
+      </c>
+      <c r="D2035" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100116/pan-minta-kpk-tak-ikut-campur-soal-masa-jabatan-ketum-partai</t>
+        </is>
+      </c>
+    </row>
+    <row r="2036">
+      <c r="A2036" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2036" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2036" t="inlineStr">
+        <is>
+          <t>Kata PDIP, NasDem, dan PKB Soal Masa Jabatan Ketum Dibatasi</t>
+        </is>
+      </c>
+      <c r="D2036" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100103/kata-pdip-nasdem-dan-pkb-soal-masa-jabatan-ketum-dibatasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2037">
+      <c r="A2037" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2037" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2037" t="inlineStr">
+        <is>
+          <t>PDIP Minta Revisi UU Pemilu Dibahas Tahun Ini</t>
+        </is>
+      </c>
+      <c r="D2037" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100100/pdip-minta-revisi-uu-pemilu-dibahas-tahun-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="2038">
+      <c r="A2038" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2038" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2038" t="inlineStr">
+        <is>
+          <t>Kemenag Buka Pendaftaran Beasiswa Indonesia Bangkit 2026</t>
+        </is>
+      </c>
+      <c r="D2038" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100093/kemenag-buka-pendaftaran-beasiswa-indonesia-bangkit-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2039">
+      <c r="A2039" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2039" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2039" t="inlineStr">
+        <is>
+          <t>Mendagri Minta Pemda Bebaskan Pajak Kendaraan Listrik</t>
+        </is>
+      </c>
+      <c r="D2039" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100076/mendagri-minta-pemda-bebaskan-pajak-kendaraan-listrik</t>
+        </is>
+      </c>
+    </row>
+    <row r="2040">
+      <c r="A2040" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2040" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2040" t="inlineStr">
+        <is>
+          <t>NasDem Usul Ambang Batas Parlemen di Atas 5 Persen</t>
+        </is>
+      </c>
+      <c r="D2040" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100071/nasdem-usul-ambang-batas-parlemen-di-atas-5-persen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2041">
+      <c r="A2041" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2041" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2041" t="inlineStr">
+        <is>
+          <t>Langkah Dedi Mulyadi Satukan Gedung Sate-Gasibu Tuai Kritik</t>
+        </is>
+      </c>
+      <c r="D2041" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100070/langkah-dedi-mulyadi-satukan-gedung-sate-gasibu-tuai-kritik</t>
+        </is>
+      </c>
+    </row>
+    <row r="2042">
+      <c r="A2042" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2042" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2042" t="inlineStr">
+        <is>
+          <t>Koalisi Sipil Desak Pemerintah Tunda Pembahasan PP Tugas TNI</t>
+        </is>
+      </c>
+      <c r="D2042" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100068/koalisi-sipil-desak-pemerintah-tunda-pembahasan-pp-tugas-tni</t>
+        </is>
+      </c>
+    </row>
+    <row r="2043">
+      <c r="A2043" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2043" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C2043" t="inlineStr">
+        <is>
+          <t>15 Negara Siap Ramaikan Semarang Night Carnival 2026</t>
+        </is>
+      </c>
+      <c r="D2043" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100066/15-negara-siap-ramaikan-semarang-night-carnival-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2044">
+      <c r="A2044" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2044" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C2044" t="inlineStr">
+        <is>
+          <t>BNI Rehabilitasi 50 Hektare Mangrove di Banyuwangi</t>
+        </is>
+      </c>
+      <c r="D2044" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100064/bni-rehabilitasi-50-hektare-mangrove-di-banyuwangi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2045">
+      <c r="A2045" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2045" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C2045" t="inlineStr">
+        <is>
+          <t>5 Aplikasi Investasi Reksa Dana Terbaik Berdasarkan Profil Risiko</t>
+        </is>
+      </c>
+      <c r="D2045" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100063/5-aplikasi-investasi-reksa-dana-terbaik-berdasarkan-profil-risiko</t>
+        </is>
+      </c>
+    </row>
+    <row r="2046">
+      <c r="A2046" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2046" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2046" t="inlineStr">
+        <is>
+          <t>Komisioner Komnas HAM Kritik Putusan PTUN soal Perkara Fadli</t>
+        </is>
+      </c>
+      <c r="D2046" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100056/komisioner-komnas-ham-kritik-putusan-ptun-soal-perkara-fadli</t>
+        </is>
+      </c>
+    </row>
+    <row r="2047">
+      <c r="A2047" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2047" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2047" t="inlineStr">
+        <is>
+          <t>KPK Usul Capres-Cawapres Harus Kader Partai, PKB: Menarik</t>
+        </is>
+      </c>
+      <c r="D2047" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100053/kpk-usul-capres-cawapres-harus-kader-partai-pkb-menarik</t>
+        </is>
+      </c>
+    </row>
+    <row r="2048">
+      <c r="A2048" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2048" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C2048" t="inlineStr">
+        <is>
+          <t>Jalan Panjang di Balik Solidaritas Lewat TKD untuk Pemulihan Banjir Sumatra</t>
+        </is>
+      </c>
+      <c r="D2048" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100052/jalan-panjang-di-balik-solidaritas-lewat-tkd-untuk-pemulihan-banjir-sumatra</t>
+        </is>
+      </c>
+    </row>
+    <row r="2049">
+      <c r="A2049" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2049" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C2049" t="inlineStr">
+        <is>
+          <t>Raja Emas Indonesia, Tempat Aman untuk Semua Transaksi Emas</t>
+        </is>
+      </c>
+      <c r="D2049" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100051/raja-emas-indonesia-tempat-aman-untuk-semua-transaksi-emas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2050">
+      <c r="A2050" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2050" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2050" t="inlineStr">
+        <is>
+          <t>PKB: Pembatasan Masa Jabatan Ketum Tak Jamin Atasi Korupsi</t>
+        </is>
+      </c>
+      <c r="D2050" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100045/pkb-pembatasan-masa-jabatan-ketum-tak-jamin-atasi-korupsi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2051">
+      <c r="A2051" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2051" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C2051" t="inlineStr">
+        <is>
+          <t>Bank Jakarta Raih Indonesia 50 Best CEO Awards dan Indonesia Best COO Awards 2026</t>
+        </is>
+      </c>
+      <c r="D2051" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100037/bank-jakarta-raih-indonesia-50-best-ceo-awards-dan-indonesia-best-coo-awards-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2052">
+      <c r="A2052" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2052" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2052" t="inlineStr">
+        <is>
+          <t>Menhum: Royalti Karya Jurnalistik Harus Masuk UU Hak Cipta</t>
+        </is>
+      </c>
+      <c r="D2052" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100035/menhum-royalti-karya-jurnalistik-harus-masuk-uu-hak-cipta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2053">
+      <c r="A2053" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2053" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2053" t="inlineStr">
+        <is>
+          <t>British national in court over 1.4kg Bali cocaine haul</t>
+        </is>
+      </c>
+      <c r="D2053" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413457/british-national-in-court-over-14kg-bali-cocaine-haul</t>
+        </is>
+      </c>
+    </row>
+    <row r="2054">
+      <c r="A2054" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2054" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C2054" t="inlineStr">
+        <is>
+          <t>Kioxia Introduces New Mainstream KIOXIA BG8 Series SSDs for PC OEMs</t>
+        </is>
+      </c>
+      <c r="D2054" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413456/kioxia-introduces-new-mainstream-kioxia-bg8-series-ssds-for-pc-oems</t>
+        </is>
+      </c>
+    </row>
+    <row r="2055">
+      <c r="A2055" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2055" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2055" t="inlineStr">
+        <is>
+          <t>Accertify Launches Global Air Travel Fraud Report Revealing Where Booking-Stage Pressure Is Most Concentrated</t>
+        </is>
+      </c>
+      <c r="D2055" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413452/accertify-launches-global-air-travel-fraud-report-revealing-where-booking-stage-pressure-is-most-concentrated</t>
+        </is>
+      </c>
+    </row>
+    <row r="2056">
+      <c r="A2056" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2056" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2056" t="inlineStr">
+        <is>
+          <t>Indonesia pushes for South China Sea CoC this year</t>
+        </is>
+      </c>
+      <c r="D2056" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413449/indonesia-pushes-for-south-china-sea-coc-this-year</t>
+        </is>
+      </c>
+    </row>
+    <row r="2057">
+      <c r="A2057" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2057" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C2057" t="inlineStr">
+        <is>
+          <t>‘Concrete in Life 2025/26’ Winners Announced – Spectacular Photographs From Around the World</t>
+        </is>
+      </c>
+      <c r="D2057" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413448/concrete-in-life-2025-26-winners-announced-spectacular-photographs-from-around-the-world</t>
+        </is>
+      </c>
+    </row>
+    <row r="2058">
+      <c r="A2058" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2058" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C2058" t="inlineStr">
+        <is>
+          <t>Two tourists airlifted to safety after being trapped on Bali cliff</t>
+        </is>
+      </c>
+      <c r="D2058" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413444/two-tourists-airlifted-to-safety-after-being-trapped-on-bali-cliff</t>
+        </is>
+      </c>
+    </row>
+    <row r="2059">
+      <c r="A2059" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2059" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2059" t="inlineStr">
+        <is>
+          <t>Indonesia seeks more teachers for Sekolah Rakyat expansion</t>
+        </is>
+      </c>
+      <c r="D2059" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413443/indonesia-seeks-more-teachers-for-sekolah-rakyat-expansion</t>
+        </is>
+      </c>
+    </row>
+    <row r="2060">
+      <c r="A2060" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2060" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2060" t="inlineStr">
+        <is>
+          <t>Indonesia anti-graft body urges two-term limits for party chiefs</t>
+        </is>
+      </c>
+      <c r="D2060" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413441/indonesia-anti-graft-body-urges-two-term-limits-for-party-chiefs</t>
+        </is>
+      </c>
+    </row>
+    <row r="2061">
+      <c r="A2061" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2061" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2061" t="inlineStr">
+        <is>
+          <t>Govt ensures full support for Hajj pilgrims: Cabinet Secretary</t>
+        </is>
+      </c>
+      <c r="D2061" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413439/govt-ensures-full-support-for-hajj-pilgrims-cabinet-secretary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2062">
+      <c r="A2062" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2062" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2062" t="inlineStr">
+        <is>
+          <t>Defense Minister urges troops to maintain community harmony</t>
+        </is>
+      </c>
+      <c r="D2062" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413437/defense-minister-urges-troops-to-maintain-community-harmony</t>
+        </is>
+      </c>
+    </row>
+    <row r="2063">
+      <c r="A2063" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2063" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C2063" t="inlineStr">
+        <is>
+          <t>Pupuk Indonesia ready to export urea to Australia amid global demand</t>
+        </is>
+      </c>
+      <c r="D2063" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413435/pupuk-indonesia-ready-to-export-urea-to-australia-amid-global-demand</t>
+        </is>
+      </c>
+    </row>
+    <row r="2064">
+      <c r="A2064" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2064" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C2064" t="inlineStr">
+        <is>
+          <t>Indonesia expands free meals to tackle stunting risk: minister</t>
+        </is>
+      </c>
+      <c r="D2064" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413433/indonesia-expands-free-meals-to-tackle-stunting-risk-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="2065">
+      <c r="A2065" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2065" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C2065" t="inlineStr">
+        <is>
+          <t>Whale Cloud and AGIBOT Announce Strategic Partnership to Accelerate Global Expansion of Embodied AI</t>
+        </is>
+      </c>
+      <c r="D2065" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413431/whale-cloud-and-agibot-announce-strategic-partnership-to-accelerate-global-expansion-of-embodied-ai</t>
+        </is>
+      </c>
+    </row>
+    <row r="2066">
+      <c r="A2066" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2066" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2066" t="inlineStr">
+        <is>
+          <t>Indonesian Police foil attempted smuggling of 68 migrants to Malaysia</t>
+        </is>
+      </c>
+      <c r="D2066" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413427/indonesian-police-foil-attempted-smuggling-of-68-migrants-to-malaysia</t>
+        </is>
+      </c>
+    </row>
+    <row r="2067">
+      <c r="A2067" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2067" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2067" t="inlineStr">
+        <is>
+          <t>Indonesia's BRIN develops railway technologies to boost transport</t>
+        </is>
+      </c>
+      <c r="D2067" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413425/indonesias-brin-develops-railway-technologies-to-boost-transport</t>
+        </is>
+      </c>
+    </row>
+    <row r="2068">
+      <c r="A2068" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2068" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2068" t="inlineStr">
+        <is>
+          <t>Danantara waiting for Hajj Village land tender results</t>
+        </is>
+      </c>
+      <c r="D2068" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413423/danantara-waiting-for-hajj-village-land-tender-results</t>
+        </is>
+      </c>
+    </row>
+    <row r="2069">
+      <c r="A2069" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2069" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C2069" t="inlineStr">
+        <is>
+          <t>Indonesia to reopen Mount Semeru climbing routes on April 24</t>
+        </is>
+      </c>
+      <c r="D2069" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413421/indonesia-to-reopen-mount-semeru-climbing-routes-on-april-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="2070">
+      <c r="A2070" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2070" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C2070" t="inlineStr">
+        <is>
+          <t>EZVIZ joins the United Nations Global Compact, starting a new chapter of its unwavering journey</t>
+        </is>
+      </c>
+      <c r="D2070" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413417/ezviz-joins-the-united-nations-global-compact-starting-a-new-chapter-of-its-unwavering-journey</t>
+        </is>
+      </c>
+    </row>
+    <row r="2071">
+      <c r="A2071" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2071" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2071" t="inlineStr">
+        <is>
+          <t>Indonesia, Philippines strengthen ties in economy, security</t>
+        </is>
+      </c>
+      <c r="D2071" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413413/indonesia-philippines-strengthen-ties-in-economy-security</t>
+        </is>
+      </c>
+    </row>
+    <row r="2072">
+      <c r="A2072" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2072" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C2072" t="inlineStr">
+        <is>
+          <t>Xinhua Silk Road: 3TREES expands global reach amid eye-catching stone paint sales</t>
+        </is>
+      </c>
+      <c r="D2072" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413411/xinhua-silk-road-3trees-expands-global-reach-amid-eye-catching-stone-paint-sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="2073">
+      <c r="A2073" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2073" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2073" t="inlineStr">
+        <is>
+          <t>Kejagung Periksa Pejabat ESDM terkait Kasus Tambang Ilegal Samin Tan</t>
+        </is>
+      </c>
+      <c r="D2073" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322382/kejagung-periksa-pejabat-esdm-terkait-kasus-tambang-ilegal-samin-tan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2074">
+      <c r="A2074" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2074" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C2074" t="inlineStr">
+        <is>
+          <t>El Nino 2026 Diprediksi Lebih Panjang, Warga Jakarta Diminta Waspada 3 Hal Ini</t>
+        </is>
+      </c>
+      <c r="D2074" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322352/el-nino-2026-diprediksi-lebih-panjang-warga-jakarta-diminta-waspada-3-hal-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="2075">
+      <c r="A2075" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2075" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2075" t="inlineStr">
+        <is>
+          <t>Wamendagri Bima Arya Dorong Sinergi Sipil-Militer Hadapi Tantangan Global</t>
+        </is>
+      </c>
+      <c r="D2075" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322342/wamendagri-bima-arya-dorong-sinergi-sipil-militer-hadapi-tantangan-global</t>
+        </is>
+      </c>
+    </row>
+    <row r="2076">
+      <c r="A2076" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2076" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C2076" t="inlineStr">
+        <is>
+          <t>Dari Duka ke Harapan, Huntara Bener Meriah Pulihkan Senyum Penyintas</t>
+        </is>
+      </c>
+      <c r="D2076" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322340/dari-duka-ke-harapan-huntara-bener-meriah-pulihkan-senyum-penyintas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2077">
+      <c r="A2077" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2077" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2077" t="inlineStr">
+        <is>
+          <t>Top 3 News: Semua Moda Transportasi Umum di Jakarta Gratis pada 24 April 2026</t>
+        </is>
+      </c>
+      <c r="D2077" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322290/top-3-news-semua-moda-transportasi-umum-di-jakarta-gratis-pada-24-april-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2078">
+      <c r="A2078" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2078" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C2078" t="inlineStr">
+        <is>
+          <t>Kasatgas PRR Tinjau Sinkhole Aceh Tengah, Apresiasi Kinerja Tim Penanganan</t>
+        </is>
+      </c>
+      <c r="D2078" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322336/kasatgas-prr-tinjau-sinkhole-aceh-tengah-apresiasi-kinerja-tim-penanganan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2079">
+      <c r="A2079" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2079" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2079" t="inlineStr">
+        <is>
+          <t>Pengakuan Ustadz Khalid Basalamah Usai Diperiksa KPK</t>
+        </is>
+      </c>
+      <c r="D2079" s="2" t="inlineStr">
+        <is>
+          <t>https://enamplus.liputan6.com/news/read/6322334/pengakuan-ustadz-khalid-basalamah-usai-diperiksa-kpk</t>
+        </is>
+      </c>
+    </row>
+    <row r="2080">
+      <c r="A2080" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2080" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2080" t="inlineStr">
+        <is>
+          <t>24 April Diperingati sebagai Hari Apa? Yuk Simak Sejarah hingga Tujuan Hari Angkutan Nasional</t>
+        </is>
+      </c>
+      <c r="D2080" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322291/24-april-diperingati-sebagai-hari-apa-yuk-simak-sejarah-hingga-tujuan-hari-angkutan-nasional</t>
+        </is>
+      </c>
+    </row>
+    <row r="2081">
+      <c r="A2081" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2081" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2081" t="inlineStr">
+        <is>
+          <t>Said Aqil Siroj: Butuh Rekalibrasi Spiritual untuk Dunia Lebih Baik</t>
+        </is>
+      </c>
+      <c r="D2081" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322309/said-aqil-siroj-butuh-rekalibrasi-spiritual-untuk-dunia-lebih-baik</t>
+        </is>
+      </c>
+    </row>
+    <row r="2082">
+      <c r="A2082" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2082" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2082" t="inlineStr">
+        <is>
+          <t>Ganjil Genap Jakarta Tetap Berlaku Jelang Akhir Pekan, Jumat 24 April 2026</t>
+        </is>
+      </c>
+      <c r="D2082" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322288/ganjil-genap-jakarta-tetap-berlaku-jelang-akhir-pekan-jumat-24-april-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2083">
+      <c r="A2083" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2083" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C2083" t="inlineStr">
+        <is>
+          <t>Cuaca Hari Ini Jumat 24 April 2026: Pagi Cerah, Jabodetabek Siang hingga Malam Mayoritas Bakal Hujan</t>
+        </is>
+      </c>
+      <c r="D2083" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322112/cuaca-hari-ini-jumat-24-april-2026-pagi-cerah-jabodetabek-siang-hingga-malam-mayoritas-bakal-hujan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2084">
+      <c r="A2084" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2084" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2084" t="inlineStr">
+        <is>
+          <t>Kejagung: Handry Sulfian Setoran Bulanan dari Samin Tan untuk Loloskan Izin Berlayar</t>
+        </is>
+      </c>
+      <c r="D2084" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322280/kejagung-handry-sulfian-setoran-bulanan-dari-samin-tan-untuk-loloskan-izin-berlayar</t>
+        </is>
+      </c>
+    </row>
+    <row r="2085">
+      <c r="A2085" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2085" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C2085" t="inlineStr">
+        <is>
+          <t>DKI Tebar Diskon PBB-P2 hingga 10 Persen pada 2026, Ini Besarannya</t>
+        </is>
+      </c>
+      <c r="D2085" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322163/dki-tebar-diskon-pbb-p2-hingga-10-persen-pada-2026-ini-besarannya</t>
+        </is>
+      </c>
+    </row>
+    <row r="2086">
+      <c r="A2086" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2086" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2086" t="inlineStr">
+        <is>
+          <t>Polda Metro Periksa Anggota Polsek Cimanggis, Diduga Broker Proyek di Bekasi</t>
+        </is>
+      </c>
+      <c r="D2086" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322255/polda-metro-periksa-anggota-polsek-cimanggis-diduga-broker-proyek-di-bekasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2087">
+      <c r="A2087" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2087" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2087" t="inlineStr">
+        <is>
+          <t>Legislator NasDem Setuju Capres dari Internal Partai: Ada Tanggung Jawab Moral</t>
+        </is>
+      </c>
+      <c r="D2087" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322253/legislator-nasdem-setuju-capres-dari-internal-partai-ada-tanggung-jawab-moral</t>
+        </is>
+      </c>
+    </row>
+    <row r="2088">
+      <c r="A2088" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2088" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C2088" t="inlineStr">
+        <is>
+          <t>Gunung Slamet Berstatus Waspada: Suhu Kawah Meningkat Drastis dan Radius Aman Diperluas</t>
+        </is>
+      </c>
+      <c r="D2088" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322258/gunung-slamet-berstatus-waspada-suhu-kawah-meningkat-drastis-dan-radius-aman-diperluas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2089">
+      <c r="A2089" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2089" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C2089" t="inlineStr">
+        <is>
+          <t>Penanaman Ribuan Bibit Pohon Mangrove di Kawasan Pesisir Rusunawa Marunda Jakut</t>
+        </is>
+      </c>
+      <c r="D2089" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322198/penanaman-ribuan-bibit-pohon-mangrove-di-kawasan-pesisir-rusunawa-marunda-jakut</t>
+        </is>
+      </c>
+    </row>
+    <row r="2090">
+      <c r="A2090" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2090" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2090" t="inlineStr">
+        <is>
+          <t>Sidang Kasus Chromebook, Nadiem Hadirkan 7 Guru dari Aceh-Papua Jadi Saksi</t>
+        </is>
+      </c>
+      <c r="D2090" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322264/sidang-kasus-chromebook-nadiem-hadirkan-7-guru-dari-aceh-papua-jadi-saksi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2091">
+      <c r="A2091" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2091" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2091" t="inlineStr">
+        <is>
+          <t>Ditjen Imigrasi Deportasi Buronan Warga Negara AS</t>
+        </is>
+      </c>
+      <c r="D2091" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322239/ditjen-imigrasi-deportasi-buronan-warga-negara-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="2092">
+      <c r="A2092" t="inlineStr">
+        <is>
+          <t>Friday, 24 April 2026</t>
+        </is>
+      </c>
+      <c r="B2092" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2092" t="inlineStr">
+        <is>
+          <t>Kejagung Tetapkan 3 Tersangka Baru Kasus Pengelolaan Tambang Ilegal Samin Tan</t>
+        </is>
+      </c>
+      <c r="D2092" s="2" t="inlineStr">
+        <is>
+          <t>https://www.liputan6.com/news/read/6322219/kejagung-tetapkan-3-tersangka-baru-kasus-pengelolaan-tambang-ilegal-samin-tan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D2018"/>
+  <autoFilter ref="A1:D2092"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -46864,6 +48492,80 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2016" r:id="rId2015"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2017" r:id="rId2016"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2018" r:id="rId2017"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2019" r:id="rId2018"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2020" r:id="rId2019"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2021" r:id="rId2020"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2022" r:id="rId2021"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2023" r:id="rId2022"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2024" r:id="rId2023"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2025" r:id="rId2024"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2026" r:id="rId2025"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2027" r:id="rId2026"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2028" r:id="rId2027"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2029" r:id="rId2028"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2030" r:id="rId2029"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2031" r:id="rId2030"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2032" r:id="rId2031"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2033" r:id="rId2032"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2034" r:id="rId2033"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2035" r:id="rId2034"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2036" r:id="rId2035"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2037" r:id="rId2036"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2038" r:id="rId2037"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2039" r:id="rId2038"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2040" r:id="rId2039"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2041" r:id="rId2040"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2042" r:id="rId2041"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2043" r:id="rId2042"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2044" r:id="rId2043"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2045" r:id="rId2044"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2046" r:id="rId2045"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2047" r:id="rId2046"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2048" r:id="rId2047"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2049" r:id="rId2048"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2050" r:id="rId2049"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2051" r:id="rId2050"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2052" r:id="rId2051"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2053" r:id="rId2052"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2054" r:id="rId2053"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2055" r:id="rId2054"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2056" r:id="rId2055"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2057" r:id="rId2056"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2058" r:id="rId2057"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2059" r:id="rId2058"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2060" r:id="rId2059"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2061" r:id="rId2060"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2062" r:id="rId2061"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2063" r:id="rId2062"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2064" r:id="rId2063"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2065" r:id="rId2064"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2066" r:id="rId2065"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2067" r:id="rId2066"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2068" r:id="rId2067"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2069" r:id="rId2068"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2070" r:id="rId2069"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2071" r:id="rId2070"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2072" r:id="rId2071"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2073" r:id="rId2072"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2074" r:id="rId2073"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2075" r:id="rId2074"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2076" r:id="rId2075"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2077" r:id="rId2076"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2078" r:id="rId2077"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2079" r:id="rId2078"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2080" r:id="rId2079"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2081" r:id="rId2080"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2082" r:id="rId2081"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2083" r:id="rId2082"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2084" r:id="rId2083"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2085" r:id="rId2084"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2086" r:id="rId2085"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2087" r:id="rId2086"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2088" r:id="rId2087"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2089" r:id="rId2088"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2090" r:id="rId2089"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2091" r:id="rId2090"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2092" r:id="rId2091"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-25
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$2166</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$2239</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2166"/>
+  <dimension ref="A1:D2239"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -48100,8 +48100,1614 @@
         </is>
       </c>
     </row>
+    <row r="2167">
+      <c r="A2167" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2167" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2167" t="inlineStr">
+        <is>
+          <t>Ketatnya 'Checking' Bagasi Jemaah Haji Indonesia di Madinah</t>
+        </is>
+      </c>
+      <c r="D2167" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8461160/ketatnya-checking-bagasi-jemaah-haji-indonesia-di-madinah</t>
+        </is>
+      </c>
+    </row>
+    <row r="2168">
+      <c r="A2168" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2168" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2168" t="inlineStr">
+        <is>
+          <t>Panduan Urutan Haji dari Awal hingga Akhir dan Waktunya</t>
+        </is>
+      </c>
+      <c r="D2168" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/sumut/foto/d-8461176/panduan-urutan-haji-dari-awal-hingga-akhir-dan-waktunya</t>
+        </is>
+      </c>
+    </row>
+    <row r="2169">
+      <c r="A2169" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2169" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2169" t="inlineStr">
+        <is>
+          <t>Kisah Marbot Naik Haji, Berjuang Menabung 15 Tahun</t>
+        </is>
+      </c>
+      <c r="D2169" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8461087/kisah-marbot-naik-haji-berjuang-menabung-15-tahun</t>
+        </is>
+      </c>
+    </row>
+    <row r="2170">
+      <c r="A2170" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2170" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2170" t="inlineStr">
+        <is>
+          <t>Saudi Buka Penghargaan Inovasi Layanan Haji-Umrah, Hadiahnya Capai Rp7,4 Miliar</t>
+        </is>
+      </c>
+      <c r="D2170" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8460860/saudi-buka-penghargaan-inovasi-layanan-haji-umrah-hadiahnya-capai-rp7-4-miliar</t>
+        </is>
+      </c>
+    </row>
+    <row r="2171">
+      <c r="A2171" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2171" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2171" t="inlineStr">
+        <is>
+          <t>Cuaca Madinah Capai 36 Derajat Celsius, Jemaah Diimbau Lakukan Ini</t>
+        </is>
+      </c>
+      <c r="D2171" s="2" t="inlineStr">
+        <is>
+          <t>https://www.detik.com/hikmah/haji-dan-umrah/d-8460855/cuaca-madinah-capai-36-derajat-celsius-jemaah-diimbau-lakukan-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="2172">
+      <c r="A2172" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2172" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2172" t="inlineStr">
+        <is>
+          <t>Redam Dampak Avtur Mahal, Pemerintah Tanggung PPN Tiket Pesawat 60 Hari</t>
+        </is>
+      </c>
+      <c r="D2172" s="2" t="inlineStr">
+        <is>
+          <t>https://finance.detik.com/berita-ekonomi-bisnis/d-8461374/redam-dampak-avtur-mahal-pemerintah-tanggung-ppn-tiket-pesawat-60-hari</t>
+        </is>
+      </c>
+    </row>
+    <row r="2173">
+      <c r="A2173" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2173" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C2173" t="inlineStr">
+        <is>
+          <t>Gilanya Sprint Race MotoGP Spanyol 2026: Marquez Juara Usai Sempat Crash!</t>
+        </is>
+      </c>
+      <c r="D2173" s="2" t="inlineStr">
+        <is>
+          <t>https://oto.detik.com/otosport/d-8461312/gilanya-sprint-race-motogp-spanyol-2026-marquez-juara-usai-sempat-crash</t>
+        </is>
+      </c>
+    </row>
+    <row r="2174">
+      <c r="A2174" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2174" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C2174" t="inlineStr">
+        <is>
+          <t>Video Rahasia Makeup Anti Cakey untuk Kulit Kering: Skin Prep yang Cukup!</t>
+        </is>
+      </c>
+      <c r="D2174" s="2" t="inlineStr">
+        <is>
+          <t>https://wolipop.detik.com/detiktv/d-8461295/video-rahasia-makeup-anti-cakey-untuk-kulit-kering-skin-prep-yang-cukup</t>
+        </is>
+      </c>
+    </row>
+    <row r="2175">
+      <c r="A2175" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2175" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C2175" t="inlineStr">
+        <is>
+          <t>Netanyahu Diam-diam Sempat Idap Kanker Prostat, Kondisi Apa Itu?</t>
+        </is>
+      </c>
+      <c r="D2175" s="2" t="inlineStr">
+        <is>
+          <t>https://health.detik.com/berita-detikhealth/d-8460960/netanyahu-diam-diam-sempat-idap-kanker-prostat-kondisi-apa-itu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2176">
+      <c r="A2176" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2176" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C2176" t="inlineStr">
+        <is>
+          <t>Barcelona Bisa Apa Tanpa Lamine Yamal?</t>
+        </is>
+      </c>
+      <c r="D2176" s="2" t="inlineStr">
+        <is>
+          <t>https://sport.detik.com/sepakbola/liga-spanyol/d-8461115/barcelona-bisa-apa-tanpa-lamine-yamal</t>
+        </is>
+      </c>
+    </row>
+    <row r="2177">
+      <c r="A2177" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2177" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2177" t="inlineStr">
+        <is>
+          <t>Rano Sebut Pembangunan Kantor Satpol PP DKI Tertunda Efisiensi</t>
+        </is>
+      </c>
+      <c r="D2177" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8461531/rano-sebut-pembangunan-kantor-satpol-pp-dki-tertunda-efisiensi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2178">
+      <c r="A2178" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2178" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C2178" t="inlineStr">
+        <is>
+          <t>DKI Belum Henti Basmi Sapu-sapu: 10 Ton Ditangkap, Penjual Diedukasi</t>
+        </is>
+      </c>
+      <c r="D2178" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8461436/dki-belum-henti-basmi-sapu-sapu-10-ton-ditangkap-penjual-diedukasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2179">
+      <c r="A2179" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2179" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2179" t="inlineStr">
+        <is>
+          <t>Diusut Unsur Pidana di Kasus PRT Tewas Usai Loncat dari Kosan Majikan</t>
+        </is>
+      </c>
+      <c r="D2179" s="2" t="inlineStr">
+        <is>
+          <t>https://news.detik.com/berita/d-8461364/diusut-unsur-pidana-di-kasus-prt-tewas-usai-loncat-dari-kosan-majikan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2180">
+      <c r="A2180" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2180" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2180" t="inlineStr">
+        <is>
+          <t>Anggota Komisi II DPR Ungkap Alasan Menunda Pembahasan RUU Pemilu</t>
+        </is>
+      </c>
+      <c r="D2180" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100363/anggota-komisi-ii-dpr-ungkap-alasan-menunda-pembahasan-ruu-pemilu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2181">
+      <c r="A2181" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2181" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C2181" t="inlineStr">
+        <is>
+          <t>Asosiasi Pengusaha Dapur Ingin MBG Berlanjut hingga 25 Tahun</t>
+        </is>
+      </c>
+      <c r="D2181" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100357/asosiasi-pengusaha-dapur-ingin-mbg-berlanjut-hingga-25-tahun</t>
+        </is>
+      </c>
+    </row>
+    <row r="2182">
+      <c r="A2182" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2182" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C2182" t="inlineStr">
+        <is>
+          <t>Kemenkes Sediakan 666 Ribu Kuota Pelatihan Penjamah Pangan untuk SPPG</t>
+        </is>
+      </c>
+      <c r="D2182" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100356/kemenkes-sediakan-666-ribu-kuota-pelatihan-penjamah-pangan-untuk-sppg</t>
+        </is>
+      </c>
+    </row>
+    <row r="2183">
+      <c r="A2183" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2183" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C2183" t="inlineStr">
+        <is>
+          <t>Sirnas Padel Open Seri II di Semarang Pecahkan Rekor Nasional</t>
+        </is>
+      </c>
+      <c r="D2183" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100355/sirnas-padel-open-seri-ii-di-semarang-pecahkan-rekor-nasional</t>
+        </is>
+      </c>
+    </row>
+    <row r="2184">
+      <c r="A2184" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2184" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2184" t="inlineStr">
+        <is>
+          <t>Wali Kota Agustina Lakukan Peremajaan 10 Armada Trans Semarang</t>
+        </is>
+      </c>
+      <c r="D2184" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100353/wali-kota-agustina-lakukan-peremajaan-10-armada-trans-semarang</t>
+        </is>
+      </c>
+    </row>
+    <row r="2185">
+      <c r="A2185" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2185" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C2185" t="inlineStr">
+        <is>
+          <t>Cegah Bakteri, Kemenkes Ingatkan SPPG Batas Waktu Masak hingga Distribusi 4 Jam</t>
+        </is>
+      </c>
+      <c r="D2185" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100349/cegah-bakteri-kemenkes-ingatkan-sppg-batas-waktu-masak-hingga-distribusi-4-jam</t>
+        </is>
+      </c>
+    </row>
+    <row r="2186">
+      <c r="A2186" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2186" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2186" t="inlineStr">
+        <is>
+          <t>Berkinerja Prima di Bidang Kesehatan, Bupati Satria Menerima Governance Awards 2026</t>
+        </is>
+      </c>
+      <c r="D2186" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100345/berkinerja-prima-di-bidang-kesehatan-bupati-satria-menerima-governance-awards-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2187">
+      <c r="A2187" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2187" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2187" t="inlineStr">
+        <is>
+          <t>Penjelasan BGN soal Anggaran Zoom Meeting Rp 5,7 M</t>
+        </is>
+      </c>
+      <c r="D2187" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100343/penjelasan-bgn-soal-anggaran-zoom-meeting-rp-57-m</t>
+        </is>
+      </c>
+    </row>
+    <row r="2188">
+      <c r="A2188" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2188" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2188" t="inlineStr">
+        <is>
+          <t>Kepala Bappisus Ungkap Temuan Banyak Dapur Pangkas Porsi MBG</t>
+        </is>
+      </c>
+      <c r="D2188" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100340/kepala-bappisus-ungkap-temuan-banyak-dapur-pangkas-porsi-mbg</t>
+        </is>
+      </c>
+    </row>
+    <row r="2189">
+      <c r="A2189" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2189" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2189" t="inlineStr">
+        <is>
+          <t>Sanksi untuk Pelaku Kekerasan Seksual di FH UI Bakal Diputus dalam 79 Hari</t>
+        </is>
+      </c>
+      <c r="D2189" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100336/sanksi-untuk-pelaku-kekerasan-seksual-di-fh-ui-bakal-diputus-dalam-79-hari</t>
+        </is>
+      </c>
+    </row>
+    <row r="2190">
+      <c r="A2190" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2190" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2190" t="inlineStr">
+        <is>
+          <t>Unpad: Keputusan untuk Tutup Prodi Hak Perguruan Tinggi</t>
+        </is>
+      </c>
+      <c r="D2190" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100335/unpad-keputusan-untuk-tutup-prodi-hak-perguruan-tinggi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2191">
+      <c r="A2191" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2191" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2191" t="inlineStr">
+        <is>
+          <t>Cara Kemensos Cari Anak Jalanan buat Sekolah Rakyat Dikritik</t>
+        </is>
+      </c>
+      <c r="D2191" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100320/cara-kemensos-cari-anak-jalanan-buat-sekolah-rakyat-dikritik</t>
+        </is>
+      </c>
+    </row>
+    <row r="2192">
+      <c r="A2192" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2192" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2192" t="inlineStr">
+        <is>
+          <t>Dave Laksono soal Pajak Kapal di Selat Malaka: Harus Dikaji Komprehensif</t>
+        </is>
+      </c>
+      <c r="D2192" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100317/dave-laksono-soal-pajak-kapal-di-selat-malaka-harus-dikaji-komprehensif</t>
+        </is>
+      </c>
+    </row>
+    <row r="2193">
+      <c r="A2193" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2193" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2193" t="inlineStr">
+        <is>
+          <t>Kemendikti Bakal Tutup Prodi yang Tak Relevan dengan Industri</t>
+        </is>
+      </c>
+      <c r="D2193" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100315/kemendikti-bakal-tutup-prodi-yang-tak-relevan-dengan-industri</t>
+        </is>
+      </c>
+    </row>
+    <row r="2194">
+      <c r="A2194" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2194" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2194" t="inlineStr">
+        <is>
+          <t>Update Kasus Kekerasan Seksual Mahasiswa Fakultas Hukum UI</t>
+        </is>
+      </c>
+      <c r="D2194" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100309/update-kasus-kekerasan-seksual-mahasiswa-fakultas-hukum-ui</t>
+        </is>
+      </c>
+    </row>
+    <row r="2195">
+      <c r="A2195" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2195" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2195" t="inlineStr">
+        <is>
+          <t>NasDem Usulkan Formula untuk Ambang Batas Parlemen</t>
+        </is>
+      </c>
+      <c r="D2195" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100300/nasdem-usulkan-formula-untuk-ambang-batas-parlemen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2196">
+      <c r="A2196" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2196" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C2196" t="inlineStr">
+        <is>
+          <t>Pemprov Lampung Perkuat Layanan Kesehatan untuk Tekan TBC</t>
+        </is>
+      </c>
+      <c r="D2196" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100297/pemprov-lampung-perkuat-layanan-kesehatan-untuk-tekan-tbc</t>
+        </is>
+      </c>
+    </row>
+    <row r="2197">
+      <c r="A2197" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2197" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2197" t="inlineStr">
+        <is>
+          <t>Bank Jakarta Salurkan Bantuan untuk Sahabat Disabilitas Binaan YaSDI</t>
+        </is>
+      </c>
+      <c r="D2197" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100296/bank-jakarta-salurkan-bantuan-untuk-sahabat-disabilitas-binaan-yasdi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2198">
+      <c r="A2198" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2198" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2198" t="inlineStr">
+        <is>
+          <t>Lagi, 1 Prajurit TNI Gugur dalam Serangan di Libanon</t>
+        </is>
+      </c>
+      <c r="D2198" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100289/lagi-1-prajurit-tni-gugur-dalam-serangan-di-libanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2199">
+      <c r="A2199" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2199" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2199" t="inlineStr">
+        <is>
+          <t>Kemensos Jaring Anak Jalanan buat Jadi Siswa Sekolah Rakyat</t>
+        </is>
+      </c>
+      <c r="D2199" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100287/kemensos-jaring-anak-jalanan-buat-jadi-siswa-sekolah-rakyat</t>
+        </is>
+      </c>
+    </row>
+    <row r="2200">
+      <c r="A2200" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2200" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C2200" t="inlineStr">
+        <is>
+          <t>Indonesia positions fishing village program to boost blue economy</t>
+        </is>
+      </c>
+      <c r="D2200" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413635/indonesia-positions-fishing-village-program-to-boost-blue-economy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2201">
+      <c r="A2201" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2201" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C2201" t="inlineStr">
+        <is>
+          <t>Indonesia eyes global market with custom automotive industry push</t>
+        </is>
+      </c>
+      <c r="D2201" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413633/indonesia-eyes-global-market-with-custom-automotive-industry-push</t>
+        </is>
+      </c>
+    </row>
+    <row r="2202">
+      <c r="A2202" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2202" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2202" t="inlineStr">
+        <is>
+          <t>Inside the Baduy’s 200 km sacred journey through the night</t>
+        </is>
+      </c>
+      <c r="D2202" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413629/inside-the-baduys-200-km-sacred-journey-through-the-night</t>
+        </is>
+      </c>
+    </row>
+    <row r="2203">
+      <c r="A2203" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2203" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C2203" t="inlineStr">
+        <is>
+          <t>MPR Deputy Speaker urges govt to boost public trust in vaccinations</t>
+        </is>
+      </c>
+      <c r="D2203" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413628/mpr-deputy-speaker-urges-govt-to-boost-public-trust-in-vaccinations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2204">
+      <c r="A2204" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2204" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C2204" t="inlineStr">
+        <is>
+          <t>Banten waives electric vehicle tax to support clean energy</t>
+        </is>
+      </c>
+      <c r="D2204" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413624/banten-waives-electric-vehicle-tax-to-support-clean-energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2205">
+      <c r="A2205" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2205" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2205" t="inlineStr">
+        <is>
+          <t>RI govt speeds up housing program for Senen rail-side community</t>
+        </is>
+      </c>
+      <c r="D2205" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413620/ri-govt-speeds-up-housing-program-for-senen-rail-side-community</t>
+        </is>
+      </c>
+    </row>
+    <row r="2206">
+      <c r="A2206" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2206" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2206" t="inlineStr">
+        <is>
+          <t>Gov't striving to expand education access to reduce dropout rates</t>
+        </is>
+      </c>
+      <c r="D2206" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413619/govt-striving-to-expand-education-access-to-reduce-dropout-rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2207">
+      <c r="A2207" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2207" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2207" t="inlineStr">
+        <is>
+          <t>Indonesia to continue school revamp, digital push in 2026</t>
+        </is>
+      </c>
+      <c r="D2207" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413617/indonesia-to-continue-school-revamp-digital-push-in-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2208">
+      <c r="A2208" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2208" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C2208" t="inlineStr">
+        <is>
+          <t>Forestry Ministry to periodically evaluate Komodo National Park quota</t>
+        </is>
+      </c>
+      <c r="D2208" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413613/forestry-ministry-to-periodically-evaluate-komodo-national-park-quota</t>
+        </is>
+      </c>
+    </row>
+    <row r="2209">
+      <c r="A2209" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2209" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2209" t="inlineStr">
+        <is>
+          <t>Indonesia prepares to repatriate fourth TNI soldier killed in Lebanon</t>
+        </is>
+      </c>
+      <c r="D2209" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413609/indonesia-prepares-to-repatriate-fourth-tni-soldier-killed-in-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2210">
+      <c r="A2210" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2210" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C2210" t="inlineStr">
+        <is>
+          <t>Indonesia targets safety training for 666,000 MBG food handlers</t>
+        </is>
+      </c>
+      <c r="D2210" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413608/indonesia-targets-safety-training-for-666000-mbg-food-handlers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2211">
+      <c r="A2211" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2211" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C2211" t="inlineStr">
+        <is>
+          <t>Ministry speeds up hygiene certification for 26 thousand MBG kitchens</t>
+        </is>
+      </c>
+      <c r="D2211" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413605/ministry-speeds-up-hygiene-certification-for-26-thousand-mbg-kitchens</t>
+        </is>
+      </c>
+    </row>
+    <row r="2212">
+      <c r="A2212" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2212" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2212" t="inlineStr">
+        <is>
+          <t>Gov't open to sharp criticism from academics, says top minister</t>
+        </is>
+      </c>
+      <c r="D2212" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413603/govt-open-to-sharp-criticism-from-academics-says-top-minister</t>
+        </is>
+      </c>
+    </row>
+    <row r="2213">
+      <c r="A2213" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2213" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C2213" t="inlineStr">
+        <is>
+          <t>Ministry identifies seven peat hotspots highly prone to wildfires</t>
+        </is>
+      </c>
+      <c r="D2213" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413601/ministry-identifies-seven-peat-hotspots-highly-prone-to-wildfires</t>
+        </is>
+      </c>
+    </row>
+    <row r="2214">
+      <c r="A2214" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2214" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2214" t="inlineStr">
+        <is>
+          <t>Indonesia's DPR presses UNIFIL safety review after personnel deaths</t>
+        </is>
+      </c>
+      <c r="D2214" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413599/indonesias-dpr-presses-unifil-safety-review-after-personnel-deaths</t>
+        </is>
+      </c>
+    </row>
+    <row r="2215">
+      <c r="A2215" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2215" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2215" t="inlineStr">
+        <is>
+          <t>Sleman's slum area transformation serves as model for other cities</t>
+        </is>
+      </c>
+      <c r="D2215" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413597/slemans-slum-area-transformation-serves-as-model-for-other-cities</t>
+        </is>
+      </c>
+    </row>
+    <row r="2216">
+      <c r="A2216" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2216" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2216" t="inlineStr">
+        <is>
+          <t>Ministry expands quality education coverage through distance learning</t>
+        </is>
+      </c>
+      <c r="D2216" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413593/ministry-expands-quality-education-coverage-through-distance-learning</t>
+        </is>
+      </c>
+    </row>
+    <row r="2217">
+      <c r="A2217" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2217" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2217" t="inlineStr">
+        <is>
+          <t>Minister proposes electric motorcycles incentive starting 2026</t>
+        </is>
+      </c>
+      <c r="D2217" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413589/minister-proposes-electric-motorcycles-incentive-starting-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2218">
+      <c r="A2218" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2218" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2218" t="inlineStr">
+        <is>
+          <t>Minister urges stronger reforms in public service across regions</t>
+        </is>
+      </c>
+      <c r="D2218" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413587/minister-urges-stronger-reforms-in-public-service-across-regions</t>
+        </is>
+      </c>
+    </row>
+    <row r="2219">
+      <c r="A2219" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2219" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C2219" t="inlineStr">
+        <is>
+          <t>Indonesia pushes rapid farmland recovery after Sumatra floods</t>
+        </is>
+      </c>
+      <c r="D2219" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413583/indonesia-pushes-rapid-farmland-recovery-after-sumatra-floods</t>
+        </is>
+      </c>
+    </row>
+    <row r="2220">
+      <c r="A2220" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2220" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2220" t="inlineStr">
+        <is>
+          <t>Menlu Iran dan PM Pakistan gelar pertemuan bahas solusi perang</t>
+        </is>
+      </c>
+      <c r="D2220" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5542493/menlu-iran-dan-pm-pakistan-gelar-pertemuan-bahas-solusi-perang</t>
+        </is>
+      </c>
+    </row>
+    <row r="2221">
+      <c r="A2221" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2221" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2221" t="inlineStr">
+        <is>
+          <t>WHO: Perbaikan sistem kesehatan di Gaza butuh Rp172 triliun</t>
+        </is>
+      </c>
+      <c r="D2221" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542479/who-perbaikan-sistem-kesehatan-di-gaza-butuh-rp172-triliun</t>
+        </is>
+      </c>
+    </row>
+    <row r="2222">
+      <c r="A2222" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2222" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2222" t="inlineStr">
+        <is>
+          <t>Jerman siapkan armada ke Mediterania untuk misi di Selat Hormuz</t>
+        </is>
+      </c>
+      <c r="D2222" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542445/jerman-siapkan-armada-ke-mediterania-untuk-misi-di-selat-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="2223">
+      <c r="A2223" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2223" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2223" t="inlineStr">
+        <is>
+          <t>Sekjen PBB sambut baik perpanjangan gencatan senjata Lebanon-Israel</t>
+        </is>
+      </c>
+      <c r="D2223" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542383/sekjen-pbb-sambut-baik-perpanjangan-gencatan-senjata-lebanon-israel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2224">
+      <c r="A2224" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2224" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2224" t="inlineStr">
+        <is>
+          <t>Iran sita dua kapal di Selat Hormuz diduga terkait dengan Israel</t>
+        </is>
+      </c>
+      <c r="D2224" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542305/iran-sita-dua-kapal-di-selat-hormuz-diduga-terkait-dengan-israel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2225">
+      <c r="A2225" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2225" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2225" t="inlineStr">
+        <is>
+          <t>Menlu Turki: Israel jadi ancaman langsung bagi keamanan global</t>
+        </is>
+      </c>
+      <c r="D2225" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542188/menlu-turki-israel-jadi-ancaman-langsung-bagi-keamanan-global</t>
+        </is>
+      </c>
+    </row>
+    <row r="2226">
+      <c r="A2226" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2226" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2226" t="inlineStr">
+        <is>
+          <t>Rusia butuh 644 pesawat baru 2030 penuhi permintaan sektor penerbangan</t>
+        </is>
+      </c>
+      <c r="D2226" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542163/rusia-butuh-644-pesawat-baru-2030-penuhi-permintaan-sektor-penerbangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2227">
+      <c r="A2227" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2227" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2227" t="inlineStr">
+        <is>
+          <t>Prajurit TNI gugur di UNIFIL, pemerintah kutuk “kejahatan perang”</t>
+        </is>
+      </c>
+      <c r="D2227" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5541948/prajurit-tni-gugur-di-unifil-pemerintah-kutuk-kejahatan-perang</t>
+        </is>
+      </c>
+    </row>
+    <row r="2228">
+      <c r="A2228" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2228" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C2228" t="inlineStr">
+        <is>
+          <t>Uni Eropa: Konflik Timur Tengah sebabkan lonjakan biaya impor energi</t>
+        </is>
+      </c>
+      <c r="D2228" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5541907/uni-eropa-konflik-timur-tengah-sebabkan-lonjakan-biaya-impor-energi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2229">
+      <c r="A2229" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2229" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2229" t="inlineStr">
+        <is>
+          <t>Praka Rico personel TNI kedua yang gugur diserang Israel pada 29 Maret</t>
+        </is>
+      </c>
+      <c r="D2229" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5541868/praka-rico-personel-tni-kedua-yang-gugur-diserang-israel-pada-29-maret</t>
+        </is>
+      </c>
+    </row>
+    <row r="2230">
+      <c r="A2230" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2230" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2230" t="inlineStr">
+        <is>
+          <t>Biaya operasi militer AS terhadap Iran tembus Rp1.000 triliun</t>
+        </is>
+      </c>
+      <c r="D2230" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5541863/biaya-operasi-militer-as-terhadap-iran-tembus-rp1000-triliun</t>
+        </is>
+      </c>
+    </row>
+    <row r="2231">
+      <c r="A2231" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2231" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2231" t="inlineStr">
+        <is>
+          <t>IMO catat 29 serangan kapal sipil di Teluk Persia-Hormuz</t>
+        </is>
+      </c>
+      <c r="D2231" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5541857/imo-catat-29-serangan-kapal-sipil-di-teluk-persia-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="2232">
+      <c r="A2232" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2232" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2232" t="inlineStr">
+        <is>
+          <t>AS tawarkan Rp172 miliar untuk informasi Hashim Finyan Rahim al-Saraji</t>
+        </is>
+      </c>
+      <c r="D2232" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5541821/as-tawarkan-rp172-miliar-untuk-informasi-hashim-finyan-rahim-al-saraji</t>
+        </is>
+      </c>
+    </row>
+    <row r="2233">
+      <c r="A2233" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2233" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2233" t="inlineStr">
+        <is>
+          <t>Upacara pemakaman jurnalis yang tewas akibat serangan Israel digelar di Baissariyeh, Lebanon</t>
+        </is>
+      </c>
+      <c r="D2233" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5541815/upacara-pemakaman-jurnalis-yang-tewas-akibat-serangan-israel-digelar-di-baissariyeh-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2234">
+      <c r="A2234" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2234" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2234" t="inlineStr">
+        <is>
+          <t>Indonesia dan tujuh negara Islam kompak kecam aksi pemukim Israel</t>
+        </is>
+      </c>
+      <c r="D2234" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5541687/indonesia-dan-tujuh-negara-islam-kompak-kecam-aksi-pemukim-israel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2235">
+      <c r="A2235" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2235" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2235" t="inlineStr">
+        <is>
+          <t>Picu ketegangan dengan Korut, Yoon Suk-yeol dituntut 30 tahun penjara</t>
+        </is>
+      </c>
+      <c r="D2235" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5541679/picu-ketegangan-dengan-korut-yoon-suk-yeol-dituntut-30-tahun-penjara</t>
+        </is>
+      </c>
+    </row>
+    <row r="2236">
+      <c r="A2236" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2236" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2236" t="inlineStr">
+        <is>
+          <t>PBB sampaikan belasungkawa atas wafatnya Praka Rico</t>
+        </is>
+      </c>
+      <c r="D2236" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5541644/pbb-sampaikan-belasungkawa-atas-wafatnya-praka-rico</t>
+        </is>
+      </c>
+    </row>
+    <row r="2237">
+      <c r="A2237" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2237" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2237" t="inlineStr">
+        <is>
+          <t>Ketika Panglima Tertinggi dianggap lebih berbahaya dari musuh</t>
+        </is>
+      </c>
+      <c r="D2237" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5541605/ketika-panglima-tertinggi-dianggap-lebih-berbahaya-dari-musuh</t>
+        </is>
+      </c>
+    </row>
+    <row r="2238">
+      <c r="A2238" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2238" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C2238" t="inlineStr">
+        <is>
+          <t>Krisis Timur Tengah ancam pasokan energi Kepulauan Marshall</t>
+        </is>
+      </c>
+      <c r="D2238" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5541601/krisis-timur-tengah-ancam-pasokan-energikepulauanmarshall</t>
+        </is>
+      </c>
+    </row>
+    <row r="2239">
+      <c r="A2239" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2239" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2239" t="inlineStr">
+        <is>
+          <t>Gencatan senjata Israel-Lebanon diperpanjang tiga pekan</t>
+        </is>
+      </c>
+      <c r="D2239" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5541512/gencatan-senjata-israel-lebanon-diperpanjang-tiga-pekan</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D2166"/>
+  <autoFilter ref="A1:D2239"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -50268,6 +51874,79 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2164" r:id="rId2163"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2165" r:id="rId2164"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2166" r:id="rId2165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2167" r:id="rId2166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2168" r:id="rId2167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2169" r:id="rId2168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2170" r:id="rId2169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2171" r:id="rId2170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2172" r:id="rId2171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2173" r:id="rId2172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2174" r:id="rId2173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2175" r:id="rId2174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2176" r:id="rId2175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2177" r:id="rId2176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2178" r:id="rId2177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2179" r:id="rId2178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2180" r:id="rId2179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2181" r:id="rId2180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2182" r:id="rId2181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2183" r:id="rId2182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2184" r:id="rId2183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2185" r:id="rId2184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2186" r:id="rId2185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2187" r:id="rId2186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2188" r:id="rId2187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2189" r:id="rId2188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2190" r:id="rId2189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2191" r:id="rId2190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2192" r:id="rId2191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2193" r:id="rId2192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2194" r:id="rId2193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2195" r:id="rId2194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2196" r:id="rId2195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2197" r:id="rId2196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2198" r:id="rId2197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2199" r:id="rId2198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2200" r:id="rId2199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2201" r:id="rId2200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2202" r:id="rId2201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2203" r:id="rId2202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2204" r:id="rId2203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2205" r:id="rId2204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2206" r:id="rId2205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2207" r:id="rId2206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2208" r:id="rId2207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2209" r:id="rId2208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2210" r:id="rId2209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2211" r:id="rId2210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2212" r:id="rId2211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2213" r:id="rId2212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2214" r:id="rId2213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2215" r:id="rId2214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2216" r:id="rId2215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2217" r:id="rId2216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2218" r:id="rId2217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2219" r:id="rId2218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2220" r:id="rId2219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2221" r:id="rId2220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2222" r:id="rId2221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2223" r:id="rId2222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2224" r:id="rId2223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2225" r:id="rId2224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2226" r:id="rId2225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2227" r:id="rId2226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2228" r:id="rId2227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2229" r:id="rId2228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2230" r:id="rId2229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2231" r:id="rId2230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2232" r:id="rId2231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2233" r:id="rId2232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2234" r:id="rId2233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2235" r:id="rId2234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2236" r:id="rId2235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2237" r:id="rId2236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2238" r:id="rId2237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2239" r:id="rId2238"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update headlines archive — 2026-04-26
</commit_message>
<xml_diff>
--- a/headlines_archive.xlsx
+++ b/headlines_archive.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Headlines Archive" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$2239</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Headlines Archive'!$A$1:$D$2364</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -439,7 +439,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D2239"/>
+  <dimension ref="A1:D2364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -49706,8 +49706,2818 @@
         </is>
       </c>
     </row>
+    <row r="2240">
+      <c r="A2240" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2240" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2240" t="inlineStr">
+        <is>
+          <t>KPAI Soroti Daycare Tak Berizin, tapi Bisa Beroperasi</t>
+        </is>
+      </c>
+      <c r="D2240" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100479/kpai-soroti-daycare-tak-berizin-tapi-bisa-beroperasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2241">
+      <c r="A2241" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2241" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2241" t="inlineStr">
+        <is>
+          <t>Daycare Beroperasi Tanpa Izin karena Pengawasan Lemah</t>
+        </is>
+      </c>
+      <c r="D2241" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100475/daycare-beroperasi-tanpa-izin-karena-pengawasan-lemah</t>
+        </is>
+      </c>
+    </row>
+    <row r="2242">
+      <c r="A2242" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2242" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2242" t="inlineStr">
+        <is>
+          <t>Dosen UGM Jadi Penasihat Daycare yang Lakukan Kekerasan</t>
+        </is>
+      </c>
+      <c r="D2242" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100464/dosen-ugm-jadi-penasihat-daycare-yang-lakukan-kekerasan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2243">
+      <c r="A2243" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2243" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2243" t="inlineStr">
+        <is>
+          <t>Respons Dedi Mulyadi soal Spanduk "Shut Up KDM"</t>
+        </is>
+      </c>
+      <c r="D2243" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100459/respons-dedi-mulyadi-soal-spanduk-shut-up-kdm</t>
+        </is>
+      </c>
+    </row>
+    <row r="2244">
+      <c r="A2244" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2244" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C2244" t="inlineStr">
+        <is>
+          <t>Memulai Era Sampah Menjadi Energi</t>
+        </is>
+      </c>
+      <c r="D2244" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100456/memulai-era-sampah-menjadi-energi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2245">
+      <c r="A2245" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2245" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C2245" t="inlineStr">
+        <is>
+          <t>Pekanbaru dan Revolusi Pengelolaan Sampah Modern</t>
+        </is>
+      </c>
+      <c r="D2245" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100455/pekanbaru-dan-revolusi-pengelolaan-sampah-modern</t>
+        </is>
+      </c>
+    </row>
+    <row r="2246">
+      <c r="A2246" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2246" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C2246" t="inlineStr">
+        <is>
+          <t>Menteri LH Apresiasi Langkah Wali Kota Pekanbaru Dorong Waste to Energy dan Penataan TPA</t>
+        </is>
+      </c>
+      <c r="D2246" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100453/menteri-lh-apresiasi-langkah-wali-kota-pekanbaru-dorong-waste-to-energy-dan-penataan-tpa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2247">
+      <c r="A2247" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2247" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2247" t="inlineStr">
+        <is>
+          <t>Turunkan Stunting dan Angka Kemiskinan, Wali Kota Pekanbaru Raih Penghargaan Kemendagri</t>
+        </is>
+      </c>
+      <c r="D2247" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100449/turunkan-stunting-dan-angka-kemiskinan-wali-kota-pekanbaru-raih-penghargaan-kemendagri</t>
+        </is>
+      </c>
+    </row>
+    <row r="2248">
+      <c r="A2248" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2248" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2248" t="inlineStr">
+        <is>
+          <t>Kekerasan di Daycare Yogyakarta, DPRD Akan Panggil Pemda</t>
+        </is>
+      </c>
+      <c r="D2248" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100442/kekerasan-di-daycare-yogyakarta-dprd-akan-panggil-pemda</t>
+        </is>
+      </c>
+    </row>
+    <row r="2249">
+      <c r="A2249" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2249" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2249" t="inlineStr">
+        <is>
+          <t>Pemkot Yogya Akan Tertibkan Daycare Buntut Dugaan Kekerasan</t>
+        </is>
+      </c>
+      <c r="D2249" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100436/pemkot-yogya-akan-tertibkan-daycare-buntut-dugaan-kekerasan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2250">
+      <c r="A2250" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2250" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2250" t="inlineStr">
+        <is>
+          <t>Legislator PDI Perjuangan Minta Revisi UU Pemilu Dibahas Tahun Ini</t>
+        </is>
+      </c>
+      <c r="D2250" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100430/legislator-pdi-perjuangan-minta-revisi-uu-pemilu-dibahas-tahun-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="2251">
+      <c r="A2251" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2251" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2251" t="inlineStr">
+        <is>
+          <t>Daycare di Yogya yang Diduga Menganiaya Anak, Belum Berizin</t>
+        </is>
+      </c>
+      <c r="D2251" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100425/daycare-di-yogya-yang-diduga-menganiaya-anak-belum-berizin</t>
+        </is>
+      </c>
+    </row>
+    <row r="2252">
+      <c r="A2252" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2252" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2252" t="inlineStr">
+        <is>
+          <t>Teddy Klaim Hunian untuk Warga Bantaran Rel Pasar Senen Hampir Rampung</t>
+        </is>
+      </c>
+      <c r="D2252" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100421/teddy-klaim-hunian-untuk-warga-bantaran-rel-pasar-senen-hampir-rampung</t>
+        </is>
+      </c>
+    </row>
+    <row r="2253">
+      <c r="A2253" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2253" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2253" t="inlineStr">
+        <is>
+          <t>Menteri PPPA Targetkan Setiap Kabupaten Kota Bentuk RBI di Seluruh Desa</t>
+        </is>
+      </c>
+      <c r="D2253" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100419/menteri-pppa-targetkan-setiap-kabupaten-kota-bentuk-rbi-di-seluruh-desa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2254">
+      <c r="A2254" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2254" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C2254" t="inlineStr">
+        <is>
+          <t>Atraksi Paramotor Ramaikan Langit CFD Depok</t>
+        </is>
+      </c>
+      <c r="D2254" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100413/atraksi-paramotor-ramaikan-langit-cfd-depok</t>
+        </is>
+      </c>
+    </row>
+    <row r="2255">
+      <c r="A2255" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2255" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2255" t="inlineStr">
+        <is>
+          <t>TNI Naikkan Pangkat Rico Pramudia, Prajurit yang Tewas di Libanon</t>
+        </is>
+      </c>
+      <c r="D2255" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100398/tni-naikkan-pangkat-rico-pramudia-prajurit-yang-tewas-di-libanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2256">
+      <c r="A2256" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2256" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2256" t="inlineStr">
+        <is>
+          <t>Kemendagri Gandeng Media, Pakar, dan Akademisi untuk Nilai Pemda Berprestasi 2026</t>
+        </is>
+      </c>
+      <c r="D2256" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100397/kemendagri-gandeng-media-pakar-dan-akademisi-untuk-nilai-pemda-berprestasi-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2257">
+      <c r="A2257" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2257" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2257" t="inlineStr">
+        <is>
+          <t>Kemendagri Siapkan Reward Bagi Daerah Berprestasi</t>
+        </is>
+      </c>
+      <c r="D2257" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100396/kemendagri-siapkan-reward-bagi-daerah-berprestasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2258">
+      <c r="A2258" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2258" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2258" t="inlineStr">
+        <is>
+          <t>Kemendagri Dorong Kompetisi Kinerja Daerah Berbasis Wilayah</t>
+        </is>
+      </c>
+      <c r="D2258" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100395/kemendagri-dorong-kompetisi-kinerja-daerah-berbasis-wilayah</t>
+        </is>
+      </c>
+    </row>
+    <row r="2259">
+      <c r="A2259" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2259" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2259" t="inlineStr">
+        <is>
+          <t>Menjemput Visi Prabowo, Wamendagri Bima Arya Bedah Strategi Akselerator Negeri dari Bumi Sriwijaya</t>
+        </is>
+      </c>
+      <c r="D2259" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.tempo.co/read/2100394/menjemput-visi-prabowo-wamendagri-bima-arya-bedah-strategi-akselerator-negeri-dari-bumi-sriwijaya</t>
+        </is>
+      </c>
+    </row>
+    <row r="2260">
+      <c r="A2260" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2260" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2260" t="inlineStr">
+        <is>
+          <t>Trump Batalkan Kunjungan Utusan AS ke Pakistan</t>
+        </is>
+      </c>
+      <c r="D2260" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100474/trump-batalkan-kunjungan-utusan-as-ke-pakistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2261">
+      <c r="A2261" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2261" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2261" t="inlineStr">
+        <is>
+          <t>Usai dari Pakistan, Menlu Iran Tiba di Oman Bahas Konflik</t>
+        </is>
+      </c>
+      <c r="D2261" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100471/usai-dari-pakistan-menlu-iran-tiba-di-oman-bahas-konflik</t>
+        </is>
+      </c>
+    </row>
+    <row r="2262">
+      <c r="A2262" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2262" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2262" t="inlineStr">
+        <is>
+          <t>Ini Senjata yang Dibawa Pelaku Penembakan di Acara Trump</t>
+        </is>
+      </c>
+      <c r="D2262" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100440/ini-senjata-yang-dibawa-pelaku-penembakan-di-acara-trump</t>
+        </is>
+      </c>
+    </row>
+    <row r="2263">
+      <c r="A2263" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2263" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2263" t="inlineStr">
+        <is>
+          <t>Pernyataan Jubir Gedung Putih Viral Usai Penembakan di AS</t>
+        </is>
+      </c>
+      <c r="D2263" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100439/pernyataan-jubir-gedung-putih-viral-usai-penembakan-di-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="2264">
+      <c r="A2264" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2264" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2264" t="inlineStr">
+        <is>
+          <t>Trump: Penembakan di Acara Gedung Putih oleh Pelaku Tunggal</t>
+        </is>
+      </c>
+      <c r="D2264" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100435/trump-penembakan-di-acara-gedung-putih-oleh-pelaku-tunggal</t>
+        </is>
+      </c>
+    </row>
+    <row r="2265">
+      <c r="A2265" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2265" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2265" t="inlineStr">
+        <is>
+          <t>Kata Donald Trump Soal Penembakan di Acara yang Dihadirinya</t>
+        </is>
+      </c>
+      <c r="D2265" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100432/kata-donald-trump-soal-penembakan-di-acara-yang-dihadirinya</t>
+        </is>
+      </c>
+    </row>
+    <row r="2266">
+      <c r="A2266" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2266" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2266" t="inlineStr">
+        <is>
+          <t>Menlu Iran Temui PM Pakistan, Bahas Apa Saja?</t>
+        </is>
+      </c>
+      <c r="D2266" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100362/menlu-iran-temui-pm-pakistan-bahas-apa-saja</t>
+        </is>
+      </c>
+    </row>
+    <row r="2267">
+      <c r="A2267" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2267" t="inlineStr">
+        <is>
+          <t>Transportation</t>
+        </is>
+      </c>
+      <c r="C2267" t="inlineStr">
+        <is>
+          <t>Bandara Internasional Imam Khomeini Iran Kembali Dibuka</t>
+        </is>
+      </c>
+      <c r="D2267" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100361/bandara-internasional-imam-khomeini-iran-kembali-dibuka</t>
+        </is>
+      </c>
+    </row>
+    <row r="2268">
+      <c r="A2268" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2268" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2268" t="inlineStr">
+        <is>
+          <t>Presiden Kolombia Kunjungi Venezuela, Bahas Soal Ini</t>
+        </is>
+      </c>
+      <c r="D2268" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100360/presiden-kolombia-kunjungi-venezuela-bahas-soal-ini</t>
+        </is>
+      </c>
+    </row>
+    <row r="2269">
+      <c r="A2269" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2269" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2269" t="inlineStr">
+        <is>
+          <t>Palestina Gelar Pemilu Lokal di Tepi Barat dan Gaza Tengah</t>
+        </is>
+      </c>
+      <c r="D2269" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100358/palestina-gelar-pemilu-lokal-di-tepi-barat-dan-gaza-tengah</t>
+        </is>
+      </c>
+    </row>
+    <row r="2270">
+      <c r="A2270" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2270" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2270" t="inlineStr">
+        <is>
+          <t>Amerika Serikat Bekukan Aset Kripto Iran Rp 5,9 Triliun</t>
+        </is>
+      </c>
+      <c r="D2270" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100348/amerika-serikat-bekukan-aset-kripto-iran-rp-59-triliun</t>
+        </is>
+      </c>
+    </row>
+    <row r="2271">
+      <c r="A2271" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2271" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2271" t="inlineStr">
+        <is>
+          <t>IMO: 29 Serangan ke Kapal Sipil di Teluk Persia-Hormuz</t>
+        </is>
+      </c>
+      <c r="D2271" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100312/imo-29-serangan-ke-kapal-sipil-di-teluk-persia-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="2272">
+      <c r="A2272" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2272" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2272" t="inlineStr">
+        <is>
+          <t>Polisi Peru Gerebek Rumah Pejabat KPU, Imbas Kisruh Pemilu</t>
+        </is>
+      </c>
+      <c r="D2272" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100311/polisi-peru-gerebek-rumah-pejabat-kpu-imbas-kisruh-pemilu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2273">
+      <c r="A2273" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2273" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2273" t="inlineStr">
+        <is>
+          <t>Netanyahu Sembuh dari Kanker Prostat, Akui Tunda Pengumuman</t>
+        </is>
+      </c>
+      <c r="D2273" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100308/netanyahu-sembuh-dari-kanker-prostat-akui-tunda-pengumuman</t>
+        </is>
+      </c>
+    </row>
+    <row r="2274">
+      <c r="A2274" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2274" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2274" t="inlineStr">
+        <is>
+          <t>Biaya Perang AS terhadap Iran Tembus Rp 1.000 Triliun</t>
+        </is>
+      </c>
+      <c r="D2274" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100299/biaya-perang-as-terhadap-iran-tembus-rp-1-000-triliun</t>
+        </is>
+      </c>
+    </row>
+    <row r="2275">
+      <c r="A2275" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2275" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2275" t="inlineStr">
+        <is>
+          <t>PM Pedro Sanchez: Spanyol Anggota NATO yang Dapat Diandalkan</t>
+        </is>
+      </c>
+      <c r="D2275" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100293/pm-pedro-sanchez-spanyol-anggota-nato-yang-dapat-diandalkan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2276">
+      <c r="A2276" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2276" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2276" t="inlineStr">
+        <is>
+          <t>Uni Eropa Usulkan Misi AL untuk Buka Kembali Selat Hormuz</t>
+        </is>
+      </c>
+      <c r="D2276" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100286/uni-eropa-usulkan-misi-al-untuk-buka-kembali-selat-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="2277">
+      <c r="A2277" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2277" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2277" t="inlineStr">
+        <is>
+          <t>Mendag AS: Baru Satu Orang Terima Visa Emas Trump</t>
+        </is>
+      </c>
+      <c r="D2277" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100284/mendag-as-baru-satu-orang-terima-visa-emas-trump</t>
+        </is>
+      </c>
+    </row>
+    <row r="2278">
+      <c r="A2278" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2278" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2278" t="inlineStr">
+        <is>
+          <t>Kemlu: Indonesia Berduka atas Gugurnya Praka Rico di Libanon</t>
+        </is>
+      </c>
+      <c r="D2278" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100281/kemlu-indonesia-berduka-atas-gugurnya-praka-rico-di-libanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2279">
+      <c r="A2279" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2279" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2279" t="inlineStr">
+        <is>
+          <t>UNIFIL: Praka Rico Gugur dalam Serangan di Libanon</t>
+        </is>
+      </c>
+      <c r="D2279" s="2" t="inlineStr">
+        <is>
+          <t>https://dunia.tempo.co/read/2100280/unifil-praka-rico-gugur-dalam-serangan-di-libanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2280">
+      <c r="A2280" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2280" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2280" t="inlineStr">
+        <is>
+          <t>Indonesia seeks UNESCO heritage committee seat support</t>
+        </is>
+      </c>
+      <c r="D2280" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413667/indonesia-seeks-unesco-heritage-committee-seat-support</t>
+        </is>
+      </c>
+    </row>
+    <row r="2281">
+      <c r="A2281" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2281" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2281" t="inlineStr">
+        <is>
+          <t>Indonesian govt drafts rules to secure local food for meal plan</t>
+        </is>
+      </c>
+      <c r="D2281" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413664/indonesian-govt-drafts-rules-to-secure-local-food-for-meal-plan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2282">
+      <c r="A2282" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2282" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C2282" t="inlineStr">
+        <is>
+          <t>Indonesia expands eye screening, cataract surgery access</t>
+        </is>
+      </c>
+      <c r="D2282" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413660/indonesia-expands-eye-screening-cataract-surgery-access</t>
+        </is>
+      </c>
+    </row>
+    <row r="2283">
+      <c r="A2283" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2283" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C2283" t="inlineStr">
+        <is>
+          <t>Indonesia's minister hails sport as key to public health push</t>
+        </is>
+      </c>
+      <c r="D2283" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413659/indonesias-minister-hails-sport-as-key-to-public-health-push</t>
+        </is>
+      </c>
+    </row>
+    <row r="2284">
+      <c r="A2284" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2284" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2284" t="inlineStr">
+        <is>
+          <t>Minister urges youth to lead science-based innovation</t>
+        </is>
+      </c>
+      <c r="D2284" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413657/minister-urges-youth-to-lead-science-based-innovation</t>
+        </is>
+      </c>
+    </row>
+    <row r="2285">
+      <c r="A2285" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2285" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C2285" t="inlineStr">
+        <is>
+          <t>Indonesia covers VAT on economy flights to cut airfares</t>
+        </is>
+      </c>
+      <c r="D2285" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413655/indonesia-covers-vat-on-economy-flights-to-cut-airfares</t>
+        </is>
+      </c>
+    </row>
+    <row r="2286">
+      <c r="A2286" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2286" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2286" t="inlineStr">
+        <is>
+          <t>Lawmaker demands full probe into Yogyakarta daycare abuse scandal</t>
+        </is>
+      </c>
+      <c r="D2286" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413652/lawmaker-demands-full-probe-into-yogyakarta-daycare-abuse-scandal</t>
+        </is>
+      </c>
+    </row>
+    <row r="2287">
+      <c r="A2287" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2287" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C2287" t="inlineStr">
+        <is>
+          <t>Minister urges graduates to safeguard digital space</t>
+        </is>
+      </c>
+      <c r="D2287" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413648/minister-urges-graduates-to-safeguard-digital-space</t>
+        </is>
+      </c>
+    </row>
+    <row r="2288">
+      <c r="A2288" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2288" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2288" t="inlineStr">
+        <is>
+          <t>UGM expert backs internship program for job seekers</t>
+        </is>
+      </c>
+      <c r="D2288" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413644/ugm-expert-backs-internship-program-for-job-seekers</t>
+        </is>
+      </c>
+    </row>
+    <row r="2289">
+      <c r="A2289" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2289" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C2289" t="inlineStr">
+        <is>
+          <t>Indonesia sees $1 mln potential in Japan pop-up store</t>
+        </is>
+      </c>
+      <c r="D2289" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413640/indonesia-sees-1-mln-potential-in-japan-pop-up-store</t>
+        </is>
+      </c>
+    </row>
+    <row r="2290">
+      <c r="A2290" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2290" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2290" t="inlineStr">
+        <is>
+          <t>Indonesia presses UN to probe peacekeeper killing in Lebanon</t>
+        </is>
+      </c>
+      <c r="D2290" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413637/indonesia-presses-un-to-probe-peacekeeper-killing-in-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2291">
+      <c r="A2291" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2291" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C2291" t="inlineStr">
+        <is>
+          <t>Indonesia positions fishing village program to boost blue economy</t>
+        </is>
+      </c>
+      <c r="D2291" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413635/indonesia-positions-fishing-village-program-to-boost-blue-economy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2292">
+      <c r="A2292" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2292" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C2292" t="inlineStr">
+        <is>
+          <t>Indonesia eyes global market with custom automotive industry push</t>
+        </is>
+      </c>
+      <c r="D2292" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413633/indonesia-eyes-global-market-with-custom-automotive-industry-push</t>
+        </is>
+      </c>
+    </row>
+    <row r="2293">
+      <c r="A2293" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2293" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2293" t="inlineStr">
+        <is>
+          <t>Inside the Baduy’s 200 km sacred journey through the night</t>
+        </is>
+      </c>
+      <c r="D2293" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413629/inside-the-baduys-200-km-sacred-journey-through-the-night</t>
+        </is>
+      </c>
+    </row>
+    <row r="2294">
+      <c r="A2294" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2294" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C2294" t="inlineStr">
+        <is>
+          <t>MPR Deputy Speaker urges govt to boost public trust in vaccinations</t>
+        </is>
+      </c>
+      <c r="D2294" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413628/mpr-deputy-speaker-urges-govt-to-boost-public-trust-in-vaccinations</t>
+        </is>
+      </c>
+    </row>
+    <row r="2295">
+      <c r="A2295" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2295" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C2295" t="inlineStr">
+        <is>
+          <t>Banten waives electric vehicle tax to support clean energy</t>
+        </is>
+      </c>
+      <c r="D2295" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413624/banten-waives-electric-vehicle-tax-to-support-clean-energy</t>
+        </is>
+      </c>
+    </row>
+    <row r="2296">
+      <c r="A2296" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2296" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2296" t="inlineStr">
+        <is>
+          <t>RI govt speeds up housing program for Senen rail-side community</t>
+        </is>
+      </c>
+      <c r="D2296" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413620/ri-govt-speeds-up-housing-program-for-senen-rail-side-community</t>
+        </is>
+      </c>
+    </row>
+    <row r="2297">
+      <c r="A2297" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2297" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2297" t="inlineStr">
+        <is>
+          <t>Gov't striving to expand education access to reduce dropout rates</t>
+        </is>
+      </c>
+      <c r="D2297" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413619/govt-striving-to-expand-education-access-to-reduce-dropout-rates</t>
+        </is>
+      </c>
+    </row>
+    <row r="2298">
+      <c r="A2298" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2298" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2298" t="inlineStr">
+        <is>
+          <t>Indonesia to continue school revamp, digital push in 2026</t>
+        </is>
+      </c>
+      <c r="D2298" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413617/indonesia-to-continue-school-revamp-digital-push-in-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2299">
+      <c r="A2299" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2299" t="inlineStr">
+        <is>
+          <t>Environment</t>
+        </is>
+      </c>
+      <c r="C2299" t="inlineStr">
+        <is>
+          <t>Forestry Ministry to periodically evaluate Komodo National Park quota</t>
+        </is>
+      </c>
+      <c r="D2299" s="2" t="inlineStr">
+        <is>
+          <t>https://en.antaranews.com/news/413613/forestry-ministry-to-periodically-evaluate-komodo-national-park-quota</t>
+        </is>
+      </c>
+    </row>
+    <row r="2300">
+      <c r="A2300" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2300" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2300" t="inlineStr">
+        <is>
+          <t>Sultan Oman, Menlu Iran bahas upaya mediasi dalam konflik regional</t>
+        </is>
+      </c>
+      <c r="D2300" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5543111/sultan-oman-menlu-iran-bahas-upaya-mediasi-dalam-konflik-regional</t>
+        </is>
+      </c>
+    </row>
+    <row r="2301">
+      <c r="A2301" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2301" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2301" t="inlineStr">
+        <is>
+          <t>Ulama Lebak serukan damai Timur Tengah permanen</t>
+        </is>
+      </c>
+      <c r="D2301" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5543055/ulama-lebak-serukan-damai-timur-tengah-permanen</t>
+        </is>
+      </c>
+    </row>
+    <row r="2302">
+      <c r="A2302" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2302" t="inlineStr">
+        <is>
+          <t>Disaster/Emergency</t>
+        </is>
+      </c>
+      <c r="C2302" t="inlineStr">
+        <is>
+          <t>Kebakaran hutan di Jepang terus meluas, 3.000 orang dievakuasi</t>
+        </is>
+      </c>
+      <c r="D2302" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5543033/kebakaran-hutan-di-jepang-terus-meluas-3000-orang-dievakuasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2303">
+      <c r="A2303" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2303" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2303" t="inlineStr">
+        <is>
+          <t>Pelaku penembakan di acara Trump mengaku incar pejabat AS</t>
+        </is>
+      </c>
+      <c r="D2303" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5543003/pelaku-penembakan-di-acara-trump-mengaku-incar-pejabat-as</t>
+        </is>
+      </c>
+    </row>
+    <row r="2304">
+      <c r="A2304" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2304" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2304" t="inlineStr">
+        <is>
+          <t>Penembakan di acara Trump terjadi di hotel tempat Reagan dulu ditembak</t>
+        </is>
+      </c>
+      <c r="D2304" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542967/penembakan-di-acara-trump-terjadi-di-hotel-tempat-reagan-dulu-ditembak</t>
+        </is>
+      </c>
+    </row>
+    <row r="2305">
+      <c r="A2305" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2305" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2305" t="inlineStr">
+        <is>
+          <t>AS bakal tolak kartu hijau pemohon pro-Palestina, pengkritik Israel</t>
+        </is>
+      </c>
+      <c r="D2305" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542941/as-bakal-tolak-kartu-hijau-pemohon-pro-palestina-pengkritik-israel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2306">
+      <c r="A2306" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2306" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2306" t="inlineStr">
+        <is>
+          <t>Polisi: Pelaku penembakan di acara Trump bersenjata senapan gentel</t>
+        </is>
+      </c>
+      <c r="D2306" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542928/polisi-pelaku-penembakan-di-acara-trump-bersenjata-senapan-gentel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2307">
+      <c r="A2307" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2307" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2307" t="inlineStr">
+        <is>
+          <t>Qatar sampaikan belasungkawa atas gugurnya anggota TNI di Lebanon</t>
+        </is>
+      </c>
+      <c r="D2307" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542780/qatar-sampaikan-belasungkawa-atas-gugurnya-anggota-tni-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2308">
+      <c r="A2308" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2308" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2308" t="inlineStr">
+        <is>
+          <t>Trump: Petugas tertembak dalam insiden jamuan makan, pelaku ditahan</t>
+        </is>
+      </c>
+      <c r="D2308" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542761/trump-petugas-tertembak-dalam-insiden-jamuan-makan-pelaku-ditahan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2309">
+      <c r="A2309" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2309" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2309" t="inlineStr">
+        <is>
+          <t>Pernyataan jubir Gedung Putih viral usai penembakan di acara wartawan</t>
+        </is>
+      </c>
+      <c r="D2309" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542740/pernyataan-jubir-gedung-putih-viral-usai-penembakan-di-acara-wartawan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2310">
+      <c r="A2310" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2310" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2310" t="inlineStr">
+        <is>
+          <t>Trump: Satu orang ditangkap usai penembakan di jamuan makan</t>
+        </is>
+      </c>
+      <c r="D2310" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542712/trump-satu-orang-ditangkap-usai-penembakan-di-jamuan-makan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2311">
+      <c r="A2311" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2311" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2311" t="inlineStr">
+        <is>
+          <t>Trump dievakuasi dari acara Gedung Putih karena insiden keamanan</t>
+        </is>
+      </c>
+      <c r="D2311" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542708/trump-dievakuasi-dari-acara-gedung-putih-karena-insiden-keamanan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2312">
+      <c r="A2312" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2312" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2312" t="inlineStr">
+        <is>
+          <t>Pezeshkian: Iran takkan berunding di bawah ancaman, blokade</t>
+        </is>
+      </c>
+      <c r="D2312" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542700/pezeshkian-iran-takkan-berunding-di-bawah-ancaman-blokade</t>
+        </is>
+      </c>
+    </row>
+    <row r="2313">
+      <c r="A2313" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2313" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2313" t="inlineStr">
+        <is>
+          <t>Trump: AS terima usulan baru dari Iran usai batalkan misi ke Pakistan</t>
+        </is>
+      </c>
+      <c r="D2313" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542693/trump-as-terima-usulan-baru-dari-iran-usai-batalkan-misi-ke-pakistan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2314">
+      <c r="A2314" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2314" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="C2314" t="inlineStr">
+        <is>
+          <t>Perayaan Hari Antariksa China tampilkan teknologi luar angkasa</t>
+        </is>
+      </c>
+      <c r="D2314" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542689/perayaan-hari-antariksa-china-tampilkan-teknologi-luar-angkasa</t>
+        </is>
+      </c>
+    </row>
+    <row r="2315">
+      <c r="A2315" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2315" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2315" t="inlineStr">
+        <is>
+          <t>Batalkan misi utusan ke Pakistan, Trump sebut AS "punya semua kartu"</t>
+        </is>
+      </c>
+      <c r="D2315" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542680/batalkan-misi-utusan-ke-pakistan-trump-sebut-as-punya-semua-kartu</t>
+        </is>
+      </c>
+    </row>
+    <row r="2316">
+      <c r="A2316" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2316" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2316" t="inlineStr">
+        <is>
+          <t>Menlu Iran dan PM Pakistan gelar pertemuan bahas solusi perang</t>
+        </is>
+      </c>
+      <c r="D2316" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/video/5542493/menlu-iran-dan-pm-pakistan-gelar-pertemuan-bahas-solusi-perang</t>
+        </is>
+      </c>
+    </row>
+    <row r="2317">
+      <c r="A2317" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2317" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+      <c r="C2317" t="inlineStr">
+        <is>
+          <t>WHO: Perbaikan sistem kesehatan di Gaza butuh Rp172 triliun</t>
+        </is>
+      </c>
+      <c r="D2317" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542479/who-perbaikan-sistem-kesehatan-di-gaza-butuh-rp172-triliun</t>
+        </is>
+      </c>
+    </row>
+    <row r="2318">
+      <c r="A2318" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2318" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2318" t="inlineStr">
+        <is>
+          <t>Jerman siapkan armada ke Mediterania untuk misi di Selat Hormuz</t>
+        </is>
+      </c>
+      <c r="D2318" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542445/jerman-siapkan-armada-ke-mediterania-untuk-misi-di-selat-hormuz</t>
+        </is>
+      </c>
+    </row>
+    <row r="2319">
+      <c r="A2319" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2319" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2319" t="inlineStr">
+        <is>
+          <t>Sekjen PBB sambut baik perpanjangan gencatan senjata Lebanon-Israel</t>
+        </is>
+      </c>
+      <c r="D2319" s="2" t="inlineStr">
+        <is>
+          <t>https://www.antaranews.com/berita/5542383/sekjen-pbb-sambut-baik-perpanjangan-gencatan-senjata-lebanon-israel</t>
+        </is>
+      </c>
+    </row>
+    <row r="2320">
+      <c r="A2320" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2320" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C2320" t="inlineStr">
+        <is>
+          <t>1000 Lebih Atlet Akuatik Setanah Air Ambil Bagian dalam Kejurnas Akuatik Indonesia 2026</t>
+        </is>
+      </c>
+      <c r="D2320" s="2" t="inlineStr">
+        <is>
+          <t>https://news.republika.co.id/berita/te3nnb456/1000-lebih-atlet-akuatik-setanah-air-ambil-bagian-dalam-kejurnas-akuatik-indonesia-2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2321">
+      <c r="A2321" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2321" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C2321" t="inlineStr">
+        <is>
+          <t>Start dari Urutan 17, Veda Ega Pratama Melesat dan Berhasil Finish Keenam di Moto 3 Spanyol</t>
+        </is>
+      </c>
+      <c r="D2321" s="2" t="inlineStr">
+        <is>
+          <t>https://news.republika.co.id/berita/te3n73409/start-dari-urutan-17-veda-ega-pratama-melesat-dan-berhasil-finish-keenam-di-moto-3-spanyol</t>
+        </is>
+      </c>
+    </row>
+    <row r="2322">
+      <c r="A2322" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2322" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2322" t="inlineStr">
+        <is>
+          <t>Tangis Haru Iringi Keberangkatan 441 Calon Jamaah Haji Asal Cimahi</t>
+        </is>
+      </c>
+      <c r="D2322" s="2" t="inlineStr">
+        <is>
+          <t>https://khazanah.republika.co.id/berita/te3lvi366/tangis-haru-iringi-keberangkatan-441-calon-jamaah-haji-asal-cimahi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2323">
+      <c r="A2323" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2323" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C2323" t="inlineStr">
+        <is>
+          <t>Talenta Digital Sumbang Rp6,5 Triliun, Jadi Mesin Ekonomi Baru</t>
+        </is>
+      </c>
+      <c r="D2323" s="2" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/te3mfu522/talenta-digital-sumbang-rp65-triliun-jadi-mesin-ekonomi-baru</t>
+        </is>
+      </c>
+    </row>
+    <row r="2324">
+      <c r="A2324" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2324" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C2324" t="inlineStr">
+        <is>
+          <t>Ketidakpastian Global Meningkat, B57+ Dorong Ekonomi Syariah Lintas Negara</t>
+        </is>
+      </c>
+      <c r="D2324" s="2" t="inlineStr">
+        <is>
+          <t>https://sharia.republika.co.id/berita/te3mcr522/ketidakpastian-global-meningkat-b57-dorong-ekonomi-syariah-lintas-negara</t>
+        </is>
+      </c>
+    </row>
+    <row r="2325">
+      <c r="A2325" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2325" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C2325" t="inlineStr">
+        <is>
+          <t>Emas Jadi Pilihan, Pembiayaan Syariah Ikut Tumbuh di Tengah Ketidakpastian Global</t>
+        </is>
+      </c>
+      <c r="D2325" s="2" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/te3m9c522/emas-jadi-pilihan-pembiayaan-syariah-ikut-tumbuh-di-tengah-ketidakpastian-global</t>
+        </is>
+      </c>
+    </row>
+    <row r="2326">
+      <c r="A2326" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2326" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2326" t="inlineStr">
+        <is>
+          <t>PPIH Siapkan 6.000 Bus Modern untuk Layani Jamaah Haji Indonesia</t>
+        </is>
+      </c>
+      <c r="D2326" s="2" t="inlineStr">
+        <is>
+          <t>https://khazanah.republika.co.id/berita/te3kkb366/ppih-siapkan-6000-bus-modern-untuk-layani-jamaah-haji-indonesia</t>
+        </is>
+      </c>
+    </row>
+    <row r="2327">
+      <c r="A2327" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2327" t="inlineStr">
+        <is>
+          <t>Entertainment</t>
+        </is>
+      </c>
+      <c r="C2327" t="inlineStr">
+        <is>
+          <t>Aksi Dalang Cilik Memainkan Wayang Golek Berlakon Somantri Duta</t>
+        </is>
+      </c>
+      <c r="D2327" s="2" t="inlineStr">
+        <is>
+          <t>https://visual.republika.co.id/berita/te3j7l375/aksi-dalang-cilik-memainkan-wayang-golek-berlakon-somantri-duta</t>
+        </is>
+      </c>
+    </row>
+    <row r="2328">
+      <c r="A2328" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2328" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C2328" t="inlineStr">
+        <is>
+          <t>Bos IEA Ungkap Perang Iran Bikin Dunia Makin Tinggalkan Minyak, Percepat Adopsi Nukir dan EBT</t>
+        </is>
+      </c>
+      <c r="D2328" s="2" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/te3lie490/bos-iea-ungkap-perang-iran-bikin-dunia-makin-tinggalkan-minyak-percepat-adopsi-nukir-dan-ebt</t>
+        </is>
+      </c>
+    </row>
+    <row r="2329">
+      <c r="A2329" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2329" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2329" t="inlineStr">
+        <is>
+          <t>Jumlah Tentara Zionis yang Bunuh Diri Terus Melonjak</t>
+        </is>
+      </c>
+      <c r="D2329" s="2" t="inlineStr">
+        <is>
+          <t>https://news.republika.co.id/berita/te3lc4393/jumlah-tentara-zionis-yang-bunuh-diri-terus-melonjak</t>
+        </is>
+      </c>
+    </row>
+    <row r="2330">
+      <c r="A2330" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2330" t="inlineStr">
+        <is>
+          <t>Business</t>
+        </is>
+      </c>
+      <c r="C2330" t="inlineStr">
+        <is>
+          <t>BNI Tegaskan Koperasi Swadharma Bukan Bagian dari Bank</t>
+        </is>
+      </c>
+      <c r="D2330" s="2" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/te3ky7472/bni-tegaskan-koperasi-swadharma-bukan-bagian-dari-bank</t>
+        </is>
+      </c>
+    </row>
+    <row r="2331">
+      <c r="A2331" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2331" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2331" t="inlineStr">
+        <is>
+          <t>KPAI: Sejumlah Daycare Hanya Berorientasi Bisnis, Pengawasan Harus Diperketat</t>
+        </is>
+      </c>
+      <c r="D2331" s="2" t="inlineStr">
+        <is>
+          <t>https://news.republika.co.id/berita/te3knh409/kpai-sejumlah-daycare-hanya-berorientasi-bisnis-pengawasan-harus-diperketat</t>
+        </is>
+      </c>
+    </row>
+    <row r="2332">
+      <c r="A2332" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2332" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2332" t="inlineStr">
+        <is>
+          <t>Trump Nyungsep saat Dievakuasi</t>
+        </is>
+      </c>
+      <c r="D2332" s="2" t="inlineStr">
+        <is>
+          <t>https://republika.co.id/page/shorts/yt-te3kj2771429142/trump-nyungsep-saat-dievakuasi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2333">
+      <c r="A2333" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2333" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C2333" t="inlineStr">
+        <is>
+          <t>Ketika Purbaya Lawan 'Suara Berisik' yang Sebut Ekonomi Indonesia Tidak Baik-Baik Saja</t>
+        </is>
+      </c>
+      <c r="D2333" s="2" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/te3kba490/ketika-purbaya-lawan-suara-berisik-yang-sebut-ekonomi-indonesia-tidak-baikbaik-saja</t>
+        </is>
+      </c>
+    </row>
+    <row r="2334">
+      <c r="A2334" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2334" t="inlineStr">
+        <is>
+          <t>Energy</t>
+        </is>
+      </c>
+      <c r="C2334" t="inlineStr">
+        <is>
+          <t>PLN Teken PJBTL Terbesar untuk Data Center di Indonesia, Siap Pasok Listrik 511 MVA ke DayOne</t>
+        </is>
+      </c>
+      <c r="D2334" s="2" t="inlineStr">
+        <is>
+          <t>https://ekonomi.republika.co.id/berita/te3jmp472/pln-teken-pjbtl-terbesar-untuk-data-center-di-indonesia-siap-pasok-listrik-511-mva-ke-dayone</t>
+        </is>
+      </c>
+    </row>
+    <row r="2335">
+      <c r="A2335" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2335" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2335" t="inlineStr">
+        <is>
+          <t>Praka Rico Gugur di Lebanon, Legislator Tekankan Perlindungan Prajurit TNI
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2335" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/18334081/praka-rico-gugur-di-lebanon-legislator-tekankan-perlindungan-prajurit-tni</t>
+        </is>
+      </c>
+    </row>
+    <row r="2336">
+      <c r="A2336" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2336" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2336" t="inlineStr">
+        <is>
+          <t>BNPP RI Gelar Kuliah Umum di NTT, Ajak Mahasiswa Bangun Masa Depan Kawasan Perbatasan
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2336" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/17583601/bnpp-ri-gelar-kuliah-umum-di-ntt-ajak-mahasiswa-bangun-masa-depan-kawasan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2337">
+      <c r="A2337" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2337" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2337" t="inlineStr">
+        <is>
+          <t>KPK Bakal Panggil 2 Tersangka Baru Kasus Kuota Haji
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2337" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/17552251/kpk-bakal-panggil-2-tersangka-baru-kasus-kuota-haji</t>
+        </is>
+      </c>
+    </row>
+    <row r="2338">
+      <c r="A2338" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2338" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2338" t="inlineStr">
+        <is>
+          <t>Dari Rumah hingga Ruang Digital, Ketua TP PKK Soroti Pentingnya Rasa Aman bagi Perempuan 
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2338" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/17510881/dari-rumah-hingga-ruang-digital-ketua-tp-pkk-soroti-pentingnya-rasa-aman</t>
+        </is>
+      </c>
+    </row>
+    <row r="2339">
+      <c r="A2339" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2339" t="inlineStr">
+        <is>
+          <t>Economy</t>
+        </is>
+      </c>
+      <c r="C2339" t="inlineStr">
+        <is>
+          <t>Rupiah Sentuh Rp 17.300, Anggota DPR Dorong Penguatan Investor Domestik
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2339" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/17380101/rupiah-sentuh-rp-17300-anggota-dpr-dorong-penguatan-investor-domestik</t>
+        </is>
+      </c>
+    </row>
+    <row r="2340">
+      <c r="A2340" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2340" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2340" t="inlineStr">
+        <is>
+          <t>PAN Setuju Pembatasan Uang Tunai di Pemilu, Dorong Revisi Aturan
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2340" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/17082931/pan-setuju-pembatasan-uang-tunai-di-pemilu-dorong-revisi-aturan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2341">
+      <c r="A2341" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2341" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2341" t="inlineStr">
+        <is>
+          <t>Kekerasan di Daycare Yogyakarta, KPAI: Korban Harus Dapat Pendampingan Psikososial
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2341" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/16300101/kekerasan-di-daycare-yogyakarta-kpai-korban-harus-dapat-pendampingan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2342">
+      <c r="A2342" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2342" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2342" t="inlineStr">
+        <is>
+          <t>Pemprov Kalteng Raih Penghargaan Bidang Pendidikan Ajang "National Governance Awards 2026"
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2342" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/16214611/pemprov-kalteng-raih-penghargaan-bidang-pendidikan-ajang-national-governance</t>
+        </is>
+      </c>
+    </row>
+    <row r="2343">
+      <c r="A2343" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2343" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2343" t="inlineStr">
+        <is>
+          <t>KemenPPPA Turunkan Tim Pendampingan Korban Kasus Kekerasan Anak Daycare Little Aresha
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2343" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/14353231/kemenpppa-turunkan-tim-pendampingan-korban-kasus-kekerasan-anak-daycare</t>
+        </is>
+      </c>
+    </row>
+    <row r="2344">
+      <c r="A2344" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2344" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2344" t="inlineStr">
+        <is>
+          <t>Anggota DPR Minta Kasus Kekerasan Anak Daycare Little Aresha Diusut Tuntas
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2344" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/14145611/anggota-dpr-minta-kasus-kekerasan-anak-daycare-little-aresha-diusut-tuntas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2345">
+      <c r="A2345" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2345" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2345" t="inlineStr">
+        <is>
+          <t>Mensos Tegaskan Bansos Tak Dipotong, Tetap Disalurkan Penuh ke Penerima
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2345" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/13323891/mensos-tegaskan-bansos-tak-dipotong-tetap-disalurkan-penuh-ke-penerima</t>
+        </is>
+      </c>
+    </row>
+    <row r="2346">
+      <c r="A2346" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2346" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2346" t="inlineStr">
+        <is>
+          <t>Mendagri Tito Pacu Daerah Berlomba Tunjukkan Kinerja lewat Apresiasi Daerah Berprestasi 2026
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2346" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/13323881/mendagri-tito-pacu-daerah-berlomba-tunjukkan-kinerja-lewat-apresiasi-daerah</t>
+        </is>
+      </c>
+    </row>
+    <row r="2347">
+      <c r="A2347" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2347" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2347" t="inlineStr">
+        <is>
+          <t>Periksa Bos Travel Haji, KPK Dalami Dugaan Penjualan Kuota Haji dan Keuntungannya
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2347" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/13260261/periksa-bos-travel-haji-kpk-dalami-dugaan-penjualan-kuota-haji-dan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2348">
+      <c r="A2348" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2348" t="inlineStr">
+        <is>
+          <t>Religion</t>
+        </is>
+      </c>
+      <c r="C2348" t="inlineStr">
+        <is>
+          <t>Update Penyelenggaraan Haji, 17.747 Jemaah Indonesia Tiba di Madinah
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2348" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/13030481/update-penyelenggaraan-haji-17747-jemaah-indonesia-tiba-di-madinah</t>
+        </is>
+      </c>
+    </row>
+    <row r="2349">
+      <c r="A2349" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2349" t="inlineStr">
+        <is>
+          <t>Defence/Security</t>
+        </is>
+      </c>
+      <c r="C2349" t="inlineStr">
+        <is>
+          <t>Kedubes Qatar Sampaikan Belasungkawa Gugurnya Praka Rico di Lebanon
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2349" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/12185471/kedubes-qatar-sampaikan-belasungkawa-gugurnya-praka-rico-di-lebanon</t>
+        </is>
+      </c>
+    </row>
+    <row r="2350">
+      <c r="A2350" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2350" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2350" t="inlineStr">
+        <is>
+          <t>Ganjar Dorong Politik Uang Dihukum Berat, Bisa Diskualifikasi hingga Sanksi Pidana
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2350" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/12064861/ganjar-dorong-politik-uang-dihukum-berat-bisa-diskualifikasi-hingga-sanksi</t>
+        </is>
+      </c>
+    </row>
+    <row r="2351">
+      <c r="A2351" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2351" t="inlineStr">
+        <is>
+          <t>Education</t>
+        </is>
+      </c>
+      <c r="C2351" t="inlineStr">
+        <is>
+          <t>PP TUNAS dan Pelajaran Sebulan Pertama: Menguji Komitmen dan Realitas
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2351" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/12010031/pp-tunas-dan-pelajaran-sebulan-pertama--menguji-komitmen-dan-realitas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2352">
+      <c r="A2352" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2352" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2352" t="inlineStr">
+        <is>
+          <t>Kasus Daycare Little Aresha, Legislator: Pelaku Harus Disanksi Tegas
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2352" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/11531361/kasus-daycare-little-aresha-legislator-pelaku-harus-disanksi-tegas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2353">
+      <c r="A2353" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2353" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2353" t="inlineStr">
+        <is>
+          <t>Respons Usulan KPK, Ganjar: Pembatasan Uang Tunai Bukan Solusi Utama Cegah Politik Uang
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2353" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/11315461/respons-usulan-kpk-ganjar-pembatasan-uang-tunai-bukan-solusi-utama-cegah</t>
+        </is>
+      </c>
+    </row>
+    <row r="2354">
+      <c r="A2354" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2354" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2354" t="inlineStr">
+        <is>
+          <t>Apresiasi Daerah Berprestasi 2026 Digelar, Mendagri Dorong Iklim Kompetitif Antardaerah
+Nasional
+26 April 2026</t>
+        </is>
+      </c>
+      <c r="D2354" s="2" t="inlineStr">
+        <is>
+          <t>https://nasional.kompas.com/read/2026/04/26/11223491/apresiasi-daerah-berprestasi-2026-digelar-mendagri-dorong-iklim-kompetitif</t>
+        </is>
+      </c>
+    </row>
+    <row r="2355">
+      <c r="A2355" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2355" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2355" t="inlineStr">
+        <is>
+          <t>1
+Polisi Tetapkan 13 Tersangka Kasus Daycare Jogja, Terungkap Ada Kamar Sempit Diisi Puluhan Bayi
+Yogyakarta</t>
+        </is>
+      </c>
+      <c r="D2355" s="2" t="inlineStr">
+        <is>
+          <t>https://yogyakarta.kompas.com/read/2026/04/26/064949578/polisi-tetapkan-13-tersangka-kasus-daycare-jogja-terungkap-ada-kamar</t>
+        </is>
+      </c>
+    </row>
+    <row r="2356">
+      <c r="A2356" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2356" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2356" t="inlineStr">
+        <is>
+          <t>2
+Trump Dievakuasi Usai Terdengar Tembakan di Jamuan Makan Gedung Putih
+Internasional</t>
+        </is>
+      </c>
+      <c r="D2356" s="2" t="inlineStr">
+        <is>
+          <t>https://internasional.kompas.com/read/2026/04/26/082440070/trump-dievakuasi-usai-terdengar-tembakan-di-jamuan-makan-gedung-putih</t>
+        </is>
+      </c>
+    </row>
+    <row r="2357">
+      <c r="A2357" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2357" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2357" t="inlineStr">
+        <is>
+          <t>3
+Oknum Penghulu KUA Bekasi Utara Sudah Diperiksa dan Disanksi Usai Tarik Pungli
+Megapolitan</t>
+        </is>
+      </c>
+      <c r="D2357" s="2" t="inlineStr">
+        <is>
+          <t>https://megapolitan.kompas.com/read/2026/04/25/22172811/oknum-penghulu-kua-bekasi-utara-sudah-diperiksa-dan-disanksi-usai-tarik</t>
+        </is>
+      </c>
+    </row>
+    <row r="2358">
+      <c r="A2358" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2358" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2358" t="inlineStr">
+        <is>
+          <t>4
+AS Batal Kirim Utusan ke Pakistan, Iran Langsung Aktifkan Pertahanan Udara
+Internasional</t>
+        </is>
+      </c>
+      <c r="D2358" s="2" t="inlineStr">
+        <is>
+          <t>https://internasional.kompas.com/read/2026/04/26/073614170/as-batal-kirim-utusan-ke-pakistan-iran-langsung-aktifkan-pertahanan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2359">
+      <c r="A2359" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2359" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2359" t="inlineStr">
+        <is>
+          <t>5
+Di Balik Terbongkarnya Kasus Daycare di Jogja, Ada Peran Eks Karyawan Ijazahnya Ditahan
+Yogyakarta</t>
+        </is>
+      </c>
+      <c r="D2359" s="2" t="inlineStr">
+        <is>
+          <t>https://yogyakarta.kompas.com/read/2026/04/25/194221878/di-balik-terbongkarnya-kasus-daycare-di-jogja-ada-peran-eks-karyawan</t>
+        </is>
+      </c>
+    </row>
+    <row r="2360">
+      <c r="A2360" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2360" t="inlineStr">
+        <is>
+          <t>Social Affairs</t>
+        </is>
+      </c>
+      <c r="C2360" t="inlineStr">
+        <is>
+          <t>6
+Polisi Ungkap Korban Kekerasan Daycare Little Aresha Jogja Capai 103 Anak, 53 Alami Kekerasan Fisik
+Yogyakarta</t>
+        </is>
+      </c>
+      <c r="D2360" s="2" t="inlineStr">
+        <is>
+          <t>https://yogyakarta.kompas.com/read/2026/04/25/185815178/polisi-ungkap-korban-kekerasan-daycare-little-aresha-jogja-capai-103-anak</t>
+        </is>
+      </c>
+    </row>
+    <row r="2361">
+      <c r="A2361" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2361" t="inlineStr">
+        <is>
+          <t>Sports</t>
+        </is>
+      </c>
+      <c r="C2361" t="inlineStr">
+        <is>
+          <t>7
+Bonus Rp 5 Miliar untuk Persib Jadi Polemik, Dedi Mulyadi Buka Suara: Saya Junjung Transparansi
+Bandung</t>
+        </is>
+      </c>
+      <c r="D2361" s="2" t="inlineStr">
+        <is>
+          <t>https://bandung.kompas.com/read/2026/04/26/100540478/bonus-rp-5-miliar-untuk-persib-jadi-polemik-dedi-mulyadi-buka-suara-saya</t>
+        </is>
+      </c>
+    </row>
+    <row r="2362">
+      <c r="A2362" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2362" t="inlineStr">
+        <is>
+          <t>Legal/Judiciary</t>
+        </is>
+      </c>
+      <c r="C2362" t="inlineStr">
+        <is>
+          <t>8
+Usai OTT KPK, SK Kepala Sekolah di Tulungagung Ditunda
+Surabaya</t>
+        </is>
+      </c>
+      <c r="D2362" s="2" t="inlineStr">
+        <is>
+          <t>https://surabaya.kompas.com/read/2026/04/25/185802278/usai-ott-kpk-sk-kepala-sekolah-di-tulungagung-ditunda</t>
+        </is>
+      </c>
+    </row>
+    <row r="2363">
+      <c r="A2363" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2363" t="inlineStr">
+        <is>
+          <t>Foreign Affairs</t>
+        </is>
+      </c>
+      <c r="C2363" t="inlineStr">
+        <is>
+          <t>9
+Trump Buka Suara soal Insiden Penembakan di Jamuan Makan Gedung Putih
+Internasional</t>
+        </is>
+      </c>
+      <c r="D2363" s="2" t="inlineStr">
+        <is>
+          <t>https://internasional.kompas.com/read/2026/04/26/101705870/trump-buka-suara-soal-insiden-penembakan-di-jamuan-makan-gedung-putih</t>
+        </is>
+      </c>
+    </row>
+    <row r="2364">
+      <c r="A2364" t="inlineStr">
+        <is>
+          <t>Sunday, 26 April 2026</t>
+        </is>
+      </c>
+      <c r="B2364" t="inlineStr">
+        <is>
+          <t>Politics</t>
+        </is>
+      </c>
+      <c r="C2364" t="inlineStr">
+        <is>
+          <t>10
+Tanggapi Santai, Dedi Mulyadi Ucapkan Terima Kasih atas Spanduk "Shut Up KDM" di GBLA
+Bandung</t>
+        </is>
+      </c>
+      <c r="D2364" s="2" t="inlineStr">
+        <is>
+          <t>https://bandung.kompas.com/read/2026/04/26/080358378/tanggapi-santai-dedi-mulyadi-ucapkan-terima-kasih-atas-spanduk-shut-up-kdm</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D2239"/>
+  <autoFilter ref="A1:D2364"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D3" r:id="rId2"/>
@@ -51947,6 +54757,131 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2237" r:id="rId2236"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2238" r:id="rId2237"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2239" r:id="rId2238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2240" r:id="rId2239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2241" r:id="rId2240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2242" r:id="rId2241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2243" r:id="rId2242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2244" r:id="rId2243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2245" r:id="rId2244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2246" r:id="rId2245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2247" r:id="rId2246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2248" r:id="rId2247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2249" r:id="rId2248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2250" r:id="rId2249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2251" r:id="rId2250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2252" r:id="rId2251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2253" r:id="rId2252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2254" r:id="rId2253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2255" r:id="rId2254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2256" r:id="rId2255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2257" r:id="rId2256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2258" r:id="rId2257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2259" r:id="rId2258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2260" r:id="rId2259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2261" r:id="rId2260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2262" r:id="rId2261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2263" r:id="rId2262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2264" r:id="rId2263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2265" r:id="rId2264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2266" r:id="rId2265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2267" r:id="rId2266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2268" r:id="rId2267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2269" r:id="rId2268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2270" r:id="rId2269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2271" r:id="rId2270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2272" r:id="rId2271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2273" r:id="rId2272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2274" r:id="rId2273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2275" r:id="rId2274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2276" r:id="rId2275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2277" r:id="rId2276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2278" r:id="rId2277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2279" r:id="rId2278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2280" r:id="rId2279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2281" r:id="rId2280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2282" r:id="rId2281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2283" r:id="rId2282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2284" r:id="rId2283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2285" r:id="rId2284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2286" r:id="rId2285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2287" r:id="rId2286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2288" r:id="rId2287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2289" r:id="rId2288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2290" r:id="rId2289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2291" r:id="rId2290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2292" r:id="rId2291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2293" r:id="rId2292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2294" r:id="rId2293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2295" r:id="rId2294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2296" r:id="rId2295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2297" r:id="rId2296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2298" r:id="rId2297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2299" r:id="rId2298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2300" r:id="rId2299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2301" r:id="rId2300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2302" r:id="rId2301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2303" r:id="rId2302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2304" r:id="rId2303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2305" r:id="rId2304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2306" r:id="rId2305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2307" r:id="rId2306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2308" r:id="rId2307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2309" r:id="rId2308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2310" r:id="rId2309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2311" r:id="rId2310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2312" r:id="rId2311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2313" r:id="rId2312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2314" r:id="rId2313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2315" r:id="rId2314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2316" r:id="rId2315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2317" r:id="rId2316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2318" r:id="rId2317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2319" r:id="rId2318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2320" r:id="rId2319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2321" r:id="rId2320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2322" r:id="rId2321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2323" r:id="rId2322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2324" r:id="rId2323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2325" r:id="rId2324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2326" r:id="rId2325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2327" r:id="rId2326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2328" r:id="rId2327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2329" r:id="rId2328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2330" r:id="rId2329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2331" r:id="rId2330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2332" r:id="rId2331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2333" r:id="rId2332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2334" r:id="rId2333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2335" r:id="rId2334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2336" r:id="rId2335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2337" r:id="rId2336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2338" r:id="rId2337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2339" r:id="rId2338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2340" r:id="rId2339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2341" r:id="rId2340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2342" r:id="rId2341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2343" r:id="rId2342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2344" r:id="rId2343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2345" r:id="rId2344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2346" r:id="rId2345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2347" r:id="rId2346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2348" r:id="rId2347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2349" r:id="rId2348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2350" r:id="rId2349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2351" r:id="rId2350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2352" r:id="rId2351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2353" r:id="rId2352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2354" r:id="rId2353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2355" r:id="rId2354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2356" r:id="rId2355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2357" r:id="rId2356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2358" r:id="rId2357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2359" r:id="rId2358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2360" r:id="rId2359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2361" r:id="rId2360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2362" r:id="rId2361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2363" r:id="rId2362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D2364" r:id="rId2363"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>